<commit_message>
Unit 3 look-over: every spec re-derived and read whole; slide fractions set display-size, warm-up text measured with real font metrics; source citations tightened; reference-sheet table widened
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xYWeLUsuszQH6z7ADE9tj
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -49,7 +49,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">MTR.5.1: Notes II — 3²·3³ is expanded into five factors of 3 before the rule is named, so the law is read off the structure rather than memorised.
+          <t xml:space="preserve">MTR.5.1: Notes II — 3²·3³ is expanded into five factors of 3 before the rule is named, so the law is read off the structure rather than memorized.
 MTR.3.1: Boards 1, 3, 4 and 7 — one law, one move, written and up on the cue; today is where the fluency for the rest of the unit is set.
 MTR.4.1: Board 5 — when the room splits between 4⁵ and 16⁵, the sixty-second re-vote before the reveal.</t>
         </r>
@@ -133,7 +133,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">MTR.5.1: Notes I — x² · x³ is expanded into five letters before the rule is restated, so the law is recognised as the one from 3.01 rather than met as a new one.
+          <t xml:space="preserve">MTR.5.1: Notes I — x² · x³ is expanded into five letters before the rule is restated, so the law is recognized as the one from 3.01 rather than met as a new one.
 MTR.3.1: Boards 1, 2 and 7 — one move each, written and up on the cue; the law has to be automatic before the negative exponents arrive tomorrow.
 MTR.4.1: Board 5 — when the room splits over whether the 5 gets squared, the sixty-second re-vote before the reveal.</t>
         </r>
@@ -5548,7 +5548,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py at commit e6ca325 on 21 September 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py at commit 8b0d7b3 on 27 September 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">https://github.com/croix18/croix18-windy-hill-a7/blob/main/a7/packages/A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation/PDFs/Slides/A7%203.01%20%20Slides.pdf</t>
@@ -6556,7 +6556,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="13">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -6624,6 +6624,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8CBAD"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -6923,7 +6931,7 @@
       </c>
       <c r="B1" s="2" t="n">
         <f aca="true">TODAY()</f>
-        <v>46286</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6932,7 +6940,7 @@
       </c>
       <c r="B3" s="4" t="str">
         <f aca="true">IF($B$42&gt;131,"The school year has ended.",IF(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$42)=TODAY(),"Today's class",IF(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$42)&lt;TODAY(),"The PM3 window (3–28 May)","Next class: "&amp;TEXT(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$42),"dddd d mmmm"))))</f>
-        <v>Next class: Wednesday 23 September</v>
+        <v>Next class: Monday 28 September</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6941,7 +6949,7 @@
       </c>
       <c r="B5" s="6" t="str">
         <f aca="false">IF($B$42&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,$B$42)&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,$B$42))</f>
-        <v>3.01   Product laws of exponents</v>
+        <v>3.04   Negative exponent law</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6950,7 +6958,7 @@
       </c>
       <c r="B6" s="6" t="str">
         <f aca="false">IF($B$42&gt;131,"",INDEX('Scope &amp; Sequence'!$S$2:$S$132,$B$42)&amp;"")</f>
-        <v>I can use the product of powers, power of a product, power of a power and identity laws to rewrite and evaluate a numerical expression.</v>
+        <v>I can rewrite a power with a negative exponent using a positive exponent, and evaluate it.</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6959,16 +6967,16 @@
       </c>
       <c r="B7" s="6" t="str">
         <f aca="false">IF($B$42&gt;131,"",INDEX('Scope &amp; Sequence'!$T$2:$T$132,$B$42)&amp;"")</f>
-        <v>How can the laws of exponents be used to write an equivalent expression?</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>How do you evaluate a numerical expression that has a negative exponent?</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="6" t="str">
         <f aca="false">IF($B$42&gt;131,"",INDEX('Scope &amp; Sequence'!$U$2:$U$132,$B$42)&amp;"")</f>
-        <v>base, exponent, power, product of powers law, power of a product law, power of a power law, identity exponent law</v>
+        <v>negative exponent law, reciprocal, opposite</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6977,7 +6985,7 @@
       </c>
       <c r="B9" s="6" t="str">
         <f aca="false">IF($B$42&gt;131,"",INDEX('Scope &amp; Sequence'!$V$2:$V$132,$B$42)&amp;"")</f>
-        <v>7.NSO.1.1 · 8.NSO.1.3</v>
+        <v>8.NSO.1.3</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6986,7 +6994,7 @@
       </c>
       <c r="B10" s="6" t="str">
         <f aca="false">IF($B$42&gt;131,"",IF(INDEX('Scope &amp; Sequence'!$Q$2:$Q$132,$B$42)&amp;""="","none",INDEX('Scope &amp; Sequence'!$Q$2:$Q$132,$B$42)&amp;"   — due "&amp;TEXT(INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$42),"ddd d mmm")))</f>
-        <v>Evaluate powers — SZQ; Multiplication with exponents — 5SK; Power rule — 8DA; Understanding exponents — BFA   — due Thu 24 Sep</v>
+        <v>Understanding negative exponents — YBB; Evaluate powers with negative exponents — WGS   — due Tue 29 Sep</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6995,7 +7003,7 @@
       </c>
       <c r="B11" s="6" t="str">
         <f aca="false">IF($B$42&gt;131,"",IFERROR(INDEX('IXL tracker'!$D$5:$D$86,MATCH(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$42),'IXL tracker'!$G$5:$G$86,0)),"nothing due"))</f>
-        <v>nothing due</v>
+        <v>Evaluate expressions using properties of exponents (ZE9)</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7004,7 +7012,7 @@
       </c>
       <c r="B12" s="6" t="str">
         <f aca="false">IF($B$42&gt;131,"",INDEX('Scope &amp; Sequence'!$Y$2:$Y$132,$B$42)&amp;"")</f>
-        <v>Aiyanna says she can use the power of a product law to evaluate (10 + (−2))³. Is she right?</v>
+        <v>Ellen says the value of 5⁻² is −25. Explain why she is wrong, and show the correct value.</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7130,11 +7138,11 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="n">
         <f aca="false">IF(($B$42+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$42+1)))</f>
-        <v>46289</v>
+        <v>46294</v>
       </c>
       <c r="B29" s="6" t="str">
         <f aca="false">IF(($B$42+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$42+1))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$42+1)))</f>
-        <v>3.02   Quotient laws of exponents</v>
+        <v>3.05   Applying exponent laws</v>
       </c>
       <c r="C29" s="8" t="str">
         <f aca="false">IF(($B$42+1)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$42+1))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$42+1)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$42+1))&amp;"")))</f>
@@ -7144,11 +7152,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="n">
         <f aca="false">IF(($B$42+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$42+2)))</f>
-        <v>46290</v>
+        <v>46295</v>
       </c>
       <c r="B30" s="6" t="str">
         <f aca="false">IF(($B$42+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$42+2))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$42+2)))</f>
-        <v>3.03   Exponential expressions</v>
+        <v>3.06+07   Evaluating and equivalent expressions with integer exponents</v>
       </c>
       <c r="C30" s="8" t="str">
         <f aca="false">IF(($B$42+2)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$42+2))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$42+2)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$42+2))&amp;"")))</f>
@@ -7158,11 +7166,11 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="n">
         <f aca="false">IF(($B$42+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$42+3)))</f>
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="B31" s="6" t="str">
         <f aca="false">IF(($B$42+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$42+3))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$42+3)))</f>
-        <v>3.04   Negative exponent law</v>
+        <v>T-A1   Thread A: the same laws with variable bases (14.1–14.2)</v>
       </c>
       <c r="C31" s="8" t="str">
         <f aca="false">IF(($B$42+3)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$42+3))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$42+3)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$42+3))&amp;"")))</f>
@@ -7172,11 +7180,11 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="n">
         <f aca="false">IF(($B$42+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$42+4)))</f>
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="B32" s="6" t="str">
         <f aca="false">IF(($B$42+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$42+4))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$42+4)))</f>
-        <v>3.05   Applying exponent laws</v>
+        <v>T-A2   Thread A: negative exponents and multiple laws, variable bases (14.3–14.4)</v>
       </c>
       <c r="C32" s="8" t="str">
         <f aca="false">IF(($B$42+4)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$42+4))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$42+4)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$42+4))&amp;"")))</f>
@@ -7186,11 +7194,11 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
         <f aca="false">IF(($B$42+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$42+5)))</f>
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="B33" s="6" t="str">
         <f aca="false">IF(($B$42+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$42+5))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$42+5)))</f>
-        <v>3.06+07   Evaluating and equivalent expressions with integer exponents</v>
+        <v>3.08   Large numbers in scientific notation</v>
       </c>
       <c r="C33" s="8" t="str">
         <f aca="false">IF(($B$42+5)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$42+5))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$42+5)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$42+5))&amp;"")))</f>
@@ -7210,7 +7218,7 @@
       </c>
       <c r="B42" s="13" t="n">
         <f aca="true">IF(TODAY()&gt;$B$43,131+1,MIN(COUNTIF('Scope &amp; Sequence'!$A$2:$A$132,"&lt;"&amp;TODAY())+1,131))</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17073,7 +17081,7 @@
       <c r="I5" s="50"/>
       <c r="J5" s="7" t="str">
         <f aca="true">IF(I5="✓","done",IF(TODAY()&lt;B5,"upcoming",IF(TODAY()&lt;G5,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>due — check scores</v>
       </c>
       <c r="K5" s="51"/>
     </row>
@@ -17103,7 +17111,7 @@
       <c r="I6" s="50"/>
       <c r="J6" s="7" t="str">
         <f aca="true">IF(I6="✓","done",IF(TODAY()&lt;B6,"upcoming",IF(TODAY()&lt;G6,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>due — check scores</v>
       </c>
       <c r="K6" s="51"/>
     </row>
@@ -17133,7 +17141,7 @@
       <c r="I7" s="50"/>
       <c r="J7" s="7" t="str">
         <f aca="true">IF(I7="✓","done",IF(TODAY()&lt;B7,"upcoming",IF(TODAY()&lt;G7,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>open</v>
       </c>
       <c r="K7" s="51"/>
     </row>
@@ -19513,13 +19521,13 @@
     <mergeCell ref="A2:K2"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J86">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$J5="done"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$J5="due — check scores"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$J5="open"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Master sheet: one-tap Drive links where the Drive index has the document's id
Same change as windy-hill-m7: tools/drive_index.csv (from Windmill drive/) gives each document's
Drive id; linked by id where known, by title search where not; the check resolves every id to its
package file and row. No index committed yet (the script has not run in his account).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xYWeLUsuszQH6z7ADE9tj
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -5548,13 +5548,13 @@
     <t xml:space="preserve">Good to know</t>
   </si>
   <si>
-    <t xml:space="preserve">Links open Google Drive. Drive has no address for a file by its folder and name, so each link is a search for the file's exact name: Drive opens showing that one file, and a tap opens it. It works wherever the file sits in your Drive and keeps working when a rebuilt file replaces it. "No results" means that file is not in your Drive yet (upload the unit's folder, unzipped); two results mean an older copy is still there — open the newer one and delete the other.</t>
+    <t xml:space="preserve">Links open Google Drive. Drive has no address for a file by its folder and name, so each link is a search for the file's exact name: Drive opens showing the one file with that name, and a tap opens it. "No results" means that file is not in your Drive yet (upload the unit's folder, unzipped); two results mean an older copy is still there — open the newer one and delete the other. It works wherever the file sits in your Drive and keeps working when a rebuilt file replaces it.</t>
   </si>
   <si>
     <t xml:space="preserve">If Drive opens in the wrong Google account, switch to the one that holds the Windy Hill folder (the round picture, top right) and tap the link again.</t>
   </si>
   <si>
-    <t xml:space="preserve">A link that reads "in folder" opens the unit's folder, not the file: every unit has a file or folder of that name (START HERE, Lessons, All Slides), so a search by name could not tell them apart.</t>
+    <t xml:space="preserve">A link that reads "in folder" opens the unit's folder, not the file: every unit has a file or folder of that name (START HERE, Lessons, All Slides), and without its address in the index a search by name could not tell them apart.</t>
   </si>
   <si>
     <t xml:space="preserve">'not built yet' means the unit's documents do not exist yet. Units 5 onward fill in as they are built; this file is regenerated from the plan each time.</t>
@@ -5569,7 +5569,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (Google Drive links) at commit c8ea8f5 on 04 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (Google Drive links, no index) at commit 0a27cc4 on 04 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%203.01%20Product%20Laws%20of%20Exponents%20-%20Slides.pdf%22</t>

</xml_diff>

<commit_message>
Master sheet: the notes name his Windy Hill Master Folder (where the script works)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xYWeLUsuszQH6z7ADE9tj
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -5540,16 +5540,16 @@
     <t xml:space="preserve">Good to know</t>
   </si>
   <si>
-    <t xml:space="preserve">Links open Google Drive, and they are live: each one looks the document's address up, in this file's hidden Drive tab, at the moment you open the file. A script in your own Google account refills that tab every hour from what is in your Drive right now, so a document that is replaced, moved or rebuilt is followed by itself — nobody remakes this sheet for that. If you edit a document, save your copy under the same file name in the folder Windy Hill &gt; My versions: the link then opens yours. Anything of your own that you name for a lesson ("A7 3.01 …") turns up under "Everything for this lesson".</t>
+    <t xml:space="preserve">Links open Google Drive, and they are live: each one looks the document's address up, in this file's hidden Drive tab, at the moment you open the file. A script in your own Google account refills that tab every hour from what is in your Drive right now, so a document that is replaced, moved or rebuilt is followed by itself — nobody remakes this sheet for that. If you edit a document, save your copy under the same file name in the folder My versions (inside your Windy Hill Master Folder): the link then opens yours. Anything of your own that you name for a lesson ("A7 3.01 …") turns up under "Everything for this lesson".</t>
   </si>
   <si>
     <t xml:space="preserve">Where your Drive does not hold a document — or before the script has ever run — its link is a search for the file's exact name instead: Drive opens showing that one file, and a tap opens it. "No results" means the file is not in your Drive yet.</t>
   </si>
   <si>
-    <t xml:space="preserve">If Drive opens in the wrong Google account, switch to the one that holds the Windy Hill folder (the round picture, top right) and tap the link again.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A copy of this file that is still an Excel file (.xlsx) has an empty Drive tab, so all of its links are searches. The live copy is the Google Sheet of the same name that the script makes in your Windy Hill folder (the Status tab of the Windy Hill Drive Index links to it).</t>
+    <t xml:space="preserve">If Drive opens in the wrong Google account, switch to one the Windy Hill Master Folder is shared with (the round picture, top right) and tap the link again.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A copy of this file that is still an Excel file (.xlsx) has an empty Drive tab, so all of its links are searches. The live copy is the Google Sheet of the same name that the script makes in your Windy Hill Master Folder (the Status tab of the Windy Hill Drive Index links to it).</t>
   </si>
   <si>
     <t xml:space="preserve">'not built yet' means the unit's documents do not exist yet. Units 5 onward fill in as they are built; this file is regenerated from the plan each time.</t>
@@ -5564,7 +5564,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit f1c1c2a on 04 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit f5174c5 on 04 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -7581,7 +7581,7 @@
         <v>1590</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="69" t="s">
         <v>1591</v>
       </c>

</xml_diff>

<commit_message>
Master sheet: the About tab says what the Drive script (v3) now does with the yellow IXL cells - carried into each new edition of the live sheet, which keeps its address
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xYWeLUsuszQH6z7ADE9tj
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -463,7 +463,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2719" uniqueCount="1838">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2720" uniqueCount="1839">
   <si>
     <t xml:space="preserve">A7 — today</t>
   </si>
@@ -5555,6 +5555,9 @@
     <t xml:space="preserve">'not built yet' means the unit's documents do not exist yet. Units 5 onward fill in as they are built; this file is regenerated from the plan each time.</t>
   </si>
   <si>
+    <t xml:space="preserve">The yellow cells in the IXL tracker are yours. In the live Google Sheet they stay: when a new edition of this sheet is published, the script puts the new contents into the same Google Sheet, so its address and your bookmark stay (should Google ever refuse, it makes a new sheet, and the Status tab of the Windy Hill Drive Index links to it), and it writes your ticks and notes back, lesson by lesson (a copy of them is kept on the Kept tab of the Windy Hill Drive Index). Anything typed anywhere else in this sheet is replaced by the next edition. An Excel copy (.xlsx) carries no ticks.</t>
+  </si>
+  <si>
     <t xml:space="preserve">IXL: every skill listed is required, to a SmartScore of 67, due at the start of the next class (ruling 28). Lessons in a row that use the same skills are one assignment, due after the last of them — the IXL due column already shows that date.</t>
   </si>
   <si>
@@ -5564,7 +5567,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit f5174c5 on 04 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit e16632a on 05 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -7168,7 +7171,7 @@
       </c>
       <c r="B1" s="2" t="n">
         <f aca="true">TODAY()</f>
-        <v>46299</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7177,7 +7180,7 @@
       </c>
       <c r="B3" s="4" t="str">
         <f aca="true">IF($B$44&gt;131,"The school year has ended.",IF(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44)=TODAY(),"Today's class",IF(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44)&lt;TODAY(),"The PM3 window (3–28 May)","Next class: "&amp;TEXT(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),"dddd d mmmm"))))</f>
-        <v>Next class: Monday 5 October</v>
+        <v>Today's class</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7494,7 +7497,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -7596,7 +7599,7 @@
         <v>1593</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="69" t="s">
         <v>1594</v>
       </c>
@@ -7606,17 +7609,22 @@
         <v>1595</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="69"/>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="69" t="s">
+        <v>1596</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="68" t="s">
-        <v>1596</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="69" t="s">
+      <c r="A24" s="69"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="68" t="s">
         <v>1597</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="69" t="s">
+        <v>1598</v>
       </c>
     </row>
   </sheetData>
@@ -7680,13 +7688,13 @@
       </c>
       <c r="N1" s="70"/>
       <c r="O1" s="70" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
       <c r="P1" s="70" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="Q1" s="70" t="s">
-        <v>1600</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7738,14 +7746,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M2" s="70" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="N2" s="70"/>
       <c r="O2" s="70" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="P2" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q2" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k999a58eef73f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22")</f>
@@ -7801,14 +7809,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M3" s="70" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="N3" s="70"/>
       <c r="O3" s="70" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="P3" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q3" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b0883f744a4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22")</f>
@@ -7864,14 +7872,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M4" s="70" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
       <c r="N4" s="70"/>
       <c r="O4" s="70" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="P4" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q4" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4e34d1ba5135",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22")</f>
@@ -7927,14 +7935,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M5" s="70" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="N5" s="70"/>
       <c r="O5" s="70" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
       <c r="P5" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q5" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k654621d73a39",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22")</f>
@@ -7990,14 +7998,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M6" s="70" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="N6" s="70"/>
       <c r="O6" s="70" t="s">
-        <v>1611</v>
+        <v>1612</v>
       </c>
       <c r="P6" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q6" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k05aafdefef87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22")</f>
@@ -8053,14 +8061,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M7" s="70" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="N7" s="70"/>
       <c r="O7" s="70" t="s">
-        <v>1613</v>
+        <v>1614</v>
       </c>
       <c r="P7" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q7" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0fe1632a0900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22")</f>
@@ -8088,10 +8096,10 @@
       <c r="M8" s="70"/>
       <c r="N8" s="70"/>
       <c r="O8" s="70" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
       <c r="P8" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q8" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kadb8b2686141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22")</f>
@@ -8119,10 +8127,10 @@
       <c r="M9" s="70"/>
       <c r="N9" s="70"/>
       <c r="O9" s="70" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="P9" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q9" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4c613b2b0958",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22")</f>
@@ -8178,14 +8186,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M10" s="70" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="N10" s="70"/>
       <c r="O10" s="70" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="P10" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q10" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd60a700332eb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22")</f>
@@ -8241,14 +8249,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M11" s="70" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
       <c r="N11" s="70"/>
       <c r="O11" s="70" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
       <c r="P11" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q11" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k509a716d7468",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22")</f>
@@ -8304,14 +8312,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M12" s="70" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="N12" s="70"/>
       <c r="O12" s="70" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="P12" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q12" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke52ff0df0d4b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22")</f>
@@ -8339,10 +8347,10 @@
       <c r="M13" s="70"/>
       <c r="N13" s="70"/>
       <c r="O13" s="70" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="P13" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q13" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf990f1c33e7d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22")</f>
@@ -8398,14 +8406,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M14" s="70" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="N14" s="70"/>
       <c r="O14" s="70" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="P14" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q14" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb93ffed6ca63",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22")</f>
@@ -8439,10 +8447,10 @@
       <c r="M15" s="70"/>
       <c r="N15" s="70"/>
       <c r="O15" s="70" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="P15" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q15" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k467ef44c3569",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22")</f>
@@ -8476,10 +8484,10 @@
       <c r="M16" s="70"/>
       <c r="N16" s="70"/>
       <c r="O16" s="70" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="P16" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q16" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1f816ed6a0ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22")</f>
@@ -8513,10 +8521,10 @@
       <c r="M17" s="70"/>
       <c r="N17" s="70"/>
       <c r="O17" s="70" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="P17" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q17" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7c17b9b2eea3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test.pdf%22")</f>
@@ -8550,10 +8558,10 @@
       <c r="M18" s="70"/>
       <c r="N18" s="70"/>
       <c r="O18" s="70" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="P18" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q18" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k584fc57b9722",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20-%20Key.pdf%22")</f>
@@ -8609,14 +8617,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M19" s="70" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="N19" s="70"/>
       <c r="O19" s="70" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="P19" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q19" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke57d72cf0716",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22")</f>
@@ -8672,14 +8680,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M20" s="70" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="N20" s="70"/>
       <c r="O20" s="70" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
       <c r="P20" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q20" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dd5b368d2b0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22")</f>
@@ -8735,14 +8743,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M21" s="70" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="N21" s="70"/>
       <c r="O21" s="70" t="s">
-        <v>1634</v>
+        <v>1635</v>
       </c>
       <c r="P21" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q21" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb2536de7152",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22")</f>
@@ -8798,14 +8806,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M22" s="70" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
       <c r="N22" s="70"/>
       <c r="O22" s="70" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="P22" s="70" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="Q22" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2f48d7f422a9",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
@@ -8861,14 +8869,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M23" s="70" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="N23" s="70"/>
       <c r="O23" s="70" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
       <c r="P23" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q23" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8fdeab195866",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
@@ -8924,14 +8932,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M24" s="70" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="N24" s="70"/>
       <c r="O24" s="70" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
       <c r="P24" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q24" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k05aafdefef87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22")</f>
@@ -8965,10 +8973,10 @@
       <c r="M25" s="70"/>
       <c r="N25" s="70"/>
       <c r="O25" s="70" t="s">
-        <v>1642</v>
+        <v>1643</v>
       </c>
       <c r="P25" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q25" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4e34d1ba5135",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22")</f>
@@ -9002,10 +9010,10 @@
       <c r="M26" s="70"/>
       <c r="N26" s="70"/>
       <c r="O26" s="70" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="P26" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q26" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k654621d73a39",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22")</f>
@@ -9039,10 +9047,10 @@
       <c r="M27" s="70"/>
       <c r="N27" s="70"/>
       <c r="O27" s="70" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
       <c r="P27" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q27" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k999a58eef73f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22")</f>
@@ -9076,10 +9084,10 @@
       <c r="M28" s="70"/>
       <c r="N28" s="70"/>
       <c r="O28" s="70" t="s">
-        <v>1645</v>
+        <v>1646</v>
       </c>
       <c r="P28" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q28" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b0883f744a4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22")</f>
@@ -9102,14 +9110,14 @@
       <c r="K29" s="70"/>
       <c r="L29" s="70"/>
       <c r="M29" s="70" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
       <c r="N29" s="70"/>
       <c r="O29" s="70" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
       <c r="P29" s="70" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="Q29" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2ed79628bc59",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
@@ -9132,14 +9140,14 @@
       <c r="K30" s="70"/>
       <c r="L30" s="70"/>
       <c r="M30" s="70" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
       <c r="N30" s="70"/>
       <c r="O30" s="70" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="P30" s="70" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="Q30" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kf1ee50ed8929",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
@@ -9162,14 +9170,14 @@
       <c r="K31" s="70"/>
       <c r="L31" s="70"/>
       <c r="M31" s="70" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="N31" s="70"/>
       <c r="O31" s="70" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="P31" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q31" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k749da75b36af",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
@@ -9192,14 +9200,14 @@
       <c r="K32" s="70"/>
       <c r="L32" s="70"/>
       <c r="M32" s="70" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="N32" s="70"/>
       <c r="O32" s="70" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="P32" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q32" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k509a716d7468",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22")</f>
@@ -9222,14 +9230,14 @@
       <c r="K33" s="70"/>
       <c r="L33" s="70"/>
       <c r="M33" s="70" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="N33" s="70"/>
       <c r="O33" s="70" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="P33" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q33" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4c613b2b0958",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22")</f>
@@ -9252,14 +9260,14 @@
       <c r="K34" s="70"/>
       <c r="L34" s="70"/>
       <c r="M34" s="70" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
       <c r="N34" s="70"/>
       <c r="O34" s="70" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="P34" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q34" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd60a700332eb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22")</f>
@@ -9284,10 +9292,10 @@
       <c r="M35" s="70"/>
       <c r="N35" s="70"/>
       <c r="O35" s="70" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="P35" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q35" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0fe1632a0900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22")</f>
@@ -9312,10 +9320,10 @@
       <c r="M36" s="70"/>
       <c r="N36" s="70"/>
       <c r="O36" s="70" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="P36" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q36" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kadb8b2686141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22")</f>
@@ -9340,10 +9348,10 @@
       <c r="M37" s="70"/>
       <c r="N37" s="70"/>
       <c r="O37" s="70" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
       <c r="P37" s="70" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="Q37" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k986a7bd5b0f8",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
@@ -9366,14 +9374,14 @@
       <c r="K38" s="70"/>
       <c r="L38" s="70"/>
       <c r="M38" s="70" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="N38" s="70"/>
       <c r="O38" s="70" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
       <c r="P38" s="70" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="Q38" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kb8fed8266c53",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
@@ -9396,14 +9404,14 @@
       <c r="K39" s="70"/>
       <c r="L39" s="70"/>
       <c r="M39" s="70" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="N39" s="70"/>
       <c r="O39" s="70" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
       <c r="P39" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q39" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb737ddcb3701",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
@@ -9426,14 +9434,14 @@
       <c r="K40" s="70"/>
       <c r="L40" s="70"/>
       <c r="M40" s="70" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="N40" s="70"/>
       <c r="O40" s="70" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="P40" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q40" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1f816ed6a0ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22")</f>
@@ -9456,14 +9464,14 @@
       <c r="K41" s="70"/>
       <c r="L41" s="70"/>
       <c r="M41" s="70" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="N41" s="70"/>
       <c r="O41" s="70" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="P41" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q41" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb93ffed6ca63",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22")</f>
@@ -9486,14 +9494,14 @@
       <c r="K42" s="70"/>
       <c r="L42" s="70"/>
       <c r="M42" s="70" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
       <c r="N42" s="70"/>
       <c r="O42" s="70" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="P42" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q42" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k467ef44c3569",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22")</f>
@@ -9516,14 +9524,14 @@
       <c r="K43" s="70"/>
       <c r="L43" s="70"/>
       <c r="M43" s="70" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
       <c r="N43" s="70"/>
       <c r="O43" s="70" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="P43" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q43" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke52ff0df0d4b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22")</f>
@@ -9546,14 +9554,14 @@
       <c r="K44" s="70"/>
       <c r="L44" s="70"/>
       <c r="M44" s="70" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
       <c r="N44" s="70"/>
       <c r="O44" s="70" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="P44" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q44" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf990f1c33e7d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22")</f>
@@ -9576,14 +9584,14 @@
       <c r="K45" s="70"/>
       <c r="L45" s="70"/>
       <c r="M45" s="70" t="s">
-        <v>1675</v>
+        <v>1676</v>
       </c>
       <c r="N45" s="70"/>
       <c r="O45" s="70" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="P45" s="70" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="Q45" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k85bc365a5352",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
@@ -9608,10 +9616,10 @@
       <c r="M46" s="70"/>
       <c r="N46" s="70"/>
       <c r="O46" s="70" t="s">
-        <v>1677</v>
+        <v>1678</v>
       </c>
       <c r="P46" s="70" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="Q46" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k19f682b91838",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
@@ -9636,10 +9644,10 @@
       <c r="M47" s="70"/>
       <c r="N47" s="70"/>
       <c r="O47" s="70" t="s">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="P47" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q47" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k44624f8b3141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
@@ -9662,14 +9670,14 @@
       <c r="K48" s="70"/>
       <c r="L48" s="70"/>
       <c r="M48" s="70" t="s">
-        <v>1679</v>
+        <v>1680</v>
       </c>
       <c r="N48" s="70"/>
       <c r="O48" s="70" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="P48" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q48" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb2536de7152",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22")</f>
@@ -9692,14 +9700,14 @@
       <c r="K49" s="70"/>
       <c r="L49" s="70"/>
       <c r="M49" s="70" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="N49" s="70"/>
       <c r="O49" s="70" t="s">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="P49" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q49" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke57d72cf0716",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22")</f>
@@ -9722,14 +9730,14 @@
       <c r="K50" s="70"/>
       <c r="L50" s="70"/>
       <c r="M50" s="70" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="N50" s="70"/>
       <c r="O50" s="70" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="P50" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q50" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dd5b368d2b0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22")</f>
@@ -9752,14 +9760,14 @@
       <c r="K51" s="70"/>
       <c r="L51" s="70"/>
       <c r="M51" s="70" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="N51" s="70"/>
       <c r="O51" s="70" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="P51" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q51" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7c17b9b2eea3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test.pdf%22")</f>
@@ -9782,14 +9790,14 @@
       <c r="K52" s="70"/>
       <c r="L52" s="70"/>
       <c r="M52" s="70" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
       <c r="N52" s="70"/>
       <c r="O52" s="70" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="P52" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q52" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k584fc57b9722",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20-%20Key.pdf%22")</f>
@@ -9814,10 +9822,10 @@
       <c r="M53" s="70"/>
       <c r="N53" s="70"/>
       <c r="O53" s="70" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="P53" s="70" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="Q53" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k395c44aceb1d",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
@@ -9842,10 +9850,10 @@
       <c r="M54" s="70"/>
       <c r="N54" s="70"/>
       <c r="O54" s="70" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="P54" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q54" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf7444edd4950",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22")</f>
@@ -9870,10 +9878,10 @@
       <c r="M55" s="70"/>
       <c r="N55" s="70"/>
       <c r="O55" s="70" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="P55" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q55" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbb6e44272bb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
@@ -9898,10 +9906,10 @@
       <c r="M56" s="70"/>
       <c r="N56" s="70"/>
       <c r="O56" s="70" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="P56" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q56" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc68dd81311bb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22")</f>
@@ -9926,10 +9934,10 @@
       <c r="M57" s="70"/>
       <c r="N57" s="70"/>
       <c r="O57" s="70" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="P57" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q57" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k70c393f4e972",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -9952,14 +9960,14 @@
       <c r="K58" s="70"/>
       <c r="L58" s="70"/>
       <c r="M58" s="70" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="N58" s="70"/>
       <c r="O58" s="70" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="P58" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q58" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1d60e486567d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -9982,14 +9990,14 @@
       <c r="K59" s="70"/>
       <c r="L59" s="70"/>
       <c r="M59" s="70" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="N59" s="70"/>
       <c r="O59" s="70" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="P59" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q59" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k40dc62cd52a5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10012,14 +10020,14 @@
       <c r="K60" s="70"/>
       <c r="L60" s="70"/>
       <c r="M60" s="70" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="N60" s="70"/>
       <c r="O60" s="70" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="P60" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q60" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42d053aa97d9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22")</f>
@@ -10042,14 +10050,14 @@
       <c r="K61" s="70"/>
       <c r="L61" s="70"/>
       <c r="M61" s="70" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="N61" s="70"/>
       <c r="O61" s="70" t="s">
-        <v>1701</v>
+        <v>1702</v>
       </c>
       <c r="P61" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q61" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3d5b3115f0ff",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22")</f>
@@ -10072,14 +10080,14 @@
       <c r="K62" s="70"/>
       <c r="L62" s="70"/>
       <c r="M62" s="70" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="N62" s="70"/>
       <c r="O62" s="70" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="P62" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q62" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b6284c3dfc8",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22")</f>
@@ -10102,14 +10110,14 @@
       <c r="K63" s="70"/>
       <c r="L63" s="70"/>
       <c r="M63" s="70" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="N63" s="70"/>
       <c r="O63" s="70" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="P63" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q63" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k751991f77144",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -10134,10 +10142,10 @@
       <c r="M64" s="70"/>
       <c r="N64" s="70"/>
       <c r="O64" s="70" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="P64" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q64" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6386e55cce43",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10160,14 +10168,14 @@
       <c r="K65" s="70"/>
       <c r="L65" s="70"/>
       <c r="M65" s="70" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="N65" s="70"/>
       <c r="O65" s="70" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="P65" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q65" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb55aff075211",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10192,10 +10200,10 @@
       <c r="M66" s="70"/>
       <c r="N66" s="70"/>
       <c r="O66" s="70" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="P66" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q66" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k78f3bd7641b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22")</f>
@@ -10220,10 +10228,10 @@
       <c r="M67" s="70"/>
       <c r="N67" s="70"/>
       <c r="O67" s="70" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="P67" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q67" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab82b01c89fe",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
@@ -10248,10 +10256,10 @@
       <c r="M68" s="70"/>
       <c r="N68" s="70"/>
       <c r="O68" s="70" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="P68" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q68" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb5633697c8e5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22")</f>
@@ -10276,10 +10284,10 @@
       <c r="M69" s="70"/>
       <c r="N69" s="70"/>
       <c r="O69" s="70" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="P69" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q69" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf724d6e842b3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -10302,14 +10310,14 @@
       <c r="K70" s="70"/>
       <c r="L70" s="70"/>
       <c r="M70" s="70" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="N70" s="70"/>
       <c r="O70" s="70" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="P70" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q70" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k36b71975bd76",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10332,14 +10340,14 @@
       <c r="K71" s="70"/>
       <c r="L71" s="70"/>
       <c r="M71" s="70" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="N71" s="70"/>
       <c r="O71" s="70" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="P71" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q71" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd7994f0255be",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10362,14 +10370,14 @@
       <c r="K72" s="70"/>
       <c r="L72" s="70"/>
       <c r="M72" s="70" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="N72" s="70"/>
       <c r="O72" s="70" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="P72" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q72" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k441c122ac61a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22")</f>
@@ -10392,14 +10400,14 @@
       <c r="K73" s="70"/>
       <c r="L73" s="70"/>
       <c r="M73" s="70" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="N73" s="70"/>
       <c r="O73" s="70" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="P73" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q73" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcad6ba0a7c20",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22")</f>
@@ -10422,14 +10430,14 @@
       <c r="K74" s="70"/>
       <c r="L74" s="70"/>
       <c r="M74" s="70" t="s">
-        <v>1721</v>
+        <v>1722</v>
       </c>
       <c r="N74" s="70"/>
       <c r="O74" s="70" t="s">
-        <v>1722</v>
+        <v>1723</v>
       </c>
       <c r="P74" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q74" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kecd875ec58e7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22")</f>
@@ -10452,14 +10460,14 @@
       <c r="K75" s="70"/>
       <c r="L75" s="70"/>
       <c r="M75" s="70" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="N75" s="70"/>
       <c r="O75" s="70" t="s">
-        <v>1724</v>
+        <v>1725</v>
       </c>
       <c r="P75" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q75" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k04385d48a56f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -10482,14 +10490,14 @@
       <c r="K76" s="70"/>
       <c r="L76" s="70"/>
       <c r="M76" s="70" t="s">
-        <v>1725</v>
+        <v>1726</v>
       </c>
       <c r="N76" s="70"/>
       <c r="O76" s="70" t="s">
-        <v>1726</v>
+        <v>1727</v>
       </c>
       <c r="P76" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q76" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kaa89f6499257",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10512,14 +10520,14 @@
       <c r="K77" s="70"/>
       <c r="L77" s="70"/>
       <c r="M77" s="70" t="s">
-        <v>1727</v>
+        <v>1728</v>
       </c>
       <c r="N77" s="70"/>
       <c r="O77" s="70" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
       <c r="P77" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q77" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc0dcbe2e82c2",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10544,10 +10552,10 @@
       <c r="M78" s="70"/>
       <c r="N78" s="70"/>
       <c r="O78" s="70" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="P78" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q78" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k368f7f8b9908",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22")</f>
@@ -10572,10 +10580,10 @@
       <c r="M79" s="70"/>
       <c r="N79" s="70"/>
       <c r="O79" s="70" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
       <c r="P79" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q79" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k53d619094fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
@@ -10598,14 +10606,14 @@
       <c r="K80" s="70"/>
       <c r="L80" s="70"/>
       <c r="M80" s="70" t="s">
-        <v>1731</v>
+        <v>1732</v>
       </c>
       <c r="N80" s="70"/>
       <c r="O80" s="70" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="P80" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q80" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf511d84233f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22")</f>
@@ -10628,14 +10636,14 @@
       <c r="K81" s="70"/>
       <c r="L81" s="70"/>
       <c r="M81" s="70" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
       <c r="N81" s="70"/>
       <c r="O81" s="70" t="s">
-        <v>1734</v>
+        <v>1735</v>
       </c>
       <c r="P81" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q81" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9da92cf1af2b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -10658,14 +10666,14 @@
       <c r="K82" s="70"/>
       <c r="L82" s="70"/>
       <c r="M82" s="70" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="N82" s="70"/>
       <c r="O82" s="70" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="P82" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q82" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k515087871fe0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10688,14 +10696,14 @@
       <c r="K83" s="70"/>
       <c r="L83" s="70"/>
       <c r="M83" s="70" t="s">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="N83" s="70"/>
       <c r="O83" s="70" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="P83" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q83" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb6acc983851",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10718,14 +10726,14 @@
       <c r="K84" s="70"/>
       <c r="L84" s="70"/>
       <c r="M84" s="70" t="s">
-        <v>1739</v>
+        <v>1740</v>
       </c>
       <c r="N84" s="70"/>
       <c r="O84" s="70" t="s">
-        <v>1740</v>
+        <v>1741</v>
       </c>
       <c r="P84" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q84" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9cdee450b988",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22")</f>
@@ -10748,14 +10756,14 @@
       <c r="K85" s="70"/>
       <c r="L85" s="70"/>
       <c r="M85" s="70" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="N85" s="70"/>
       <c r="O85" s="70" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="P85" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q85" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kac1e5e18d498",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
@@ -10778,14 +10786,14 @@
       <c r="K86" s="70"/>
       <c r="L86" s="70"/>
       <c r="M86" s="70" t="s">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="N86" s="70"/>
       <c r="O86" s="70" t="s">
-        <v>1744</v>
+        <v>1745</v>
       </c>
       <c r="P86" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q86" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb5db6608070",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22")</f>
@@ -10810,10 +10818,10 @@
       <c r="M87" s="70"/>
       <c r="N87" s="70"/>
       <c r="O87" s="70" t="s">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="P87" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q87" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf2a43f4ef780",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -10838,10 +10846,10 @@
       <c r="M88" s="70"/>
       <c r="N88" s="70"/>
       <c r="O88" s="70" t="s">
-        <v>1746</v>
+        <v>1747</v>
       </c>
       <c r="P88" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q88" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k86b940633ffd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10866,10 +10874,10 @@
       <c r="M89" s="70"/>
       <c r="N89" s="70"/>
       <c r="O89" s="70" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
       <c r="P89" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q89" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf341ebe84b57",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10892,14 +10900,14 @@
       <c r="K90" s="70"/>
       <c r="L90" s="70"/>
       <c r="M90" s="70" t="s">
-        <v>1748</v>
+        <v>1749</v>
       </c>
       <c r="N90" s="70"/>
       <c r="O90" s="70" t="s">
-        <v>1749</v>
+        <v>1750</v>
       </c>
       <c r="P90" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q90" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7383ee3f2ec5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22")</f>
@@ -10922,14 +10930,14 @@
       <c r="K91" s="70"/>
       <c r="L91" s="70"/>
       <c r="M91" s="70" t="s">
-        <v>1750</v>
+        <v>1751</v>
       </c>
       <c r="N91" s="70"/>
       <c r="O91" s="70" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
       <c r="P91" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q91" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5cae8f95e8bd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
@@ -10952,14 +10960,14 @@
       <c r="K92" s="70"/>
       <c r="L92" s="70"/>
       <c r="M92" s="70" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="N92" s="70"/>
       <c r="O92" s="70" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="P92" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q92" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0ecee6c15886",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22")</f>
@@ -10982,14 +10990,14 @@
       <c r="K93" s="70"/>
       <c r="L93" s="70"/>
       <c r="M93" s="70" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="N93" s="70"/>
       <c r="O93" s="70" t="s">
-        <v>1755</v>
+        <v>1756</v>
       </c>
       <c r="P93" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q93" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k874b463422ce",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11014,10 +11022,10 @@
       <c r="M94" s="70"/>
       <c r="N94" s="70"/>
       <c r="O94" s="70" t="s">
-        <v>1756</v>
+        <v>1757</v>
       </c>
       <c r="P94" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q94" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k07aa4ed88482",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11040,14 +11048,14 @@
       <c r="K95" s="70"/>
       <c r="L95" s="70"/>
       <c r="M95" s="70" t="s">
-        <v>1757</v>
+        <v>1758</v>
       </c>
       <c r="N95" s="70"/>
       <c r="O95" s="70" t="s">
-        <v>1758</v>
+        <v>1759</v>
       </c>
       <c r="P95" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q95" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k444ff4b9a71a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11070,14 +11078,14 @@
       <c r="K96" s="70"/>
       <c r="L96" s="70"/>
       <c r="M96" s="70" t="s">
-        <v>1759</v>
+        <v>1760</v>
       </c>
       <c r="N96" s="70"/>
       <c r="O96" s="70" t="s">
-        <v>1760</v>
+        <v>1761</v>
       </c>
       <c r="P96" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q96" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42b7580a8cb9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22")</f>
@@ -11102,10 +11110,10 @@
       <c r="M97" s="70"/>
       <c r="N97" s="70"/>
       <c r="O97" s="70" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
       <c r="P97" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q97" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8e5410dc08f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11130,10 +11138,10 @@
       <c r="M98" s="70"/>
       <c r="N98" s="70"/>
       <c r="O98" s="70" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="P98" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q98" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb0df0c43cf87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22")</f>
@@ -11158,10 +11166,10 @@
       <c r="M99" s="70"/>
       <c r="N99" s="70"/>
       <c r="O99" s="70" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
       <c r="P99" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q99" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kde315e91893f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11186,10 +11194,10 @@
       <c r="M100" s="70"/>
       <c r="N100" s="70"/>
       <c r="O100" s="70" t="s">
-        <v>1764</v>
+        <v>1765</v>
       </c>
       <c r="P100" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q100" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf9cc95eccf07",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11212,14 +11220,14 @@
       <c r="K101" s="70"/>
       <c r="L101" s="70"/>
       <c r="M101" s="70" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
       <c r="N101" s="70"/>
       <c r="O101" s="70" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="P101" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q101" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd674be572fbd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11242,14 +11250,14 @@
       <c r="K102" s="70"/>
       <c r="L102" s="70"/>
       <c r="M102" s="70" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="N102" s="70"/>
       <c r="O102" s="70" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="P102" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q102" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4f3c12075c6f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22")</f>
@@ -11272,14 +11280,14 @@
       <c r="K103" s="70"/>
       <c r="L103" s="70"/>
       <c r="M103" s="70" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
       <c r="N103" s="70"/>
       <c r="O103" s="70" t="s">
-        <v>1770</v>
+        <v>1771</v>
       </c>
       <c r="P103" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q103" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k856d2d13cd04",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11302,14 +11310,14 @@
       <c r="K104" s="70"/>
       <c r="L104" s="70"/>
       <c r="M104" s="70" t="s">
-        <v>1771</v>
+        <v>1772</v>
       </c>
       <c r="N104" s="70"/>
       <c r="O104" s="70" t="s">
-        <v>1772</v>
+        <v>1773</v>
       </c>
       <c r="P104" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q104" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k160e960d09c4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22")</f>
@@ -11332,14 +11340,14 @@
       <c r="K105" s="70"/>
       <c r="L105" s="70"/>
       <c r="M105" s="70" t="s">
-        <v>1773</v>
+        <v>1774</v>
       </c>
       <c r="N105" s="70"/>
       <c r="O105" s="70" t="s">
-        <v>1774</v>
+        <v>1775</v>
       </c>
       <c r="P105" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q105" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd3a48013b455",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11362,14 +11370,14 @@
       <c r="K106" s="70"/>
       <c r="L106" s="70"/>
       <c r="M106" s="70" t="s">
-        <v>1775</v>
+        <v>1776</v>
       </c>
       <c r="N106" s="70"/>
       <c r="O106" s="70" t="s">
-        <v>1776</v>
+        <v>1777</v>
       </c>
       <c r="P106" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q106" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f26b556436e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11392,14 +11400,14 @@
       <c r="K107" s="70"/>
       <c r="L107" s="70"/>
       <c r="M107" s="70" t="s">
-        <v>1777</v>
+        <v>1778</v>
       </c>
       <c r="N107" s="70"/>
       <c r="O107" s="70" t="s">
-        <v>1778</v>
+        <v>1779</v>
       </c>
       <c r="P107" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q107" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3a6534dc5a62",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11424,10 +11432,10 @@
       <c r="M108" s="70"/>
       <c r="N108" s="70"/>
       <c r="O108" s="70" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
       <c r="P108" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q108" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ka5734698aa50",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22")</f>
@@ -11452,10 +11460,10 @@
       <c r="M109" s="70"/>
       <c r="N109" s="70"/>
       <c r="O109" s="70" t="s">
-        <v>1780</v>
+        <v>1781</v>
       </c>
       <c r="P109" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q109" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3bd1b440e87a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11478,14 +11486,14 @@
       <c r="K110" s="70"/>
       <c r="L110" s="70"/>
       <c r="M110" s="70" t="s">
-        <v>1781</v>
+        <v>1782</v>
       </c>
       <c r="N110" s="70"/>
       <c r="O110" s="70" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="P110" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q110" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k52493b74eb28",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22")</f>
@@ -11508,14 +11516,14 @@
       <c r="K111" s="70"/>
       <c r="L111" s="70"/>
       <c r="M111" s="70" t="s">
-        <v>1783</v>
+        <v>1784</v>
       </c>
       <c r="N111" s="70"/>
       <c r="O111" s="70" t="s">
-        <v>1784</v>
+        <v>1785</v>
       </c>
       <c r="P111" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q111" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3fa800b9318b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11538,14 +11546,14 @@
       <c r="K112" s="70"/>
       <c r="L112" s="70"/>
       <c r="M112" s="70" t="s">
-        <v>1785</v>
+        <v>1786</v>
       </c>
       <c r="N112" s="70"/>
       <c r="O112" s="70" t="s">
-        <v>1786</v>
+        <v>1787</v>
       </c>
       <c r="P112" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q112" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b2764e691f7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11570,10 +11578,10 @@
       <c r="M113" s="70"/>
       <c r="N113" s="70"/>
       <c r="O113" s="70" t="s">
-        <v>1787</v>
+        <v>1788</v>
       </c>
       <c r="P113" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q113" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9afa96310f5f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11598,10 +11606,10 @@
       <c r="M114" s="70"/>
       <c r="N114" s="70"/>
       <c r="O114" s="70" t="s">
-        <v>1788</v>
+        <v>1789</v>
       </c>
       <c r="P114" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q114" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3eb4a6e4e0a9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22")</f>
@@ -11624,14 +11632,14 @@
       <c r="K115" s="70"/>
       <c r="L115" s="70"/>
       <c r="M115" s="70" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="N115" s="70"/>
       <c r="O115" s="70" t="s">
-        <v>1790</v>
+        <v>1791</v>
       </c>
       <c r="P115" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q115" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3786dea98f2a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11654,14 +11662,14 @@
       <c r="K116" s="70"/>
       <c r="L116" s="70"/>
       <c r="M116" s="70" t="s">
-        <v>1791</v>
+        <v>1792</v>
       </c>
       <c r="N116" s="70"/>
       <c r="O116" s="70" t="s">
-        <v>1792</v>
+        <v>1793</v>
       </c>
       <c r="P116" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q116" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8424cc4e78b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22")</f>
@@ -11684,14 +11692,14 @@
       <c r="K117" s="70"/>
       <c r="L117" s="70"/>
       <c r="M117" s="70" t="s">
-        <v>1793</v>
+        <v>1794</v>
       </c>
       <c r="N117" s="70"/>
       <c r="O117" s="70" t="s">
-        <v>1794</v>
+        <v>1795</v>
       </c>
       <c r="P117" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q117" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf325ac36b969",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11714,14 +11722,14 @@
       <c r="K118" s="70"/>
       <c r="L118" s="70"/>
       <c r="M118" s="70" t="s">
-        <v>1795</v>
+        <v>1796</v>
       </c>
       <c r="N118" s="70"/>
       <c r="O118" s="70" t="s">
-        <v>1796</v>
+        <v>1797</v>
       </c>
       <c r="P118" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q118" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4ec5ffc67bf1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11744,14 +11752,14 @@
       <c r="K119" s="70"/>
       <c r="L119" s="70"/>
       <c r="M119" s="70" t="s">
-        <v>1797</v>
+        <v>1798</v>
       </c>
       <c r="N119" s="70"/>
       <c r="O119" s="70" t="s">
-        <v>1798</v>
+        <v>1799</v>
       </c>
       <c r="P119" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q119" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k006e6e337926",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11774,14 +11782,14 @@
       <c r="K120" s="70"/>
       <c r="L120" s="70"/>
       <c r="M120" s="70" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="N120" s="70"/>
       <c r="O120" s="70" t="s">
-        <v>1800</v>
+        <v>1801</v>
       </c>
       <c r="P120" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q120" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k94da89c1d16d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22")</f>
@@ -11804,14 +11812,14 @@
       <c r="K121" s="70"/>
       <c r="L121" s="70"/>
       <c r="M121" s="70" t="s">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="N121" s="70"/>
       <c r="O121" s="70" t="s">
-        <v>1802</v>
+        <v>1803</v>
       </c>
       <c r="P121" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q121" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9b79f94a3042",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11834,14 +11842,14 @@
       <c r="K122" s="70"/>
       <c r="L122" s="70"/>
       <c r="M122" s="70" t="s">
-        <v>1803</v>
+        <v>1804</v>
       </c>
       <c r="N122" s="70"/>
       <c r="O122" s="70" t="s">
-        <v>1804</v>
+        <v>1805</v>
       </c>
       <c r="P122" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q122" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b57aec5f42c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22")</f>
@@ -11864,14 +11872,14 @@
       <c r="K123" s="70"/>
       <c r="L123" s="70"/>
       <c r="M123" s="70" t="s">
-        <v>1805</v>
+        <v>1806</v>
       </c>
       <c r="N123" s="70"/>
       <c r="O123" s="70" t="s">
-        <v>1806</v>
+        <v>1807</v>
       </c>
       <c r="P123" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q123" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k524993898ff0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11894,14 +11902,14 @@
       <c r="K124" s="70"/>
       <c r="L124" s="70"/>
       <c r="M124" s="70" t="s">
-        <v>1807</v>
+        <v>1808</v>
       </c>
       <c r="N124" s="70"/>
       <c r="O124" s="70" t="s">
-        <v>1808</v>
+        <v>1809</v>
       </c>
       <c r="P124" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q124" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k71038ca67fed",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11926,10 +11934,10 @@
       <c r="M125" s="70"/>
       <c r="N125" s="70"/>
       <c r="O125" s="70" t="s">
-        <v>1809</v>
+        <v>1810</v>
       </c>
       <c r="P125" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q125" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab565ddcecfd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11954,10 +11962,10 @@
       <c r="M126" s="70"/>
       <c r="N126" s="70"/>
       <c r="O126" s="70" t="s">
-        <v>1810</v>
+        <v>1811</v>
       </c>
       <c r="P126" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q126" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kda9320d99fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22")</f>
@@ -11980,14 +11988,14 @@
       <c r="K127" s="70"/>
       <c r="L127" s="70"/>
       <c r="M127" s="70" t="s">
-        <v>1811</v>
+        <v>1812</v>
       </c>
       <c r="N127" s="70"/>
       <c r="O127" s="70" t="s">
-        <v>1812</v>
+        <v>1813</v>
       </c>
       <c r="P127" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q127" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k577a4eca3248",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12010,14 +12018,14 @@
       <c r="K128" s="70"/>
       <c r="L128" s="70"/>
       <c r="M128" s="70" t="s">
-        <v>1813</v>
+        <v>1814</v>
       </c>
       <c r="N128" s="70"/>
       <c r="O128" s="70" t="s">
-        <v>1814</v>
+        <v>1815</v>
       </c>
       <c r="P128" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q128" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dbd9d8294a0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22")</f>
@@ -12042,10 +12050,10 @@
       <c r="M129" s="70"/>
       <c r="N129" s="70"/>
       <c r="O129" s="70" t="s">
-        <v>1815</v>
+        <v>1816</v>
       </c>
       <c r="P129" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q129" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k858285f0484a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12070,10 +12078,10 @@
       <c r="M130" s="70"/>
       <c r="N130" s="70"/>
       <c r="O130" s="70" t="s">
-        <v>1816</v>
+        <v>1817</v>
       </c>
       <c r="P130" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q130" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3386b404a0cc",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12098,10 +12106,10 @@
       <c r="M131" s="70"/>
       <c r="N131" s="70"/>
       <c r="O131" s="70" t="s">
-        <v>1817</v>
+        <v>1818</v>
       </c>
       <c r="P131" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q131" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1fdcada6b7d5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12126,10 +12134,10 @@
       <c r="M132" s="70"/>
       <c r="N132" s="70"/>
       <c r="O132" s="70" t="s">
-        <v>1818</v>
+        <v>1819</v>
       </c>
       <c r="P132" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q132" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k66ad104dc3f4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22")</f>
@@ -12152,10 +12160,10 @@
       <c r="M133" s="70"/>
       <c r="N133" s="70"/>
       <c r="O133" s="70" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="P133" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q133" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f9d2ee2e87b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12178,10 +12186,10 @@
       <c r="M134" s="70"/>
       <c r="N134" s="70"/>
       <c r="O134" s="70" t="s">
-        <v>1820</v>
+        <v>1821</v>
       </c>
       <c r="P134" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q134" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k2e021d1404f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22")</f>
@@ -12204,10 +12212,10 @@
       <c r="M135" s="70"/>
       <c r="N135" s="70"/>
       <c r="O135" s="70" t="s">
-        <v>1821</v>
+        <v>1822</v>
       </c>
       <c r="P135" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q135" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7f727f839de9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12230,10 +12238,10 @@
       <c r="M136" s="70"/>
       <c r="N136" s="70"/>
       <c r="O136" s="70" t="s">
-        <v>1822</v>
+        <v>1823</v>
       </c>
       <c r="P136" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q136" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc9f54d815229",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12256,10 +12264,10 @@
       <c r="M137" s="70"/>
       <c r="N137" s="70"/>
       <c r="O137" s="70" t="s">
-        <v>1823</v>
+        <v>1824</v>
       </c>
       <c r="P137" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q137" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k814de685731b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12282,10 +12290,10 @@
       <c r="M138" s="70"/>
       <c r="N138" s="70"/>
       <c r="O138" s="70" t="s">
-        <v>1824</v>
+        <v>1825</v>
       </c>
       <c r="P138" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q138" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbeebbf583a30",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22")</f>
@@ -12308,10 +12316,10 @@
       <c r="M139" s="70"/>
       <c r="N139" s="70"/>
       <c r="O139" s="70" t="s">
-        <v>1825</v>
+        <v>1826</v>
       </c>
       <c r="P139" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q139" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kae76dda4b45d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12334,10 +12342,10 @@
       <c r="M140" s="70"/>
       <c r="N140" s="70"/>
       <c r="O140" s="70" t="s">
-        <v>1826</v>
+        <v>1827</v>
       </c>
       <c r="P140" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q140" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1228a3dffde6",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22")</f>
@@ -12360,10 +12368,10 @@
       <c r="M141" s="70"/>
       <c r="N141" s="70"/>
       <c r="O141" s="70" t="s">
-        <v>1827</v>
+        <v>1828</v>
       </c>
       <c r="P141" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q141" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k47f0af99bd1e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12386,10 +12394,10 @@
       <c r="M142" s="70"/>
       <c r="N142" s="70"/>
       <c r="O142" s="70" t="s">
-        <v>1828</v>
+        <v>1829</v>
       </c>
       <c r="P142" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q142" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcee0b8f57c67",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12412,10 +12420,10 @@
       <c r="M143" s="70"/>
       <c r="N143" s="70"/>
       <c r="O143" s="70" t="s">
-        <v>1829</v>
+        <v>1830</v>
       </c>
       <c r="P143" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q143" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k59fb8b4ed900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12438,10 +12446,10 @@
       <c r="M144" s="70"/>
       <c r="N144" s="70"/>
       <c r="O144" s="70" t="s">
-        <v>1830</v>
+        <v>1831</v>
       </c>
       <c r="P144" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q144" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1a00a0a22804",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22")</f>
@@ -12464,10 +12472,10 @@
       <c r="M145" s="70"/>
       <c r="N145" s="70"/>
       <c r="O145" s="70" t="s">
-        <v>1831</v>
+        <v>1832</v>
       </c>
       <c r="P145" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q145" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k29d47d551984",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12490,10 +12498,10 @@
       <c r="M146" s="70"/>
       <c r="N146" s="70"/>
       <c r="O146" s="70" t="s">
-        <v>1832</v>
+        <v>1833</v>
       </c>
       <c r="P146" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q146" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdc81e4a42f98",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12516,10 +12524,10 @@
       <c r="M147" s="70"/>
       <c r="N147" s="70"/>
       <c r="O147" s="70" t="s">
-        <v>1833</v>
+        <v>1834</v>
       </c>
       <c r="P147" s="70" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="Q147" s="70" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc34b261fea84",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12552,16 +12560,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="72" t="s">
-        <v>1834</v>
+        <v>1835</v>
       </c>
       <c r="B1" s="72" t="s">
-        <v>1835</v>
+        <v>1836</v>
       </c>
       <c r="C1" s="72" t="s">
-        <v>1836</v>
+        <v>1837</v>
       </c>
       <c r="D1" s="72" t="s">
-        <v>1837</v>
+        <v>1838</v>
       </c>
     </row>
   </sheetData>
@@ -20338,7 +20346,7 @@
       <c r="I11" s="50"/>
       <c r="J11" s="7" t="str">
         <f aca="true">IF(I11="✓","done",IF(TODAY()&lt;B11,"upcoming",IF(TODAY()&lt;G11,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>open</v>
       </c>
       <c r="K11" s="51"/>
     </row>

</xml_diff>

<commit_message>
Ruling 41: a deck is its Slides file — no HTML decks, no console; Units 3 and 4 rebuilt (kit 6831bc5); master sheet rebuilt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xYWeLUsuszQH6z7ADE9tj
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -5567,7 +5567,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit e16632a on 05 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit cbeda99 on 06 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="B1" s="2" t="n">
         <f aca="true">TODAY()</f>
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="B5" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,$B$44)&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,$B$44))</f>
-        <v>T-A1   Thread A: the same laws with variable bases (14.1–14.2)</v>
+        <v>T-A2   Thread A: negative exponents and multiple laws, variable bases (14.3–14.4)</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7198,16 +7198,16 @@
       </c>
       <c r="B6" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$T$2:$T$132,$B$44)&amp;"")</f>
-        <v>I can multiply and divide monomials, and raise a monomial to a power, by applying the laws of exponents to variable bases.</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>I can rewrite an algebraic expression with negative exponents using only positive exponents, and apply several laws of exponents to a monomial expression.</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$U$2:$U$132,$B$44)&amp;"")</f>
-        <v>Do the laws of exponents change when the base is a variable?</v>
+        <v>What does a negative exponent on a variable mean, and how do several laws combine in one expression?</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7216,7 +7216,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$V$2:$V$132,$B$44)&amp;"")</f>
-        <v>monomial, coefficient, like bases</v>
+        <v>negative exponent law, simplified form</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7234,25 +7234,25 @@
       </c>
       <c r="B10" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IF(INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;""="","none",INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;"   — due "&amp;TEXT(INDEX('Scope &amp; Sequence'!$S$2:$S$132,$B$44),"ddd d mmm")))</f>
-        <v>Multiply powers: variable bases — TR9; Powers of a power: variable bases — 2CU; Divide monomials with positive exponents — C8L   — due Tue 6 Oct</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>Variables with negative exponents — 2NL; Multiply and divide powers: variable bases — 85P   — due Wed 7 Oct</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IFERROR(INDEX('IXL tracker'!$D$5:$D$86,MATCH(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),'IXL tracker'!$G$5:$G$86,0)),"nothing due"))</f>
-        <v>nothing due</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>Multiply powers: variable bases (TR9); Powers of a power: variable bases (2CU); Divide monomials with positive exponents (C8L)</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$Z$2:$Z$132,$B$44)&amp;"")</f>
-        <v>Rachel writes (15xy²)³ as 15 · 15 · 15 · x · x · x · y · y · y · y · y · y. Justina writes it as 3,375x³y⁶. Who is correct? Explain.</v>
+        <v>How are x³ and x⁻³ related? Explain, and give the value of each when x = 2.</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7387,11 +7387,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="n">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+1)))</f>
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B30" s="6" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+1))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+1)))</f>
-        <v>T-A2   Thread A: negative exponents and multiple laws, variable bases (14.3–14.4)</v>
+        <v>3.08   Large numbers in scientific notation</v>
       </c>
       <c r="C30" s="8" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+1))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+1)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+1))&amp;"")))</f>
@@ -7401,49 +7401,49 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="n">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+2)))</f>
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B31" s="6" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+2))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+2)))</f>
-        <v>3.08   Large numbers in scientific notation</v>
+        <v>off   State test — no class</v>
       </c>
       <c r="C31" s="8" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+2))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+2)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+2))&amp;"")))</f>
-        <v>open</v>
+        <v>—</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="n">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+3)))</f>
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B32" s="6" t="str">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+3))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+3)))</f>
-        <v>off   State test — no class</v>
+        <v>3.09   Small numbers in scientific notation; how many times larger</v>
       </c>
       <c r="C32" s="8" t="str">
         <f aca="false">IF(($B$44+3)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+3))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+3)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+3))&amp;"")))</f>
-        <v>—</v>
+        <v>open</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+4)))</f>
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="B33" s="6" t="str">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+4))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+4)))</f>
-        <v>3.09   Small numbers in scientific notation; how many times larger</v>
+        <v>spiral   Spiral day — mixed retrieval from the unit just finished and the two before it</v>
       </c>
       <c r="C33" s="8" t="str">
         <f aca="false">IF(($B$44+4)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+4))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+4)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+4))&amp;"")))</f>
-        <v>open</v>
+        <v>Unit Review</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="n">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+5)))</f>
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B34" s="6" t="str">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+5))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+5)))</f>
@@ -7467,7 +7467,7 @@
       </c>
       <c r="B44" s="13" t="n">
         <f aca="true">IF(TODAY()&gt;$B$45,131+1,MIN(COUNTIF('Scope &amp; Sequence'!$A$2:$A$132,"&lt;"&amp;TODAY())+1,131))</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20346,7 +20346,7 @@
       <c r="I11" s="50"/>
       <c r="J11" s="7" t="str">
         <f aca="true">IF(I11="✓","done",IF(TODAY()&lt;B11,"upcoming",IF(TODAY()&lt;G11,"open","due — check scores")))</f>
-        <v>open</v>
+        <v>due — check scores</v>
       </c>
       <c r="K11" s="51"/>
     </row>
@@ -20376,7 +20376,7 @@
       <c r="I12" s="50"/>
       <c r="J12" s="7" t="str">
         <f aca="true">IF(I12="✓","done",IF(TODAY()&lt;B12,"upcoming",IF(TODAY()&lt;G12,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>open</v>
       </c>
       <c r="K12" s="51"/>
     </row>

</xml_diff>

<commit_message>
Ruling 43: a practice problem never repeats what the lesson already showed — Units 3 and 4 rewritten, rebuilt and installed at 0 findings (kit 050fc2b)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xYWeLUsuszQH6z7ADE9tj
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -78,7 +78,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">MTR.2.1: Notes II and board 9 — the same expression is carried to the end by two different plans, written side by side, and the two answers are compared.
+          <t xml:space="preserve">MTR.2.1: Notes II and board 9 — one expression is carried to the end by two different plans, written side by side, and the two answers are compared.
 MTR.3.1: Boards 1 through 4 — four multi-law expressions, one each, written without a reference sheet.
 MTR.6.1: Board 5 — a sixth power over 2¹⁰ lands on 4; students say why an answer that small is reasonable before they trust it.</t>
         </r>
@@ -93,7 +93,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">MTR.5.1: Notes I — the halving table; students fill 2⁻¹, 2⁻² and 2⁻³ from the pattern before the rule is named.
-MTR.4.1: Board 5 — when the room splits between 1/25 and −25, the sixty-second re-vote before the reveal.
+MTR.4.1: Board 5 — when the room splits between 1/49 and −49, the sixty-second re-vote before the reveal.
 MTR.6.1: Board 1 — a reciprocal of 8³ is a small positive number, so −512 cannot be right; students say why.</t>
         </r>
       </text>
@@ -107,7 +107,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">MTR.5.1: Notes I — 3.04's halving table redone with a fraction base, so the flip appears as the next line of a pattern the class already owns rather than a second rule.
-MTR.4.1: Board 5 — when the room splits between (−8/7)³ and (8/7)³, the sixty-second re-vote before the reveal: is the reciprocal of −7/8 positive or negative?
+MTR.4.1: Board 5 — when the room splits between (−10/7)³ and (10/7)³, the sixty-second re-vote before the reveal: is the reciprocal of −7/10 positive or negative?
 MTR.6.1: Board 3 — a base between −1 and 0 raised to a negative even power; students say which side of 1 the value lands on before computing it.</t>
         </r>
       </text>
@@ -122,7 +122,7 @@
           </rPr>
           <t xml:space="preserve">MTR.2.1: Notes I — two students' plans for one expression are written side by side and both are carried to the end, so the value is seen to be independent of the route.
 MTR.5.1: Notes III and boards 4, 7 and 8 — 8, 4 and 16 are rewritten as powers of 2, which is the only way expressions with different bases can be compared at all.
-MTR.6.1: Board 9 — Xavier's claim is tested rather than believed; the student converts the second expression and finds 2⁻⁶.</t>
+MTR.6.1: Board 9 — Xavier's claim is tested rather than believed; the student converts the second expression and finds 3⁻⁸.</t>
         </r>
       </text>
     </comment>
@@ -150,7 +150,7 @@
           </rPr>
           <t xml:space="preserve">MTR.5.1: Notes I — 3.04's halving table rewritten with a letter, so x⁻¹ = 1/x is the next line of a pattern the class already owns.
 MTR.6.1: Board 4 — two negative exponents on two different letters; students say how many factors end up under the bar before they write anything.
-MTR.4.1: Board 6 — when the room splits over whether the 2 gets squared, the sixty-second re-vote before the reveal.</t>
+MTR.4.1: Board 6 — when the room splits over whether the 3 gets squared, the sixty-second re-vote before the reveal.</t>
         </r>
       </text>
     </comment>
@@ -234,7 +234,7 @@
           </rPr>
           <t xml:space="preserve">MTR.5.1: Notes I — the radical bar is recognised as a grouping symbol by comparing √(9 + 16) with √9 + √16, so the rule is derived from the difference rather than announced.
 MTR.6.1: Boards 3 and 6 — students say whether a negative answer is possible at all before they evaluate, which is the whole square-root-versus-cube-root distinction.
-MTR.4.1: Board 5 — when the room splits between 5 and 7 on √(9 + 16), the sixty-second re-vote before the reveal.</t>
+MTR.4.1: Board 5 — when the room splits between 13 and 17 on √(25 + 144), the sixty-second re-vote before the reveal.</t>
         </r>
       </text>
     </comment>
@@ -286,7 +286,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to say that both students are right and that 2⁰ is 1. Read the boards, not the papers.</t>
+          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to say that both students are right and that 6⁰ is 1. Read the boards, not the papers.</t>
         </r>
       </text>
     </comment>
@@ -346,7 +346,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to say that both forms are the same expression and show that 15³ is 3,375. Read the boards, not the papers.</t>
+          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to say that both forms are the same expression and show that 14³ is 2,744. Read the boards, not the papers.</t>
         </r>
       </text>
     </comment>
@@ -358,7 +358,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to name x⁻³ as the reciprocal of x³ and give both values at x = 2. Read the boards, not the papers.</t>
+          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to name x⁻⁵ as the reciprocal of x⁵ and give both values at x = 2. Read the boards, not the papers.</t>
         </r>
       </text>
     </comment>
@@ -370,7 +370,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to say both things — equal in value, and not in scientific notation — and give 2 × 10⁶. Read the boards, not the papers.</t>
+          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to say both things — equal in value, and not in scientific notation — and give 7 × 10⁷. Read the boards, not the papers.</t>
         </r>
       </text>
     </comment>
@@ -394,7 +394,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to name both of Devon's mistakes separately and give 3.413 × 10⁵. Read the boards, not the papers.</t>
+          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to name both of Devon's mistakes separately and give 6.619 × 10⁴. Read the boards, not the papers.</t>
         </r>
       </text>
     </comment>
@@ -418,7 +418,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to say what the rule for a sum actually is, not only that Ellis used the wrong one, and give 1.240 × 10³. Read the boards, not the papers.</t>
+          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to say what the rule for a sum actually is, not only that Ellis used the wrong one, and give 9.150 × 10³. Read the boards, not the papers.</t>
         </r>
       </text>
     </comment>
@@ -615,10 +615,10 @@
 MA.K12.MTR.4.1 Engage in discussions that reflect on the mathematical thinking of self and others.</t>
   </si>
   <si>
-    <t xml:space="preserve">Aiyanna says she can use the power of a product law to evaluate (10 + (−2))³. Is she right?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No — (10 + (−2))³ = 8³ = 512</t>
+    <t xml:space="preserve">Aiyanna says she can use the power of a product law to evaluate (9 + (−3))³. Is she right?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No — (9 + (−3))³ = 6³ = 216</t>
   </si>
   <si>
     <t xml:space="preserve">3.1 Product Laws of Exponents</t>
@@ -650,10 +650,10 @@
 MA.K12.MTR.4.1 Engage in discussions that reflect on the mathematical thinking of self and others.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hannah cancels 2³/2³ to 1. Sebastian subtracts to 2⁰. Who is right?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Both — 2⁰ = 1</t>
+    <t xml:space="preserve">Hannah cancels 6²/6² to 1. Sebastian subtracts to 6⁰. Who is right?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both — 6⁰ = 1</t>
   </si>
   <si>
     <t xml:space="preserve">3.2 Quotient Laws of Exponents</t>
@@ -685,10 +685,10 @@
 MA.K12.MTR.6.1 Assess the reasonableness of solutions.</t>
   </si>
   <si>
-    <t xml:space="preserve">Winston writes (2⁶/2⁴)³ = (2²)³. Yvette writes (2⁶/2⁴)³ = 2¹⁸/2¹². Do they get the same value? Explain.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes — both give 2⁶ = 64</t>
+    <t xml:space="preserve">Winston writes (4⁷/4⁴)² = (4³)². Yvette writes (4⁷/4⁴)² = 4¹⁴/4⁸. Do they get the same value? Explain.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes — both give 4⁶ = 4,096</t>
   </si>
   <si>
     <t xml:space="preserve">3.3 Exponential Expressions</t>
@@ -726,10 +726,10 @@
 MA.K12.MTR.6.1 Assess the reasonableness of solutions.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ellen says the value of 5⁻² is −25. Explain why she is wrong, and show the correct value.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5⁻² = 1/5² = 1/25</t>
+    <t xml:space="preserve">Ellen says the value of 12⁻² is −144. Explain why she is wrong, and show the correct value.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12⁻² = 1/12² = 1/144</t>
   </si>
   <si>
     <t xml:space="preserve">3.4 Negative Exponent Law</t>
@@ -756,10 +756,10 @@
     <t xml:space="preserve">reciprocal of a fraction, rational base with a negative exponent</t>
   </si>
   <si>
-    <t xml:space="preserve">Marco says (−2/3)⁻⁵ can be rewritten as (2/3)⁵ because 'two negatives make a positive.' Is he right?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No — (−2/3)⁻⁵ = (−3/2)⁵</t>
+    <t xml:space="preserve">Marco says (−4/11)⁻⁷ can be rewritten as (4/11)⁷ because 'two negatives make a positive.' Is he right?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No — (−4/11)⁻⁷ = (−11/4)⁷</t>
   </si>
   <si>
     <t xml:space="preserve">3.5 Applying Exponent Laws</t>
@@ -788,10 +788,10 @@
 MA.K12.MTR.6.1 Assess the reasonableness of solutions.</t>
   </si>
   <si>
-    <t xml:space="preserve">Xavier says (1/4)²·2⁻³ and (1/2)⁴·4⁻¹ are equivalent because both can be written as 2⁻⁷. Do you agree?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No — the second is 2⁻⁶, not 2⁻⁷</t>
+    <t xml:space="preserve">Xavier says (1/9)²·3⁻⁵ and (1/3)⁶·9⁻¹ are equivalent because both can be written as 3⁻⁹. Do you agree?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No — the second is 3⁻⁸, not 3⁻⁹</t>
   </si>
   <si>
     <t xml:space="preserve">3.6 Evaluating Numerical Expressions with Integer Exponents
@@ -831,10 +831,10 @@
     <t xml:space="preserve">MA.8.AR.1.1 — Apply the Laws of Exponents to generate equivalent algebraic expressions, limited to integer exponents and monomial bases.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rachel writes (15xy²)³ as 15 · 15 · 15 · x · x · x · y · y · y · y · y · y. Justina writes it as 3,375x³y⁶. Who is correct? Explain.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Both are correct; 15³ = 3,375, x · x · x = x³, and six y's make y⁶.</t>
+    <t xml:space="preserve">Rachel writes (14a³b)³ as 14 · 14 · 14 · a · a · a · a · a · a · a · a · a · b · b · b. Justina writes it as 2,744a⁹b³. Who is correct? Explain.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both are correct; 14³ = 2,744, nine a's make a⁹, and b · b · b = b³.</t>
   </si>
   <si>
     <t xml:space="preserve">14.1 Applying Exponent Laws to Algebraic Expressions – Part 1
@@ -859,10 +859,10 @@
     <t xml:space="preserve">negative exponent law, simplified form</t>
   </si>
   <si>
-    <t xml:space="preserve">How are x³ and x⁻³ related? Explain, and give the value of each when x = 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x⁻³ is the reciprocal of x³. When x = 2: x³ = 8 and x⁻³ = 1/8.</t>
+    <t xml:space="preserve">How are x⁵ and x⁻⁵ related? Explain, and give the value of each when x = 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x⁻⁵ is the reciprocal of x⁵. When x = 2: x⁵ = 32 and x⁻⁵ = 1/32.</t>
   </si>
   <si>
     <t xml:space="preserve">14.3 Algebraic Expressions with Negative Exponents
@@ -898,10 +898,10 @@
 MA.K12.MTR.6.1 Assess the reasonableness of solutions.</t>
   </si>
   <si>
-    <t xml:space="preserve">Marcus writes 2,000,000 as 20 × 10⁵. Is his expression equal to 2,000,000? Is it scientific notation? Explain.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equal, yes. Scientific notation, no: 20 is not less than 10. 2 × 10⁶.</t>
+    <t xml:space="preserve">Marcus writes 70,000,000 as 70 × 10⁶. Is his expression equal to 70,000,000? Is it scientific notation? Explain.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equal, yes. Scientific notation, no: 70 is not less than 10. 7 × 10⁷.</t>
   </si>
   <si>
     <t xml:space="preserve">3.8 Writing Large Numbers in Scientific Notation</t>
@@ -987,10 +987,10 @@
     <t xml:space="preserve">MA.8.NSO.1.5 — Add, subtract, multiply and divide numbers expressed in scientific notation with procedural fluency.</t>
   </si>
   <si>
-    <t xml:space="preserve">Devon writes (1.3 × 10³) + (3.4 × 10⁵) = 4.7 × 10⁸. Name the two mistakes he made, and give the correct sum.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.413 × 10⁵</t>
+    <t xml:space="preserve">Devon writes (1.9 × 10²) + (6.6 × 10⁴) = 8.5 × 10⁶. Name the two mistakes he made, and give the correct sum.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.619 × 10⁴</t>
   </si>
   <si>
     <t xml:space="preserve">4.1 Adding and Subtracting Numbers Expressed in Scientific Notation</t>
@@ -1053,10 +1053,10 @@
 MA.K12.MTR.4.1 Engage in discussions that reflect on the mathematical thinking of self and others.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ellis says that because 1,234 has 4 significant digits and 5.6 has 2, the sum 1,234 + 5.6 must be written with 2 significant digits, as 1.2 × 10³. Explain why he is wrong, and give the correct sum.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,240 = 1.240 × 10³</t>
+    <t xml:space="preserve">Ellis says that because 9,145 has 4 significant digits and 4.8 has 2, the sum 9,145 + 4.8 must be written with 2 significant digits, as 9.1 × 10³. Explain why he is wrong, and give the correct sum.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9,150 = 9.150 × 10³</t>
   </si>
   <si>
     <t xml:space="preserve">4.4 Solving Real-World Problems Involving Numbers Expressed in Scientific Notation</t>
@@ -1142,10 +1142,10 @@
 MA.K12.MTR.4.1 Engage in discussions that reflect on the mathematical thinking of self and others.</t>
   </si>
   <si>
-    <t xml:space="preserve">A plan costs 15 dollars plus 4 dollars for each of 6 gigabytes. Another costs 15 dollars for each of 4 lines, plus 6 dollars of tax. Find both totals, and say why the key words could not have told you.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">39 dollars and 66 dollars</t>
+    <t xml:space="preserve">One pizza order costs 13 dollars plus 2 dollars for each of 5 toppings. Another costs 13 dollars for each of 2 pizzas, plus 5 dollars for delivery. Find both totals, and say why the key words could not have told you.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23 dollars and 31 dollars</t>
   </si>
   <si>
     <t xml:space="preserve">4.7 / 4.8 Evaluating Real-World Problems Using the Order of Operations – Parts 1, 2</t>
@@ -5567,7 +5567,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit cbeda99 on 06 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit e613d4b on 07 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="B1" s="2" t="n">
         <f aca="true">TODAY()</f>
-        <v>46301</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="B5" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,$B$44)&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,$B$44))</f>
-        <v>T-A2   Thread A: negative exponents and multiple laws, variable bases (14.3–14.4)</v>
+        <v>3.08   Large numbers in scientific notation</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7198,7 +7198,7 @@
       </c>
       <c r="B6" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$T$2:$T$132,$B$44)&amp;"")</f>
-        <v>I can rewrite an algebraic expression with negative exponents using only positive exponents, and apply several laws of exponents to a monomial expression.</v>
+        <v>I can write a large number in scientific notation, read one back into standard form, and find how many times larger one number is than another.</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7207,7 +7207,7 @@
       </c>
       <c r="B7" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$U$2:$U$132,$B$44)&amp;"")</f>
-        <v>What does a negative exponent on a variable mean, and how do several laws combine in one expression?</v>
+        <v>How does a power of 10 let us write a very large number briefly, and compare two of them?</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7216,7 +7216,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$V$2:$V$132,$B$44)&amp;"")</f>
-        <v>negative exponent law, simplified form</v>
+        <v>scientific notation, standard form, coefficient</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="B9" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$W$2:$W$132,$B$44)&amp;"")</f>
-        <v>8.AR.1.1</v>
+        <v>8.NSO.1.4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="B10" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IF(INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;""="","none",INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;"   — due "&amp;TEXT(INDEX('Scope &amp; Sequence'!$S$2:$S$132,$B$44),"ddd d mmm")))</f>
-        <v>Variables with negative exponents — 2NL; Multiply and divide powers: variable bases — 85P   — due Wed 7 Oct</v>
+        <v>Convert between standard and scientific notation: large numbers — 2AL; Compare large numbers — WEZ; Powers of ten — LJQ   — due Fri 9 Oct</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7243,16 +7243,16 @@
       </c>
       <c r="B11" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IFERROR(INDEX('IXL tracker'!$D$5:$D$86,MATCH(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),'IXL tracker'!$G$5:$G$86,0)),"nothing due"))</f>
-        <v>Multiply powers: variable bases (TR9); Powers of a power: variable bases (2CU); Divide monomials with positive exponents (C8L)</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>Variables with negative exponents (2NL); Multiply and divide powers: variable bases (85P)</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$Z$2:$Z$132,$B$44)&amp;"")</f>
-        <v>How are x³ and x⁻³ related? Explain, and give the value of each when x = 2.</v>
+        <v>Marcus writes 70,000,000 as 70 × 10⁶. Is his expression equal to 70,000,000? Is it scientific notation? Explain.</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7387,49 +7387,49 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="n">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+1)))</f>
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B30" s="6" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+1))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+1)))</f>
-        <v>3.08   Large numbers in scientific notation</v>
+        <v>off   State test — no class</v>
       </c>
       <c r="C30" s="8" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+1))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+1)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+1))&amp;"")))</f>
-        <v>open</v>
+        <v>—</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="n">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+2)))</f>
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B31" s="6" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+2))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+2)))</f>
-        <v>off   State test — no class</v>
+        <v>3.09   Small numbers in scientific notation; how many times larger</v>
       </c>
       <c r="C31" s="8" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+2))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+2)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+2))&amp;"")))</f>
-        <v>—</v>
+        <v>open</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="n">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+3)))</f>
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="B32" s="6" t="str">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+3))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+3)))</f>
-        <v>3.09   Small numbers in scientific notation; how many times larger</v>
+        <v>spiral   Spiral day — mixed retrieval from the unit just finished and the two before it</v>
       </c>
       <c r="C32" s="8" t="str">
         <f aca="false">IF(($B$44+3)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+3))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+3)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+3))&amp;"")))</f>
-        <v>open</v>
+        <v>Unit Review</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+4)))</f>
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B33" s="6" t="str">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+4))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+4)))</f>
@@ -7443,15 +7443,15 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="n">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+5)))</f>
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B34" s="6" t="str">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+5))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+5)))</f>
-        <v>spiral   Spiral day — mixed retrieval from the unit just finished and the two before it</v>
+        <v>3.X1   Unit 3 exam, day 1</v>
       </c>
       <c r="C34" s="8" t="str">
         <f aca="false">IF(($B$44+5)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+5))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+5)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+5))&amp;"")))</f>
-        <v>Unit Review</v>
+        <v>Unit Assessment</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7467,7 +7467,7 @@
       </c>
       <c r="B44" s="13" t="n">
         <f aca="true">IF(TODAY()&gt;$B$45,131+1,MIN(COUNTIF('Scope &amp; Sequence'!$A$2:$A$132,"&lt;"&amp;TODAY())+1,131))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20376,7 +20376,7 @@
       <c r="I12" s="50"/>
       <c r="J12" s="7" t="str">
         <f aca="true">IF(I12="✓","done",IF(TODAY()&lt;B12,"upcoming",IF(TODAY()&lt;G12,"open","due — check scores")))</f>
-        <v>open</v>
+        <v>due — check scores</v>
       </c>
       <c r="K12" s="51"/>
     </row>
@@ -20406,7 +20406,7 @@
       <c r="I13" s="50"/>
       <c r="J13" s="7" t="str">
         <f aca="true">IF(I13="✓","done",IF(TODAY()&lt;B13,"upcoming",IF(TODAY()&lt;G13,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>open</v>
       </c>
       <c r="K13" s="51"/>
     </row>

</xml_diff>

<commit_message>
Ruling 43, second pass: 3.01 board 6, 3.T1 board 2, 3.T2 board 2 and independent 5, 4.02 board 9 get numbers of their own; Units 3 and 4 rebuilt at 0 findings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xYWeLUsuszQH6z7ADE9tj
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -406,7 +406,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to name Marcus's error and Sara's error separately and give 3 × 10⁵. Read the boards, not the papers.</t>
+          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the student has to name Marcus's error and Sara's error separately and give 3 × 10⁸. Read the boards, not the papers.</t>
         </r>
       </text>
     </comment>
@@ -1014,10 +1014,10 @@
     <t xml:space="preserve">product of powers law, quotient of powers law, regrouping a product</t>
   </si>
   <si>
-    <t xml:space="preserve">For (7.2 × 10⁹) ÷ (2.4 × 10⁴), Marcus writes 4.8 × 10⁵ and Sara writes 3 × 10¹³. Name what each one did wrong, and give the correct quotient.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 × 10⁵</t>
+    <t xml:space="preserve">For (7.2 × 10¹¹) ÷ (2.4 × 10³), Marcus writes 4.8 × 10⁸ and Sara writes 3 × 10¹⁴. Name what each one did wrong, and give the correct quotient.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 × 10⁸</t>
   </si>
   <si>
     <t xml:space="preserve">4.2 Multiplying Numbers Expressed in Scientific Notation
@@ -5567,7 +5567,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit e613d4b on 07 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit ec6b272 on 07 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>

</xml_diff>

<commit_message>
A7 Unit 3 test: the last question is cut at Croix's word (he sat the paper: 17:27, did not know it) — 40 points, 20 questions, one transfer item; kit ecff0e2e848e; Unit 3 rebuilt at 0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xYWeLUsuszQH6z7ADE9tj
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -463,7 +463,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2720" uniqueCount="1839">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2716" uniqueCount="1839">
   <si>
     <t xml:space="preserve">A7 — today</t>
   </si>
@@ -5567,7 +5567,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit ec6b272 on 07 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 3eda8d2 on 08 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="B1" s="2" t="n">
         <f aca="true">TODAY()</f>
-        <v>46302</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7189,25 +7189,25 @@
       </c>
       <c r="B5" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,$B$44)&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,$B$44))</f>
-        <v>3.08   Large numbers in scientific notation</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>off   State test — no class</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$T$2:$T$132,$B$44)&amp;"")</f>
-        <v>I can write a large number in scientific notation, read one back into standard form, and find how many times larger one number is than another.</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v/>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$U$2:$U$132,$B$44)&amp;"")</f>
-        <v>How does a power of 10 let us write a very large number briefly, and compare two of them?</v>
+        <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7216,7 +7216,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$V$2:$V$132,$B$44)&amp;"")</f>
-        <v>scientific notation, standard form, coefficient</v>
+        <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7225,34 +7225,34 @@
       </c>
       <c r="B9" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$W$2:$W$132,$B$44)&amp;"")</f>
-        <v>8.NSO.1.4</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IF(INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;""="","none",INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;"   — due "&amp;TEXT(INDEX('Scope &amp; Sequence'!$S$2:$S$132,$B$44),"ddd d mmm")))</f>
-        <v>Convert between standard and scientific notation: large numbers — 2AL; Compare large numbers — WEZ; Powers of ten — LJQ   — due Fri 9 Oct</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>none</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IFERROR(INDEX('IXL tracker'!$D$5:$D$86,MATCH(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),'IXL tracker'!$G$5:$G$86,0)),"nothing due"))</f>
-        <v>Variables with negative exponents (2NL); Multiply and divide powers: variable bases (85P)</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>nothing due</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$Z$2:$Z$132,$B$44)&amp;"")</f>
-        <v>Marcus writes 70,000,000 as 70 × 10⁶. Is his expression equal to 70,000,000? Is it scientific notation? Explain.</v>
+        <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7266,7 +7266,7 @@
       </c>
       <c r="B15" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$B$2:$B$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,$B$44),INDEX('Scope &amp; Sequence'!$F$2:$F$132,$B$44)&amp;"")))</f>
-        <v>open</v>
+        <v>—</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7275,7 +7275,7 @@
       </c>
       <c r="B16" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$C$2:$C$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$C$2:$C$132,$B$44),INDEX('Scope &amp; Sequence'!$G$2:$G$132,$B$44)&amp;"")))</f>
-        <v>open</v>
+        <v>—</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="B17" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$D$2:$D$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$D$2:$D$132,$B$44),INDEX('Scope &amp; Sequence'!$H$2:$H$132,$B$44)&amp;"")))</f>
-        <v>open</v>
+        <v>—</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7293,7 +7293,7 @@
       </c>
       <c r="B18" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$E$2:$E$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$E$2:$E$132,$B$44),INDEX('Scope &amp; Sequence'!$I$2:$I$132,$B$44)&amp;"")))</f>
-        <v>open</v>
+        <v>—</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="B19" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$F$2:$F$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$F$2:$F$132,$B$44),INDEX('Scope &amp; Sequence'!$J$2:$J$132,$B$44)&amp;"")))</f>
-        <v>open</v>
+        <v>—</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="B20" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$G$2:$G$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$G$2:$G$132,$B$44),INDEX('Scope &amp; Sequence'!$K$2:$K$132,$B$44)&amp;"")))</f>
-        <v>key</v>
+        <v>—</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="B21" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$H$2:$H$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$H$2:$H$132,$B$44),INDEX('Scope &amp; Sequence'!$L$2:$L$132,$B$44)&amp;"")))</f>
-        <v>open</v>
+        <v>—</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7329,7 +7329,7 @@
       </c>
       <c r="B22" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$I$2:$I$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$I$2:$I$132,$B$44),INDEX('Scope &amp; Sequence'!$M$2:$M$132,$B$44)&amp;"")))</f>
-        <v>key</v>
+        <v>—</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="B23" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$J$2:$J$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$J$2:$J$132,$B$44),INDEX('Scope &amp; Sequence'!$N$2:$N$132,$B$44)&amp;"")))</f>
-        <v>open</v>
+        <v>—</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7347,7 +7347,7 @@
       </c>
       <c r="B24" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$K$2:$K$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$K$2:$K$132,$B$44),INDEX('Scope &amp; Sequence'!$O$2:$O$132,$B$44)&amp;"")))</f>
-        <v>key</v>
+        <v>—</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7365,7 +7365,7 @@
       </c>
       <c r="B26" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$M$2:$M$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$M$2:$M$132,$B$44),INDEX('Scope &amp; Sequence'!$Q$2:$Q$132,$B$44)&amp;"")))</f>
-        <v>search</v>
+        <v>—</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7387,35 +7387,35 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="n">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+1)))</f>
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B30" s="6" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+1))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+1)))</f>
-        <v>off   State test — no class</v>
+        <v>3.09   Small numbers in scientific notation; how many times larger</v>
       </c>
       <c r="C30" s="8" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+1))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+1)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+1))&amp;"")))</f>
-        <v>—</v>
+        <v>open</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="n">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+2)))</f>
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="B31" s="6" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+2))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+2)))</f>
-        <v>3.09   Small numbers in scientific notation; how many times larger</v>
+        <v>spiral   Spiral day — mixed retrieval from the unit just finished and the two before it</v>
       </c>
       <c r="C31" s="8" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+2))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+2)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+2))&amp;"")))</f>
-        <v>open</v>
+        <v>Unit Review</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="n">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+3)))</f>
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B32" s="6" t="str">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+3))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+3)))</f>
@@ -7429,25 +7429,25 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+4)))</f>
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B33" s="6" t="str">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+4))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+4)))</f>
-        <v>spiral   Spiral day — mixed retrieval from the unit just finished and the two before it</v>
+        <v>3.X1   Unit 3 exam, day 1</v>
       </c>
       <c r="C33" s="8" t="str">
         <f aca="false">IF(($B$44+4)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+4))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+4)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+4))&amp;"")))</f>
-        <v>Unit Review</v>
+        <v>Unit Assessment</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="n">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+5)))</f>
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B34" s="6" t="str">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+5))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+5)))</f>
-        <v>3.X1   Unit 3 exam, day 1</v>
+        <v>3.X2   Unit 3 exam, day 2</v>
       </c>
       <c r="C34" s="8" t="str">
         <f aca="false">IF(($B$44+5)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+5))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+5)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+5))&amp;"")))</f>
@@ -7467,7 +7467,7 @@
       </c>
       <c r="B44" s="13" t="n">
         <f aca="true">IF(TODAY()&gt;$B$45,131+1,MIN(COUNTIF('Scope &amp; Sequence'!$A$2:$A$132,"&lt;"&amp;TODAY())+1,131))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23082,7 +23082,7 @@
       </c>
       <c r="J11" s="47" t="n">
         <f aca="false">IF(SUMIF('Unit tests'!$E:$E,A11,'Unit tests'!$C:$C)=0,"",SUMIF('Unit tests'!$E:$E,A11,'Unit tests'!$C:$C))</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K11" s="6" t="s">
         <v>975</v>
@@ -24796,7 +24796,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12"/>
@@ -24915,8 +24915,8 @@
         <v>46311</v>
       </c>
       <c r="D6" s="47" t="n">
-        <f aca="false">C46</f>
-        <v>41</v>
+        <f aca="false">C45</f>
+        <v>40</v>
       </c>
       <c r="E6" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$12,"open")</f>
@@ -24950,7 +24950,7 @@
         <v>46325</v>
       </c>
       <c r="D7" s="47" t="n">
-        <f aca="false">C70</f>
+        <f aca="false">C69</f>
         <v>34</v>
       </c>
       <c r="E7" s="8" t="str">
@@ -25287,12 +25287,12 @@
         <v>955</v>
       </c>
       <c r="J25" s="47" t="n">
-        <f aca="false">SUMIF($E$25:$E$45,I25,$C$25:$C$45)</f>
+        <f aca="false">SUMIF($E$25:$E$44,I25,$C$25:$C$44)</f>
         <v>9</v>
       </c>
       <c r="K25" s="55" t="n">
-        <f aca="false">J25/$C$46</f>
-        <v>0.219512195121951</v>
+        <f aca="false">J25/$C$45</f>
+        <v>0.225</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25319,12 +25319,12 @@
         <v>961</v>
       </c>
       <c r="J26" s="47" t="n">
-        <f aca="false">SUMIF($E$25:$E$45,I26,$C$25:$C$45)</f>
+        <f aca="false">SUMIF($E$25:$E$44,I26,$C$25:$C$44)</f>
         <v>11</v>
       </c>
       <c r="K26" s="55" t="n">
-        <f aca="false">J26/$C$46</f>
-        <v>0.268292682926829</v>
+        <f aca="false">J26/$C$45</f>
+        <v>0.275</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25349,12 +25349,12 @@
         <v>966</v>
       </c>
       <c r="J27" s="47" t="n">
-        <f aca="false">SUMIF($E$25:$E$45,I27,$C$25:$C$45)</f>
+        <f aca="false">SUMIF($E$25:$E$44,I27,$C$25:$C$44)</f>
         <v>9</v>
       </c>
       <c r="K27" s="55" t="n">
-        <f aca="false">J27/$C$46</f>
-        <v>0.219512195121951</v>
+        <f aca="false">J27/$C$45</f>
+        <v>0.225</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25379,12 +25379,12 @@
         <v>972</v>
       </c>
       <c r="J28" s="47" t="n">
-        <f aca="false">SUMIF($E$25:$E$45,I28,$C$25:$C$45)</f>
-        <v>12</v>
+        <f aca="false">SUMIF($E$25:$E$44,I28,$C$25:$C$44)</f>
+        <v>11</v>
       </c>
       <c r="K28" s="55" t="n">
-        <f aca="false">J28/$C$46</f>
-        <v>0.292682926829268</v>
+        <f aca="false">J28/$C$45</f>
+        <v>0.275</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25708,80 +25708,91 @@
       <c r="G44" s="47"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="47" t="n">
-        <v>21</v>
-      </c>
-      <c r="B45" s="47"/>
-      <c r="C45" s="47" t="n">
+      <c r="B45" s="5" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C45" s="56" t="n">
+        <f aca="false">SUM(C25:C44)</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>1252</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="12" t="s">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>1236</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>1208</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>1237</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>1238</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>1239</v>
+      </c>
+      <c r="I50" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="J50" s="54" t="s">
+        <v>1208</v>
+      </c>
+      <c r="K50" s="54" t="s">
+        <v>1240</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="D45" s="7" t="s">
-        <v>1249</v>
-      </c>
-      <c r="E45" s="7" t="s">
-        <v>972</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>1245</v>
-      </c>
-      <c r="G45" s="47" t="s">
-        <v>1247</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="5" t="s">
-        <v>1251</v>
-      </c>
-      <c r="C46" s="56" t="n">
-        <f aca="false">SUM(C25:C45)</f>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="s">
-        <v>1252</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="12" t="s">
-        <v>1234</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="9" t="s">
-        <v>1235</v>
-      </c>
-      <c r="B51" s="9" t="s">
+      <c r="B51" s="47" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C51" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>1253</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="F51" s="7" t="s">
         <v>1236</v>
       </c>
-      <c r="C51" s="9" t="s">
-        <v>1208</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>1237</v>
-      </c>
-      <c r="E51" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>1238</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>1239</v>
-      </c>
-      <c r="I51" s="54" t="s">
-        <v>6</v>
-      </c>
-      <c r="J51" s="54" t="s">
-        <v>1208</v>
-      </c>
-      <c r="K51" s="54" t="s">
-        <v>1240</v>
+      <c r="G51" s="47"/>
+      <c r="I51" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="J51" s="47" t="n">
+        <f aca="false">SUMIF($E$51:$E$68,I51,$C$51:$C$68)</f>
+        <v>12</v>
+      </c>
+      <c r="K51" s="55" t="n">
+        <f aca="false">J51/$C$69</f>
+        <v>0.352941176470588</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B52" s="47" t="s">
         <v>1241</v>
@@ -25800,26 +25811,24 @@
       </c>
       <c r="G52" s="47"/>
       <c r="I52" s="7" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="J52" s="47" t="n">
-        <f aca="false">SUMIF($E$52:$E$69,I52,$C$52:$C$69)</f>
-        <v>12</v>
+        <f aca="false">SUMIF($E$51:$E$68,I52,$C$51:$C$68)</f>
+        <v>9</v>
       </c>
       <c r="K52" s="55" t="n">
-        <f aca="false">J52/$C$70</f>
-        <v>0.352941176470588</v>
+        <f aca="false">J52/$C$69</f>
+        <v>0.264705882352941</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="47" t="n">
-        <v>2</v>
-      </c>
-      <c r="B53" s="47" t="s">
-        <v>1241</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B53" s="47"/>
       <c r="C53" s="47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D53" s="7" t="s">
         <v>1253</v>
@@ -25828,24 +25837,24 @@
         <v>976</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>1236</v>
+        <v>1244</v>
       </c>
       <c r="G53" s="47"/>
       <c r="I53" s="7" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="J53" s="47" t="n">
-        <f aca="false">SUMIF($E$52:$E$69,I53,$C$52:$C$69)</f>
-        <v>9</v>
+        <f aca="false">SUMIF($E$51:$E$68,I53,$C$51:$C$68)</f>
+        <v>13</v>
       </c>
       <c r="K53" s="55" t="n">
-        <f aca="false">J53/$C$70</f>
-        <v>0.264705882352941</v>
+        <f aca="false">J53/$C$69</f>
+        <v>0.382352941176471</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B54" s="47"/>
       <c r="C54" s="47" t="n">
@@ -25861,21 +25870,10 @@
         <v>1244</v>
       </c>
       <c r="G54" s="47"/>
-      <c r="I54" s="7" t="s">
-        <v>986</v>
-      </c>
-      <c r="J54" s="47" t="n">
-        <f aca="false">SUMIF($E$52:$E$69,I54,$C$52:$C$69)</f>
-        <v>13</v>
-      </c>
-      <c r="K54" s="55" t="n">
-        <f aca="false">J54/$C$70</f>
-        <v>0.382352941176471</v>
-      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="47" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B55" s="47"/>
       <c r="C55" s="47" t="n">
@@ -25888,13 +25886,13 @@
         <v>976</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="G55" s="47"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B56" s="47"/>
       <c r="C56" s="47" t="n">
@@ -25909,38 +25907,40 @@
       <c r="F56" s="7" t="s">
         <v>1245</v>
       </c>
-      <c r="G56" s="47"/>
+      <c r="G56" s="47" t="s">
+        <v>1247</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="47" t="n">
-        <v>6</v>
-      </c>
-      <c r="B57" s="47"/>
+        <v>7</v>
+      </c>
+      <c r="B57" s="47" t="s">
+        <v>1243</v>
+      </c>
       <c r="C57" s="47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>1245</v>
-      </c>
-      <c r="G57" s="47" t="s">
-        <v>1247</v>
-      </c>
+        <v>1236</v>
+      </c>
+      <c r="G57" s="47"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B58" s="47" t="s">
-        <v>1243</v>
+        <v>1250</v>
       </c>
       <c r="C58" s="47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D58" s="7" t="s">
         <v>1254</v>
@@ -25955,7 +25955,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B59" s="47" t="s">
         <v>1250</v>
@@ -25976,13 +25976,11 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="47" t="n">
-        <v>9</v>
-      </c>
-      <c r="B60" s="47" t="s">
-        <v>1250</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B60" s="47"/>
       <c r="C60" s="47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D60" s="7" t="s">
         <v>1254</v>
@@ -25991,13 +25989,13 @@
         <v>982</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>1236</v>
+        <v>1245</v>
       </c>
       <c r="G60" s="47"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B61" s="47"/>
       <c r="C61" s="47" t="n">
@@ -26010,38 +26008,40 @@
         <v>982</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="G61" s="47"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="47" t="n">
-        <v>11</v>
-      </c>
-      <c r="B62" s="47"/>
+        <v>12</v>
+      </c>
+      <c r="B62" s="47" t="s">
+        <v>1241</v>
+      </c>
       <c r="C62" s="47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D62" s="7" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>1244</v>
+        <v>1236</v>
       </c>
       <c r="G62" s="47"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="47" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B63" s="47" t="s">
-        <v>1241</v>
+        <v>1243</v>
       </c>
       <c r="C63" s="47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D63" s="7" t="s">
         <v>1255</v>
@@ -26056,13 +26056,13 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="47" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B64" s="47" t="s">
-        <v>1243</v>
+        <v>1250</v>
       </c>
       <c r="C64" s="47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D64" s="7" t="s">
         <v>1255</v>
@@ -26077,13 +26077,11 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="47" t="n">
-        <v>14</v>
-      </c>
-      <c r="B65" s="47" t="s">
-        <v>1250</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="B65" s="47"/>
       <c r="C65" s="47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D65" s="7" t="s">
         <v>1255</v>
@@ -26092,13 +26090,13 @@
         <v>986</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>1236</v>
+        <v>1244</v>
       </c>
       <c r="G65" s="47"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="47" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B66" s="47"/>
       <c r="C66" s="47" t="n">
@@ -26117,7 +26115,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="47" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B67" s="47"/>
       <c r="C67" s="47" t="n">
@@ -26130,13 +26128,13 @@
         <v>986</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="G67" s="47"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="47" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B68" s="47"/>
       <c r="C68" s="47" t="n">
@@ -26151,35 +26149,16 @@
       <c r="F68" s="7" t="s">
         <v>1245</v>
       </c>
-      <c r="G68" s="47"/>
+      <c r="G68" s="47" t="s">
+        <v>1247</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="47" t="n">
-        <v>18</v>
-      </c>
-      <c r="B69" s="47"/>
-      <c r="C69" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D69" s="7" t="s">
-        <v>1255</v>
-      </c>
-      <c r="E69" s="7" t="s">
-        <v>986</v>
-      </c>
-      <c r="F69" s="7" t="s">
-        <v>1245</v>
-      </c>
-      <c r="G69" s="47" t="s">
-        <v>1247</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B70" s="5" t="s">
+      <c r="B69" s="5" t="s">
         <v>1251</v>
       </c>
-      <c r="C70" s="56" t="n">
-        <f aca="false">SUM(C52:C69)</f>
+      <c r="C69" s="56" t="n">
+        <f aca="false">SUM(C51:C68)</f>
         <v>34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
A7 Unit 3 test: the four questions answered in a sentence are cut at Croix's word — 36 points, 16 questions, no transfer item (the key says so); START HERE dates the two thread days; kit 6c8dd856e5c1; Unit 3 rebuilt at 0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xYWeLUsuszQH6z7ADE9tj
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -463,7 +463,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2716" uniqueCount="1839">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2703" uniqueCount="1839">
   <si>
     <t xml:space="preserve">A7 — today</t>
   </si>
@@ -4344,25 +4344,25 @@
     <t xml:space="preserve">Integer Exponents</t>
   </si>
   <si>
+    <t xml:space="preserve">Variable Bases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scientific Notation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a–b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit 4 test — question map</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operations in Scientific Notation</t>
+  </si>
+  <si>
     <t xml:space="preserve">yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variable Bases</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scientific Notation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a–b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unit 4 test — question map</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operations in Scientific Notation</t>
   </si>
   <si>
     <t xml:space="preserve">Real-World Problems and Significant Digits</t>
@@ -5567,7 +5567,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 3eda8d2 on 08 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit ada85db on 08 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -23012,7 +23012,7 @@
       </c>
       <c r="J9" s="47" t="n">
         <f aca="false">IF(SUMIF('Unit tests'!$E:$E,A9,'Unit tests'!$C:$C)=0,"",SUMIF('Unit tests'!$E:$E,A9,'Unit tests'!$C:$C))</f>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K9" s="6" t="s">
         <v>965</v>
@@ -23048,7 +23048,7 @@
       </c>
       <c r="J10" s="47" t="n">
         <f aca="false">IF(SUMIF('Unit tests'!$E:$E,A10,'Unit tests'!$C:$C)=0,"",SUMIF('Unit tests'!$E:$E,A10,'Unit tests'!$C:$C))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K10" s="6" t="s">
         <v>878</v>
@@ -23082,7 +23082,7 @@
       </c>
       <c r="J11" s="47" t="n">
         <f aca="false">IF(SUMIF('Unit tests'!$E:$E,A11,'Unit tests'!$C:$C)=0,"",SUMIF('Unit tests'!$E:$E,A11,'Unit tests'!$C:$C))</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K11" s="6" t="s">
         <v>975</v>
@@ -24796,7 +24796,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12"/>
@@ -24915,8 +24915,8 @@
         <v>46311</v>
       </c>
       <c r="D6" s="47" t="n">
-        <f aca="false">C45</f>
-        <v>40</v>
+        <f aca="false">C41</f>
+        <v>36</v>
       </c>
       <c r="E6" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$12,"open")</f>
@@ -24950,7 +24950,7 @@
         <v>46325</v>
       </c>
       <c r="D7" s="47" t="n">
-        <f aca="false">C69</f>
+        <f aca="false">C65</f>
         <v>34</v>
       </c>
       <c r="E7" s="8" t="str">
@@ -25287,12 +25287,12 @@
         <v>955</v>
       </c>
       <c r="J25" s="47" t="n">
-        <f aca="false">SUMIF($E$25:$E$44,I25,$C$25:$C$44)</f>
+        <f aca="false">SUMIF($E$25:$E$40,I25,$C$25:$C$40)</f>
         <v>9</v>
       </c>
       <c r="K25" s="55" t="n">
-        <f aca="false">J25/$C$45</f>
-        <v>0.225</v>
+        <f aca="false">J25/$C$41</f>
+        <v>0.25</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25319,12 +25319,12 @@
         <v>961</v>
       </c>
       <c r="J26" s="47" t="n">
-        <f aca="false">SUMIF($E$25:$E$44,I26,$C$25:$C$44)</f>
-        <v>11</v>
+        <f aca="false">SUMIF($E$25:$E$40,I26,$C$25:$C$40)</f>
+        <v>9</v>
       </c>
       <c r="K26" s="55" t="n">
-        <f aca="false">J26/$C$45</f>
-        <v>0.275</v>
+        <f aca="false">J26/$C$41</f>
+        <v>0.25</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25349,12 +25349,12 @@
         <v>966</v>
       </c>
       <c r="J27" s="47" t="n">
-        <f aca="false">SUMIF($E$25:$E$44,I27,$C$25:$C$44)</f>
-        <v>9</v>
+        <f aca="false">SUMIF($E$25:$E$40,I27,$C$25:$C$40)</f>
+        <v>8</v>
       </c>
       <c r="K27" s="55" t="n">
-        <f aca="false">J27/$C$45</f>
-        <v>0.225</v>
+        <f aca="false">J27/$C$41</f>
+        <v>0.222222222222222</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25379,12 +25379,12 @@
         <v>972</v>
       </c>
       <c r="J28" s="47" t="n">
-        <f aca="false">SUMIF($E$25:$E$44,I28,$C$25:$C$44)</f>
-        <v>11</v>
+        <f aca="false">SUMIF($E$25:$E$40,I28,$C$25:$C$40)</f>
+        <v>10</v>
       </c>
       <c r="K28" s="55" t="n">
-        <f aca="false">J28/$C$45</f>
-        <v>0.275</v>
+        <f aca="false">J28/$C$41</f>
+        <v>0.277777777777778</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25471,18 +25471,20 @@
       <c r="A33" s="47" t="n">
         <v>9</v>
       </c>
-      <c r="B33" s="47"/>
+      <c r="B33" s="47" t="s">
+        <v>1241</v>
+      </c>
       <c r="C33" s="47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>961</v>
+        <v>966</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>1245</v>
+        <v>1236</v>
       </c>
       <c r="G33" s="47"/>
     </row>
@@ -25490,41 +25492,39 @@
       <c r="A34" s="47" t="n">
         <v>10</v>
       </c>
-      <c r="B34" s="47"/>
+      <c r="B34" s="47" t="s">
+        <v>1243</v>
+      </c>
       <c r="C34" s="47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>961</v>
+        <v>966</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>1245</v>
-      </c>
-      <c r="G34" s="47" t="s">
-        <v>1247</v>
-      </c>
+        <v>1236</v>
+      </c>
+      <c r="G34" s="47"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="47" t="n">
         <v>11</v>
       </c>
-      <c r="B35" s="47" t="s">
-        <v>1241</v>
-      </c>
+      <c r="B35" s="47"/>
       <c r="C35" s="47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>966</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>1236</v>
+        <v>1244</v>
       </c>
       <c r="G35" s="47"/>
     </row>
@@ -25533,16 +25533,16 @@
         <v>12</v>
       </c>
       <c r="B36" s="47" t="s">
-        <v>1243</v>
+        <v>1241</v>
       </c>
       <c r="C36" s="47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>1248</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>1236</v>
@@ -25553,18 +25553,20 @@
       <c r="A37" s="47" t="n">
         <v>13</v>
       </c>
-      <c r="B37" s="47"/>
+      <c r="B37" s="47" t="s">
+        <v>1249</v>
+      </c>
       <c r="C37" s="47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>1248</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>1244</v>
+        <v>1236</v>
       </c>
       <c r="G37" s="47"/>
     </row>
@@ -25580,10 +25582,10 @@
         <v>1248</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="G38" s="47"/>
     </row>
@@ -25592,13 +25594,13 @@
         <v>15</v>
       </c>
       <c r="B39" s="47" t="s">
-        <v>1241</v>
+        <v>1249</v>
       </c>
       <c r="C39" s="47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>972</v>
@@ -25612,314 +25614,314 @@
       <c r="A40" s="47" t="n">
         <v>16</v>
       </c>
-      <c r="B40" s="47" t="s">
-        <v>1250</v>
-      </c>
+      <c r="B40" s="47"/>
       <c r="C40" s="47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="E40" s="7" t="s">
         <v>972</v>
       </c>
       <c r="F40" s="7" t="s">
+        <v>1245</v>
+      </c>
+      <c r="G40" s="47"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="5" t="s">
+        <v>1250</v>
+      </c>
+      <c r="C41" s="56" t="n">
+        <f aca="false">SUM(C25:C40)</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>1251</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="12" t="s">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B46" s="9" t="s">
         <v>1236</v>
       </c>
-      <c r="G40" s="47"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="47" t="n">
-        <v>17</v>
-      </c>
-      <c r="B41" s="47"/>
-      <c r="C41" s="47" t="n">
+      <c r="C46" s="9" t="s">
+        <v>1208</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>1237</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>1238</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>1239</v>
+      </c>
+      <c r="I46" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="J46" s="54" t="s">
+        <v>1208</v>
+      </c>
+      <c r="K46" s="54" t="s">
+        <v>1240</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="7" t="s">
-        <v>1249</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>972</v>
-      </c>
-      <c r="F41" s="7" t="s">
+      <c r="B47" s="47" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C47" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>1252</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>1236</v>
+      </c>
+      <c r="G47" s="47"/>
+      <c r="I47" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="J47" s="47" t="n">
+        <f aca="false">SUMIF($E$47:$E$64,I47,$C$47:$C$64)</f>
+        <v>12</v>
+      </c>
+      <c r="K47" s="55" t="n">
+        <f aca="false">J47/$C$65</f>
+        <v>0.352941176470588</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="47" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C48" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>1252</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>1236</v>
+      </c>
+      <c r="G48" s="47"/>
+      <c r="I48" s="7" t="s">
+        <v>982</v>
+      </c>
+      <c r="J48" s="47" t="n">
+        <f aca="false">SUMIF($E$47:$E$64,I48,$C$47:$C$64)</f>
+        <v>9</v>
+      </c>
+      <c r="K48" s="55" t="n">
+        <f aca="false">J48/$C$65</f>
+        <v>0.264705882352941</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="B49" s="47"/>
+      <c r="C49" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>1252</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="F49" s="7" t="s">
         <v>1244</v>
       </c>
-      <c r="G41" s="47"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="47" t="n">
-        <v>18</v>
-      </c>
-      <c r="B42" s="47" t="s">
-        <v>1250</v>
-      </c>
-      <c r="C42" s="47" t="n">
-        <v>2</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>1249</v>
-      </c>
-      <c r="E42" s="7" t="s">
-        <v>972</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>1236</v>
-      </c>
-      <c r="G42" s="47"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="47" t="n">
-        <v>19</v>
-      </c>
-      <c r="B43" s="47"/>
-      <c r="C43" s="47" t="n">
+      <c r="G49" s="47"/>
+      <c r="I49" s="7" t="s">
+        <v>986</v>
+      </c>
+      <c r="J49" s="47" t="n">
+        <f aca="false">SUMIF($E$47:$E$64,I49,$C$47:$C$64)</f>
+        <v>13</v>
+      </c>
+      <c r="K49" s="55" t="n">
+        <f aca="false">J49/$C$65</f>
+        <v>0.382352941176471</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="B50" s="47"/>
+      <c r="C50" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="D43" s="7" t="s">
-        <v>1249</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>972</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>1245</v>
-      </c>
-      <c r="G43" s="47"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="47" t="n">
-        <v>20</v>
-      </c>
-      <c r="B44" s="47"/>
-      <c r="C44" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>1249</v>
-      </c>
-      <c r="E44" s="7" t="s">
-        <v>972</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>1245</v>
-      </c>
-      <c r="G44" s="47"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="5" t="s">
-        <v>1251</v>
-      </c>
-      <c r="C45" s="56" t="n">
-        <f aca="false">SUM(C25:C44)</f>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
+      <c r="D50" s="7" t="s">
         <v>1252</v>
       </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="12" t="s">
-        <v>1234</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="9" t="s">
-        <v>1235</v>
-      </c>
-      <c r="B50" s="9" t="s">
-        <v>1236</v>
-      </c>
-      <c r="C50" s="9" t="s">
-        <v>1208</v>
-      </c>
-      <c r="D50" s="9" t="s">
-        <v>1237</v>
-      </c>
-      <c r="E50" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F50" s="9" t="s">
-        <v>1238</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>1239</v>
-      </c>
-      <c r="I50" s="54" t="s">
-        <v>6</v>
-      </c>
-      <c r="J50" s="54" t="s">
-        <v>1208</v>
-      </c>
-      <c r="K50" s="54" t="s">
-        <v>1240</v>
-      </c>
+      <c r="E50" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>1244</v>
+      </c>
+      <c r="G50" s="47"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="47" t="n">
+        <v>5</v>
+      </c>
+      <c r="B51" s="47"/>
+      <c r="C51" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="B51" s="47" t="s">
-        <v>1241</v>
-      </c>
-      <c r="C51" s="47" t="n">
-        <v>4</v>
-      </c>
       <c r="D51" s="7" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E51" s="7" t="s">
         <v>976</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>1236</v>
+        <v>1245</v>
       </c>
       <c r="G51" s="47"/>
-      <c r="I51" s="7" t="s">
-        <v>976</v>
-      </c>
-      <c r="J51" s="47" t="n">
-        <f aca="false">SUMIF($E$51:$E$68,I51,$C$51:$C$68)</f>
-        <v>12</v>
-      </c>
-      <c r="K51" s="55" t="n">
-        <f aca="false">J51/$C$69</f>
-        <v>0.352941176470588</v>
-      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="47" t="n">
-        <v>2</v>
-      </c>
-      <c r="B52" s="47" t="s">
-        <v>1241</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B52" s="47"/>
       <c r="C52" s="47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D52" s="7" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E52" s="7" t="s">
         <v>976</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>1236</v>
-      </c>
-      <c r="G52" s="47"/>
-      <c r="I52" s="7" t="s">
-        <v>982</v>
-      </c>
-      <c r="J52" s="47" t="n">
-        <f aca="false">SUMIF($E$51:$E$68,I52,$C$51:$C$68)</f>
-        <v>9</v>
-      </c>
-      <c r="K52" s="55" t="n">
-        <f aca="false">J52/$C$69</f>
-        <v>0.264705882352941</v>
+        <v>1245</v>
+      </c>
+      <c r="G52" s="47" t="s">
+        <v>1253</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="47" t="n">
+        <v>7</v>
+      </c>
+      <c r="B53" s="47" t="s">
+        <v>1243</v>
+      </c>
+      <c r="C53" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="B53" s="47"/>
-      <c r="C53" s="47" t="n">
-        <v>1</v>
-      </c>
       <c r="D53" s="7" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>1244</v>
+        <v>1236</v>
       </c>
       <c r="G53" s="47"/>
-      <c r="I53" s="7" t="s">
-        <v>986</v>
-      </c>
-      <c r="J53" s="47" t="n">
-        <f aca="false">SUMIF($E$51:$E$68,I53,$C$51:$C$68)</f>
-        <v>13</v>
-      </c>
-      <c r="K53" s="55" t="n">
-        <f aca="false">J53/$C$69</f>
-        <v>0.382352941176471</v>
-      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="47" t="n">
-        <v>4</v>
-      </c>
-      <c r="B54" s="47"/>
+        <v>8</v>
+      </c>
+      <c r="B54" s="47" t="s">
+        <v>1249</v>
+      </c>
       <c r="C54" s="47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>1244</v>
+        <v>1236</v>
       </c>
       <c r="G54" s="47"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="47" t="n">
-        <v>5</v>
-      </c>
-      <c r="B55" s="47"/>
+        <v>9</v>
+      </c>
+      <c r="B55" s="47" t="s">
+        <v>1249</v>
+      </c>
       <c r="C55" s="47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>1245</v>
+        <v>1236</v>
       </c>
       <c r="G55" s="47"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="47" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B56" s="47"/>
       <c r="C56" s="47" t="n">
         <v>1</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>1245</v>
       </c>
-      <c r="G56" s="47" t="s">
-        <v>1247</v>
-      </c>
+      <c r="G56" s="47"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="47" t="n">
-        <v>7</v>
-      </c>
-      <c r="B57" s="47" t="s">
-        <v>1243</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B57" s="47"/>
       <c r="C57" s="47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D57" s="7" t="s">
         <v>1254</v>
@@ -25928,25 +25930,25 @@
         <v>982</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>1236</v>
+        <v>1244</v>
       </c>
       <c r="G57" s="47"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="47" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B58" s="47" t="s">
-        <v>1250</v>
+        <v>1241</v>
       </c>
       <c r="C58" s="47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>1236</v>
@@ -25955,19 +25957,19 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="47" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B59" s="47" t="s">
-        <v>1250</v>
+        <v>1243</v>
       </c>
       <c r="C59" s="47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>1236</v>
@@ -25976,36 +25978,38 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="47" t="n">
-        <v>10</v>
-      </c>
-      <c r="B60" s="47"/>
+        <v>14</v>
+      </c>
+      <c r="B60" s="47" t="s">
+        <v>1249</v>
+      </c>
       <c r="C60" s="47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>1245</v>
+        <v>1236</v>
       </c>
       <c r="G60" s="47"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="47" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B61" s="47"/>
       <c r="C61" s="47" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>1244</v>
@@ -26014,13 +26018,11 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="47" t="n">
-        <v>12</v>
-      </c>
-      <c r="B62" s="47" t="s">
-        <v>1241</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B62" s="47"/>
       <c r="C62" s="47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D62" s="7" t="s">
         <v>1255</v>
@@ -26029,19 +26031,17 @@
         <v>986</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>1236</v>
+        <v>1244</v>
       </c>
       <c r="G62" s="47"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="47" t="n">
-        <v>13</v>
-      </c>
-      <c r="B63" s="47" t="s">
-        <v>1243</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="B63" s="47"/>
       <c r="C63" s="47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D63" s="7" t="s">
         <v>1255</v>
@@ -26050,19 +26050,17 @@
         <v>986</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>1236</v>
+        <v>1245</v>
       </c>
       <c r="G63" s="47"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="47" t="n">
-        <v>14</v>
-      </c>
-      <c r="B64" s="47" t="s">
-        <v>1250</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="B64" s="47"/>
       <c r="C64" s="47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64" s="7" t="s">
         <v>1255</v>
@@ -26071,94 +26069,18 @@
         <v>986</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>1236</v>
-      </c>
-      <c r="G64" s="47"/>
+        <v>1245</v>
+      </c>
+      <c r="G64" s="47" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="47" t="n">
-        <v>15</v>
-      </c>
-      <c r="B65" s="47"/>
-      <c r="C65" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="7" t="s">
-        <v>1255</v>
-      </c>
-      <c r="E65" s="7" t="s">
-        <v>986</v>
-      </c>
-      <c r="F65" s="7" t="s">
-        <v>1244</v>
-      </c>
-      <c r="G65" s="47"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="47" t="n">
-        <v>16</v>
-      </c>
-      <c r="B66" s="47"/>
-      <c r="C66" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="7" t="s">
-        <v>1255</v>
-      </c>
-      <c r="E66" s="7" t="s">
-        <v>986</v>
-      </c>
-      <c r="F66" s="7" t="s">
-        <v>1244</v>
-      </c>
-      <c r="G66" s="47"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="47" t="n">
-        <v>17</v>
-      </c>
-      <c r="B67" s="47"/>
-      <c r="C67" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="7" t="s">
-        <v>1255</v>
-      </c>
-      <c r="E67" s="7" t="s">
-        <v>986</v>
-      </c>
-      <c r="F67" s="7" t="s">
-        <v>1245</v>
-      </c>
-      <c r="G67" s="47"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="47" t="n">
-        <v>18</v>
-      </c>
-      <c r="B68" s="47"/>
-      <c r="C68" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D68" s="7" t="s">
-        <v>1255</v>
-      </c>
-      <c r="E68" s="7" t="s">
-        <v>986</v>
-      </c>
-      <c r="F68" s="7" t="s">
-        <v>1245</v>
-      </c>
-      <c r="G68" s="47" t="s">
-        <v>1247</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="5" t="s">
-        <v>1251</v>
-      </c>
-      <c r="C69" s="56" t="n">
-        <f aca="false">SUM(C51:C68)</f>
+      <c r="B65" s="5" t="s">
+        <v>1250</v>
+      </c>
+      <c r="C65" s="56" t="n">
+        <f aca="false">SUM(C47:C64)</f>
         <v>34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Windmill 077e6ff vendored: the vocabulary slide (after the warm-up answers, before Notes; L['vocab'] drives it) and deckkit.choices laying out any count of math options; Unit 4 rebuilt and reinstalled at 0 findings
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7ovt6yLjh6QuFV9HBMV4N
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -5557,7 +5557,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 972a435e on 16 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 2ada52dd on 17 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -7161,7 +7161,7 @@
       </c>
       <c r="B1" s="2" t="n">
         <f aca="true">TODAY()</f>
-        <v>46311</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="B3" s="4" t="str">
         <f aca="true">IF($B$44&gt;131,"The school year has ended.",IF(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44)=TODAY(),"Today's class",IF(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44)&lt;TODAY(),"The PM3 window (3–28 May)","Next class: "&amp;TEXT(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),"dddd d mmmm"))))</f>
-        <v>Today's class</v>
+        <v>Next class: Monday 19 October</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="B5" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,$B$44)&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,$B$44))</f>
-        <v>4.01   Add and subtract in scientific notation</v>
+        <v>4.02+03   Multiply and divide in scientific notation</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7188,16 +7188,16 @@
       </c>
       <c r="B6" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$T$2:$T$132,$B$44)&amp;"")</f>
-        <v>I can add and subtract two numbers written in scientific notation, and write the answer in scientific notation.</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>I can multiply and divide two numbers written in scientific notation, and write the answer in scientific notation.</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$U$2:$U$132,$B$44)&amp;"")</f>
-        <v>Why must two numbers written in scientific notation carry the same power of ten before they can be added?</v>
+        <v>Why must the powers of ten match to add, but not to multiply?</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7206,7 +7206,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$V$2:$V$132,$B$44)&amp;"")</f>
-        <v>scientific notation, coefficient, common power of ten</v>
+        <v>product of powers law, quotient of powers law, regrouping a product</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7218,13 +7218,13 @@
         <v>8.NSO.1.5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IF(INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;""="","none",INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;"   — due "&amp;TEXT(INDEX('Scope &amp; Sequence'!$S$2:$S$132,$B$44),"ddd d mmm")))</f>
-        <v>Add and subtract numbers written in scientific notation — HUR   — due Mon 19 Oct</v>
+        <v>Multiply numbers written in scientific notation — YZU; Divide numbers written in scientific notation — SGT   — due Tue 20 Oct</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="B11" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IFERROR(INDEX('IXL tracker'!$D$5:$D$86,MATCH(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),'IXL tracker'!$G$5:$G$86,0)),"nothing due"))</f>
-        <v>nothing due</v>
+        <v>Add and subtract numbers written in scientific notation (HUR)</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="B12" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$Z$2:$Z$132,$B$44)&amp;"")</f>
-        <v>Devon writes (1.9 × 10²) + (6.6 × 10⁴) = 8.5 × 10⁶. Name the two mistakes he made, and give the correct sum.</v>
+        <v>For (7.2 × 10¹¹) ÷ (2.4 × 10³), Marcus writes 4.8 × 10⁸ and Sara writes 3 × 10¹⁴. Name what each one did wrong, and give the correct quotient.</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7377,11 +7377,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="n">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+1)))</f>
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="B30" s="6" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+1))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+1)))</f>
-        <v>4.02+03   Multiply and divide in scientific notation</v>
+        <v>4.04   Real-world scientific notation; significant digits</v>
       </c>
       <c r="C30" s="8" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+1))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+1)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+1))&amp;"")))</f>
@@ -7391,11 +7391,11 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="n">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+2)))</f>
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B31" s="6" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+2))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+2)))</f>
-        <v>4.04   Real-world scientific notation; significant digits</v>
+        <v>4.05   Expressions with radicals (perfect squares to 225, cubes −125 to 125)</v>
       </c>
       <c r="C31" s="8" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+2))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+2)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+2))&amp;"")))</f>
@@ -7405,11 +7405,11 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="n">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+3)))</f>
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B32" s="6" t="str">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+3))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+3)))</f>
-        <v>4.05   Expressions with radicals (perfect squares to 225, cubes −125 to 125)</v>
+        <v>4.06   Order of operations with exponents and radicals</v>
       </c>
       <c r="C32" s="8" t="str">
         <f aca="false">IF(($B$44+3)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+3))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+3)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+3))&amp;"")))</f>
@@ -7419,11 +7419,11 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+4)))</f>
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B33" s="6" t="str">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+4))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+4)))</f>
-        <v>4.06   Order of operations with exponents and radicals</v>
+        <v>4.07+08   Real-world order-of-operations problems</v>
       </c>
       <c r="C33" s="8" t="str">
         <f aca="false">IF(($B$44+4)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+4))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+4)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+4))&amp;"")))</f>
@@ -7433,15 +7433,15 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="n">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+5)))</f>
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="B34" s="6" t="str">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+5))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+5)))</f>
-        <v>4.07+08   Real-world order-of-operations problems</v>
+        <v>4.X1   Unit 4 exam, day 1</v>
       </c>
       <c r="C34" s="8" t="str">
         <f aca="false">IF(($B$44+5)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+5))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+5)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+5))&amp;"")))</f>
-        <v>open</v>
+        <v>Unit Assessment</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7457,7 +7457,7 @@
       </c>
       <c r="B44" s="13" t="n">
         <f aca="true">IF(TODAY()&gt;$B$45,131+1,MIN(COUNTIF('Scope &amp; Sequence'!$A$2:$A$132,"&lt;"&amp;TODAY())+1,131))</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
A7 Unit 5 papers: Reference Sheet (the FAST conversion lines), Unit Review with an SSDD floor plan, test Forms A, B and practice (19 q / 24 pts; transfer items 8 and 19); whole unit at 0 findings and installed. Unit title shortened to 'Multi-Step Proportional Relationships' so package paths unzip on Windows; the master-sheet tools read Form A's map and link Form A's paper when a unit ships parallel forms
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7ovt6yLjh6QuFV9HBMV4N
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -619,7 +619,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2887" uniqueCount="1928">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2893" uniqueCount="1932">
   <si>
     <t xml:space="preserve">A7 — today</t>
   </si>
@@ -1521,19 +1521,19 @@
     <t xml:space="preserve">Unit 5 exam, day 1</t>
   </si>
   <si>
+    <t xml:space="preserve">5.X2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit 5 exam, day 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.01+02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Triangle Inequality Theorem; converse of the Pythagorean Theorem</t>
+  </si>
+  <si>
     <t xml:space="preserve">not built yet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.X2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unit 5 exam, day 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.01+02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Triangle Inequality Theorem; converse of the Pythagorean Theorem</t>
   </si>
   <si>
     <t xml:space="preserve">Triangle inequality — 2N5; Converse of the Pythagorean theorem: is it a right triangle? — EQZ</t>
@@ -5970,7 +5970,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit a7c79ddb on 18 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 892ae8e7 on 18 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -6090,111 +6090,117 @@
     <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%204.06%22</t>
   </si>
   <si>
+    <t xml:space="preserve">'Unit tests'!E8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%204.07%22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Unit tests'!F8</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Unit tests'!G8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%204.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Unit tests'!H8</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Unit tests'!I8</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.02%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!G2</t>
   </si>
   <si>
     <t xml:space="preserve">folder</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!H2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.02%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.06%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!I2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.08%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!J2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.06%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.10%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!K2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.08%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!L2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.10%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!M2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!N2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.03%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!G3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!H3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.03%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.05%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!I3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.06%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!J3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.05%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.T1%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!K3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.06%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.T2%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!L3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.T1%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!M3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.T2%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!N3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!G4</t>
   </si>
   <si>
@@ -6204,39 +6210,39 @@
     <t xml:space="preserve">'Units'!I4</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!J4</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.02%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!K4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!L4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.02%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.05%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!M4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!N4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.05%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!G5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!H5</t>
   </si>
   <si>
@@ -6249,49 +6255,55 @@
     <t xml:space="preserve">'Units'!K5</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!L5</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.03%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!M5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!N5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.03%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.06%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!G6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.08%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!H6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.06%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%209.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!I6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.08%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%209.03%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!J6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%209.01%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!K6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%209.03%22</t>
+    <t xml:space="preserve">'Units'!L6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Units'!M6</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!N6</t>
@@ -6306,301 +6318,307 @@
     <t xml:space="preserve">'Units 1–2 decks'!E2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.02%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.04%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.05%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.06%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.02%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!E3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.09%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!F3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.05%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.10%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!G3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.06%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.09%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.10%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.02%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!E4</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.03%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F4</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.04%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.05%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!H4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.02%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!C5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.03%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.08%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.04%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.05%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.08%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!H5</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.03%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C6</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.04%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!D6</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.06%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.01%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.03%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!G6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.08%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!H6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.06%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C7</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D7</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E7</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.08%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F7</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G7</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.04%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H7</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.06%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C8</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.07%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!D8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.09%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!E8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.T1%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!F8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.06%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.T2%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!G8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.09%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C9</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.T1%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D9</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.T2%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.05%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!E9</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.07%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F9</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!G9</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.01%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H9</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.05%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!C10</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.07%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.02%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D10</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.03b%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E10</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.04%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F10</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.05%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!G10</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.02%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.06%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!H10</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.03b%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!C11</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.08%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D11</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.05%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2016.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!E11</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.06%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2016.03%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!F11</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G11</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.08%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H11</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2016.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2017.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!C12</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2016.03%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2017.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D12</t>
@@ -6612,13 +6630,7 @@
     <t xml:space="preserve">'Units 1–2 decks'!F12</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2017.01%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2017.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!H12</t>
@@ -7097,11 +7109,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8069,7 +8081,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q156"/>
+  <dimension ref="A1:Q160"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9268,8 +9280,8 @@
         <v>1684</v>
       </c>
       <c r="Q22" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b4473b65910",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k11cedfe615ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9331,8 +9343,8 @@
         <v>1684</v>
       </c>
       <c r="Q23" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1c81628b7541",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k34f09723e09c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9368,8 +9380,8 @@
         <v>1684</v>
       </c>
       <c r="Q24" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k60f05a144797",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b4473b65910",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9402,11 +9414,11 @@
         <v>1722</v>
       </c>
       <c r="P25" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q25" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2f48d7f422a9",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1c81628b7541",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9458,18 +9470,18 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M26" s="69" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="N26" s="69"/>
       <c r="O26" s="69" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="P26" s="69" t="s">
         <v>1684</v>
       </c>
       <c r="Q26" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8fdeab195866",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k60f05a144797",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9521,18 +9533,18 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M27" s="69" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="N27" s="69"/>
       <c r="O27" s="69" t="s">
+        <v>1726</v>
+      </c>
+      <c r="P27" s="69" t="s">
         <v>1727</v>
       </c>
-      <c r="P27" s="69" t="s">
-        <v>1684</v>
-      </c>
       <c r="Q27" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k05aafdefef87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2f48d7f422a9",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9594,8 +9606,8 @@
         <v>1684</v>
       </c>
       <c r="Q28" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4e34d1ba5135",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8fdeab195866",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9657,8 +9669,8 @@
         <v>1684</v>
       </c>
       <c r="Q29" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k654621d73a39",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k05aafdefef87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9720,8 +9732,8 @@
         <v>1684</v>
       </c>
       <c r="Q30" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k999a58eef73f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4e34d1ba5135",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9783,64 +9795,82 @@
         <v>1684</v>
       </c>
       <c r="Q31" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b0883f744a4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k654621d73a39",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="70" t="n">
         <v>46331</v>
       </c>
-      <c r="B32" s="69"/>
+      <c r="B32" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k11cedfe615ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22</v>
+      </c>
       <c r="C32" s="69"/>
       <c r="D32" s="69"/>
       <c r="E32" s="69"/>
       <c r="F32" s="69"/>
-      <c r="G32" s="69"/>
+      <c r="G32" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k34f09723e09c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22</v>
+      </c>
       <c r="H32" s="69"/>
       <c r="I32" s="69"/>
       <c r="J32" s="69"/>
       <c r="K32" s="69"/>
-      <c r="L32" s="69"/>
+      <c r="L32" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k57de004b2b0a",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
+      </c>
       <c r="M32" s="69"/>
       <c r="N32" s="69"/>
       <c r="O32" s="69" t="s">
         <v>1736</v>
       </c>
       <c r="P32" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q32" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2ed79628bc59",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k999a58eef73f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="70" t="n">
         <v>46332</v>
       </c>
-      <c r="B33" s="69"/>
+      <c r="B33" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k11cedfe615ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22</v>
+      </c>
       <c r="C33" s="69"/>
       <c r="D33" s="69"/>
       <c r="E33" s="69"/>
       <c r="F33" s="69"/>
-      <c r="G33" s="69"/>
+      <c r="G33" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k34f09723e09c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22</v>
+      </c>
       <c r="H33" s="69"/>
       <c r="I33" s="69"/>
       <c r="J33" s="69"/>
       <c r="K33" s="69"/>
-      <c r="L33" s="69"/>
+      <c r="L33" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k57de004b2b0a",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
+      </c>
       <c r="M33" s="69"/>
       <c r="N33" s="69"/>
       <c r="O33" s="69" t="s">
         <v>1737</v>
       </c>
       <c r="P33" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q33" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kf1ee50ed8929",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b0883f744a4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9866,11 +9896,11 @@
         <v>1739</v>
       </c>
       <c r="P34" s="69" t="s">
-        <v>1684</v>
+        <v>1727</v>
       </c>
       <c r="Q34" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k749da75b36af",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2ed79628bc59",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9896,11 +9926,11 @@
         <v>1741</v>
       </c>
       <c r="P35" s="69" t="s">
-        <v>1684</v>
+        <v>1727</v>
       </c>
       <c r="Q35" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k509a716d7468",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kf1ee50ed8929",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9929,8 +9959,8 @@
         <v>1684</v>
       </c>
       <c r="Q36" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4c613b2b0958",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k749da75b36af",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9959,8 +9989,8 @@
         <v>1684</v>
       </c>
       <c r="Q37" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd60a700332eb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k509a716d7468",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9989,8 +10019,8 @@
         <v>1684</v>
       </c>
       <c r="Q38" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0fe1632a0900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4c613b2b0958",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10019,8 +10049,8 @@
         <v>1684</v>
       </c>
       <c r="Q39" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kadb8b2686141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd60a700332eb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10046,11 +10076,11 @@
         <v>1751</v>
       </c>
       <c r="P40" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q40" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k986a7bd5b0f8",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0fe1632a0900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10076,11 +10106,11 @@
         <v>1753</v>
       </c>
       <c r="P41" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q41" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kb8fed8266c53",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kadb8b2686141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10104,11 +10134,11 @@
         <v>1754</v>
       </c>
       <c r="P42" s="69" t="s">
-        <v>1684</v>
+        <v>1727</v>
       </c>
       <c r="Q42" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb737ddcb3701",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k986a7bd5b0f8",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10132,11 +10162,11 @@
         <v>1755</v>
       </c>
       <c r="P43" s="69" t="s">
-        <v>1684</v>
+        <v>1727</v>
       </c>
       <c r="Q43" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1f816ed6a0ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kb8fed8266c53",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10163,8 +10193,8 @@
         <v>1684</v>
       </c>
       <c r="Q44" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb93ffed6ca63",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb737ddcb3701",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10191,8 +10221,8 @@
         <v>1684</v>
       </c>
       <c r="Q45" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k467ef44c3569",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1f816ed6a0ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10221,8 +10251,8 @@
         <v>1684</v>
       </c>
       <c r="Q46" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke52ff0df0d4b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb93ffed6ca63",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10251,8 +10281,8 @@
         <v>1684</v>
       </c>
       <c r="Q47" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf990f1c33e7d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k467ef44c3569",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10278,11 +10308,11 @@
         <v>1763</v>
       </c>
       <c r="P48" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q48" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k85bc365a5352",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke52ff0df0d4b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10308,11 +10338,11 @@
         <v>1765</v>
       </c>
       <c r="P49" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q49" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k19f682b91838",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf990f1c33e7d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10338,11 +10368,11 @@
         <v>1767</v>
       </c>
       <c r="P50" s="69" t="s">
-        <v>1684</v>
+        <v>1727</v>
       </c>
       <c r="Q50" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k44624f8b3141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k85bc365a5352",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10366,11 +10396,11 @@
         <v>1768</v>
       </c>
       <c r="P51" s="69" t="s">
-        <v>1684</v>
+        <v>1727</v>
       </c>
       <c r="Q51" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb2536de7152",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k19f682b91838",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10397,8 +10427,8 @@
         <v>1684</v>
       </c>
       <c r="Q52" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke57d72cf0716",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k44624f8b3141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10425,8 +10455,8 @@
         <v>1684</v>
       </c>
       <c r="Q53" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dd5b368d2b0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb2536de7152",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10453,8 +10483,8 @@
         <v>1684</v>
       </c>
       <c r="Q54" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7c17b9b2eea3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke57d72cf0716",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10481,8 +10511,8 @@
         <v>1684</v>
       </c>
       <c r="Q55" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k584fc57b9722",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dd5b368d2b0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10508,11 +10538,11 @@
         <v>1774</v>
       </c>
       <c r="P56" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q56" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k395c44aceb1d",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7c17b9b2eea3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test.pdf%22</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10538,11 +10568,11 @@
         <v>1776</v>
       </c>
       <c r="P57" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q57" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k57de004b2b0a",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k584fc57b9722",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10568,11 +10598,11 @@
         <v>1778</v>
       </c>
       <c r="P58" s="69" t="s">
-        <v>1684</v>
+        <v>1727</v>
       </c>
       <c r="Q58" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbcf7b890879b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k395c44aceb1d",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10598,11 +10628,11 @@
         <v>1780</v>
       </c>
       <c r="P59" s="69" t="s">
-        <v>1684</v>
+        <v>1727</v>
       </c>
       <c r="Q59" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k60f05a144797",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k57de004b2b0a",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10631,8 +10661,8 @@
         <v>1684</v>
       </c>
       <c r="Q60" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b4473b65910",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbcf7b890879b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10661,8 +10691,8 @@
         <v>1684</v>
       </c>
       <c r="Q61" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1c81628b7541",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k60f05a144797",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10688,11 +10718,11 @@
         <v>1786</v>
       </c>
       <c r="P62" s="69" t="s">
-        <v>1723</v>
+        <v>1684</v>
       </c>
       <c r="Q62" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k5fd6e0a77786",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b4473b65910",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10719,8 +10749,8 @@
         <v>1684</v>
       </c>
       <c r="Q63" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf7444edd4950",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1c81628b7541",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10747,8 +10777,8 @@
         <v>1684</v>
       </c>
       <c r="Q64" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbb6e44272bb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k11cedfe615ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10775,8 +10805,8 @@
         <v>1684</v>
       </c>
       <c r="Q65" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc68dd81311bb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k34f09723e09c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10800,11 +10830,11 @@
         <v>1790</v>
       </c>
       <c r="P66" s="69" t="s">
-        <v>1684</v>
+        <v>1727</v>
       </c>
       <c r="Q66" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k70c393f4e972",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k5fd6e0a77786",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10831,8 +10861,8 @@
         <v>1684</v>
       </c>
       <c r="Q67" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1d60e486567d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf7444edd4950",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10859,8 +10889,8 @@
         <v>1684</v>
       </c>
       <c r="Q68" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k40dc62cd52a5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbb6e44272bb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10887,8 +10917,8 @@
         <v>1684</v>
       </c>
       <c r="Q69" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42d053aa97d9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc68dd81311bb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10917,8 +10947,8 @@
         <v>1684</v>
       </c>
       <c r="Q70" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3d5b3115f0ff",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k70c393f4e972",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10947,8 +10977,8 @@
         <v>1684</v>
       </c>
       <c r="Q71" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b6284c3dfc8",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1d60e486567d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10977,8 +11007,8 @@
         <v>1684</v>
       </c>
       <c r="Q72" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k751991f77144",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k40dc62cd52a5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11007,8 +11037,8 @@
         <v>1684</v>
       </c>
       <c r="Q73" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6386e55cce43",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42d053aa97d9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11037,8 +11067,8 @@
         <v>1684</v>
       </c>
       <c r="Q74" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb55aff075211",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3d5b3115f0ff",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11067,8 +11097,8 @@
         <v>1684</v>
       </c>
       <c r="Q75" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k78f3bd7641b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b6284c3dfc8",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11097,8 +11127,8 @@
         <v>1684</v>
       </c>
       <c r="Q76" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab82b01c89fe",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k751991f77144",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11127,8 +11157,8 @@
         <v>1684</v>
       </c>
       <c r="Q77" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb5633697c8e5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6386e55cce43",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11155,8 +11185,8 @@
         <v>1684</v>
       </c>
       <c r="Q78" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf724d6e842b3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb55aff075211",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11183,8 +11213,8 @@
         <v>1684</v>
       </c>
       <c r="Q79" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k36b71975bd76",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k78f3bd7641b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11213,8 +11243,8 @@
         <v>1684</v>
       </c>
       <c r="Q80" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd7994f0255be",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab82b01c89fe",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11243,8 +11273,8 @@
         <v>1684</v>
       </c>
       <c r="Q81" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k441c122ac61a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb5633697c8e5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11273,8 +11303,8 @@
         <v>1684</v>
       </c>
       <c r="Q82" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcad6ba0a7c20",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf724d6e842b3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11303,8 +11333,8 @@
         <v>1684</v>
       </c>
       <c r="Q83" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kecd875ec58e7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k36b71975bd76",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11333,8 +11363,8 @@
         <v>1684</v>
       </c>
       <c r="Q84" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k04385d48a56f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd7994f0255be",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11363,8 +11393,8 @@
         <v>1684</v>
       </c>
       <c r="Q85" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kaa89f6499257",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k441c122ac61a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11393,8 +11423,8 @@
         <v>1684</v>
       </c>
       <c r="Q86" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc0dcbe2e82c2",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcad6ba0a7c20",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11421,8 +11451,8 @@
         <v>1684</v>
       </c>
       <c r="Q87" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k368f7f8b9908",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kecd875ec58e7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11449,8 +11479,8 @@
         <v>1684</v>
       </c>
       <c r="Q88" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k53d619094fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k04385d48a56f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11477,8 +11507,8 @@
         <v>1684</v>
       </c>
       <c r="Q89" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf511d84233f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kaa89f6499257",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11507,8 +11537,8 @@
         <v>1684</v>
       </c>
       <c r="Q90" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9da92cf1af2b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc0dcbe2e82c2",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11537,8 +11567,8 @@
         <v>1684</v>
       </c>
       <c r="Q91" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k515087871fe0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k368f7f8b9908",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11567,8 +11597,8 @@
         <v>1684</v>
       </c>
       <c r="Q92" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb6acc983851",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k53d619094fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11597,8 +11627,8 @@
         <v>1684</v>
       </c>
       <c r="Q93" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9cdee450b988",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf511d84233f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11625,8 +11655,8 @@
         <v>1684</v>
       </c>
       <c r="Q94" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kac1e5e18d498",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9da92cf1af2b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11655,8 +11685,8 @@
         <v>1684</v>
       </c>
       <c r="Q95" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb5db6608070",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k515087871fe0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11685,8 +11715,8 @@
         <v>1684</v>
       </c>
       <c r="Q96" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf2a43f4ef780",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb6acc983851",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11713,8 +11743,8 @@
         <v>1684</v>
       </c>
       <c r="Q97" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k86b940633ffd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9cdee450b988",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11741,8 +11771,8 @@
         <v>1684</v>
       </c>
       <c r="Q98" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf341ebe84b57",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kac1e5e18d498",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11769,8 +11799,8 @@
         <v>1684</v>
       </c>
       <c r="Q99" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7383ee3f2ec5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb5db6608070",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11797,8 +11827,8 @@
         <v>1684</v>
       </c>
       <c r="Q100" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5cae8f95e8bd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf2a43f4ef780",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11827,8 +11857,8 @@
         <v>1684</v>
       </c>
       <c r="Q101" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0ecee6c15886",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k86b940633ffd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11857,8 +11887,8 @@
         <v>1684</v>
       </c>
       <c r="Q102" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k874b463422ce",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf341ebe84b57",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11887,8 +11917,8 @@
         <v>1684</v>
       </c>
       <c r="Q103" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k07aa4ed88482",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7383ee3f2ec5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11917,8 +11947,8 @@
         <v>1684</v>
       </c>
       <c r="Q104" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k444ff4b9a71a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5cae8f95e8bd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11947,8 +11977,8 @@
         <v>1684</v>
       </c>
       <c r="Q105" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42b7580a8cb9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0ecee6c15886",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11977,8 +12007,8 @@
         <v>1684</v>
       </c>
       <c r="Q106" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8e5410dc08f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k874b463422ce",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12007,8 +12037,8 @@
         <v>1684</v>
       </c>
       <c r="Q107" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb0df0c43cf87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k07aa4ed88482",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12035,8 +12065,8 @@
         <v>1684</v>
       </c>
       <c r="Q108" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kde315e91893f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k444ff4b9a71a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12063,8 +12093,8 @@
         <v>1684</v>
       </c>
       <c r="Q109" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf9cc95eccf07",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42b7580a8cb9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12093,8 +12123,8 @@
         <v>1684</v>
       </c>
       <c r="Q110" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd674be572fbd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8e5410dc08f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12123,8 +12153,8 @@
         <v>1684</v>
       </c>
       <c r="Q111" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4f3c12075c6f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb0df0c43cf87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12153,8 +12183,8 @@
         <v>1684</v>
       </c>
       <c r="Q112" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k856d2d13cd04",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kde315e91893f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12181,8 +12211,8 @@
         <v>1684</v>
       </c>
       <c r="Q113" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k160e960d09c4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf9cc95eccf07",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12209,8 +12239,8 @@
         <v>1684</v>
       </c>
       <c r="Q114" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd3a48013b455",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd674be572fbd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12239,8 +12269,8 @@
         <v>1684</v>
       </c>
       <c r="Q115" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f26b556436e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4f3c12075c6f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12269,8 +12299,8 @@
         <v>1684</v>
       </c>
       <c r="Q116" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3a6534dc5a62",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k856d2d13cd04",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12299,8 +12329,8 @@
         <v>1684</v>
       </c>
       <c r="Q117" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ka5734698aa50",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k160e960d09c4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12329,8 +12359,8 @@
         <v>1684</v>
       </c>
       <c r="Q118" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3bd1b440e87a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd3a48013b455",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12359,8 +12389,8 @@
         <v>1684</v>
       </c>
       <c r="Q119" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k52493b74eb28",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f26b556436e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12389,8 +12419,8 @@
         <v>1684</v>
       </c>
       <c r="Q120" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3fa800b9318b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3a6534dc5a62",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12419,8 +12449,8 @@
         <v>1684</v>
       </c>
       <c r="Q121" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b2764e691f7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ka5734698aa50",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12449,8 +12479,8 @@
         <v>1684</v>
       </c>
       <c r="Q122" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9afa96310f5f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3bd1b440e87a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12479,8 +12509,8 @@
         <v>1684</v>
       </c>
       <c r="Q123" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3eb4a6e4e0a9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k52493b74eb28",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12509,8 +12539,8 @@
         <v>1684</v>
       </c>
       <c r="Q124" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3786dea98f2a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3fa800b9318b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12537,8 +12567,8 @@
         <v>1684</v>
       </c>
       <c r="Q125" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8424cc4e78b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b2764e691f7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12565,8 +12595,8 @@
         <v>1684</v>
       </c>
       <c r="Q126" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf325ac36b969",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9afa96310f5f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12595,8 +12625,8 @@
         <v>1684</v>
       </c>
       <c r="Q127" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4ec5ffc67bf1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3eb4a6e4e0a9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12625,8 +12655,8 @@
         <v>1684</v>
       </c>
       <c r="Q128" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k006e6e337926",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3786dea98f2a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12653,8 +12683,8 @@
         <v>1684</v>
       </c>
       <c r="Q129" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k94da89c1d16d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8424cc4e78b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12681,8 +12711,8 @@
         <v>1684</v>
       </c>
       <c r="Q130" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9b79f94a3042",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf325ac36b969",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12709,8 +12739,8 @@
         <v>1684</v>
       </c>
       <c r="Q131" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b57aec5f42c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4ec5ffc67bf1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12737,8 +12767,8 @@
         <v>1684</v>
       </c>
       <c r="Q132" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k524993898ff0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k006e6e337926",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12763,8 +12793,8 @@
         <v>1684</v>
       </c>
       <c r="Q133" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k71038ca67fed",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k94da89c1d16d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12789,8 +12819,8 @@
         <v>1684</v>
       </c>
       <c r="Q134" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab565ddcecfd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9b79f94a3042",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12815,8 +12845,8 @@
         <v>1684</v>
       </c>
       <c r="Q135" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kda9320d99fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b57aec5f42c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12841,8 +12871,8 @@
         <v>1684</v>
       </c>
       <c r="Q136" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k577a4eca3248",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k524993898ff0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12867,8 +12897,8 @@
         <v>1684</v>
       </c>
       <c r="Q137" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dbd9d8294a0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k71038ca67fed",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12893,8 +12923,8 @@
         <v>1684</v>
       </c>
       <c r="Q138" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k858285f0484a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab565ddcecfd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12919,8 +12949,8 @@
         <v>1684</v>
       </c>
       <c r="Q139" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3386b404a0cc",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kda9320d99fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12945,8 +12975,8 @@
         <v>1684</v>
       </c>
       <c r="Q140" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1fdcada6b7d5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k577a4eca3248",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12971,8 +13001,8 @@
         <v>1684</v>
       </c>
       <c r="Q141" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k66ad104dc3f4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dbd9d8294a0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12997,8 +13027,8 @@
         <v>1684</v>
       </c>
       <c r="Q142" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f9d2ee2e87b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k858285f0484a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13023,8 +13053,8 @@
         <v>1684</v>
       </c>
       <c r="Q143" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k2e021d1404f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3386b404a0cc",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13049,8 +13079,8 @@
         <v>1684</v>
       </c>
       <c r="Q144" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7f727f839de9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1fdcada6b7d5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13075,8 +13105,8 @@
         <v>1684</v>
       </c>
       <c r="Q145" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc9f54d815229",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k66ad104dc3f4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13101,8 +13131,8 @@
         <v>1684</v>
       </c>
       <c r="Q146" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k814de685731b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f9d2ee2e87b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13127,8 +13157,8 @@
         <v>1684</v>
       </c>
       <c r="Q147" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbeebbf583a30",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k2e021d1404f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13153,8 +13183,8 @@
         <v>1684</v>
       </c>
       <c r="Q148" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kae76dda4b45d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7f727f839de9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13179,8 +13209,8 @@
         <v>1684</v>
       </c>
       <c r="Q149" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1228a3dffde6",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc9f54d815229",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13205,8 +13235,8 @@
         <v>1684</v>
       </c>
       <c r="Q150" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k47f0af99bd1e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k814de685731b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13231,8 +13261,8 @@
         <v>1684</v>
       </c>
       <c r="Q151" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcee0b8f57c67",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbeebbf583a30",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13257,8 +13287,8 @@
         <v>1684</v>
       </c>
       <c r="Q152" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k59fb8b4ed900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kae76dda4b45d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13283,8 +13313,8 @@
         <v>1684</v>
       </c>
       <c r="Q153" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1a00a0a22804",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1228a3dffde6",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13309,8 +13339,8 @@
         <v>1684</v>
       </c>
       <c r="Q154" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k29d47d551984",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k47f0af99bd1e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13335,8 +13365,8 @@
         <v>1684</v>
       </c>
       <c r="Q155" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdc81e4a42f98",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcee0b8f57c67",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13361,6 +13391,110 @@
         <v>1684</v>
       </c>
       <c r="Q156" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k59fb8b4ed900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="69"/>
+      <c r="B157" s="69"/>
+      <c r="C157" s="69"/>
+      <c r="D157" s="69"/>
+      <c r="E157" s="69"/>
+      <c r="F157" s="69"/>
+      <c r="G157" s="69"/>
+      <c r="H157" s="69"/>
+      <c r="I157" s="69"/>
+      <c r="J157" s="69"/>
+      <c r="K157" s="69"/>
+      <c r="L157" s="69"/>
+      <c r="M157" s="69"/>
+      <c r="N157" s="69"/>
+      <c r="O157" s="69" t="s">
+        <v>1924</v>
+      </c>
+      <c r="P157" s="69" t="s">
+        <v>1684</v>
+      </c>
+      <c r="Q157" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1a00a0a22804",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="69"/>
+      <c r="B158" s="69"/>
+      <c r="C158" s="69"/>
+      <c r="D158" s="69"/>
+      <c r="E158" s="69"/>
+      <c r="F158" s="69"/>
+      <c r="G158" s="69"/>
+      <c r="H158" s="69"/>
+      <c r="I158" s="69"/>
+      <c r="J158" s="69"/>
+      <c r="K158" s="69"/>
+      <c r="L158" s="69"/>
+      <c r="M158" s="69"/>
+      <c r="N158" s="69"/>
+      <c r="O158" s="69" t="s">
+        <v>1925</v>
+      </c>
+      <c r="P158" s="69" t="s">
+        <v>1684</v>
+      </c>
+      <c r="Q158" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k29d47d551984",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="69"/>
+      <c r="B159" s="69"/>
+      <c r="C159" s="69"/>
+      <c r="D159" s="69"/>
+      <c r="E159" s="69"/>
+      <c r="F159" s="69"/>
+      <c r="G159" s="69"/>
+      <c r="H159" s="69"/>
+      <c r="I159" s="69"/>
+      <c r="J159" s="69"/>
+      <c r="K159" s="69"/>
+      <c r="L159" s="69"/>
+      <c r="M159" s="69"/>
+      <c r="N159" s="69"/>
+      <c r="O159" s="69" t="s">
+        <v>1926</v>
+      </c>
+      <c r="P159" s="69" t="s">
+        <v>1684</v>
+      </c>
+      <c r="Q159" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdc81e4a42f98",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="69"/>
+      <c r="B160" s="69"/>
+      <c r="C160" s="69"/>
+      <c r="D160" s="69"/>
+      <c r="E160" s="69"/>
+      <c r="F160" s="69"/>
+      <c r="G160" s="69"/>
+      <c r="H160" s="69"/>
+      <c r="I160" s="69"/>
+      <c r="J160" s="69"/>
+      <c r="K160" s="69"/>
+      <c r="L160" s="69"/>
+      <c r="M160" s="69"/>
+      <c r="N160" s="69"/>
+      <c r="O160" s="69" t="s">
+        <v>1927</v>
+      </c>
+      <c r="P160" s="69" t="s">
+        <v>1684</v>
+      </c>
+      <c r="Q160" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc34b261fea84",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
         <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
@@ -13391,16 +13525,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="71" t="s">
-        <v>1924</v>
+        <v>1928</v>
       </c>
       <c r="B1" s="71" t="s">
-        <v>1925</v>
+        <v>1929</v>
       </c>
       <c r="C1" s="71" t="s">
-        <v>1926</v>
+        <v>1930</v>
       </c>
       <c r="D1" s="71" t="s">
-        <v>1927</v>
+        <v>1931</v>
       </c>
     </row>
   </sheetData>
@@ -16075,19 +16209,26 @@
       <c r="E32" s="33" t="s">
         <v>287</v>
       </c>
-      <c r="F32" s="43" t="s">
-        <v>288</v>
+      <c r="F32" s="34" t="str">
+        <f aca="false">HYPERLINK(Links!$B$32,"Unit Assessment")</f>
+        <v>Unit Assessment</v>
       </c>
       <c r="G32" s="30"/>
       <c r="H32" s="30"/>
       <c r="I32" s="30"/>
       <c r="J32" s="30"/>
-      <c r="K32" s="30"/>
+      <c r="K32" s="34" t="str">
+        <f aca="false">HYPERLINK(Links!$G$32,"Assessment key")</f>
+        <v>Assessment key</v>
+      </c>
       <c r="L32" s="30"/>
       <c r="M32" s="30"/>
       <c r="N32" s="30"/>
       <c r="O32" s="30"/>
-      <c r="P32" s="30"/>
+      <c r="P32" s="34" t="str">
+        <f aca="false">HYPERLINK(Links!$L$32,"folder")</f>
+        <v>folder</v>
+      </c>
       <c r="Q32" s="30"/>
       <c r="R32" s="33"/>
       <c r="S32" s="35"/>
@@ -16112,24 +16253,31 @@
         <v>5</v>
       </c>
       <c r="D33" s="32" t="s">
+        <v>288</v>
+      </c>
+      <c r="E33" s="33" t="s">
         <v>289</v>
       </c>
-      <c r="E33" s="33" t="s">
-        <v>290</v>
-      </c>
-      <c r="F33" s="43" t="s">
-        <v>288</v>
+      <c r="F33" s="34" t="str">
+        <f aca="false">HYPERLINK(Links!$B$33,"Unit Assessment")</f>
+        <v>Unit Assessment</v>
       </c>
       <c r="G33" s="30"/>
       <c r="H33" s="30"/>
       <c r="I33" s="30"/>
       <c r="J33" s="30"/>
-      <c r="K33" s="30"/>
+      <c r="K33" s="34" t="str">
+        <f aca="false">HYPERLINK(Links!$G$33,"Assessment key")</f>
+        <v>Assessment key</v>
+      </c>
       <c r="L33" s="30"/>
       <c r="M33" s="30"/>
       <c r="N33" s="30"/>
       <c r="O33" s="30"/>
-      <c r="P33" s="30"/>
+      <c r="P33" s="34" t="str">
+        <f aca="false">HYPERLINK(Links!$L$33,"folder")</f>
+        <v>folder</v>
+      </c>
       <c r="Q33" s="30"/>
       <c r="R33" s="33"/>
       <c r="S33" s="35"/>
@@ -16154,13 +16302,13 @@
         <v>6</v>
       </c>
       <c r="D34" s="39" t="s">
+        <v>290</v>
+      </c>
+      <c r="E34" s="40" t="s">
         <v>291</v>
       </c>
-      <c r="E34" s="40" t="s">
+      <c r="F34" s="43" t="s">
         <v>292</v>
-      </c>
-      <c r="F34" s="44" t="s">
-        <v>288</v>
       </c>
       <c r="G34" s="37"/>
       <c r="H34" s="37"/>
@@ -16214,8 +16362,8 @@
       <c r="E35" s="40" t="s">
         <v>298</v>
       </c>
-      <c r="F35" s="44" t="s">
-        <v>288</v>
+      <c r="F35" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G35" s="37"/>
       <c r="H35" s="37"/>
@@ -16269,8 +16417,8 @@
       <c r="E36" s="40" t="s">
         <v>304</v>
       </c>
-      <c r="F36" s="44" t="s">
-        <v>288</v>
+      <c r="F36" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G36" s="37"/>
       <c r="H36" s="37"/>
@@ -16324,8 +16472,8 @@
       <c r="E37" s="40" t="s">
         <v>308</v>
       </c>
-      <c r="F37" s="44" t="s">
-        <v>288</v>
+      <c r="F37" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G37" s="37"/>
       <c r="H37" s="37"/>
@@ -16379,8 +16527,8 @@
       <c r="E38" s="40" t="s">
         <v>314</v>
       </c>
-      <c r="F38" s="44" t="s">
-        <v>288</v>
+      <c r="F38" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G38" s="37"/>
       <c r="H38" s="37"/>
@@ -16434,8 +16582,8 @@
       <c r="E39" s="40" t="s">
         <v>318</v>
       </c>
-      <c r="F39" s="44" t="s">
-        <v>288</v>
+      <c r="F39" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G39" s="37"/>
       <c r="H39" s="37"/>
@@ -16489,8 +16637,8 @@
       <c r="E40" s="40" t="s">
         <v>324</v>
       </c>
-      <c r="F40" s="44" t="s">
-        <v>288</v>
+      <c r="F40" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G40" s="37"/>
       <c r="H40" s="37"/>
@@ -16544,8 +16692,8 @@
       <c r="E41" s="40" t="s">
         <v>330</v>
       </c>
-      <c r="F41" s="44" t="s">
-        <v>288</v>
+      <c r="F41" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G41" s="37"/>
       <c r="H41" s="37"/>
@@ -16639,8 +16787,8 @@
       <c r="E43" s="33" t="s">
         <v>336</v>
       </c>
-      <c r="F43" s="43" t="s">
-        <v>288</v>
+      <c r="F43" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G43" s="30"/>
       <c r="H43" s="30"/>
@@ -16681,8 +16829,8 @@
       <c r="E44" s="33" t="s">
         <v>338</v>
       </c>
-      <c r="F44" s="43" t="s">
-        <v>288</v>
+      <c r="F44" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G44" s="30"/>
       <c r="H44" s="30"/>
@@ -16764,7 +16912,7 @@
         <v>342</v>
       </c>
       <c r="F46" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G46" s="16"/>
       <c r="H46" s="16"/>
@@ -16819,7 +16967,7 @@
         <v>348</v>
       </c>
       <c r="F47" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G47" s="16"/>
       <c r="H47" s="16"/>
@@ -16874,7 +17022,7 @@
         <v>354</v>
       </c>
       <c r="F48" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G48" s="16"/>
       <c r="H48" s="16"/>
@@ -16929,7 +17077,7 @@
         <v>360</v>
       </c>
       <c r="F49" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G49" s="16"/>
       <c r="H49" s="16"/>
@@ -16984,7 +17132,7 @@
         <v>366</v>
       </c>
       <c r="F50" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G50" s="16"/>
       <c r="H50" s="16"/>
@@ -17038,8 +17186,8 @@
       <c r="E51" s="33" t="s">
         <v>372</v>
       </c>
-      <c r="F51" s="43" t="s">
-        <v>288</v>
+      <c r="F51" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G51" s="30"/>
       <c r="H51" s="30"/>
@@ -17080,8 +17228,8 @@
       <c r="E52" s="33" t="s">
         <v>374</v>
       </c>
-      <c r="F52" s="43" t="s">
-        <v>288</v>
+      <c r="F52" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G52" s="30"/>
       <c r="H52" s="30"/>
@@ -17248,8 +17396,8 @@
       <c r="E56" s="40" t="s">
         <v>388</v>
       </c>
-      <c r="F56" s="44" t="s">
-        <v>288</v>
+      <c r="F56" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G56" s="37"/>
       <c r="H56" s="37"/>
@@ -17303,8 +17451,8 @@
       <c r="E57" s="40" t="s">
         <v>394</v>
       </c>
-      <c r="F57" s="44" t="s">
-        <v>288</v>
+      <c r="F57" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G57" s="37"/>
       <c r="H57" s="37"/>
@@ -17358,8 +17506,8 @@
       <c r="E58" s="40" t="s">
         <v>398</v>
       </c>
-      <c r="F58" s="44" t="s">
-        <v>288</v>
+      <c r="F58" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G58" s="37"/>
       <c r="H58" s="37"/>
@@ -17413,8 +17561,8 @@
       <c r="E59" s="40" t="s">
         <v>404</v>
       </c>
-      <c r="F59" s="44" t="s">
-        <v>288</v>
+      <c r="F59" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G59" s="37"/>
       <c r="H59" s="37"/>
@@ -17468,8 +17616,8 @@
       <c r="E60" s="40" t="s">
         <v>408</v>
       </c>
-      <c r="F60" s="44" t="s">
-        <v>288</v>
+      <c r="F60" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G60" s="37"/>
       <c r="H60" s="37"/>
@@ -17524,7 +17672,7 @@
         <v>414</v>
       </c>
       <c r="F61" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G61" s="16"/>
       <c r="H61" s="16"/>
@@ -17579,7 +17727,7 @@
         <v>420</v>
       </c>
       <c r="F62" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G62" s="16"/>
       <c r="H62" s="16"/>
@@ -17833,8 +17981,8 @@
       <c r="E68" s="33" t="s">
         <v>426</v>
       </c>
-      <c r="F68" s="43" t="s">
-        <v>288</v>
+      <c r="F68" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G68" s="30"/>
       <c r="H68" s="30"/>
@@ -17875,8 +18023,8 @@
       <c r="E69" s="33" t="s">
         <v>428</v>
       </c>
-      <c r="F69" s="43" t="s">
-        <v>288</v>
+      <c r="F69" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G69" s="30"/>
       <c r="H69" s="30"/>
@@ -17917,8 +18065,8 @@
       <c r="E70" s="40" t="s">
         <v>430</v>
       </c>
-      <c r="F70" s="44" t="s">
-        <v>288</v>
+      <c r="F70" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G70" s="37"/>
       <c r="H70" s="37"/>
@@ -17972,8 +18120,8 @@
       <c r="E71" s="40" t="s">
         <v>436</v>
       </c>
-      <c r="F71" s="44" t="s">
-        <v>288</v>
+      <c r="F71" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G71" s="37"/>
       <c r="H71" s="37"/>
@@ -18027,8 +18175,8 @@
       <c r="E72" s="40" t="s">
         <v>442</v>
       </c>
-      <c r="F72" s="44" t="s">
-        <v>288</v>
+      <c r="F72" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G72" s="37"/>
       <c r="H72" s="37"/>
@@ -18082,8 +18230,8 @@
       <c r="E73" s="40" t="s">
         <v>448</v>
       </c>
-      <c r="F73" s="44" t="s">
-        <v>288</v>
+      <c r="F73" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G73" s="37"/>
       <c r="H73" s="37"/>
@@ -18137,8 +18285,8 @@
       <c r="E74" s="40" t="s">
         <v>454</v>
       </c>
-      <c r="F74" s="44" t="s">
-        <v>288</v>
+      <c r="F74" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G74" s="37"/>
       <c r="H74" s="37"/>
@@ -18192,8 +18340,8 @@
       <c r="E75" s="40" t="s">
         <v>458</v>
       </c>
-      <c r="F75" s="44" t="s">
-        <v>288</v>
+      <c r="F75" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G75" s="37"/>
       <c r="H75" s="37"/>
@@ -18247,8 +18395,8 @@
       <c r="E76" s="40" t="s">
         <v>464</v>
       </c>
-      <c r="F76" s="44" t="s">
-        <v>288</v>
+      <c r="F76" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G76" s="37"/>
       <c r="H76" s="37"/>
@@ -18302,8 +18450,8 @@
       <c r="E77" s="40" t="s">
         <v>470</v>
       </c>
-      <c r="F77" s="44" t="s">
-        <v>288</v>
+      <c r="F77" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G77" s="37"/>
       <c r="H77" s="37"/>
@@ -18357,8 +18505,8 @@
       <c r="E78" s="33" t="s">
         <v>476</v>
       </c>
-      <c r="F78" s="43" t="s">
-        <v>288</v>
+      <c r="F78" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G78" s="30"/>
       <c r="H78" s="30"/>
@@ -18399,8 +18547,8 @@
       <c r="E79" s="33" t="s">
         <v>478</v>
       </c>
-      <c r="F79" s="43" t="s">
-        <v>288</v>
+      <c r="F79" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G79" s="30"/>
       <c r="H79" s="30"/>
@@ -18442,7 +18590,7 @@
         <v>480</v>
       </c>
       <c r="F80" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G80" s="16"/>
       <c r="H80" s="16"/>
@@ -18497,7 +18645,7 @@
         <v>486</v>
       </c>
       <c r="F81" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G81" s="16"/>
       <c r="H81" s="16"/>
@@ -18552,7 +18700,7 @@
         <v>490</v>
       </c>
       <c r="F82" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G82" s="16"/>
       <c r="H82" s="16"/>
@@ -18607,7 +18755,7 @@
         <v>494</v>
       </c>
       <c r="F83" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G83" s="16"/>
       <c r="H83" s="16"/>
@@ -18662,7 +18810,7 @@
         <v>498</v>
       </c>
       <c r="F84" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G84" s="16"/>
       <c r="H84" s="16"/>
@@ -18717,7 +18865,7 @@
         <v>504</v>
       </c>
       <c r="F85" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G85" s="16"/>
       <c r="H85" s="16"/>
@@ -18772,7 +18920,7 @@
         <v>510</v>
       </c>
       <c r="F86" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G86" s="16"/>
       <c r="H86" s="16"/>
@@ -18826,8 +18974,8 @@
       <c r="E87" s="33" t="s">
         <v>514</v>
       </c>
-      <c r="F87" s="43" t="s">
-        <v>288</v>
+      <c r="F87" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G87" s="30"/>
       <c r="H87" s="30"/>
@@ -18868,8 +19016,8 @@
       <c r="E88" s="33" t="s">
         <v>516</v>
       </c>
-      <c r="F88" s="43" t="s">
-        <v>288</v>
+      <c r="F88" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G88" s="30"/>
       <c r="H88" s="30"/>
@@ -18950,8 +19098,8 @@
       <c r="E90" s="40" t="s">
         <v>518</v>
       </c>
-      <c r="F90" s="44" t="s">
-        <v>288</v>
+      <c r="F90" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G90" s="37"/>
       <c r="H90" s="37"/>
@@ -19005,8 +19153,8 @@
       <c r="E91" s="40" t="s">
         <v>524</v>
       </c>
-      <c r="F91" s="44" t="s">
-        <v>288</v>
+      <c r="F91" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G91" s="37"/>
       <c r="H91" s="37"/>
@@ -19060,8 +19208,8 @@
       <c r="E92" s="40" t="s">
         <v>528</v>
       </c>
-      <c r="F92" s="44" t="s">
-        <v>288</v>
+      <c r="F92" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G92" s="37"/>
       <c r="H92" s="37"/>
@@ -19115,8 +19263,8 @@
       <c r="E93" s="40" t="s">
         <v>534</v>
       </c>
-      <c r="F93" s="44" t="s">
-        <v>288</v>
+      <c r="F93" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G93" s="37"/>
       <c r="H93" s="37"/>
@@ -19210,8 +19358,8 @@
       <c r="E95" s="40" t="s">
         <v>537</v>
       </c>
-      <c r="F95" s="44" t="s">
-        <v>288</v>
+      <c r="F95" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G95" s="37"/>
       <c r="H95" s="37"/>
@@ -19265,8 +19413,8 @@
       <c r="E96" s="40" t="s">
         <v>543</v>
       </c>
-      <c r="F96" s="44" t="s">
-        <v>288</v>
+      <c r="F96" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G96" s="37"/>
       <c r="H96" s="37"/>
@@ -19360,8 +19508,8 @@
       <c r="E98" s="33" t="s">
         <v>549</v>
       </c>
-      <c r="F98" s="43" t="s">
-        <v>288</v>
+      <c r="F98" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G98" s="30"/>
       <c r="H98" s="30"/>
@@ -19402,8 +19550,8 @@
       <c r="E99" s="33" t="s">
         <v>551</v>
       </c>
-      <c r="F99" s="43" t="s">
-        <v>288</v>
+      <c r="F99" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G99" s="30"/>
       <c r="H99" s="30"/>
@@ -19485,7 +19633,7 @@
         <v>553</v>
       </c>
       <c r="F101" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G101" s="16"/>
       <c r="H101" s="16"/>
@@ -19540,7 +19688,7 @@
         <v>559</v>
       </c>
       <c r="F102" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G102" s="16"/>
       <c r="H102" s="16"/>
@@ -19595,7 +19743,7 @@
         <v>565</v>
       </c>
       <c r="F103" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G103" s="16"/>
       <c r="H103" s="16"/>
@@ -19650,7 +19798,7 @@
         <v>571</v>
       </c>
       <c r="F104" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G104" s="16"/>
       <c r="H104" s="16"/>
@@ -19705,7 +19853,7 @@
         <v>577</v>
       </c>
       <c r="F105" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G105" s="16"/>
       <c r="H105" s="16"/>
@@ -19760,7 +19908,7 @@
         <v>583</v>
       </c>
       <c r="F106" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G106" s="16"/>
       <c r="H106" s="16"/>
@@ -19815,7 +19963,7 @@
         <v>589</v>
       </c>
       <c r="F107" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G107" s="16"/>
       <c r="H107" s="16"/>
@@ -19869,8 +20017,8 @@
       <c r="E108" s="33" t="s">
         <v>595</v>
       </c>
-      <c r="F108" s="43" t="s">
-        <v>288</v>
+      <c r="F108" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G108" s="30"/>
       <c r="H108" s="30"/>
@@ -19911,8 +20059,8 @@
       <c r="E109" s="33" t="s">
         <v>597</v>
       </c>
-      <c r="F109" s="43" t="s">
-        <v>288</v>
+      <c r="F109" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G109" s="30"/>
       <c r="H109" s="30"/>
@@ -19953,8 +20101,8 @@
       <c r="E110" s="40" t="s">
         <v>599</v>
       </c>
-      <c r="F110" s="44" t="s">
-        <v>288</v>
+      <c r="F110" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G110" s="37"/>
       <c r="H110" s="37"/>
@@ -20008,8 +20156,8 @@
       <c r="E111" s="40" t="s">
         <v>603</v>
       </c>
-      <c r="F111" s="44" t="s">
-        <v>288</v>
+      <c r="F111" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G111" s="37"/>
       <c r="H111" s="37"/>
@@ -20063,8 +20211,8 @@
       <c r="E112" s="40" t="s">
         <v>609</v>
       </c>
-      <c r="F112" s="44" t="s">
-        <v>288</v>
+      <c r="F112" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G112" s="37"/>
       <c r="H112" s="37"/>
@@ -20118,8 +20266,8 @@
       <c r="E113" s="33" t="s">
         <v>615</v>
       </c>
-      <c r="F113" s="43" t="s">
-        <v>288</v>
+      <c r="F113" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G113" s="30"/>
       <c r="H113" s="30"/>
@@ -20160,8 +20308,8 @@
       <c r="E114" s="33" t="s">
         <v>617</v>
       </c>
-      <c r="F114" s="43" t="s">
-        <v>288</v>
+      <c r="F114" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G114" s="30"/>
       <c r="H114" s="30"/>
@@ -20203,7 +20351,7 @@
         <v>619</v>
       </c>
       <c r="F115" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G115" s="16"/>
       <c r="H115" s="16"/>
@@ -20258,7 +20406,7 @@
         <v>625</v>
       </c>
       <c r="F116" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G116" s="16"/>
       <c r="H116" s="16"/>
@@ -20313,7 +20461,7 @@
         <v>629</v>
       </c>
       <c r="F117" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G117" s="16"/>
       <c r="H117" s="16"/>
@@ -20368,7 +20516,7 @@
         <v>635</v>
       </c>
       <c r="F118" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G118" s="16"/>
       <c r="H118" s="16"/>
@@ -20423,7 +20571,7 @@
         <v>639</v>
       </c>
       <c r="F119" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G119" s="16"/>
       <c r="H119" s="16"/>
@@ -20478,7 +20626,7 @@
         <v>643</v>
       </c>
       <c r="F120" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G120" s="16"/>
       <c r="H120" s="16"/>
@@ -20533,7 +20681,7 @@
         <v>649</v>
       </c>
       <c r="F121" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G121" s="16"/>
       <c r="H121" s="16"/>
@@ -20588,7 +20736,7 @@
         <v>655</v>
       </c>
       <c r="F122" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G122" s="16"/>
       <c r="H122" s="16"/>
@@ -20642,8 +20790,8 @@
       <c r="E123" s="40" t="s">
         <v>659</v>
       </c>
-      <c r="F123" s="44" t="s">
-        <v>288</v>
+      <c r="F123" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G123" s="37"/>
       <c r="H123" s="37"/>
@@ -20697,8 +20845,8 @@
       <c r="E124" s="40" t="s">
         <v>665</v>
       </c>
-      <c r="F124" s="44" t="s">
-        <v>288</v>
+      <c r="F124" s="43" t="s">
+        <v>292</v>
       </c>
       <c r="G124" s="37"/>
       <c r="H124" s="37"/>
@@ -20752,8 +20900,8 @@
       <c r="E125" s="33" t="s">
         <v>671</v>
       </c>
-      <c r="F125" s="43" t="s">
-        <v>288</v>
+      <c r="F125" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G125" s="30"/>
       <c r="H125" s="30"/>
@@ -20794,8 +20942,8 @@
       <c r="E126" s="33" t="s">
         <v>673</v>
       </c>
-      <c r="F126" s="43" t="s">
-        <v>288</v>
+      <c r="F126" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G126" s="30"/>
       <c r="H126" s="30"/>
@@ -20837,7 +20985,7 @@
         <v>675</v>
       </c>
       <c r="F127" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G127" s="16"/>
       <c r="H127" s="16"/>
@@ -20892,7 +21040,7 @@
         <v>681</v>
       </c>
       <c r="F128" s="45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G128" s="16"/>
       <c r="H128" s="16"/>
@@ -20986,8 +21134,8 @@
       <c r="E130" s="33" t="s">
         <v>687</v>
       </c>
-      <c r="F130" s="43" t="s">
-        <v>288</v>
+      <c r="F130" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G130" s="30"/>
       <c r="H130" s="30"/>
@@ -21028,8 +21176,8 @@
       <c r="E131" s="33" t="s">
         <v>689</v>
       </c>
-      <c r="F131" s="43" t="s">
-        <v>288</v>
+      <c r="F131" s="44" t="s">
+        <v>292</v>
       </c>
       <c r="G131" s="30"/>
       <c r="H131" s="30"/>
@@ -26030,18 +26178,24 @@
         <f aca="false">C90</f>
         <v>24</v>
       </c>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
+      <c r="E8" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$22,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="F8" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$23,"open")</f>
+        <v>open</v>
+      </c>
       <c r="G8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$22,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$24,"open")</f>
         <v>open</v>
       </c>
       <c r="H8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$23,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$25,"open")</f>
         <v>open</v>
       </c>
       <c r="I8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$24,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$26,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -26057,7 +26211,7 @@
       </c>
       <c r="D9" s="46"/>
       <c r="E9" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F9" s="52"/>
       <c r="G9" s="52"/>
@@ -26076,7 +26230,7 @@
       </c>
       <c r="D10" s="46"/>
       <c r="E10" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F10" s="52"/>
       <c r="G10" s="52"/>
@@ -26095,7 +26249,7 @@
       </c>
       <c r="D11" s="46"/>
       <c r="E11" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F11" s="52"/>
       <c r="G11" s="52"/>
@@ -26114,7 +26268,7 @@
       </c>
       <c r="D12" s="46"/>
       <c r="E12" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F12" s="52"/>
       <c r="G12" s="52"/>
@@ -26133,7 +26287,7 @@
       </c>
       <c r="D13" s="46"/>
       <c r="E13" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F13" s="52"/>
       <c r="G13" s="52"/>
@@ -26152,7 +26306,7 @@
       </c>
       <c r="D14" s="46"/>
       <c r="E14" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F14" s="52"/>
       <c r="G14" s="52"/>
@@ -26171,7 +26325,7 @@
       </c>
       <c r="D15" s="46"/>
       <c r="E15" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F15" s="52"/>
       <c r="G15" s="52"/>
@@ -26190,7 +26344,7 @@
       </c>
       <c r="D16" s="46"/>
       <c r="E16" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="52"/>
@@ -26209,7 +26363,7 @@
       </c>
       <c r="D17" s="46"/>
       <c r="E17" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F17" s="52"/>
       <c r="G17" s="52"/>
@@ -26228,7 +26382,7 @@
       </c>
       <c r="D18" s="46"/>
       <c r="E18" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F18" s="52"/>
       <c r="G18" s="52"/>
@@ -29936,35 +30090,35 @@
         <v>1620</v>
       </c>
       <c r="G2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$25,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$27,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$26,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$28,"open")</f>
         <v>open</v>
       </c>
       <c r="I2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$27,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$29,"open")</f>
         <v>open</v>
       </c>
       <c r="J2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$28,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$30,"open")</f>
         <v>open</v>
       </c>
       <c r="K2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$29,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$31,"open")</f>
         <v>open</v>
       </c>
       <c r="L2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$30,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$32,"open")</f>
         <v>open</v>
       </c>
       <c r="M2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$31,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$33,"open")</f>
         <v>open</v>
       </c>
       <c r="N2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$32,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$34,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -29984,35 +30138,35 @@
         <v>1620</v>
       </c>
       <c r="G3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$33,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$35,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$34,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$36,"open")</f>
         <v>open</v>
       </c>
       <c r="I3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$35,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$37,"open")</f>
         <v>open</v>
       </c>
       <c r="J3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$36,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$38,"open")</f>
         <v>open</v>
       </c>
       <c r="K3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$37,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$39,"open")</f>
         <v>open</v>
       </c>
       <c r="L3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$38,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$40,"open")</f>
         <v>open</v>
       </c>
       <c r="M3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$39,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$41,"open")</f>
         <v>open</v>
       </c>
       <c r="N3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$40,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$42,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -30037,35 +30191,35 @@
         <v>1623</v>
       </c>
       <c r="G4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$41,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$43,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$42,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$44,"open")</f>
         <v>open</v>
       </c>
       <c r="I4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$43,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$45,"open")</f>
         <v>open</v>
       </c>
       <c r="J4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$44,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$46,"open")</f>
         <v>open</v>
       </c>
       <c r="K4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$45,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$47,"open")</f>
         <v>open</v>
       </c>
       <c r="L4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$46,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$48,"open")</f>
         <v>open</v>
       </c>
       <c r="M4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$47,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$49,"open")</f>
         <v>open</v>
       </c>
       <c r="N4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$48,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$50,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -30090,35 +30244,35 @@
         <v>1623</v>
       </c>
       <c r="G5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$49,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$51,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$50,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$52,"open")</f>
         <v>open</v>
       </c>
       <c r="I5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$51,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$53,"open")</f>
         <v>open</v>
       </c>
       <c r="J5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$52,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$54,"open")</f>
         <v>open</v>
       </c>
       <c r="K5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$53,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$55,"open")</f>
         <v>open</v>
       </c>
       <c r="L5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$54,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$56,"open")</f>
         <v>open</v>
       </c>
       <c r="M5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$55,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$57,"open")</f>
         <v>open</v>
       </c>
       <c r="N5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$56,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$58,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -30143,29 +30297,35 @@
         <v>1620</v>
       </c>
       <c r="G6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$57,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$59,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$58,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$60,"open")</f>
         <v>open</v>
       </c>
       <c r="I6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$59,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$61,"open")</f>
         <v>open</v>
       </c>
       <c r="J6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$60,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$62,"open")</f>
         <v>open</v>
       </c>
       <c r="K6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$61,"open")</f>
-        <v>open</v>
-      </c>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
+        <f aca="false">HYPERLINK(Links!$Q$63,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="L6" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$64,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="M6" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$65,"open")</f>
+        <v>open</v>
+      </c>
       <c r="N6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$62,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$66,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -30187,7 +30347,7 @@
         <v>12</v>
       </c>
       <c r="F7" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
@@ -30216,7 +30376,7 @@
         <v>7</v>
       </c>
       <c r="F8" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
@@ -30245,7 +30405,7 @@
         <v>5</v>
       </c>
       <c r="F9" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
@@ -30274,7 +30434,7 @@
         <v>9</v>
       </c>
       <c r="F10" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
@@ -30303,7 +30463,7 @@
         <v>10</v>
       </c>
       <c r="F11" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
@@ -30332,7 +30492,7 @@
         <v>10</v>
       </c>
       <c r="F12" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
@@ -30361,7 +30521,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
@@ -30390,7 +30550,7 @@
         <v>9</v>
       </c>
       <c r="F14" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
@@ -30419,7 +30579,7 @@
         <v>5</v>
       </c>
       <c r="F15" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
@@ -30448,7 +30608,7 @@
         <v>8</v>
       </c>
       <c r="F16" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
@@ -30477,7 +30637,7 @@
         <v>4</v>
       </c>
       <c r="F17" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
@@ -30506,7 +30666,7 @@
         <v>5</v>
       </c>
       <c r="F18" s="52" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
@@ -30585,27 +30745,27 @@
         <v>1640</v>
       </c>
       <c r="C2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$63,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$67,"open")</f>
         <v>open</v>
       </c>
       <c r="D2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$64,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$68,"open")</f>
         <v>open</v>
       </c>
       <c r="E2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$65,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$69,"open")</f>
         <v>open</v>
       </c>
       <c r="F2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$66,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$70,"open")</f>
         <v>open</v>
       </c>
       <c r="G2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$67,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$71,"open")</f>
         <v>open</v>
       </c>
       <c r="H2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$68,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$72,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30617,27 +30777,27 @@
         <v>1641</v>
       </c>
       <c r="C3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$69,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$73,"open")</f>
         <v>open</v>
       </c>
       <c r="D3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$70,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$74,"open")</f>
         <v>open</v>
       </c>
       <c r="E3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$71,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$75,"open")</f>
         <v>open</v>
       </c>
       <c r="F3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$72,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$76,"open")</f>
         <v>open</v>
       </c>
       <c r="G3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$73,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$77,"open")</f>
         <v>open</v>
       </c>
       <c r="H3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$74,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$78,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30649,27 +30809,27 @@
         <v>1642</v>
       </c>
       <c r="C4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$75,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$79,"open")</f>
         <v>open</v>
       </c>
       <c r="D4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$76,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$80,"open")</f>
         <v>open</v>
       </c>
       <c r="E4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$77,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$81,"open")</f>
         <v>open</v>
       </c>
       <c r="F4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$78,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$82,"open")</f>
         <v>open</v>
       </c>
       <c r="G4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$79,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$83,"open")</f>
         <v>open</v>
       </c>
       <c r="H4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$80,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$84,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30681,27 +30841,27 @@
         <v>1643</v>
       </c>
       <c r="C5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$81,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$85,"open")</f>
         <v>open</v>
       </c>
       <c r="D5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$82,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$86,"open")</f>
         <v>open</v>
       </c>
       <c r="E5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$83,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$87,"open")</f>
         <v>open</v>
       </c>
       <c r="F5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$84,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$88,"open")</f>
         <v>open</v>
       </c>
       <c r="G5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$85,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$89,"open")</f>
         <v>open</v>
       </c>
       <c r="H5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$86,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$90,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30713,27 +30873,27 @@
         <v>1644</v>
       </c>
       <c r="C6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$87,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$91,"open")</f>
         <v>open</v>
       </c>
       <c r="D6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$88,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$92,"open")</f>
         <v>open</v>
       </c>
       <c r="E6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$89,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$93,"open")</f>
         <v>open</v>
       </c>
       <c r="F6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$90,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$94,"open")</f>
         <v>open</v>
       </c>
       <c r="G6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$91,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$95,"open")</f>
         <v>open</v>
       </c>
       <c r="H6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$92,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$96,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30745,27 +30905,27 @@
         <v>1645</v>
       </c>
       <c r="C7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$93,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$97,"open")</f>
         <v>open</v>
       </c>
       <c r="D7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$94,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$98,"open")</f>
         <v>open</v>
       </c>
       <c r="E7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$95,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$99,"open")</f>
         <v>open</v>
       </c>
       <c r="F7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$96,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$100,"open")</f>
         <v>open</v>
       </c>
       <c r="G7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$97,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$101,"open")</f>
         <v>open</v>
       </c>
       <c r="H7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$98,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$102,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30777,27 +30937,27 @@
         <v>1646</v>
       </c>
       <c r="C8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$99,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$103,"open")</f>
         <v>open</v>
       </c>
       <c r="D8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$100,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$104,"open")</f>
         <v>open</v>
       </c>
       <c r="E8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$101,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$105,"open")</f>
         <v>open</v>
       </c>
       <c r="F8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$102,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$106,"open")</f>
         <v>open</v>
       </c>
       <c r="G8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$103,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$107,"open")</f>
         <v>open</v>
       </c>
       <c r="H8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$104,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$108,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30809,27 +30969,27 @@
         <v>1647</v>
       </c>
       <c r="C9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$105,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$109,"open")</f>
         <v>open</v>
       </c>
       <c r="D9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$106,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$110,"open")</f>
         <v>open</v>
       </c>
       <c r="E9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$107,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$111,"open")</f>
         <v>open</v>
       </c>
       <c r="F9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$108,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$112,"open")</f>
         <v>open</v>
       </c>
       <c r="G9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$109,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$113,"open")</f>
         <v>open</v>
       </c>
       <c r="H9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$110,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$114,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30841,27 +31001,27 @@
         <v>1648</v>
       </c>
       <c r="C10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$111,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$115,"open")</f>
         <v>open</v>
       </c>
       <c r="D10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$112,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$116,"open")</f>
         <v>open</v>
       </c>
       <c r="E10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$113,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$117,"open")</f>
         <v>open</v>
       </c>
       <c r="F10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$114,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$118,"open")</f>
         <v>open</v>
       </c>
       <c r="G10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$115,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$119,"open")</f>
         <v>open</v>
       </c>
       <c r="H10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$116,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$120,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30873,27 +31033,27 @@
         <v>1649</v>
       </c>
       <c r="C11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$117,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$121,"open")</f>
         <v>open</v>
       </c>
       <c r="D11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$118,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$122,"open")</f>
         <v>open</v>
       </c>
       <c r="E11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$119,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$123,"open")</f>
         <v>open</v>
       </c>
       <c r="F11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$120,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$124,"open")</f>
         <v>open</v>
       </c>
       <c r="G11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$121,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$125,"open")</f>
         <v>open</v>
       </c>
       <c r="H11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$122,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$126,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30905,27 +31065,27 @@
         <v>1650</v>
       </c>
       <c r="C12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$123,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$127,"open")</f>
         <v>open</v>
       </c>
       <c r="D12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$124,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$128,"open")</f>
         <v>open</v>
       </c>
       <c r="E12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$125,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$129,"open")</f>
         <v>open</v>
       </c>
       <c r="F12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$126,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$130,"open")</f>
         <v>open</v>
       </c>
       <c r="G12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$127,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$131,"open")</f>
         <v>open</v>
       </c>
       <c r="H12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$128,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$132,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30937,27 +31097,27 @@
         <v>1651</v>
       </c>
       <c r="C13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$129,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$133,"open")</f>
         <v>open</v>
       </c>
       <c r="D13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$130,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$134,"open")</f>
         <v>open</v>
       </c>
       <c r="E13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$131,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$135,"open")</f>
         <v>open</v>
       </c>
       <c r="F13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$132,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$136,"open")</f>
         <v>open</v>
       </c>
       <c r="G13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$133,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$137,"open")</f>
         <v>open</v>
       </c>
       <c r="H13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$134,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$138,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -30969,27 +31129,27 @@
         <v>1652</v>
       </c>
       <c r="C14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$135,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$139,"open")</f>
         <v>open</v>
       </c>
       <c r="D14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$136,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$140,"open")</f>
         <v>open</v>
       </c>
       <c r="E14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$137,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$141,"open")</f>
         <v>open</v>
       </c>
       <c r="F14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$138,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$142,"open")</f>
         <v>open</v>
       </c>
       <c r="G14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$139,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$143,"open")</f>
         <v>open</v>
       </c>
       <c r="H14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$140,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$144,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -31001,27 +31161,27 @@
         <v>1653</v>
       </c>
       <c r="C15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$141,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$145,"open")</f>
         <v>open</v>
       </c>
       <c r="D15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$142,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$146,"open")</f>
         <v>open</v>
       </c>
       <c r="E15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$143,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$147,"open")</f>
         <v>open</v>
       </c>
       <c r="F15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$144,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$148,"open")</f>
         <v>open</v>
       </c>
       <c r="G15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$145,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$149,"open")</f>
         <v>open</v>
       </c>
       <c r="H15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$146,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$150,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -31033,27 +31193,27 @@
         <v>1654</v>
       </c>
       <c r="C16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$147,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$151,"open")</f>
         <v>open</v>
       </c>
       <c r="D16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$148,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$152,"open")</f>
         <v>open</v>
       </c>
       <c r="E16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$149,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$153,"open")</f>
         <v>open</v>
       </c>
       <c r="F16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$150,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$154,"open")</f>
         <v>open</v>
       </c>
       <c r="G16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$151,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$155,"open")</f>
         <v>open</v>
       </c>
       <c r="H16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$152,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$156,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -31065,21 +31225,21 @@
         <v>1655</v>
       </c>
       <c r="C17" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$153,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$157,"open")</f>
         <v>open</v>
       </c>
       <c r="D17" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$154,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$158,"open")</f>
         <v>open</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$155,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$159,"open")</f>
         <v>open</v>
       </c>
       <c r="G17" s="7"/>
       <c r="H17" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$156,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$160,"open")</f>
         <v>open</v>
       </c>
     </row>

</xml_diff>

<commit_message>
A7 Unit 5 reviewed before shipping (Barton, adversarial, FAST educator — audit §8): the Q8 transfer surface pulled off the review and the 5.10 set; per-form key notes; Q3 and Q10 as FAST multiselects with the B1G-M misconceptions as choices; Q14 across systems; 'tanks the trip uses'; 5.04 teaches the scale from one pair before the exit asks it; US spellings; standard notes as the state writes them; kit prints Variation in the lines TE. 0 findings, installed, sheet 0 problems
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7ovt6yLjh6QuFV9HBMV4N
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -25,7 +25,7 @@
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'IXL tracker'!$A$4:$K$86</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Scope &amp; Sequence'!$A$1:$AB$132</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Standards!$A$1:$K$61</definedName>
-    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Vocabulary!$A$1:$E$71</definedName>
+    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Vocabulary!$A$1:$E$72</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -302,7 +302,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">MTR.1.1: Example 2 and its Your Turn: a distance, then a time — the first problem that does not stop at the first answer
+          <t xml:space="preserve">MTR.1.1: Example 2 and its Your Turn: the scale is not printed, and the room has to make it from one pair before the question can start
 MTR.4.1: boards 4 and 6 split; the sixty-second re-vote
 MTR.7.1: every board is a plan, a map or a model: the scale is a real object's, and the answer is checked against what a room or a car could be</t>
         </r>
@@ -316,7 +316,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">MTR.6.1: Notes II and board 6: the estimate before the arithmetic — a centimetre is shorter than an inch, so fewer inches; a yard is nearly a metre, so about 270 cm
+          <t xml:space="preserve">MTR.6.1: Notes II and board 6: the estimate before the arithmetic — a centimeter is shorter than an inch, so fewer inches; a yard is nearly a meter, so about 270 cm
 MTR.4.1: boards 4 and 6 split; the sixty-second re-vote on which ratio
 MTR.3.1: boards 5–6: two conversions in a row, each one a form of 1, with the units cancelling on the paper</t>
         </r>
@@ -332,7 +332,7 @@
           </rPr>
           <t xml:space="preserve">MTR.5.1: Notes II: yesterday's k² and today's 144 are the same structure, and the room is asked to say so
 MTR.4.1: boards 4 and 6 split; the sixty-second re-vote
-MTR.6.1: every mass and volume board says its estimate first — fewer kilograms than pounds, more litres than gallons</t>
+MTR.6.1: every mass and volume board says its estimate first — fewer kilograms than pounds, more liters than gallons</t>
         </r>
       </text>
     </comment>
@@ -346,7 +346,7 @@
           </rPr>
           <t xml:space="preserve">MTR.1.1: Notes I and board 4: a problem whose first answer (miles per tank) is not the answer, and the room keeps going
 MTR.6.1: Notes II and board 6: 'which is faster?' is refused until the units match; the answer is checked against the estimate that a mile is longer
-MTR.7.1: boards 8–9: a plan's area in square metres and a choice of car — the unit's whole toolkit on one real question</t>
+MTR.7.1: boards 8–9: a plan's area in square meters and a choice of car — the unit's whole toolkit on one real question</t>
         </r>
       </text>
     </comment>
@@ -574,7 +574,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the scale read as a rate (7.5 ft per inch), the height from it (30 ft), the area from the two real dimensions (787.5 ft²), and a sentence naming which step is the scale factor. A board that scales 3.5 × 4 = 14 in² by 7.5 has not gone to real units first.</t>
+          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the scale made from the pair (7.5 ft per inch, as Example 2 did), the height from it (30 ft), the area from the two real dimensions (787.5 ft²), and a sentence naming which step uses the scale. A board that scales 3.5 × 4 = 14 in² by 7.5 has not gone to real units first.</t>
         </r>
       </text>
     </comment>
@@ -586,7 +586,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the error named (Jo multiplied by the ratio whose 1 is inches, when she had centimetres), the estimate that catches it (inches are longer, so fewer of them), and the fix (30 × 0.39 = 11.7 in). A board that writes the right number with no sentence about the direction has not met the lesson.</t>
+          <t xml:space="preserve">What to look for: Board 9 is written work and it is the exit evidence: the error named (Jo multiplied by the ratio whose 1 is inches, when she had centimeters), the estimate that catches it (inches are longer, so fewer of them), and the fix (30 × 0.39 = 11.7 in). A board that writes the right number with no sentence about the direction has not met the lesson.</t>
         </r>
       </text>
     </comment>
@@ -619,7 +619,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2893" uniqueCount="1932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2896" uniqueCount="1934">
   <si>
     <t xml:space="preserve">A7 — today</t>
   </si>
@@ -1394,7 +1394,7 @@
     <t xml:space="preserve">A room is 2 in by 3 in on a plan at 1 in : 4 ft. Why is its real area not 6 × 4 square feet?</t>
   </si>
   <si>
-    <t xml:space="preserve">floor plan, scale (two units), unit rate of a scale</t>
+    <t xml:space="preserve">floor plan, scale (two units), unit rate of a scale, scale with one unit</t>
   </si>
   <si>
     <t xml:space="preserve">MA.K12.MTR.1.1 Actively participate in effortful learning both individually and collectively.
@@ -1402,10 +1402,10 @@
 MA.K12.MTR.7.1 Apply mathematics to real-world contexts.</t>
   </si>
   <si>
-    <t xml:space="preserve">Andrew's drawing shows a wall 3.5 in wide; the real wall is 26.25 ft wide. The drawn height is 4 in. Find the real height and the wall's real area, and say which step uses the scale factor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 ft high; 787.5 ft². The scale factor (7.5 ft per in) is the step from 4 in to 30 ft.</t>
+    <t xml:space="preserve">On Andrew's drawing a wall is 3.5 in wide and 4 in tall; the real wall is 26.25 ft wide. Find the real height and the real area, and say which step uses the scale.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 ft high; 787.5 ft². The scale (7.5 ft per in) is the step from 4 in to 30 ft.</t>
   </si>
   <si>
     <t xml:space="preserve">5.4 Solving Problems Involving Real-World Scale Drawings</t>
@@ -1443,7 +1443,7 @@
     <t xml:space="preserve">1 in = 2.54 cm and 1 cm = 0.39 in. Jo converts 30 cm to inches by multiplying by 2.54 and gets 76.2 in. Name the error and fix it.</t>
   </si>
   <si>
-    <t xml:space="preserve">She used the inches ratio on centimetres. Inches are bigger, so fewer: 11.7 in.</t>
+    <t xml:space="preserve">She used the inches ratio on centimeters. Inches are bigger, so fewer: 11.7 in.</t>
   </si>
   <si>
     <t xml:space="preserve">5.6 Currency Conversions
@@ -1487,7 +1487,7 @@
     <t xml:space="preserve">I can solve a problem that takes two or more proportional steps, including a unit conversion, and compare two rates given in different units.</t>
   </si>
   <si>
-    <t xml:space="preserve">A car does 100 km/h and another does 65 mi/h. Why can't you say which is faster yet?</t>
+    <t xml:space="preserve">A car gets 100 km/h and another does 65 mi/h. Why can't you say which is faster yet?</t>
   </si>
   <si>
     <t xml:space="preserve">unit rate, proportional, per</t>
@@ -5697,6 +5697,12 @@
     <t xml:space="preserve">the scale written per 1 drawing unit: ¼ in : 1 ft is 1 in : 4 ft</t>
   </si>
   <si>
+    <t xml:space="preserve">scale with one unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 : 50 — no units: 1 cm of model is 50 cm of car. 1 in : 4 ft is 1 : 48 this way, and 48 is the scale factor</t>
+  </si>
+  <si>
     <t xml:space="preserve">customary</t>
   </si>
   <si>
@@ -5706,7 +5712,7 @@
     <t xml:space="preserve">metric</t>
   </si>
   <si>
-    <t xml:space="preserve">the centimetre–metre–kilometre–kilogram–litre system</t>
+    <t xml:space="preserve">the centimeter–meter–kilometer–kilogram–liter system</t>
   </si>
   <si>
     <t xml:space="preserve">conversion ratio</t>
@@ -5970,7 +5976,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 892ae8e7 on 18 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 97bd28d6 on 18 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -7943,12 +7949,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="67" t="s">
-        <v>1656</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="68" t="s">
-        <v>1657</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7956,52 +7962,52 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="67" t="s">
-        <v>1658</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="68" t="s">
-        <v>1659</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="68" t="s">
-        <v>1660</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="68" t="s">
-        <v>1661</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="68" t="s">
-        <v>1662</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="68" t="s">
-        <v>1663</v>
+        <v>1665</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="68" t="s">
-        <v>1664</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="68" t="s">
-        <v>1665</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="68" t="s">
-        <v>1666</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="68" t="s">
-        <v>1667</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8009,47 +8015,47 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="67" t="s">
-        <v>1668</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="68" t="s">
-        <v>1669</v>
+        <v>1671</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="68" t="s">
-        <v>1670</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="68" t="s">
-        <v>1671</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="68" t="s">
-        <v>1672</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="68" t="s">
-        <v>1673</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="68" t="s">
-        <v>1674</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="68" t="s">
-        <v>1675</v>
+        <v>1677</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="68" t="s">
-        <v>1676</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8057,12 +8063,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="67" t="s">
-        <v>1677</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="68" t="s">
-        <v>1678</v>
+        <v>1680</v>
       </c>
     </row>
   </sheetData>
@@ -8126,13 +8132,13 @@
       </c>
       <c r="N1" s="69"/>
       <c r="O1" s="69" t="s">
-        <v>1679</v>
+        <v>1681</v>
       </c>
       <c r="P1" s="69" t="s">
-        <v>1680</v>
+        <v>1682</v>
       </c>
       <c r="Q1" s="69" t="s">
-        <v>1681</v>
+        <v>1683</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8184,14 +8190,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M2" s="69" t="s">
-        <v>1682</v>
+        <v>1684</v>
       </c>
       <c r="N2" s="69"/>
       <c r="O2" s="69" t="s">
-        <v>1683</v>
+        <v>1685</v>
       </c>
       <c r="P2" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q2" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k999a58eef73f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22")</f>
@@ -8247,14 +8253,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M3" s="69" t="s">
-        <v>1685</v>
+        <v>1687</v>
       </c>
       <c r="N3" s="69"/>
       <c r="O3" s="69" t="s">
+        <v>1688</v>
+      </c>
+      <c r="P3" s="69" t="s">
         <v>1686</v>
-      </c>
-      <c r="P3" s="69" t="s">
-        <v>1684</v>
       </c>
       <c r="Q3" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b0883f744a4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22")</f>
@@ -8310,14 +8316,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M4" s="69" t="s">
-        <v>1687</v>
+        <v>1689</v>
       </c>
       <c r="N4" s="69"/>
       <c r="O4" s="69" t="s">
-        <v>1688</v>
+        <v>1690</v>
       </c>
       <c r="P4" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q4" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4e34d1ba5135",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22")</f>
@@ -8373,14 +8379,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M5" s="69" t="s">
-        <v>1689</v>
+        <v>1691</v>
       </c>
       <c r="N5" s="69"/>
       <c r="O5" s="69" t="s">
-        <v>1690</v>
+        <v>1692</v>
       </c>
       <c r="P5" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q5" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k654621d73a39",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22")</f>
@@ -8436,14 +8442,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M6" s="69" t="s">
-        <v>1691</v>
+        <v>1693</v>
       </c>
       <c r="N6" s="69"/>
       <c r="O6" s="69" t="s">
-        <v>1692</v>
+        <v>1694</v>
       </c>
       <c r="P6" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q6" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k05aafdefef87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22")</f>
@@ -8499,14 +8505,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M7" s="69" t="s">
-        <v>1693</v>
+        <v>1695</v>
       </c>
       <c r="N7" s="69"/>
       <c r="O7" s="69" t="s">
-        <v>1694</v>
+        <v>1696</v>
       </c>
       <c r="P7" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q7" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0fe1632a0900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22")</f>
@@ -8534,10 +8540,10 @@
       <c r="M8" s="69"/>
       <c r="N8" s="69"/>
       <c r="O8" s="69" t="s">
-        <v>1695</v>
+        <v>1697</v>
       </c>
       <c r="P8" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q8" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kadb8b2686141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22")</f>
@@ -8565,10 +8571,10 @@
       <c r="M9" s="69"/>
       <c r="N9" s="69"/>
       <c r="O9" s="69" t="s">
-        <v>1696</v>
+        <v>1698</v>
       </c>
       <c r="P9" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q9" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4c613b2b0958",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22")</f>
@@ -8624,14 +8630,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M10" s="69" t="s">
-        <v>1697</v>
+        <v>1699</v>
       </c>
       <c r="N10" s="69"/>
       <c r="O10" s="69" t="s">
-        <v>1698</v>
+        <v>1700</v>
       </c>
       <c r="P10" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q10" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd60a700332eb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22")</f>
@@ -8687,14 +8693,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M11" s="69" t="s">
-        <v>1699</v>
+        <v>1701</v>
       </c>
       <c r="N11" s="69"/>
       <c r="O11" s="69" t="s">
-        <v>1700</v>
+        <v>1702</v>
       </c>
       <c r="P11" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q11" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k509a716d7468",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22")</f>
@@ -8750,14 +8756,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M12" s="69" t="s">
-        <v>1701</v>
+        <v>1703</v>
       </c>
       <c r="N12" s="69"/>
       <c r="O12" s="69" t="s">
-        <v>1702</v>
+        <v>1704</v>
       </c>
       <c r="P12" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q12" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke52ff0df0d4b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22")</f>
@@ -8785,10 +8791,10 @@
       <c r="M13" s="69"/>
       <c r="N13" s="69"/>
       <c r="O13" s="69" t="s">
-        <v>1703</v>
+        <v>1705</v>
       </c>
       <c r="P13" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q13" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf990f1c33e7d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22")</f>
@@ -8844,14 +8850,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
       <c r="M14" s="69" t="s">
-        <v>1704</v>
+        <v>1706</v>
       </c>
       <c r="N14" s="69"/>
       <c r="O14" s="69" t="s">
-        <v>1705</v>
+        <v>1707</v>
       </c>
       <c r="P14" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q14" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb93ffed6ca63",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22")</f>
@@ -8885,10 +8891,10 @@
       <c r="M15" s="69"/>
       <c r="N15" s="69"/>
       <c r="O15" s="69" t="s">
-        <v>1706</v>
+        <v>1708</v>
       </c>
       <c r="P15" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q15" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k467ef44c3569",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22")</f>
@@ -8922,10 +8928,10 @@
       <c r="M16" s="69"/>
       <c r="N16" s="69"/>
       <c r="O16" s="69" t="s">
-        <v>1707</v>
+        <v>1709</v>
       </c>
       <c r="P16" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q16" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1f816ed6a0ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22")</f>
@@ -8959,10 +8965,10 @@
       <c r="M17" s="69"/>
       <c r="N17" s="69"/>
       <c r="O17" s="69" t="s">
-        <v>1708</v>
+        <v>1710</v>
       </c>
       <c r="P17" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q17" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7c17b9b2eea3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test.pdf%22")</f>
@@ -9018,14 +9024,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M18" s="69" t="s">
-        <v>1709</v>
+        <v>1711</v>
       </c>
       <c r="N18" s="69"/>
       <c r="O18" s="69" t="s">
-        <v>1710</v>
+        <v>1712</v>
       </c>
       <c r="P18" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q18" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k584fc57b9722",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20-%20Key.pdf%22")</f>
@@ -9081,14 +9087,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M19" s="69" t="s">
-        <v>1711</v>
+        <v>1713</v>
       </c>
       <c r="N19" s="69"/>
       <c r="O19" s="69" t="s">
-        <v>1712</v>
+        <v>1714</v>
       </c>
       <c r="P19" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q19" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke57d72cf0716",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22")</f>
@@ -9144,14 +9150,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M20" s="69" t="s">
-        <v>1713</v>
+        <v>1715</v>
       </c>
       <c r="N20" s="69"/>
       <c r="O20" s="69" t="s">
-        <v>1714</v>
+        <v>1716</v>
       </c>
       <c r="P20" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q20" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dd5b368d2b0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22")</f>
@@ -9207,14 +9213,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M21" s="69" t="s">
-        <v>1715</v>
+        <v>1717</v>
       </c>
       <c r="N21" s="69"/>
       <c r="O21" s="69" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="P21" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q21" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb2536de7152",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22")</f>
@@ -9270,14 +9276,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M22" s="69" t="s">
-        <v>1717</v>
+        <v>1719</v>
       </c>
       <c r="N22" s="69"/>
       <c r="O22" s="69" t="s">
-        <v>1718</v>
+        <v>1720</v>
       </c>
       <c r="P22" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q22" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k11cedfe615ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22")</f>
@@ -9333,14 +9339,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
       <c r="M23" s="69" t="s">
-        <v>1719</v>
+        <v>1721</v>
       </c>
       <c r="N23" s="69"/>
       <c r="O23" s="69" t="s">
-        <v>1720</v>
+        <v>1722</v>
       </c>
       <c r="P23" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q23" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k34f09723e09c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
@@ -9374,10 +9380,10 @@
       <c r="M24" s="69"/>
       <c r="N24" s="69"/>
       <c r="O24" s="69" t="s">
-        <v>1721</v>
+        <v>1723</v>
       </c>
       <c r="P24" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q24" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b4473b65910",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22")</f>
@@ -9411,10 +9417,10 @@
       <c r="M25" s="69"/>
       <c r="N25" s="69"/>
       <c r="O25" s="69" t="s">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="P25" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q25" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1c81628b7541",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22")</f>
@@ -9470,14 +9476,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M26" s="69" t="s">
-        <v>1723</v>
+        <v>1725</v>
       </c>
       <c r="N26" s="69"/>
       <c r="O26" s="69" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="P26" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q26" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k60f05a144797",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22")</f>
@@ -9533,14 +9539,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M27" s="69" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="N27" s="69"/>
       <c r="O27" s="69" t="s">
-        <v>1726</v>
+        <v>1728</v>
       </c>
       <c r="P27" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q27" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2f48d7f422a9",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
@@ -9596,14 +9602,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M28" s="69" t="s">
-        <v>1728</v>
+        <v>1730</v>
       </c>
       <c r="N28" s="69"/>
       <c r="O28" s="69" t="s">
-        <v>1729</v>
+        <v>1731</v>
       </c>
       <c r="P28" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q28" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8fdeab195866",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
@@ -9659,14 +9665,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M29" s="69" t="s">
-        <v>1730</v>
+        <v>1732</v>
       </c>
       <c r="N29" s="69"/>
       <c r="O29" s="69" t="s">
-        <v>1731</v>
+        <v>1733</v>
       </c>
       <c r="P29" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q29" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k05aafdefef87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22")</f>
@@ -9722,14 +9728,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M30" s="69" t="s">
-        <v>1732</v>
+        <v>1734</v>
       </c>
       <c r="N30" s="69"/>
       <c r="O30" s="69" t="s">
-        <v>1733</v>
+        <v>1735</v>
       </c>
       <c r="P30" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q30" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4e34d1ba5135",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22")</f>
@@ -9785,14 +9791,14 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M31" s="69" t="s">
-        <v>1734</v>
+        <v>1736</v>
       </c>
       <c r="N31" s="69"/>
       <c r="O31" s="69" t="s">
-        <v>1735</v>
+        <v>1737</v>
       </c>
       <c r="P31" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q31" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k654621d73a39",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22")</f>
@@ -9826,10 +9832,10 @@
       <c r="M32" s="69"/>
       <c r="N32" s="69"/>
       <c r="O32" s="69" t="s">
-        <v>1736</v>
+        <v>1738</v>
       </c>
       <c r="P32" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q32" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k999a58eef73f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22")</f>
@@ -9863,10 +9869,10 @@
       <c r="M33" s="69"/>
       <c r="N33" s="69"/>
       <c r="O33" s="69" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="P33" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q33" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b0883f744a4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22")</f>
@@ -9889,14 +9895,14 @@
       <c r="K34" s="69"/>
       <c r="L34" s="69"/>
       <c r="M34" s="69" t="s">
-        <v>1738</v>
+        <v>1740</v>
       </c>
       <c r="N34" s="69"/>
       <c r="O34" s="69" t="s">
-        <v>1739</v>
+        <v>1741</v>
       </c>
       <c r="P34" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q34" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2ed79628bc59",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
@@ -9919,14 +9925,14 @@
       <c r="K35" s="69"/>
       <c r="L35" s="69"/>
       <c r="M35" s="69" t="s">
-        <v>1740</v>
+        <v>1742</v>
       </c>
       <c r="N35" s="69"/>
       <c r="O35" s="69" t="s">
-        <v>1741</v>
+        <v>1743</v>
       </c>
       <c r="P35" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q35" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kf1ee50ed8929",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
@@ -9949,14 +9955,14 @@
       <c r="K36" s="69"/>
       <c r="L36" s="69"/>
       <c r="M36" s="69" t="s">
-        <v>1742</v>
+        <v>1744</v>
       </c>
       <c r="N36" s="69"/>
       <c r="O36" s="69" t="s">
-        <v>1743</v>
+        <v>1745</v>
       </c>
       <c r="P36" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q36" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k749da75b36af",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
@@ -9979,14 +9985,14 @@
       <c r="K37" s="69"/>
       <c r="L37" s="69"/>
       <c r="M37" s="69" t="s">
-        <v>1744</v>
+        <v>1746</v>
       </c>
       <c r="N37" s="69"/>
       <c r="O37" s="69" t="s">
-        <v>1745</v>
+        <v>1747</v>
       </c>
       <c r="P37" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q37" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k509a716d7468",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22")</f>
@@ -10009,14 +10015,14 @@
       <c r="K38" s="69"/>
       <c r="L38" s="69"/>
       <c r="M38" s="69" t="s">
-        <v>1746</v>
+        <v>1748</v>
       </c>
       <c r="N38" s="69"/>
       <c r="O38" s="69" t="s">
-        <v>1747</v>
+        <v>1749</v>
       </c>
       <c r="P38" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q38" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4c613b2b0958",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22")</f>
@@ -10039,14 +10045,14 @@
       <c r="K39" s="69"/>
       <c r="L39" s="69"/>
       <c r="M39" s="69" t="s">
-        <v>1748</v>
+        <v>1750</v>
       </c>
       <c r="N39" s="69"/>
       <c r="O39" s="69" t="s">
-        <v>1749</v>
+        <v>1751</v>
       </c>
       <c r="P39" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q39" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd60a700332eb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22")</f>
@@ -10069,14 +10075,14 @@
       <c r="K40" s="69"/>
       <c r="L40" s="69"/>
       <c r="M40" s="69" t="s">
-        <v>1750</v>
+        <v>1752</v>
       </c>
       <c r="N40" s="69"/>
       <c r="O40" s="69" t="s">
-        <v>1751</v>
+        <v>1753</v>
       </c>
       <c r="P40" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q40" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0fe1632a0900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22")</f>
@@ -10099,14 +10105,14 @@
       <c r="K41" s="69"/>
       <c r="L41" s="69"/>
       <c r="M41" s="69" t="s">
-        <v>1752</v>
+        <v>1754</v>
       </c>
       <c r="N41" s="69"/>
       <c r="O41" s="69" t="s">
-        <v>1753</v>
+        <v>1755</v>
       </c>
       <c r="P41" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q41" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kadb8b2686141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22")</f>
@@ -10131,10 +10137,10 @@
       <c r="M42" s="69"/>
       <c r="N42" s="69"/>
       <c r="O42" s="69" t="s">
-        <v>1754</v>
+        <v>1756</v>
       </c>
       <c r="P42" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q42" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k986a7bd5b0f8",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
@@ -10159,10 +10165,10 @@
       <c r="M43" s="69"/>
       <c r="N43" s="69"/>
       <c r="O43" s="69" t="s">
-        <v>1755</v>
+        <v>1757</v>
       </c>
       <c r="P43" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q43" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kb8fed8266c53",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
@@ -10187,10 +10193,10 @@
       <c r="M44" s="69"/>
       <c r="N44" s="69"/>
       <c r="O44" s="69" t="s">
-        <v>1756</v>
+        <v>1758</v>
       </c>
       <c r="P44" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q44" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb737ddcb3701",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
@@ -10215,10 +10221,10 @@
       <c r="M45" s="69"/>
       <c r="N45" s="69"/>
       <c r="O45" s="69" t="s">
-        <v>1757</v>
+        <v>1759</v>
       </c>
       <c r="P45" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q45" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1f816ed6a0ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22")</f>
@@ -10241,14 +10247,14 @@
       <c r="K46" s="69"/>
       <c r="L46" s="69"/>
       <c r="M46" s="69" t="s">
-        <v>1758</v>
+        <v>1760</v>
       </c>
       <c r="N46" s="69"/>
       <c r="O46" s="69" t="s">
-        <v>1759</v>
+        <v>1761</v>
       </c>
       <c r="P46" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q46" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb93ffed6ca63",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22")</f>
@@ -10271,14 +10277,14 @@
       <c r="K47" s="69"/>
       <c r="L47" s="69"/>
       <c r="M47" s="69" t="s">
-        <v>1760</v>
+        <v>1762</v>
       </c>
       <c r="N47" s="69"/>
       <c r="O47" s="69" t="s">
-        <v>1761</v>
+        <v>1763</v>
       </c>
       <c r="P47" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q47" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k467ef44c3569",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22")</f>
@@ -10301,14 +10307,14 @@
       <c r="K48" s="69"/>
       <c r="L48" s="69"/>
       <c r="M48" s="69" t="s">
-        <v>1762</v>
+        <v>1764</v>
       </c>
       <c r="N48" s="69"/>
       <c r="O48" s="69" t="s">
-        <v>1763</v>
+        <v>1765</v>
       </c>
       <c r="P48" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q48" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke52ff0df0d4b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22")</f>
@@ -10331,14 +10337,14 @@
       <c r="K49" s="69"/>
       <c r="L49" s="69"/>
       <c r="M49" s="69" t="s">
-        <v>1764</v>
+        <v>1766</v>
       </c>
       <c r="N49" s="69"/>
       <c r="O49" s="69" t="s">
-        <v>1765</v>
+        <v>1767</v>
       </c>
       <c r="P49" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q49" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf990f1c33e7d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22")</f>
@@ -10361,14 +10367,14 @@
       <c r="K50" s="69"/>
       <c r="L50" s="69"/>
       <c r="M50" s="69" t="s">
-        <v>1766</v>
+        <v>1768</v>
       </c>
       <c r="N50" s="69"/>
       <c r="O50" s="69" t="s">
-        <v>1767</v>
+        <v>1769</v>
       </c>
       <c r="P50" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q50" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k85bc365a5352",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
@@ -10393,10 +10399,10 @@
       <c r="M51" s="69"/>
       <c r="N51" s="69"/>
       <c r="O51" s="69" t="s">
-        <v>1768</v>
+        <v>1770</v>
       </c>
       <c r="P51" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q51" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k19f682b91838",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
@@ -10421,10 +10427,10 @@
       <c r="M52" s="69"/>
       <c r="N52" s="69"/>
       <c r="O52" s="69" t="s">
-        <v>1769</v>
+        <v>1771</v>
       </c>
       <c r="P52" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q52" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k44624f8b3141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
@@ -10449,10 +10455,10 @@
       <c r="M53" s="69"/>
       <c r="N53" s="69"/>
       <c r="O53" s="69" t="s">
-        <v>1770</v>
+        <v>1772</v>
       </c>
       <c r="P53" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q53" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb2536de7152",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22")</f>
@@ -10477,10 +10483,10 @@
       <c r="M54" s="69"/>
       <c r="N54" s="69"/>
       <c r="O54" s="69" t="s">
-        <v>1771</v>
+        <v>1773</v>
       </c>
       <c r="P54" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q54" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke57d72cf0716",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22")</f>
@@ -10505,10 +10511,10 @@
       <c r="M55" s="69"/>
       <c r="N55" s="69"/>
       <c r="O55" s="69" t="s">
-        <v>1772</v>
+        <v>1774</v>
       </c>
       <c r="P55" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q55" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dd5b368d2b0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22")</f>
@@ -10531,14 +10537,14 @@
       <c r="K56" s="69"/>
       <c r="L56" s="69"/>
       <c r="M56" s="69" t="s">
-        <v>1773</v>
+        <v>1775</v>
       </c>
       <c r="N56" s="69"/>
       <c r="O56" s="69" t="s">
-        <v>1774</v>
+        <v>1776</v>
       </c>
       <c r="P56" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q56" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7c17b9b2eea3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test.pdf%22")</f>
@@ -10561,14 +10567,14 @@
       <c r="K57" s="69"/>
       <c r="L57" s="69"/>
       <c r="M57" s="69" t="s">
-        <v>1775</v>
+        <v>1777</v>
       </c>
       <c r="N57" s="69"/>
       <c r="O57" s="69" t="s">
-        <v>1776</v>
+        <v>1778</v>
       </c>
       <c r="P57" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q57" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k584fc57b9722",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20-%20Key.pdf%22")</f>
@@ -10591,14 +10597,14 @@
       <c r="K58" s="69"/>
       <c r="L58" s="69"/>
       <c r="M58" s="69" t="s">
-        <v>1777</v>
+        <v>1779</v>
       </c>
       <c r="N58" s="69"/>
       <c r="O58" s="69" t="s">
-        <v>1778</v>
+        <v>1780</v>
       </c>
       <c r="P58" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q58" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k395c44aceb1d",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
@@ -10621,14 +10627,14 @@
       <c r="K59" s="69"/>
       <c r="L59" s="69"/>
       <c r="M59" s="69" t="s">
-        <v>1779</v>
+        <v>1781</v>
       </c>
       <c r="N59" s="69"/>
       <c r="O59" s="69" t="s">
-        <v>1780</v>
+        <v>1782</v>
       </c>
       <c r="P59" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q59" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k57de004b2b0a",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
@@ -10651,14 +10657,14 @@
       <c r="K60" s="69"/>
       <c r="L60" s="69"/>
       <c r="M60" s="69" t="s">
-        <v>1781</v>
+        <v>1783</v>
       </c>
       <c r="N60" s="69"/>
       <c r="O60" s="69" t="s">
-        <v>1782</v>
+        <v>1784</v>
       </c>
       <c r="P60" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q60" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbcf7b890879b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
@@ -10681,14 +10687,14 @@
       <c r="K61" s="69"/>
       <c r="L61" s="69"/>
       <c r="M61" s="69" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
       <c r="N61" s="69"/>
       <c r="O61" s="69" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
       <c r="P61" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q61" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k60f05a144797",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22")</f>
@@ -10711,14 +10717,14 @@
       <c r="K62" s="69"/>
       <c r="L62" s="69"/>
       <c r="M62" s="69" t="s">
-        <v>1785</v>
+        <v>1787</v>
       </c>
       <c r="N62" s="69"/>
       <c r="O62" s="69" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
       <c r="P62" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q62" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b4473b65910",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22")</f>
@@ -10743,10 +10749,10 @@
       <c r="M63" s="69"/>
       <c r="N63" s="69"/>
       <c r="O63" s="69" t="s">
-        <v>1787</v>
+        <v>1789</v>
       </c>
       <c r="P63" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q63" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1c81628b7541",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22")</f>
@@ -10771,10 +10777,10 @@
       <c r="M64" s="69"/>
       <c r="N64" s="69"/>
       <c r="O64" s="69" t="s">
-        <v>1788</v>
+        <v>1790</v>
       </c>
       <c r="P64" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q64" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k11cedfe615ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22")</f>
@@ -10799,10 +10805,10 @@
       <c r="M65" s="69"/>
       <c r="N65" s="69"/>
       <c r="O65" s="69" t="s">
-        <v>1789</v>
+        <v>1791</v>
       </c>
       <c r="P65" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q65" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k34f09723e09c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
@@ -10827,10 +10833,10 @@
       <c r="M66" s="69"/>
       <c r="N66" s="69"/>
       <c r="O66" s="69" t="s">
-        <v>1790</v>
+        <v>1792</v>
       </c>
       <c r="P66" s="69" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="Q66" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k5fd6e0a77786",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
@@ -10855,10 +10861,10 @@
       <c r="M67" s="69"/>
       <c r="N67" s="69"/>
       <c r="O67" s="69" t="s">
-        <v>1791</v>
+        <v>1793</v>
       </c>
       <c r="P67" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q67" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf7444edd4950",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22")</f>
@@ -10883,10 +10889,10 @@
       <c r="M68" s="69"/>
       <c r="N68" s="69"/>
       <c r="O68" s="69" t="s">
-        <v>1792</v>
+        <v>1794</v>
       </c>
       <c r="P68" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q68" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbb6e44272bb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
@@ -10911,10 +10917,10 @@
       <c r="M69" s="69"/>
       <c r="N69" s="69"/>
       <c r="O69" s="69" t="s">
-        <v>1793</v>
+        <v>1795</v>
       </c>
       <c r="P69" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q69" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc68dd81311bb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22")</f>
@@ -10937,14 +10943,14 @@
       <c r="K70" s="69"/>
       <c r="L70" s="69"/>
       <c r="M70" s="69" t="s">
-        <v>1794</v>
+        <v>1796</v>
       </c>
       <c r="N70" s="69"/>
       <c r="O70" s="69" t="s">
-        <v>1795</v>
+        <v>1797</v>
       </c>
       <c r="P70" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q70" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k70c393f4e972",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -10967,14 +10973,14 @@
       <c r="K71" s="69"/>
       <c r="L71" s="69"/>
       <c r="M71" s="69" t="s">
-        <v>1796</v>
+        <v>1798</v>
       </c>
       <c r="N71" s="69"/>
       <c r="O71" s="69" t="s">
-        <v>1797</v>
+        <v>1799</v>
       </c>
       <c r="P71" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q71" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1d60e486567d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -10997,14 +11003,14 @@
       <c r="K72" s="69"/>
       <c r="L72" s="69"/>
       <c r="M72" s="69" t="s">
-        <v>1798</v>
+        <v>1800</v>
       </c>
       <c r="N72" s="69"/>
       <c r="O72" s="69" t="s">
-        <v>1799</v>
+        <v>1801</v>
       </c>
       <c r="P72" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q72" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k40dc62cd52a5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11027,14 +11033,14 @@
       <c r="K73" s="69"/>
       <c r="L73" s="69"/>
       <c r="M73" s="69" t="s">
-        <v>1800</v>
+        <v>1802</v>
       </c>
       <c r="N73" s="69"/>
       <c r="O73" s="69" t="s">
-        <v>1801</v>
+        <v>1803</v>
       </c>
       <c r="P73" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q73" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42d053aa97d9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22")</f>
@@ -11057,14 +11063,14 @@
       <c r="K74" s="69"/>
       <c r="L74" s="69"/>
       <c r="M74" s="69" t="s">
-        <v>1802</v>
+        <v>1804</v>
       </c>
       <c r="N74" s="69"/>
       <c r="O74" s="69" t="s">
-        <v>1803</v>
+        <v>1805</v>
       </c>
       <c r="P74" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q74" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3d5b3115f0ff",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11087,14 +11093,14 @@
       <c r="K75" s="69"/>
       <c r="L75" s="69"/>
       <c r="M75" s="69" t="s">
-        <v>1804</v>
+        <v>1806</v>
       </c>
       <c r="N75" s="69"/>
       <c r="O75" s="69" t="s">
-        <v>1805</v>
+        <v>1807</v>
       </c>
       <c r="P75" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q75" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b6284c3dfc8",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22")</f>
@@ -11117,14 +11123,14 @@
       <c r="K76" s="69"/>
       <c r="L76" s="69"/>
       <c r="M76" s="69" t="s">
-        <v>1806</v>
+        <v>1808</v>
       </c>
       <c r="N76" s="69"/>
       <c r="O76" s="69" t="s">
-        <v>1807</v>
+        <v>1809</v>
       </c>
       <c r="P76" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q76" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k751991f77144",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11147,14 +11153,14 @@
       <c r="K77" s="69"/>
       <c r="L77" s="69"/>
       <c r="M77" s="69" t="s">
-        <v>1808</v>
+        <v>1810</v>
       </c>
       <c r="N77" s="69"/>
       <c r="O77" s="69" t="s">
-        <v>1809</v>
+        <v>1811</v>
       </c>
       <c r="P77" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q77" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6386e55cce43",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11179,10 +11185,10 @@
       <c r="M78" s="69"/>
       <c r="N78" s="69"/>
       <c r="O78" s="69" t="s">
-        <v>1810</v>
+        <v>1812</v>
       </c>
       <c r="P78" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q78" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb55aff075211",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11207,10 +11213,10 @@
       <c r="M79" s="69"/>
       <c r="N79" s="69"/>
       <c r="O79" s="69" t="s">
-        <v>1811</v>
+        <v>1813</v>
       </c>
       <c r="P79" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q79" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k78f3bd7641b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22")</f>
@@ -11233,14 +11239,14 @@
       <c r="K80" s="69"/>
       <c r="L80" s="69"/>
       <c r="M80" s="69" t="s">
-        <v>1812</v>
+        <v>1814</v>
       </c>
       <c r="N80" s="69"/>
       <c r="O80" s="69" t="s">
-        <v>1813</v>
+        <v>1815</v>
       </c>
       <c r="P80" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q80" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab82b01c89fe",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11263,14 +11269,14 @@
       <c r="K81" s="69"/>
       <c r="L81" s="69"/>
       <c r="M81" s="69" t="s">
-        <v>1814</v>
+        <v>1816</v>
       </c>
       <c r="N81" s="69"/>
       <c r="O81" s="69" t="s">
-        <v>1815</v>
+        <v>1817</v>
       </c>
       <c r="P81" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q81" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb5633697c8e5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22")</f>
@@ -11293,14 +11299,14 @@
       <c r="K82" s="69"/>
       <c r="L82" s="69"/>
       <c r="M82" s="69" t="s">
-        <v>1816</v>
+        <v>1818</v>
       </c>
       <c r="N82" s="69"/>
       <c r="O82" s="69" t="s">
-        <v>1817</v>
+        <v>1819</v>
       </c>
       <c r="P82" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q82" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf724d6e842b3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11323,14 +11329,14 @@
       <c r="K83" s="69"/>
       <c r="L83" s="69"/>
       <c r="M83" s="69" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="N83" s="69"/>
       <c r="O83" s="69" t="s">
-        <v>1819</v>
+        <v>1821</v>
       </c>
       <c r="P83" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q83" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k36b71975bd76",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11353,14 +11359,14 @@
       <c r="K84" s="69"/>
       <c r="L84" s="69"/>
       <c r="M84" s="69" t="s">
-        <v>1820</v>
+        <v>1822</v>
       </c>
       <c r="N84" s="69"/>
       <c r="O84" s="69" t="s">
-        <v>1821</v>
+        <v>1823</v>
       </c>
       <c r="P84" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q84" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd7994f0255be",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11383,14 +11389,14 @@
       <c r="K85" s="69"/>
       <c r="L85" s="69"/>
       <c r="M85" s="69" t="s">
-        <v>1822</v>
+        <v>1824</v>
       </c>
       <c r="N85" s="69"/>
       <c r="O85" s="69" t="s">
-        <v>1823</v>
+        <v>1825</v>
       </c>
       <c r="P85" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q85" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k441c122ac61a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22")</f>
@@ -11413,14 +11419,14 @@
       <c r="K86" s="69"/>
       <c r="L86" s="69"/>
       <c r="M86" s="69" t="s">
-        <v>1824</v>
+        <v>1826</v>
       </c>
       <c r="N86" s="69"/>
       <c r="O86" s="69" t="s">
-        <v>1825</v>
+        <v>1827</v>
       </c>
       <c r="P86" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q86" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcad6ba0a7c20",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11445,10 +11451,10 @@
       <c r="M87" s="69"/>
       <c r="N87" s="69"/>
       <c r="O87" s="69" t="s">
-        <v>1826</v>
+        <v>1828</v>
       </c>
       <c r="P87" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q87" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kecd875ec58e7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22")</f>
@@ -11473,10 +11479,10 @@
       <c r="M88" s="69"/>
       <c r="N88" s="69"/>
       <c r="O88" s="69" t="s">
-        <v>1827</v>
+        <v>1829</v>
       </c>
       <c r="P88" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q88" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k04385d48a56f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11501,10 +11507,10 @@
       <c r="M89" s="69"/>
       <c r="N89" s="69"/>
       <c r="O89" s="69" t="s">
-        <v>1828</v>
+        <v>1830</v>
       </c>
       <c r="P89" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q89" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kaa89f6499257",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11527,14 +11533,14 @@
       <c r="K90" s="69"/>
       <c r="L90" s="69"/>
       <c r="M90" s="69" t="s">
-        <v>1829</v>
+        <v>1831</v>
       </c>
       <c r="N90" s="69"/>
       <c r="O90" s="69" t="s">
-        <v>1830</v>
+        <v>1832</v>
       </c>
       <c r="P90" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q90" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc0dcbe2e82c2",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11557,14 +11563,14 @@
       <c r="K91" s="69"/>
       <c r="L91" s="69"/>
       <c r="M91" s="69" t="s">
-        <v>1831</v>
+        <v>1833</v>
       </c>
       <c r="N91" s="69"/>
       <c r="O91" s="69" t="s">
-        <v>1832</v>
+        <v>1834</v>
       </c>
       <c r="P91" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q91" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k368f7f8b9908",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22")</f>
@@ -11587,14 +11593,14 @@
       <c r="K92" s="69"/>
       <c r="L92" s="69"/>
       <c r="M92" s="69" t="s">
-        <v>1833</v>
+        <v>1835</v>
       </c>
       <c r="N92" s="69"/>
       <c r="O92" s="69" t="s">
-        <v>1834</v>
+        <v>1836</v>
       </c>
       <c r="P92" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q92" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k53d619094fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11617,14 +11623,14 @@
       <c r="K93" s="69"/>
       <c r="L93" s="69"/>
       <c r="M93" s="69" t="s">
-        <v>1835</v>
+        <v>1837</v>
       </c>
       <c r="N93" s="69"/>
       <c r="O93" s="69" t="s">
-        <v>1836</v>
+        <v>1838</v>
       </c>
       <c r="P93" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q93" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf511d84233f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22")</f>
@@ -11649,10 +11655,10 @@
       <c r="M94" s="69"/>
       <c r="N94" s="69"/>
       <c r="O94" s="69" t="s">
-        <v>1837</v>
+        <v>1839</v>
       </c>
       <c r="P94" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q94" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9da92cf1af2b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11675,14 +11681,14 @@
       <c r="K95" s="69"/>
       <c r="L95" s="69"/>
       <c r="M95" s="69" t="s">
-        <v>1838</v>
+        <v>1840</v>
       </c>
       <c r="N95" s="69"/>
       <c r="O95" s="69" t="s">
-        <v>1839</v>
+        <v>1841</v>
       </c>
       <c r="P95" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q95" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k515087871fe0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11705,14 +11711,14 @@
       <c r="K96" s="69"/>
       <c r="L96" s="69"/>
       <c r="M96" s="69" t="s">
-        <v>1840</v>
+        <v>1842</v>
       </c>
       <c r="N96" s="69"/>
       <c r="O96" s="69" t="s">
-        <v>1841</v>
+        <v>1843</v>
       </c>
       <c r="P96" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q96" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb6acc983851",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11737,10 +11743,10 @@
       <c r="M97" s="69"/>
       <c r="N97" s="69"/>
       <c r="O97" s="69" t="s">
-        <v>1842</v>
+        <v>1844</v>
       </c>
       <c r="P97" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q97" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9cdee450b988",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22")</f>
@@ -11765,10 +11771,10 @@
       <c r="M98" s="69"/>
       <c r="N98" s="69"/>
       <c r="O98" s="69" t="s">
-        <v>1843</v>
+        <v>1845</v>
       </c>
       <c r="P98" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q98" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kac1e5e18d498",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11793,10 +11799,10 @@
       <c r="M99" s="69"/>
       <c r="N99" s="69"/>
       <c r="O99" s="69" t="s">
-        <v>1844</v>
+        <v>1846</v>
       </c>
       <c r="P99" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q99" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb5db6608070",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22")</f>
@@ -11821,10 +11827,10 @@
       <c r="M100" s="69"/>
       <c r="N100" s="69"/>
       <c r="O100" s="69" t="s">
-        <v>1845</v>
+        <v>1847</v>
       </c>
       <c r="P100" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q100" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf2a43f4ef780",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -11847,14 +11853,14 @@
       <c r="K101" s="69"/>
       <c r="L101" s="69"/>
       <c r="M101" s="69" t="s">
-        <v>1846</v>
+        <v>1848</v>
       </c>
       <c r="N101" s="69"/>
       <c r="O101" s="69" t="s">
-        <v>1847</v>
+        <v>1849</v>
       </c>
       <c r="P101" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q101" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k86b940633ffd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11877,14 +11883,14 @@
       <c r="K102" s="69"/>
       <c r="L102" s="69"/>
       <c r="M102" s="69" t="s">
-        <v>1848</v>
+        <v>1850</v>
       </c>
       <c r="N102" s="69"/>
       <c r="O102" s="69" t="s">
-        <v>1849</v>
+        <v>1851</v>
       </c>
       <c r="P102" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q102" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf341ebe84b57",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -11907,14 +11913,14 @@
       <c r="K103" s="69"/>
       <c r="L103" s="69"/>
       <c r="M103" s="69" t="s">
-        <v>1850</v>
+        <v>1852</v>
       </c>
       <c r="N103" s="69"/>
       <c r="O103" s="69" t="s">
-        <v>1851</v>
+        <v>1853</v>
       </c>
       <c r="P103" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q103" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7383ee3f2ec5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22")</f>
@@ -11937,14 +11943,14 @@
       <c r="K104" s="69"/>
       <c r="L104" s="69"/>
       <c r="M104" s="69" t="s">
-        <v>1852</v>
+        <v>1854</v>
       </c>
       <c r="N104" s="69"/>
       <c r="O104" s="69" t="s">
-        <v>1853</v>
+        <v>1855</v>
       </c>
       <c r="P104" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q104" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5cae8f95e8bd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
@@ -11967,14 +11973,14 @@
       <c r="K105" s="69"/>
       <c r="L105" s="69"/>
       <c r="M105" s="69" t="s">
-        <v>1854</v>
+        <v>1856</v>
       </c>
       <c r="N105" s="69"/>
       <c r="O105" s="69" t="s">
-        <v>1855</v>
+        <v>1857</v>
       </c>
       <c r="P105" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q105" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0ecee6c15886",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22")</f>
@@ -11997,14 +12003,14 @@
       <c r="K106" s="69"/>
       <c r="L106" s="69"/>
       <c r="M106" s="69" t="s">
-        <v>1856</v>
+        <v>1858</v>
       </c>
       <c r="N106" s="69"/>
       <c r="O106" s="69" t="s">
-        <v>1857</v>
+        <v>1859</v>
       </c>
       <c r="P106" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q106" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k874b463422ce",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12027,14 +12033,14 @@
       <c r="K107" s="69"/>
       <c r="L107" s="69"/>
       <c r="M107" s="69" t="s">
-        <v>1858</v>
+        <v>1860</v>
       </c>
       <c r="N107" s="69"/>
       <c r="O107" s="69" t="s">
-        <v>1859</v>
+        <v>1861</v>
       </c>
       <c r="P107" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q107" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k07aa4ed88482",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12059,10 +12065,10 @@
       <c r="M108" s="69"/>
       <c r="N108" s="69"/>
       <c r="O108" s="69" t="s">
-        <v>1860</v>
+        <v>1862</v>
       </c>
       <c r="P108" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q108" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k444ff4b9a71a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12087,10 +12093,10 @@
       <c r="M109" s="69"/>
       <c r="N109" s="69"/>
       <c r="O109" s="69" t="s">
-        <v>1861</v>
+        <v>1863</v>
       </c>
       <c r="P109" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q109" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42b7580a8cb9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22")</f>
@@ -12113,14 +12119,14 @@
       <c r="K110" s="69"/>
       <c r="L110" s="69"/>
       <c r="M110" s="69" t="s">
-        <v>1862</v>
+        <v>1864</v>
       </c>
       <c r="N110" s="69"/>
       <c r="O110" s="69" t="s">
-        <v>1863</v>
+        <v>1865</v>
       </c>
       <c r="P110" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q110" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8e5410dc08f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12143,14 +12149,14 @@
       <c r="K111" s="69"/>
       <c r="L111" s="69"/>
       <c r="M111" s="69" t="s">
-        <v>1864</v>
+        <v>1866</v>
       </c>
       <c r="N111" s="69"/>
       <c r="O111" s="69" t="s">
-        <v>1865</v>
+        <v>1867</v>
       </c>
       <c r="P111" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q111" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb0df0c43cf87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22")</f>
@@ -12173,14 +12179,14 @@
       <c r="K112" s="69"/>
       <c r="L112" s="69"/>
       <c r="M112" s="69" t="s">
-        <v>1866</v>
+        <v>1868</v>
       </c>
       <c r="N112" s="69"/>
       <c r="O112" s="69" t="s">
-        <v>1867</v>
+        <v>1869</v>
       </c>
       <c r="P112" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q112" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kde315e91893f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12205,10 +12211,10 @@
       <c r="M113" s="69"/>
       <c r="N113" s="69"/>
       <c r="O113" s="69" t="s">
-        <v>1868</v>
+        <v>1870</v>
       </c>
       <c r="P113" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q113" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf9cc95eccf07",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12233,10 +12239,10 @@
       <c r="M114" s="69"/>
       <c r="N114" s="69"/>
       <c r="O114" s="69" t="s">
-        <v>1869</v>
+        <v>1871</v>
       </c>
       <c r="P114" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q114" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd674be572fbd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12259,14 +12265,14 @@
       <c r="K115" s="69"/>
       <c r="L115" s="69"/>
       <c r="M115" s="69" t="s">
-        <v>1870</v>
+        <v>1872</v>
       </c>
       <c r="N115" s="69"/>
       <c r="O115" s="69" t="s">
-        <v>1871</v>
+        <v>1873</v>
       </c>
       <c r="P115" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q115" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4f3c12075c6f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22")</f>
@@ -12289,14 +12295,14 @@
       <c r="K116" s="69"/>
       <c r="L116" s="69"/>
       <c r="M116" s="69" t="s">
-        <v>1872</v>
+        <v>1874</v>
       </c>
       <c r="N116" s="69"/>
       <c r="O116" s="69" t="s">
-        <v>1873</v>
+        <v>1875</v>
       </c>
       <c r="P116" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q116" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k856d2d13cd04",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12319,14 +12325,14 @@
       <c r="K117" s="69"/>
       <c r="L117" s="69"/>
       <c r="M117" s="69" t="s">
-        <v>1874</v>
+        <v>1876</v>
       </c>
       <c r="N117" s="69"/>
       <c r="O117" s="69" t="s">
-        <v>1875</v>
+        <v>1877</v>
       </c>
       <c r="P117" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q117" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k160e960d09c4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22")</f>
@@ -12349,14 +12355,14 @@
       <c r="K118" s="69"/>
       <c r="L118" s="69"/>
       <c r="M118" s="69" t="s">
-        <v>1876</v>
+        <v>1878</v>
       </c>
       <c r="N118" s="69"/>
       <c r="O118" s="69" t="s">
-        <v>1877</v>
+        <v>1879</v>
       </c>
       <c r="P118" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q118" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd3a48013b455",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12379,14 +12385,14 @@
       <c r="K119" s="69"/>
       <c r="L119" s="69"/>
       <c r="M119" s="69" t="s">
-        <v>1878</v>
+        <v>1880</v>
       </c>
       <c r="N119" s="69"/>
       <c r="O119" s="69" t="s">
-        <v>1879</v>
+        <v>1881</v>
       </c>
       <c r="P119" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q119" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f26b556436e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12409,14 +12415,14 @@
       <c r="K120" s="69"/>
       <c r="L120" s="69"/>
       <c r="M120" s="69" t="s">
-        <v>1880</v>
+        <v>1882</v>
       </c>
       <c r="N120" s="69"/>
       <c r="O120" s="69" t="s">
-        <v>1881</v>
+        <v>1883</v>
       </c>
       <c r="P120" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q120" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3a6534dc5a62",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12439,14 +12445,14 @@
       <c r="K121" s="69"/>
       <c r="L121" s="69"/>
       <c r="M121" s="69" t="s">
-        <v>1882</v>
+        <v>1884</v>
       </c>
       <c r="N121" s="69"/>
       <c r="O121" s="69" t="s">
-        <v>1883</v>
+        <v>1885</v>
       </c>
       <c r="P121" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q121" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ka5734698aa50",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22")</f>
@@ -12469,14 +12475,14 @@
       <c r="K122" s="69"/>
       <c r="L122" s="69"/>
       <c r="M122" s="69" t="s">
-        <v>1884</v>
+        <v>1886</v>
       </c>
       <c r="N122" s="69"/>
       <c r="O122" s="69" t="s">
-        <v>1885</v>
+        <v>1887</v>
       </c>
       <c r="P122" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q122" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3bd1b440e87a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12499,14 +12505,14 @@
       <c r="K123" s="69"/>
       <c r="L123" s="69"/>
       <c r="M123" s="69" t="s">
-        <v>1886</v>
+        <v>1888</v>
       </c>
       <c r="N123" s="69"/>
       <c r="O123" s="69" t="s">
-        <v>1887</v>
+        <v>1889</v>
       </c>
       <c r="P123" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q123" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k52493b74eb28",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22")</f>
@@ -12529,14 +12535,14 @@
       <c r="K124" s="69"/>
       <c r="L124" s="69"/>
       <c r="M124" s="69" t="s">
-        <v>1888</v>
+        <v>1890</v>
       </c>
       <c r="N124" s="69"/>
       <c r="O124" s="69" t="s">
-        <v>1889</v>
+        <v>1891</v>
       </c>
       <c r="P124" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q124" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3fa800b9318b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12561,10 +12567,10 @@
       <c r="M125" s="69"/>
       <c r="N125" s="69"/>
       <c r="O125" s="69" t="s">
-        <v>1890</v>
+        <v>1892</v>
       </c>
       <c r="P125" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q125" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b2764e691f7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12589,10 +12595,10 @@
       <c r="M126" s="69"/>
       <c r="N126" s="69"/>
       <c r="O126" s="69" t="s">
-        <v>1891</v>
+        <v>1893</v>
       </c>
       <c r="P126" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q126" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9afa96310f5f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12615,14 +12621,14 @@
       <c r="K127" s="69"/>
       <c r="L127" s="69"/>
       <c r="M127" s="69" t="s">
-        <v>1892</v>
+        <v>1894</v>
       </c>
       <c r="N127" s="69"/>
       <c r="O127" s="69" t="s">
-        <v>1893</v>
+        <v>1895</v>
       </c>
       <c r="P127" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q127" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3eb4a6e4e0a9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22")</f>
@@ -12645,14 +12651,14 @@
       <c r="K128" s="69"/>
       <c r="L128" s="69"/>
       <c r="M128" s="69" t="s">
-        <v>1894</v>
+        <v>1896</v>
       </c>
       <c r="N128" s="69"/>
       <c r="O128" s="69" t="s">
-        <v>1895</v>
+        <v>1897</v>
       </c>
       <c r="P128" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q128" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3786dea98f2a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12677,10 +12683,10 @@
       <c r="M129" s="69"/>
       <c r="N129" s="69"/>
       <c r="O129" s="69" t="s">
-        <v>1896</v>
+        <v>1898</v>
       </c>
       <c r="P129" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q129" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8424cc4e78b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22")</f>
@@ -12705,10 +12711,10 @@
       <c r="M130" s="69"/>
       <c r="N130" s="69"/>
       <c r="O130" s="69" t="s">
-        <v>1897</v>
+        <v>1899</v>
       </c>
       <c r="P130" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q130" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf325ac36b969",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12733,10 +12739,10 @@
       <c r="M131" s="69"/>
       <c r="N131" s="69"/>
       <c r="O131" s="69" t="s">
-        <v>1898</v>
+        <v>1900</v>
       </c>
       <c r="P131" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q131" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4ec5ffc67bf1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12761,10 +12767,10 @@
       <c r="M132" s="69"/>
       <c r="N132" s="69"/>
       <c r="O132" s="69" t="s">
-        <v>1899</v>
+        <v>1901</v>
       </c>
       <c r="P132" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q132" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k006e6e337926",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12787,10 +12793,10 @@
       <c r="M133" s="69"/>
       <c r="N133" s="69"/>
       <c r="O133" s="69" t="s">
-        <v>1900</v>
+        <v>1902</v>
       </c>
       <c r="P133" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q133" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k94da89c1d16d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22")</f>
@@ -12813,10 +12819,10 @@
       <c r="M134" s="69"/>
       <c r="N134" s="69"/>
       <c r="O134" s="69" t="s">
-        <v>1901</v>
+        <v>1903</v>
       </c>
       <c r="P134" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q134" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9b79f94a3042",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12839,10 +12845,10 @@
       <c r="M135" s="69"/>
       <c r="N135" s="69"/>
       <c r="O135" s="69" t="s">
-        <v>1902</v>
+        <v>1904</v>
       </c>
       <c r="P135" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q135" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b57aec5f42c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22")</f>
@@ -12865,10 +12871,10 @@
       <c r="M136" s="69"/>
       <c r="N136" s="69"/>
       <c r="O136" s="69" t="s">
-        <v>1903</v>
+        <v>1905</v>
       </c>
       <c r="P136" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q136" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k524993898ff0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -12891,10 +12897,10 @@
       <c r="M137" s="69"/>
       <c r="N137" s="69"/>
       <c r="O137" s="69" t="s">
-        <v>1904</v>
+        <v>1906</v>
       </c>
       <c r="P137" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q137" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k71038ca67fed",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12917,10 +12923,10 @@
       <c r="M138" s="69"/>
       <c r="N138" s="69"/>
       <c r="O138" s="69" t="s">
-        <v>1905</v>
+        <v>1907</v>
       </c>
       <c r="P138" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q138" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab565ddcecfd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -12943,10 +12949,10 @@
       <c r="M139" s="69"/>
       <c r="N139" s="69"/>
       <c r="O139" s="69" t="s">
-        <v>1906</v>
+        <v>1908</v>
       </c>
       <c r="P139" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q139" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kda9320d99fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22")</f>
@@ -12969,10 +12975,10 @@
       <c r="M140" s="69"/>
       <c r="N140" s="69"/>
       <c r="O140" s="69" t="s">
-        <v>1907</v>
+        <v>1909</v>
       </c>
       <c r="P140" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q140" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k577a4eca3248",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22")</f>
@@ -12995,10 +13001,10 @@
       <c r="M141" s="69"/>
       <c r="N141" s="69"/>
       <c r="O141" s="69" t="s">
-        <v>1908</v>
+        <v>1910</v>
       </c>
       <c r="P141" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q141" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dbd9d8294a0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22")</f>
@@ -13021,10 +13027,10 @@
       <c r="M142" s="69"/>
       <c r="N142" s="69"/>
       <c r="O142" s="69" t="s">
-        <v>1909</v>
+        <v>1911</v>
       </c>
       <c r="P142" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q142" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k858285f0484a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -13047,10 +13053,10 @@
       <c r="M143" s="69"/>
       <c r="N143" s="69"/>
       <c r="O143" s="69" t="s">
-        <v>1910</v>
+        <v>1912</v>
       </c>
       <c r="P143" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q143" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3386b404a0cc",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -13073,10 +13079,10 @@
       <c r="M144" s="69"/>
       <c r="N144" s="69"/>
       <c r="O144" s="69" t="s">
-        <v>1911</v>
+        <v>1913</v>
       </c>
       <c r="P144" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q144" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1fdcada6b7d5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -13099,10 +13105,10 @@
       <c r="M145" s="69"/>
       <c r="N145" s="69"/>
       <c r="O145" s="69" t="s">
-        <v>1912</v>
+        <v>1914</v>
       </c>
       <c r="P145" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q145" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k66ad104dc3f4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22")</f>
@@ -13125,10 +13131,10 @@
       <c r="M146" s="69"/>
       <c r="N146" s="69"/>
       <c r="O146" s="69" t="s">
-        <v>1913</v>
+        <v>1915</v>
       </c>
       <c r="P146" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q146" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f9d2ee2e87b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
@@ -13151,10 +13157,10 @@
       <c r="M147" s="69"/>
       <c r="N147" s="69"/>
       <c r="O147" s="69" t="s">
-        <v>1914</v>
+        <v>1916</v>
       </c>
       <c r="P147" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q147" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k2e021d1404f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22")</f>
@@ -13177,10 +13183,10 @@
       <c r="M148" s="69"/>
       <c r="N148" s="69"/>
       <c r="O148" s="69" t="s">
-        <v>1915</v>
+        <v>1917</v>
       </c>
       <c r="P148" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q148" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7f727f839de9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -13203,10 +13209,10 @@
       <c r="M149" s="69"/>
       <c r="N149" s="69"/>
       <c r="O149" s="69" t="s">
-        <v>1916</v>
+        <v>1918</v>
       </c>
       <c r="P149" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q149" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc9f54d815229",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -13229,10 +13235,10 @@
       <c r="M150" s="69"/>
       <c r="N150" s="69"/>
       <c r="O150" s="69" t="s">
-        <v>1917</v>
+        <v>1919</v>
       </c>
       <c r="P150" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q150" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k814de685731b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -13255,10 +13261,10 @@
       <c r="M151" s="69"/>
       <c r="N151" s="69"/>
       <c r="O151" s="69" t="s">
-        <v>1918</v>
+        <v>1920</v>
       </c>
       <c r="P151" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q151" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbeebbf583a30",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22")</f>
@@ -13281,10 +13287,10 @@
       <c r="M152" s="69"/>
       <c r="N152" s="69"/>
       <c r="O152" s="69" t="s">
-        <v>1919</v>
+        <v>1921</v>
       </c>
       <c r="P152" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q152" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kae76dda4b45d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22")</f>
@@ -13307,10 +13313,10 @@
       <c r="M153" s="69"/>
       <c r="N153" s="69"/>
       <c r="O153" s="69" t="s">
-        <v>1920</v>
+        <v>1922</v>
       </c>
       <c r="P153" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q153" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1228a3dffde6",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22")</f>
@@ -13333,10 +13339,10 @@
       <c r="M154" s="69"/>
       <c r="N154" s="69"/>
       <c r="O154" s="69" t="s">
-        <v>1921</v>
+        <v>1923</v>
       </c>
       <c r="P154" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q154" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k47f0af99bd1e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -13359,10 +13365,10 @@
       <c r="M155" s="69"/>
       <c r="N155" s="69"/>
       <c r="O155" s="69" t="s">
-        <v>1922</v>
+        <v>1924</v>
       </c>
       <c r="P155" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q155" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcee0b8f57c67",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -13385,10 +13391,10 @@
       <c r="M156" s="69"/>
       <c r="N156" s="69"/>
       <c r="O156" s="69" t="s">
-        <v>1923</v>
+        <v>1925</v>
       </c>
       <c r="P156" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q156" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k59fb8b4ed900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -13411,10 +13417,10 @@
       <c r="M157" s="69"/>
       <c r="N157" s="69"/>
       <c r="O157" s="69" t="s">
-        <v>1924</v>
+        <v>1926</v>
       </c>
       <c r="P157" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q157" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1a00a0a22804",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22")</f>
@@ -13437,10 +13443,10 @@
       <c r="M158" s="69"/>
       <c r="N158" s="69"/>
       <c r="O158" s="69" t="s">
-        <v>1925</v>
+        <v>1927</v>
       </c>
       <c r="P158" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q158" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k29d47d551984",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
@@ -13463,10 +13469,10 @@
       <c r="M159" s="69"/>
       <c r="N159" s="69"/>
       <c r="O159" s="69" t="s">
-        <v>1926</v>
+        <v>1928</v>
       </c>
       <c r="P159" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q159" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdc81e4a42f98",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
@@ -13489,10 +13495,10 @@
       <c r="M160" s="69"/>
       <c r="N160" s="69"/>
       <c r="O160" s="69" t="s">
-        <v>1927</v>
+        <v>1929</v>
       </c>
       <c r="P160" s="69" t="s">
-        <v>1684</v>
+        <v>1686</v>
       </c>
       <c r="Q160" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc34b261fea84",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
@@ -13525,16 +13531,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="71" t="s">
-        <v>1928</v>
+        <v>1930</v>
       </c>
       <c r="B1" s="71" t="s">
-        <v>1929</v>
+        <v>1931</v>
       </c>
       <c r="C1" s="71" t="s">
-        <v>1930</v>
+        <v>1932</v>
       </c>
       <c r="D1" s="71" t="s">
-        <v>1931</v>
+        <v>1933</v>
       </c>
     </row>
   </sheetData>
@@ -27557,7 +27563,7 @@
         <v>1029</v>
       </c>
       <c r="F80" s="7" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="G80" s="46"/>
     </row>
@@ -28707,7 +28713,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -29725,10 +29731,10 @@
         <v>5</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="C60" s="65" t="n">
-        <v>46328</v>
+        <v>46325</v>
       </c>
       <c r="D60" s="66" t="s">
         <v>1587</v>
@@ -29793,10 +29799,10 @@
         <v>5</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="C64" s="65" t="n">
-        <v>46329</v>
+        <v>46328</v>
       </c>
       <c r="D64" s="66" t="s">
         <v>1595</v>
@@ -29878,10 +29884,10 @@
         <v>5</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="C69" s="65" t="n">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="D69" s="66" t="s">
         <v>1605</v>
@@ -29924,8 +29930,25 @@
         <v>1610</v>
       </c>
     </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="46" t="n">
+        <v>5</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="C72" s="65" t="n">
+        <v>46330</v>
+      </c>
+      <c r="D72" s="66" t="s">
+        <v>1611</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>1612</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E71"/>
+  <autoFilter ref="A1:E72"/>
   <hyperlinks>
     <hyperlink ref="C2" location="'Scope &amp; Sequence'!A2" display="#'Scope &amp; Sequence'.A2"/>
     <hyperlink ref="C3" location="'Scope &amp; Sequence'!A2" display="#'Scope &amp; Sequence'.A2"/>
@@ -29985,18 +30008,19 @@
     <hyperlink ref="C57" location="'Scope &amp; Sequence'!A28" display="#'Scope &amp; Sequence'.A28"/>
     <hyperlink ref="C58" location="'Scope &amp; Sequence'!A28" display="#'Scope &amp; Sequence'.A28"/>
     <hyperlink ref="C59" location="'Scope &amp; Sequence'!A28" display="#'Scope &amp; Sequence'.A28"/>
-    <hyperlink ref="C60" location="'Scope &amp; Sequence'!A29" display="#'Scope &amp; Sequence'.A29"/>
+    <hyperlink ref="C60" location="'Scope &amp; Sequence'!A28" display="#'Scope &amp; Sequence'.A28"/>
     <hyperlink ref="C61" location="'Scope &amp; Sequence'!A29" display="#'Scope &amp; Sequence'.A29"/>
     <hyperlink ref="C62" location="'Scope &amp; Sequence'!A29" display="#'Scope &amp; Sequence'.A29"/>
     <hyperlink ref="C63" location="'Scope &amp; Sequence'!A29" display="#'Scope &amp; Sequence'.A29"/>
-    <hyperlink ref="C64" location="'Scope &amp; Sequence'!A30" display="#'Scope &amp; Sequence'.A30"/>
+    <hyperlink ref="C64" location="'Scope &amp; Sequence'!A29" display="#'Scope &amp; Sequence'.A29"/>
     <hyperlink ref="C65" location="'Scope &amp; Sequence'!A30" display="#'Scope &amp; Sequence'.A30"/>
     <hyperlink ref="C66" location="'Scope &amp; Sequence'!A30" display="#'Scope &amp; Sequence'.A30"/>
     <hyperlink ref="C67" location="'Scope &amp; Sequence'!A30" display="#'Scope &amp; Sequence'.A30"/>
     <hyperlink ref="C68" location="'Scope &amp; Sequence'!A30" display="#'Scope &amp; Sequence'.A30"/>
-    <hyperlink ref="C69" location="'Scope &amp; Sequence'!A31" display="#'Scope &amp; Sequence'.A31"/>
+    <hyperlink ref="C69" location="'Scope &amp; Sequence'!A30" display="#'Scope &amp; Sequence'.A30"/>
     <hyperlink ref="C70" location="'Scope &amp; Sequence'!A31" display="#'Scope &amp; Sequence'.A31"/>
     <hyperlink ref="C71" location="'Scope &amp; Sequence'!A31" display="#'Scope &amp; Sequence'.A31"/>
+    <hyperlink ref="C72" location="'Scope &amp; Sequence'!A31" display="#'Scope &amp; Sequence'.A31"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -30035,7 +30059,7 @@
         <v>30</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1611</v>
+        <v>1613</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>958</v>
@@ -30044,34 +30068,34 @@
         <v>959</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>1612</v>
+        <v>1614</v>
       </c>
       <c r="F1" s="9" t="s">
         <v>705</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>1613</v>
+        <v>1615</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>1614</v>
+        <v>1616</v>
       </c>
       <c r="I1" s="9" t="s">
         <v>1245</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>1615</v>
+        <v>1617</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>1244</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>1616</v>
+        <v>1618</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>1617</v>
+        <v>1619</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>1618</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30079,7 +30103,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>1619</v>
+        <v>1621</v>
       </c>
       <c r="C2" s="52" t="s">
         <v>1247</v>
@@ -30087,7 +30111,7 @@
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
       <c r="F2" s="6" t="s">
-        <v>1620</v>
+        <v>1622</v>
       </c>
       <c r="G2" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$27,"folder")</f>
@@ -30127,7 +30151,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1621</v>
+        <v>1623</v>
       </c>
       <c r="C3" s="52" t="s">
         <v>1247</v>
@@ -30135,7 +30159,7 @@
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
       <c r="F3" s="6" t="s">
-        <v>1620</v>
+        <v>1622</v>
       </c>
       <c r="G3" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$35,"folder")</f>
@@ -30175,7 +30199,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>1622</v>
+        <v>1624</v>
       </c>
       <c r="C4" s="51" t="n">
         <v>46288</v>
@@ -30188,7 +30212,7 @@
         <v>16</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>1623</v>
+        <v>1625</v>
       </c>
       <c r="G4" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$43,"folder")</f>
@@ -30228,7 +30252,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>1624</v>
+        <v>1626</v>
       </c>
       <c r="C5" s="51" t="n">
         <v>46311</v>
@@ -30241,7 +30265,7 @@
         <v>8</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>1623</v>
+        <v>1625</v>
       </c>
       <c r="G5" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$51,"folder")</f>
@@ -30281,7 +30305,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>1625</v>
+        <v>1627</v>
       </c>
       <c r="C6" s="51" t="n">
         <v>46323</v>
@@ -30294,7 +30318,7 @@
         <v>8</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>1620</v>
+        <v>1622</v>
       </c>
       <c r="G6" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$59,"folder")</f>
@@ -30334,7 +30358,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>1626</v>
+        <v>1628</v>
       </c>
       <c r="C7" s="51" t="n">
         <v>46335</v>
@@ -30363,7 +30387,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>1627</v>
+        <v>1629</v>
       </c>
       <c r="C8" s="51" t="n">
         <v>46359</v>
@@ -30392,7 +30416,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>1628</v>
+        <v>1630</v>
       </c>
       <c r="C9" s="51" t="n">
         <v>46373</v>
@@ -30421,7 +30445,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>1629</v>
+        <v>1631</v>
       </c>
       <c r="C10" s="51" t="n">
         <v>46398</v>
@@ -30450,7 +30474,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>1630</v>
+        <v>1632</v>
       </c>
       <c r="C11" s="51" t="n">
         <v>46412</v>
@@ -30479,7 +30503,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>1631</v>
+        <v>1633</v>
       </c>
       <c r="C12" s="51" t="n">
         <v>46426</v>
@@ -30508,7 +30532,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="C13" s="51" t="n">
         <v>46441</v>
@@ -30537,7 +30561,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="C14" s="51" t="n">
         <v>46457</v>
@@ -30566,7 +30590,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="C15" s="51" t="n">
         <v>46477</v>
@@ -30595,7 +30619,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>1635</v>
+        <v>1637</v>
       </c>
       <c r="C16" s="51" t="n">
         <v>46484</v>
@@ -30624,7 +30648,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>1636</v>
+        <v>1638</v>
       </c>
       <c r="C17" s="51" t="n">
         <v>46497</v>
@@ -30653,7 +30677,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>1637</v>
+        <v>1639</v>
       </c>
       <c r="C18" s="51" t="n">
         <v>46503</v>
@@ -30679,7 +30703,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>1638</v>
+        <v>1640</v>
       </c>
     </row>
   </sheetData>
@@ -30728,7 +30752,7 @@
         <v>15</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="G1" s="9" t="s">
         <v>16</v>
@@ -30742,7 +30766,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>1640</v>
+        <v>1642</v>
       </c>
       <c r="C2" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$67,"open")</f>
@@ -30774,7 +30798,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>1641</v>
+        <v>1643</v>
       </c>
       <c r="C3" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$73,"open")</f>
@@ -30806,7 +30830,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>1642</v>
+        <v>1644</v>
       </c>
       <c r="C4" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$79,"open")</f>
@@ -30838,7 +30862,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>1643</v>
+        <v>1645</v>
       </c>
       <c r="C5" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$85,"open")</f>
@@ -30870,7 +30894,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>1644</v>
+        <v>1646</v>
       </c>
       <c r="C6" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$91,"open")</f>
@@ -30902,7 +30926,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>1645</v>
+        <v>1647</v>
       </c>
       <c r="C7" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$97,"open")</f>
@@ -30934,7 +30958,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>1646</v>
+        <v>1648</v>
       </c>
       <c r="C8" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$103,"open")</f>
@@ -30966,7 +30990,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>1647</v>
+        <v>1649</v>
       </c>
       <c r="C9" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$109,"open")</f>
@@ -30998,7 +31022,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>1648</v>
+        <v>1650</v>
       </c>
       <c r="C10" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$115,"open")</f>
@@ -31030,7 +31054,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>1649</v>
+        <v>1651</v>
       </c>
       <c r="C11" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$121,"open")</f>
@@ -31062,7 +31086,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>1650</v>
+        <v>1652</v>
       </c>
       <c r="C12" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$127,"open")</f>
@@ -31094,7 +31118,7 @@
         <v>2</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>1651</v>
+        <v>1653</v>
       </c>
       <c r="C13" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$133,"open")</f>
@@ -31126,7 +31150,7 @@
         <v>2</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>1652</v>
+        <v>1654</v>
       </c>
       <c r="C14" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$139,"open")</f>
@@ -31158,7 +31182,7 @@
         <v>2</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="C15" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$145,"open")</f>
@@ -31190,7 +31214,7 @@
         <v>2</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>1654</v>
+        <v>1656</v>
       </c>
       <c r="C16" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$151,"open")</f>
@@ -31222,7 +31246,7 @@
         <v>2</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>1655</v>
+        <v>1657</v>
       </c>
       <c r="C17" s="8" t="str">
         <f aca="false">HYPERLINK(Links!$Q$157,"open")</f>

</xml_diff>

<commit_message>
A7 Unit 5: the mathematics of every stem, board, prompt and choice typeset in LaTeX (Croix: 'rewrite the math to be in latex') — tools/texify_u5.py did the pass; title-slide boxes and asks stay plain; long math rows split into sentences; kit vendored (inline math on the baseline at text size; quantities as words on the Lexend papers). 0 findings, installed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7ovt6yLjh6QuFV9HBMV4N
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -5664,7 +5664,7 @@
     <t xml:space="preserve">k squared</t>
   </si>
   <si>
-    <t xml:space="preserve">k², k times k: the number an area is multiplied by when every length is multiplied by k</t>
+    <t xml:space="preserve">k², k times k: what an area is multiplied by when every length is multiplied by k</t>
   </si>
   <si>
     <t xml:space="preserve">perimeter ratio</t>
@@ -5688,13 +5688,13 @@
     <t xml:space="preserve">scale (two units)</t>
   </si>
   <si>
-    <t xml:space="preserve">a ratio such as ¼ in : 1 ft — a drawing length and the real length it stands for</t>
+    <t xml:space="preserve">a ratio such as (1/4) in : 1 ft — a drawing length and the real length it stands for</t>
   </si>
   <si>
     <t xml:space="preserve">unit rate of a scale</t>
   </si>
   <si>
-    <t xml:space="preserve">the scale written per 1 drawing unit: ¼ in : 1 ft is 1 in : 4 ft</t>
+    <t xml:space="preserve">the scale written per 1 drawing unit: (1/4) in : 1 ft is 1 in : 4 ft</t>
   </si>
   <si>
     <t xml:space="preserve">scale with one unit</t>
@@ -5976,7 +5976,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 97bd28d6 on 18 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit dea2f836 on 18 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>

</xml_diff>

<commit_message>
Ruling 49 in the toolchain: a unit built as the practice test alone — kit, START HERE, master sheet and its check, the teacher copy's random-set bar
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7ovt6yLjh6QuFV9HBMV4N
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -5896,7 +5896,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit f8972665 on 24 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 59ae2d29 on 24 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -8117,8 +8117,8 @@
         <v>1668</v>
       </c>
       <c r="Q2" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k999a58eef73f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b09413fba3b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test.pdf%22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8180,8 +8180,8 @@
         <v>1668</v>
       </c>
       <c r="Q3" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b0883f744a4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb7a4b26081c5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9711,8 +9711,8 @@
         <v>1668</v>
       </c>
       <c r="Q32" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k999a58eef73f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b09413fba3b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test.pdf%22</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9741,8 +9741,8 @@
         <v>1668</v>
       </c>
       <c r="Q33" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b0883f744a4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Test%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb7a4b26081c5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
A7 Unit 6 installed and its practice page built, on Windmill c9c3e8a (Croix: "Fix it. I give you permission") — the kit gives a wrapping IXL skill name the rows it needs, so T-B1 slide 35 no longer overprints and build_all.py u6 --install ran at 0 gate and 0 check findings (161 files, 13 zips, the question bank reference); master sheet regenerated, 0 problems. The practice page and the teacher copy built by run.py after every check: u6_check sound on 3,000 sets, verify, 31 of 31 planted errors caught, the lock, the variety floor, the kit's browser check. The teacher copy prints the test as random sets with the paper's shape: no set number on a student's sheet, points on the head, sections and parts, the follow-through line, the key with its set number and the score tracker. Both kits vendored at c9c3e8a; NOTES.md brought up to date.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Be467MLKJu6DjkSsjpM7D
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -801,7 +801,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3011" uniqueCount="1991">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3030" uniqueCount="2001">
   <si>
     <t xml:space="preserve">A7 — today</t>
   </si>
@@ -1885,79 +1885,79 @@
     <t xml:space="preserve">Unit 6 exam</t>
   </si>
   <si>
+    <t xml:space="preserve">T-B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thread B: angle pairs — supplementary, complementary, vertical, adjacent (16.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identify complementary, supplementary, vertical, adjacent, and congruent angles — HGV; Find measures of complementary, supplementary, vertical, and adjacent angles — R2B; Write and solve equations using angle relationships — DBV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I can name an angle pair and use it to find a missing angle, with an equation when the angles are expressions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When two angles are neighbours or opposites, what does one tell you about the other?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adjacent angles, vertical angles, complementary angles, supplementary angles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.GR.1.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MA.8.GR.1.4 — Solve mathematical problems involving the relationships between supplementary, complementary, vertical or adjacent angles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can two vertical angles be complementary? Always, sometimes or never? Explain.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sometimes — only when each is 45°.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.1 Angle Relationships</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-B2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thread B: interior and exterior angles of a triangle (16.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Find missing angles in triangles — JFJ; Exterior Angle Theorem — FMP; Triangle Angle-Sum Theorem — 6Q6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I can find a missing angle of a triangle, inside or outside, with the Triangle Sum and the Exterior Angle Theorem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why do the three angles of every triangle add to the same number?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interior angle, exterior angle, remote interior angles, Triangle Sum Theorem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.GR.1.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MA.8.GR.1.5 — Solve problems involving the relationships of interior and exterior angles of a triangle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why is an exterior angle of a triangle always bigger than either of its remote interior angles? Explain.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It is the two remote angles added, each more than 0°.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.2 Angle Relationships in Triangles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equations with like terms and the distributive property</t>
+  </si>
+  <si>
     <t xml:space="preserve">not built yet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-B1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thread B: angle pairs — supplementary, complementary, vertical, adjacent (16.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identify complementary, supplementary, vertical, adjacent, and congruent angles — HGV; Find measures of complementary, supplementary, vertical, and adjacent angles — R2B; Write and solve equations using angle relationships — DBV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I can name an angle pair and use it to find a missing angle, with an equation when the angles are expressions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">When two angles are neighbours or opposites, what does one tell you about the other?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adjacent angles, vertical angles, complementary angles, supplementary angles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.GR.1.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MA.8.GR.1.4 — Solve mathematical problems involving the relationships between supplementary, complementary, vertical or adjacent angles.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Can two vertical angles be complementary? Always, sometimes or never? Explain.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sometimes — only when each is 45°.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16.1 Angle Relationships</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-B2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thread B: interior and exterior angles of a triangle (16.2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Find missing angles in triangles — JFJ; Exterior Angle Theorem — FMP; Triangle Angle-Sum Theorem — 6Q6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I can find a missing angle of a triangle, inside or outside, with the Triangle Sum and the Exterior Angle Theorem.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Why do the three angles of every triangle add to the same number?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">interior angle, exterior angle, remote interior angles, Triangle Sum Theorem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.GR.1.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MA.8.GR.1.5 — Solve problems involving the relationships of interior and exterior angles of a triangle.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Why is an exterior angle of a triangle always bigger than either of its remote interior angles? Explain.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">It is the two remote angles added, each more than 0°.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16.2 Angle Relationships in Triangles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equations with like terms and the distributive property</t>
   </si>
   <si>
     <t xml:space="preserve">Solve equations involving like terms — Q2B; Solve equations using the distributive property — QWE; Solve two-step equations: word problems — 8CZ</t>
@@ -6340,7 +6340,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 292d4c00 on 25 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 28e8a92c on 25 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -6484,67 +6484,91 @@
     <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.04%22</t>
   </si>
   <si>
+    <t xml:space="preserve">'Unit tests'!E9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.06%22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Unit tests'!F9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.08%22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Unit tests'!G9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.10%22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Unit tests'!H9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Unit tests'!I9</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!G2</t>
   </si>
   <si>
     <t xml:space="preserve">folder</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.06%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!H2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.08%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.03%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!I2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%205.10%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!J2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.05%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!K2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.06%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!L2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!M2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.03%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!N2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.T1%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!G3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.05%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.T2%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!H3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.06%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!I3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.07%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!J3</t>
@@ -6553,22 +6577,25 @@
     <t xml:space="preserve">'Units'!K3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.T1%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.02%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!L3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%206.T2%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.03%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!M3</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.04%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!N3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.05%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!G4</t>
@@ -6577,382 +6604,385 @@
     <t xml:space="preserve">'Units'!H4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.02%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!I4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.03%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.08%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!J4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.04%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!K4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.05%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!L4</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!M4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!N4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.08%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!G5</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!H5</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!I5</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.02%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!J5</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.04%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!K5</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.05%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!L5</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.07%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!M5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.01%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!N5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.02%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!G6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!H6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.05%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.02%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!I6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%207.07%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!J6</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.05%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!K6</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.06%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!L6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!M6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.02%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.09%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!N6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.04%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.10%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!G7</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.05%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units'!H7</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.06%22</t>
+    <t xml:space="preserve">'Units'!I7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.01%22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Units'!J7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.03%22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Units'!K7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.04%22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Units'!L7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.06%22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Units'!M7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!N7</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.07%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.08%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!C2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.09%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!D2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2010.10%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F2</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.04%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%209.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!H2</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.03%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%209.03%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!C3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.04%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!D3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.06%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.07%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!F3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2012.08%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!G3</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.06%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H3</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.07%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.09%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%208.04%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%209.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.T1%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!F4</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%209.03%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.T2%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!G4</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H4</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.05%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.01%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.07%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!D5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.04%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.06%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G5</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.09%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H5</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!C6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.T1%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!D6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2013.T2%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.01%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.05%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!G6</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2014.07%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.02%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!H6</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.03b%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C7</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.04%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!D7</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.05%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E7</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.06%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F7</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.07%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G7</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.08%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H7</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2016.01%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C8</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2016.03%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units 1–2 decks'!D8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.01%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.02%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2017.01%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!F8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.03b%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2017.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!G8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.04%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H8</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.05%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!C9</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.06%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!D9</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.07%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!E9</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2015.08%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!F9</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2016.01%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!G9</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2016.03%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!H9</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!C10</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2017.01%22</t>
-  </si>
-  <si>
     <t xml:space="preserve">'Units 1–2 decks'!D10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2017.04%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units 1–2 decks'!E10</t>
@@ -7476,11 +7506,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8448,7 +8478,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q163"/>
+  <dimension ref="A1:Q173"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9889,11 +9919,11 @@
         <v>1786</v>
       </c>
       <c r="P27" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q27" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2f48d7f422a9",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k88746a6374d1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test.pdf%22</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9945,18 +9975,18 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M28" s="69" t="s">
-        <v>1788</v>
+        <v>1787</v>
       </c>
       <c r="N28" s="69"/>
       <c r="O28" s="69" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="P28" s="69" t="s">
         <v>1744</v>
       </c>
       <c r="Q28" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8fdeab195866",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb1431270c320",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10008,18 +10038,18 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M29" s="69" t="s">
-        <v>1790</v>
+        <v>1789</v>
       </c>
       <c r="N29" s="69"/>
       <c r="O29" s="69" t="s">
-        <v>1791</v>
+        <v>1790</v>
       </c>
       <c r="P29" s="69" t="s">
         <v>1744</v>
       </c>
       <c r="Q29" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k05aafdefef87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k556b588e59f3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10071,18 +10101,18 @@
         <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
       <c r="M30" s="69" t="s">
-        <v>1792</v>
+        <v>1791</v>
       </c>
       <c r="N30" s="69"/>
       <c r="O30" s="69" t="s">
-        <v>1793</v>
+        <v>1792</v>
       </c>
       <c r="P30" s="69" t="s">
         <v>1744</v>
       </c>
       <c r="Q30" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4e34d1ba5135",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k971f54462233",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10112,14 +10142,14 @@
       <c r="M31" s="69"/>
       <c r="N31" s="69"/>
       <c r="O31" s="69" t="s">
-        <v>1794</v>
+        <v>1793</v>
       </c>
       <c r="P31" s="69" t="s">
         <v>1744</v>
       </c>
       <c r="Q31" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k654621d73a39",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k517d65d34a41",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10149,14 +10179,14 @@
       <c r="M32" s="69"/>
       <c r="N32" s="69"/>
       <c r="O32" s="69" t="s">
+        <v>1794</v>
+      </c>
+      <c r="P32" s="69" t="s">
         <v>1795</v>
       </c>
-      <c r="P32" s="69" t="s">
-        <v>1744</v>
-      </c>
       <c r="Q32" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b09413fba3b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2f48d7f422a9",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10218,8 +10248,8 @@
         <v>1744</v>
       </c>
       <c r="Q33" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb7a4b26081c5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8fdeab195866",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10278,11 +10308,11 @@
         <v>1799</v>
       </c>
       <c r="P34" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q34" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2ed79628bc59",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k05aafdefef87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10341,11 +10371,11 @@
         <v>1801</v>
       </c>
       <c r="P35" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q35" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kf1ee50ed8929",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4e34d1ba5135",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10407,8 +10437,8 @@
         <v>1744</v>
       </c>
       <c r="Q36" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k749da75b36af",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k654621d73a39",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10470,8 +10500,8 @@
         <v>1744</v>
       </c>
       <c r="Q37" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k509a716d7468",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6b09413fba3b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test.pdf%22</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10533,36 +10563,45 @@
         <v>1744</v>
       </c>
       <c r="Q38" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4c613b2b0958",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb7a4b26081c5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20Equations%20and%20Inequalities%20-%20Practice%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="70" t="n">
         <v>46343</v>
       </c>
-      <c r="B39" s="69"/>
+      <c r="B39" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k88746a6374d1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test.pdf%22</v>
+      </c>
       <c r="C39" s="69"/>
       <c r="D39" s="69"/>
       <c r="E39" s="69"/>
       <c r="F39" s="69"/>
-      <c r="G39" s="69"/>
+      <c r="G39" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb1431270c320",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test%20-%20Key.pdf%22</v>
+      </c>
       <c r="H39" s="69"/>
       <c r="I39" s="69"/>
       <c r="J39" s="69"/>
       <c r="K39" s="69"/>
-      <c r="L39" s="69"/>
+      <c r="L39" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k68565bb7197c",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder</v>
+      </c>
       <c r="M39" s="69"/>
       <c r="N39" s="69"/>
       <c r="O39" s="69" t="s">
         <v>1808</v>
       </c>
       <c r="P39" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q39" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd60a700332eb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k2ed79628bc59",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%201%20-%20Equations%20and%20Inequalities%22%20type:folder</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10621,11 +10660,11 @@
         <v>1810</v>
       </c>
       <c r="P40" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q40" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0fe1632a0900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kf1ee50ed8929",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10687,8 +10726,8 @@
         <v>1744</v>
       </c>
       <c r="Q41" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kadb8b2686141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k749da75b36af",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10712,11 +10751,11 @@
         <v>1813</v>
       </c>
       <c r="P42" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q42" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k986a7bd5b0f8",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k509a716d7468",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10742,11 +10781,11 @@
         <v>1815</v>
       </c>
       <c r="P43" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q43" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kb8fed8266c53",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4c613b2b0958",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10773,8 +10812,8 @@
         <v>1744</v>
       </c>
       <c r="Q44" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb737ddcb3701",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd60a700332eb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10803,8 +10842,8 @@
         <v>1744</v>
       </c>
       <c r="Q45" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1f816ed6a0ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0fe1632a0900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test.pdf%22</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10833,8 +10872,8 @@
         <v>1744</v>
       </c>
       <c r="Q46" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb93ffed6ca63",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kadb8b2686141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%20-%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10860,11 +10899,11 @@
         <v>1822</v>
       </c>
       <c r="P47" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q47" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k467ef44c3569",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k986a7bd5b0f8",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%202%20-%20Real%20Numbers%2C%20Square%20Roots%20and%20Cube%20Roots%22%20type:folder</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10890,11 +10929,11 @@
         <v>1824</v>
       </c>
       <c r="P48" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q48" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke52ff0df0d4b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("kb8fed8266c53",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10921,8 +10960,8 @@
         <v>1744</v>
       </c>
       <c r="Q49" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf990f1c33e7d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb737ddcb3701",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10948,11 +10987,11 @@
         <v>1827</v>
       </c>
       <c r="P50" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q50" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k85bc365a5352",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1f816ed6a0ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10978,11 +11017,11 @@
         <v>1829</v>
       </c>
       <c r="P51" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q51" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k19f682b91838",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb93ffed6ca63",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11009,8 +11048,8 @@
         <v>1744</v>
       </c>
       <c r="Q52" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k44624f8b3141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k467ef44c3569",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11037,8 +11076,8 @@
         <v>1744</v>
       </c>
       <c r="Q53" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb2536de7152",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke52ff0df0d4b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test.pdf%22</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11065,8 +11104,8 @@
         <v>1744</v>
       </c>
       <c r="Q54" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke57d72cf0716",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf990f1c33e7d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20Exponents%20and%20Scientific%20Notation%20-%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11090,11 +11129,11 @@
         <v>1833</v>
       </c>
       <c r="P55" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q55" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dd5b368d2b0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k85bc365a5352",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%203%20-%20Exponents%20and%20Scientific%20Notation%22%20type:folder</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11118,11 +11157,11 @@
         <v>1834</v>
       </c>
       <c r="P56" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q56" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1aeb0889327f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20Form%20A.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20Form%20A.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k19f682b91838",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11149,8 +11188,8 @@
         <v>1744</v>
       </c>
       <c r="Q57" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k758e62e8ec43",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20Form%20A%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k44624f8b3141",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11176,11 +11215,11 @@
         <v>1837</v>
       </c>
       <c r="P58" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q58" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k395c44aceb1d",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb2536de7152",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11206,11 +11245,11 @@
         <v>1839</v>
       </c>
       <c r="P59" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q59" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k57de004b2b0a",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ke57d72cf0716",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11239,8 +11278,8 @@
         <v>1744</v>
       </c>
       <c r="Q60" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbcf7b890879b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dd5b368d2b0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11269,8 +11308,8 @@
         <v>1744</v>
       </c>
       <c r="Q61" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k60f05a144797",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1aeb0889327f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20Form%20A.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20Form%20A.pdf%22</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11299,8 +11338,8 @@
         <v>1744</v>
       </c>
       <c r="Q62" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b4473b65910",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k758e62e8ec43",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20Solving%20Problems%20with%20Rational%20Numbers%20-%20Test%20Form%20A%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11324,11 +11363,11 @@
         <v>1846</v>
       </c>
       <c r="P63" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q63" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1c81628b7541",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k395c44aceb1d",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%204%20-%20Solving%20Problems%20with%20Rational%20Numbers%22%20type:folder</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11352,11 +11391,11 @@
         <v>1847</v>
       </c>
       <c r="P64" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q64" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k11cedfe615ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k57de004b2b0a",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11385,8 +11424,8 @@
         <v>1744</v>
       </c>
       <c r="Q65" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k34f09723e09c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbcf7b890879b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11412,11 +11451,11 @@
         <v>1851</v>
       </c>
       <c r="P66" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q66" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k5fd6e0a77786",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k60f05a144797",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11442,11 +11481,11 @@
         <v>1853</v>
       </c>
       <c r="P67" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q67" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k68565bb7197c",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b4473b65910",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11475,8 +11514,8 @@
         <v>1744</v>
       </c>
       <c r="Q68" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k2483cb64a2dc",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1c81628b7541",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11502,11 +11541,11 @@
         <v>1857</v>
       </c>
       <c r="P69" s="69" t="s">
-        <v>1787</v>
+        <v>1744</v>
       </c>
       <c r="Q69" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k9cdbb0b8f97f",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k11cedfe615ec",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A.pdf%22</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11535,8 +11574,8 @@
         <v>1744</v>
       </c>
       <c r="Q70" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf7444edd4950",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k34f09723e09c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20Multi-Step%20Proportional%20Relationships%20-%20Test%20Form%20A%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11562,11 +11601,11 @@
         <v>1861</v>
       </c>
       <c r="P71" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q71" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbb6e44272bb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k5fd6e0a77786",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%205%20-%20Multi-Step%20Proportional%20Relationships%22%20type:folder</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11592,11 +11631,11 @@
         <v>1863</v>
       </c>
       <c r="P72" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q72" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc68dd81311bb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k68565bb7197c",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11623,8 +11662,8 @@
         <v>1744</v>
       </c>
       <c r="Q73" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k70c393f4e972",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k2483cb64a2dc",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11651,8 +11690,8 @@
         <v>1744</v>
       </c>
       <c r="Q74" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1d60e486567d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k517d65d34a41",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Reference%20Sheet.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Reference%20Sheet.pdf%22</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11681,8 +11720,8 @@
         <v>1744</v>
       </c>
       <c r="Q75" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k40dc62cd52a5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k556b588e59f3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Review.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Review.pdf%22</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11711,8 +11750,8 @@
         <v>1744</v>
       </c>
       <c r="Q76" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42d053aa97d9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k971f54462233",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Review%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Review%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11741,8 +11780,8 @@
         <v>1744</v>
       </c>
       <c r="Q77" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3d5b3115f0ff",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k88746a6374d1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test.pdf%22</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11771,8 +11810,8 @@
         <v>1744</v>
       </c>
       <c r="Q78" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b6284c3dfc8",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb1431270c320",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20Relationships%20in%20Triangles%20-%20Practice%20Test%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11798,11 +11837,11 @@
         <v>1875</v>
       </c>
       <c r="P79" s="69" t="s">
-        <v>1744</v>
+        <v>1795</v>
       </c>
       <c r="Q79" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k751991f77144",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/drive/folders/"&amp;VLOOKUP("k5d305f221214",Drive!$A:$B,2,0),"https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%20Unit%206%20-%20Relationships%20in%20Triangles%22%20type:folder</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11831,8 +11870,8 @@
         <v>1744</v>
       </c>
       <c r="Q80" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6386e55cce43",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf7444edd4950",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11859,8 +11898,8 @@
         <v>1744</v>
       </c>
       <c r="Q81" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb55aff075211",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbb6e44272bb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11887,8 +11926,8 @@
         <v>1744</v>
       </c>
       <c r="Q82" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k78f3bd7641b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc68dd81311bb",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11917,8 +11956,8 @@
         <v>1744</v>
       </c>
       <c r="Q83" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab82b01c89fe",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k70c393f4e972",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11947,8 +11986,8 @@
         <v>1744</v>
       </c>
       <c r="Q84" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb5633697c8e5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1d60e486567d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11977,8 +12016,8 @@
         <v>1744</v>
       </c>
       <c r="Q85" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf724d6e842b3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k40dc62cd52a5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.01%20Rewriting%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12007,8 +12046,8 @@
         <v>1744</v>
       </c>
       <c r="Q86" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k36b71975bd76",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42d053aa97d9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12035,8 +12074,8 @@
         <v>1744</v>
       </c>
       <c r="Q87" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd7994f0255be",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3d5b3115f0ff",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12063,8 +12102,8 @@
         <v>1744</v>
       </c>
       <c r="Q88" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k441c122ac61a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b6284c3dfc8",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12093,8 +12132,8 @@
         <v>1744</v>
       </c>
       <c r="Q89" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcad6ba0a7c20",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k751991f77144",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12123,8 +12162,8 @@
         <v>1744</v>
       </c>
       <c r="Q90" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kecd875ec58e7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k6386e55cce43",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12153,8 +12192,8 @@
         <v>1744</v>
       </c>
       <c r="Q91" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k04385d48a56f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb55aff075211",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.02%20Repeating%20Decimals%20to%20Fractions%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12183,8 +12222,8 @@
         <v>1744</v>
       </c>
       <c r="Q92" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kaa89f6499257",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k78f3bd7641b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12213,8 +12252,8 @@
         <v>1744</v>
       </c>
       <c r="Q93" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc0dcbe2e82c2",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab82b01c89fe",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12241,8 +12280,8 @@
         <v>1744</v>
       </c>
       <c r="Q94" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k368f7f8b9908",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb5633697c8e5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12271,8 +12310,8 @@
         <v>1744</v>
       </c>
       <c r="Q95" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k53d619094fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf724d6e842b3",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12301,8 +12340,8 @@
         <v>1744</v>
       </c>
       <c r="Q96" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf511d84233f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k36b71975bd76",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12331,8 +12370,8 @@
         <v>1744</v>
       </c>
       <c r="Q97" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9da92cf1af2b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd7994f0255be",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.03%20Two-Step%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12361,8 +12400,8 @@
         <v>1744</v>
       </c>
       <c r="Q98" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k515087871fe0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k441c122ac61a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12391,8 +12430,8 @@
         <v>1744</v>
       </c>
       <c r="Q99" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb6acc983851",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcad6ba0a7c20",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12419,8 +12458,8 @@
         <v>1744</v>
       </c>
       <c r="Q100" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9cdee450b988",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kecd875ec58e7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12447,8 +12486,8 @@
         <v>1744</v>
       </c>
       <c r="Q101" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kac1e5e18d498",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k04385d48a56f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12475,8 +12514,8 @@
         <v>1744</v>
       </c>
       <c r="Q102" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb5db6608070",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kaa89f6499257",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12503,8 +12542,8 @@
         <v>1744</v>
       </c>
       <c r="Q103" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf2a43f4ef780",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc0dcbe2e82c2",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.04%20Two-Step%20Equations%20in%20Context%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12531,8 +12570,8 @@
         <v>1744</v>
       </c>
       <c r="Q104" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k86b940633ffd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k368f7f8b9908",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12559,8 +12598,8 @@
         <v>1744</v>
       </c>
       <c r="Q105" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf341ebe84b57",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k53d619094fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12587,8 +12626,8 @@
         <v>1744</v>
       </c>
       <c r="Q106" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7383ee3f2ec5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf511d84233f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12615,8 +12654,8 @@
         <v>1744</v>
       </c>
       <c r="Q107" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5cae8f95e8bd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9da92cf1af2b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12645,8 +12684,8 @@
         <v>1744</v>
       </c>
       <c r="Q108" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0ecee6c15886",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k515087871fe0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12675,8 +12714,8 @@
         <v>1744</v>
       </c>
       <c r="Q109" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k874b463422ce",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb6acc983851",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.05%20Solving%20Problems%20with%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12705,8 +12744,8 @@
         <v>1744</v>
       </c>
       <c r="Q110" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k07aa4ed88482",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9cdee450b988",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12735,8 +12774,8 @@
         <v>1744</v>
       </c>
       <c r="Q111" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k444ff4b9a71a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kac1e5e18d498",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12765,8 +12804,8 @@
         <v>1744</v>
       </c>
       <c r="Q112" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42b7580a8cb9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdb5db6608070",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12795,8 +12834,8 @@
         <v>1744</v>
       </c>
       <c r="Q113" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8e5410dc08f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf2a43f4ef780",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12825,8 +12864,8 @@
         <v>1744</v>
       </c>
       <c r="Q114" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb0df0c43cf87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k86b940633ffd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12855,8 +12894,8 @@
         <v>1744</v>
       </c>
       <c r="Q115" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kde315e91893f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf341ebe84b57",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.06%20Writing%20Equations%20from%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12885,8 +12924,8 @@
         <v>1744</v>
       </c>
       <c r="Q116" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf9cc95eccf07",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7383ee3f2ec5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12915,8 +12954,8 @@
         <v>1744</v>
       </c>
       <c r="Q117" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd674be572fbd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5cae8f95e8bd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12943,8 +12982,8 @@
         <v>1744</v>
       </c>
       <c r="Q118" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4f3c12075c6f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0ecee6c15886",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12973,8 +13012,8 @@
         <v>1744</v>
       </c>
       <c r="Q119" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k856d2d13cd04",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k874b463422ce",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13003,8 +13042,8 @@
         <v>1744</v>
       </c>
       <c r="Q120" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k160e960d09c4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k07aa4ed88482",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13031,8 +13070,8 @@
         <v>1744</v>
       </c>
       <c r="Q121" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd3a48013b455",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k444ff4b9a71a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.07%20Writing%20and%20Solving%20Equations%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13059,8 +13098,8 @@
         <v>1744</v>
       </c>
       <c r="Q122" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f26b556436e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k42b7580a8cb9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13087,8 +13126,8 @@
         <v>1744</v>
       </c>
       <c r="Q123" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3a6534dc5a62",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8e5410dc08f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13115,8 +13154,8 @@
         <v>1744</v>
       </c>
       <c r="Q124" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ka5734698aa50",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kb0df0c43cf87",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13143,8 +13182,8 @@
         <v>1744</v>
       </c>
       <c r="Q125" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3bd1b440e87a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kde315e91893f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13171,8 +13210,8 @@
         <v>1744</v>
       </c>
       <c r="Q126" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k52493b74eb28",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf9cc95eccf07",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13199,8 +13238,8 @@
         <v>1744</v>
       </c>
       <c r="Q127" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3fa800b9318b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd674be572fbd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.08%20Determining%20Solutions%20to%20Inequalities%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13227,8 +13266,8 @@
         <v>1744</v>
       </c>
       <c r="Q128" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b2764e691f7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4f3c12075c6f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13255,8 +13294,8 @@
         <v>1744</v>
       </c>
       <c r="Q129" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9afa96310f5f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k856d2d13cd04",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13283,8 +13322,8 @@
         <v>1744</v>
       </c>
       <c r="Q130" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3eb4a6e4e0a9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k160e960d09c4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13311,8 +13350,8 @@
         <v>1744</v>
       </c>
       <c r="Q131" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3786dea98f2a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kd3a48013b455",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13339,8 +13378,8 @@
         <v>1744</v>
       </c>
       <c r="Q132" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8424cc4e78b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f26b556436e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13365,8 +13404,8 @@
         <v>1744</v>
       </c>
       <c r="Q133" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf325ac36b969",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3a6534dc5a62",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.09%20Inequalities%20with%20the%20Distributive%20Property%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13391,8 +13430,8 @@
         <v>1744</v>
       </c>
       <c r="Q134" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4ec5ffc67bf1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("ka5734698aa50",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13417,8 +13456,8 @@
         <v>1744</v>
       </c>
       <c r="Q135" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k006e6e337926",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3bd1b440e87a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13443,8 +13482,8 @@
         <v>1744</v>
       </c>
       <c r="Q136" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k94da89c1d16d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k52493b74eb28",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13469,8 +13508,8 @@
         <v>1744</v>
       </c>
       <c r="Q137" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9b79f94a3042",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3fa800b9318b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13495,8 +13534,8 @@
         <v>1744</v>
       </c>
       <c r="Q138" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b57aec5f42c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k5b2764e691f7",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13521,8 +13560,8 @@
         <v>1744</v>
       </c>
       <c r="Q139" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k524993898ff0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9afa96310f5f",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%201.10%20Inequalities%20in%20Real-World%20Contexts%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13547,8 +13586,8 @@
         <v>1744</v>
       </c>
       <c r="Q140" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k71038ca67fed",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3eb4a6e4e0a9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13573,8 +13612,8 @@
         <v>1744</v>
       </c>
       <c r="Q141" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab565ddcecfd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3786dea98f2a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13599,8 +13638,8 @@
         <v>1744</v>
       </c>
       <c r="Q142" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kda9320d99fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k8424cc4e78b1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13625,8 +13664,8 @@
         <v>1744</v>
       </c>
       <c r="Q143" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k577a4eca3248",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kf325ac36b969",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13651,8 +13690,8 @@
         <v>1744</v>
       </c>
       <c r="Q144" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dbd9d8294a0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4ec5ffc67bf1",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13677,8 +13716,8 @@
         <v>1744</v>
       </c>
       <c r="Q145" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k858285f0484a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k006e6e337926",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.01%20Square%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13703,8 +13742,8 @@
         <v>1744</v>
       </c>
       <c r="Q146" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3386b404a0cc",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k94da89c1d16d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13729,8 +13768,8 @@
         <v>1744</v>
       </c>
       <c r="Q147" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1fdcada6b7d5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k9b79f94a3042",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13755,8 +13794,8 @@
         <v>1744</v>
       </c>
       <c r="Q148" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k66ad104dc3f4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k4b57aec5f42c",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13781,8 +13820,8 @@
         <v>1744</v>
       </c>
       <c r="Q149" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f9d2ee2e87b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k524993898ff0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13807,8 +13846,8 @@
         <v>1744</v>
       </c>
       <c r="Q150" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k2e021d1404f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k71038ca67fed",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13833,8 +13872,8 @@
         <v>1744</v>
       </c>
       <c r="Q151" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7f727f839de9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kab565ddcecfd",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.02%20Square%20Values%20and%20Square%20Roots%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13859,8 +13898,8 @@
         <v>1744</v>
       </c>
       <c r="Q152" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc9f54d815229",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kda9320d99fb4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13885,8 +13924,8 @@
         <v>1744</v>
       </c>
       <c r="Q153" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k814de685731b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k577a4eca3248",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13911,8 +13950,8 @@
         <v>1744</v>
       </c>
       <c r="Q154" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbeebbf583a30",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0dbd9d8294a0",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13937,8 +13976,8 @@
         <v>1744</v>
       </c>
       <c r="Q155" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kae76dda4b45d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k858285f0484a",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13963,8 +14002,8 @@
         <v>1744</v>
       </c>
       <c r="Q156" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1228a3dffde6",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k3386b404a0cc",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13989,8 +14028,8 @@
         <v>1744</v>
       </c>
       <c r="Q157" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k47f0af99bd1e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1fdcada6b7d5",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.03%20Cube%20Values%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14015,8 +14054,8 @@
         <v>1744</v>
       </c>
       <c r="Q158" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcee0b8f57c67",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k66ad104dc3f4",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Slides.pdf%22</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14041,8 +14080,8 @@
         <v>1744</v>
       </c>
       <c r="Q159" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k59fb8b4ed900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k0f9d2ee2e87b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14067,8 +14106,8 @@
         <v>1744</v>
       </c>
       <c r="Q160" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1a00a0a22804",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k2e021d1404f9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14093,8 +14132,8 @@
         <v>1744</v>
       </c>
       <c r="Q161" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k29d47d551984",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k7f727f839de9",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14119,8 +14158,8 @@
         <v>1744</v>
       </c>
       <c r="Q162" s="69" t="str">
-        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdc81e4a42f98",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
-        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc9f54d815229",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14145,6 +14184,266 @@
         <v>1744</v>
       </c>
       <c r="Q163" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k814de685731b",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.04%20Approximating%20Irrational%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="69"/>
+      <c r="B164" s="69"/>
+      <c r="C164" s="69"/>
+      <c r="D164" s="69"/>
+      <c r="E164" s="69"/>
+      <c r="F164" s="69"/>
+      <c r="G164" s="69"/>
+      <c r="H164" s="69"/>
+      <c r="I164" s="69"/>
+      <c r="J164" s="69"/>
+      <c r="K164" s="69"/>
+      <c r="L164" s="69"/>
+      <c r="M164" s="69"/>
+      <c r="N164" s="69"/>
+      <c r="O164" s="69" t="s">
+        <v>1987</v>
+      </c>
+      <c r="P164" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q164" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kbeebbf583a30",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Slides.pdf%22</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="69"/>
+      <c r="B165" s="69"/>
+      <c r="C165" s="69"/>
+      <c r="D165" s="69"/>
+      <c r="E165" s="69"/>
+      <c r="F165" s="69"/>
+      <c r="G165" s="69"/>
+      <c r="H165" s="69"/>
+      <c r="I165" s="69"/>
+      <c r="J165" s="69"/>
+      <c r="K165" s="69"/>
+      <c r="L165" s="69"/>
+      <c r="M165" s="69"/>
+      <c r="N165" s="69"/>
+      <c r="O165" s="69" t="s">
+        <v>1988</v>
+      </c>
+      <c r="P165" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q165" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kae76dda4b45d",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Teacher%20Edition.pdf%22</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="69"/>
+      <c r="B166" s="69"/>
+      <c r="C166" s="69"/>
+      <c r="D166" s="69"/>
+      <c r="E166" s="69"/>
+      <c r="F166" s="69"/>
+      <c r="G166" s="69"/>
+      <c r="H166" s="69"/>
+      <c r="I166" s="69"/>
+      <c r="J166" s="69"/>
+      <c r="K166" s="69"/>
+      <c r="L166" s="69"/>
+      <c r="M166" s="69"/>
+      <c r="N166" s="69"/>
+      <c r="O166" s="69" t="s">
+        <v>1989</v>
+      </c>
+      <c r="P166" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q166" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1228a3dffde6",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank.pdf%22</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="69"/>
+      <c r="B167" s="69"/>
+      <c r="C167" s="69"/>
+      <c r="D167" s="69"/>
+      <c r="E167" s="69"/>
+      <c r="F167" s="69"/>
+      <c r="G167" s="69"/>
+      <c r="H167" s="69"/>
+      <c r="I167" s="69"/>
+      <c r="J167" s="69"/>
+      <c r="K167" s="69"/>
+      <c r="L167" s="69"/>
+      <c r="M167" s="69"/>
+      <c r="N167" s="69"/>
+      <c r="O167" s="69" t="s">
+        <v>1990</v>
+      </c>
+      <c r="P167" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q167" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k47f0af99bd1e",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank.pdf%22</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="69"/>
+      <c r="B168" s="69"/>
+      <c r="C168" s="69"/>
+      <c r="D168" s="69"/>
+      <c r="E168" s="69"/>
+      <c r="F168" s="69"/>
+      <c r="G168" s="69"/>
+      <c r="H168" s="69"/>
+      <c r="I168" s="69"/>
+      <c r="J168" s="69"/>
+      <c r="K168" s="69"/>
+      <c r="L168" s="69"/>
+      <c r="M168" s="69"/>
+      <c r="N168" s="69"/>
+      <c r="O168" s="69" t="s">
+        <v>1991</v>
+      </c>
+      <c r="P168" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q168" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kcee0b8f57c67",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Question%20Bank%20-%20Key.pdf%22</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="69"/>
+      <c r="B169" s="69"/>
+      <c r="C169" s="69"/>
+      <c r="D169" s="69"/>
+      <c r="E169" s="69"/>
+      <c r="F169" s="69"/>
+      <c r="G169" s="69"/>
+      <c r="H169" s="69"/>
+      <c r="I169" s="69"/>
+      <c r="J169" s="69"/>
+      <c r="K169" s="69"/>
+      <c r="L169" s="69"/>
+      <c r="M169" s="69"/>
+      <c r="N169" s="69"/>
+      <c r="O169" s="69" t="s">
+        <v>1992</v>
+      </c>
+      <c r="P169" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q169" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k59fb8b4ed900",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.05%20Rational%20and%20Irrational%20Numbers%20on%20the%20Number%20Line%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="69"/>
+      <c r="B170" s="69"/>
+      <c r="C170" s="69"/>
+      <c r="D170" s="69"/>
+      <c r="E170" s="69"/>
+      <c r="F170" s="69"/>
+      <c r="G170" s="69"/>
+      <c r="H170" s="69"/>
+      <c r="I170" s="69"/>
+      <c r="J170" s="69"/>
+      <c r="K170" s="69"/>
+      <c r="L170" s="69"/>
+      <c r="M170" s="69"/>
+      <c r="N170" s="69"/>
+      <c r="O170" s="69" t="s">
+        <v>1993</v>
+      </c>
+      <c r="P170" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q170" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k1a00a0a22804",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Slides.pdf%22</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="69"/>
+      <c r="B171" s="69"/>
+      <c r="C171" s="69"/>
+      <c r="D171" s="69"/>
+      <c r="E171" s="69"/>
+      <c r="F171" s="69"/>
+      <c r="G171" s="69"/>
+      <c r="H171" s="69"/>
+      <c r="I171" s="69"/>
+      <c r="J171" s="69"/>
+      <c r="K171" s="69"/>
+      <c r="L171" s="69"/>
+      <c r="M171" s="69"/>
+      <c r="N171" s="69"/>
+      <c r="O171" s="69" t="s">
+        <v>1994</v>
+      </c>
+      <c r="P171" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q171" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("k29d47d551984",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Teacher%20Edition.pdf%22</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="69"/>
+      <c r="B172" s="69"/>
+      <c r="C172" s="69"/>
+      <c r="D172" s="69"/>
+      <c r="E172" s="69"/>
+      <c r="F172" s="69"/>
+      <c r="G172" s="69"/>
+      <c r="H172" s="69"/>
+      <c r="I172" s="69"/>
+      <c r="J172" s="69"/>
+      <c r="K172" s="69"/>
+      <c r="L172" s="69"/>
+      <c r="M172" s="69"/>
+      <c r="N172" s="69"/>
+      <c r="O172" s="69" t="s">
+        <v>1995</v>
+      </c>
+      <c r="P172" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q172" s="69" t="str">
+        <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kdc81e4a42f98",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22")</f>
+        <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank.pdf%22</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="69"/>
+      <c r="B173" s="69"/>
+      <c r="C173" s="69"/>
+      <c r="D173" s="69"/>
+      <c r="E173" s="69"/>
+      <c r="F173" s="69"/>
+      <c r="G173" s="69"/>
+      <c r="H173" s="69"/>
+      <c r="I173" s="69"/>
+      <c r="J173" s="69"/>
+      <c r="K173" s="69"/>
+      <c r="L173" s="69"/>
+      <c r="M173" s="69"/>
+      <c r="N173" s="69"/>
+      <c r="O173" s="69" t="s">
+        <v>1996</v>
+      </c>
+      <c r="P173" s="69" t="s">
+        <v>1744</v>
+      </c>
+      <c r="Q173" s="69" t="str">
         <f aca="false">IFERROR("https://drive.google.com/file/d/"&amp;VLOOKUP("kc34b261fea84",Drive!$A:$B,2,0)&amp;"/view","https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22")</f>
         <v>https://drive.google.com/drive/search?q=title:%22A7%202.06%20Plotting%2C%20Ordering%20and%20Comparing%20Real%20Numbers%20-%20Additional%20Question%20Bank%20-%20Key.pdf%22</v>
       </c>
@@ -14175,16 +14474,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="71" t="s">
-        <v>1987</v>
+        <v>1997</v>
       </c>
       <c r="B1" s="71" t="s">
-        <v>1988</v>
+        <v>1998</v>
       </c>
       <c r="C1" s="71" t="s">
-        <v>1989</v>
+        <v>1999</v>
       </c>
       <c r="D1" s="71" t="s">
-        <v>1990</v>
+        <v>2000</v>
       </c>
     </row>
   </sheetData>
@@ -17429,19 +17728,26 @@
       <c r="E39" s="33" t="s">
         <v>345</v>
       </c>
-      <c r="F39" s="43" t="s">
-        <v>346</v>
+      <c r="F39" s="34" t="str">
+        <f aca="false">HYPERLINK(Links!$B$39,"Unit Assessment")</f>
+        <v>Unit Assessment</v>
       </c>
       <c r="G39" s="30"/>
       <c r="H39" s="30"/>
       <c r="I39" s="30"/>
       <c r="J39" s="30"/>
-      <c r="K39" s="30"/>
+      <c r="K39" s="34" t="str">
+        <f aca="false">HYPERLINK(Links!$G$39,"Assessment key")</f>
+        <v>Assessment key</v>
+      </c>
       <c r="L39" s="30"/>
       <c r="M39" s="30"/>
       <c r="N39" s="30"/>
       <c r="O39" s="30"/>
-      <c r="P39" s="30"/>
+      <c r="P39" s="34" t="str">
+        <f aca="false">HYPERLINK(Links!$L$39,"folder")</f>
+        <v>folder</v>
+      </c>
       <c r="Q39" s="30"/>
       <c r="R39" s="33"/>
       <c r="S39" s="35"/>
@@ -17466,10 +17772,10 @@
         <v>6</v>
       </c>
       <c r="D40" s="39" t="s">
+        <v>346</v>
+      </c>
+      <c r="E40" s="40" t="s">
         <v>347</v>
-      </c>
-      <c r="E40" s="40" t="s">
-        <v>348</v>
       </c>
       <c r="F40" s="41" t="str">
         <f aca="false">HYPERLINK(Links!$B$40,"open")</f>
@@ -17520,37 +17826,37 @@
         <v>search</v>
       </c>
       <c r="R40" s="40" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="S40" s="42" t="n">
         <v>46345</v>
       </c>
       <c r="T40" s="40" t="s">
+        <v>349</v>
+      </c>
+      <c r="U40" s="40" t="s">
         <v>350</v>
       </c>
-      <c r="U40" s="40" t="s">
+      <c r="V40" s="40" t="s">
         <v>351</v>
       </c>
-      <c r="V40" s="40" t="s">
+      <c r="W40" s="40" t="s">
         <v>352</v>
       </c>
-      <c r="W40" s="40" t="s">
+      <c r="X40" s="40" t="s">
         <v>353</v>
-      </c>
-      <c r="X40" s="40" t="s">
-        <v>354</v>
       </c>
       <c r="Y40" s="40" t="s">
         <v>219</v>
       </c>
       <c r="Z40" s="40" t="s">
+        <v>354</v>
+      </c>
+      <c r="AA40" s="40" t="s">
         <v>355</v>
       </c>
-      <c r="AA40" s="40" t="s">
+      <c r="AB40" s="40" t="s">
         <v>356</v>
-      </c>
-      <c r="AB40" s="40" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17564,10 +17870,10 @@
         <v>6</v>
       </c>
       <c r="D41" s="39" t="s">
+        <v>357</v>
+      </c>
+      <c r="E41" s="40" t="s">
         <v>358</v>
-      </c>
-      <c r="E41" s="40" t="s">
-        <v>359</v>
       </c>
       <c r="F41" s="41" t="str">
         <f aca="false">HYPERLINK(Links!$B$41,"open")</f>
@@ -17618,37 +17924,37 @@
         <v>search</v>
       </c>
       <c r="R41" s="40" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="S41" s="42" t="n">
         <v>46346</v>
       </c>
       <c r="T41" s="40" t="s">
+        <v>360</v>
+      </c>
+      <c r="U41" s="40" t="s">
         <v>361</v>
       </c>
-      <c r="U41" s="40" t="s">
+      <c r="V41" s="40" t="s">
         <v>362</v>
       </c>
-      <c r="V41" s="40" t="s">
+      <c r="W41" s="40" t="s">
         <v>363</v>
       </c>
-      <c r="W41" s="40" t="s">
+      <c r="X41" s="40" t="s">
         <v>364</v>
-      </c>
-      <c r="X41" s="40" t="s">
-        <v>365</v>
       </c>
       <c r="Y41" s="40" t="s">
         <v>219</v>
       </c>
       <c r="Z41" s="40" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA41" s="40" t="s">
         <v>366</v>
       </c>
-      <c r="AA41" s="40" t="s">
+      <c r="AB41" s="40" t="s">
         <v>367</v>
-      </c>
-      <c r="AB41" s="40" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17702,13 +18008,13 @@
         <v>11</v>
       </c>
       <c r="D43" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="E43" s="19" t="s">
         <v>369</v>
       </c>
-      <c r="E43" s="19" t="s">
+      <c r="F43" s="43" t="s">
         <v>370</v>
-      </c>
-      <c r="F43" s="44" t="s">
-        <v>346</v>
       </c>
       <c r="G43" s="16"/>
       <c r="H43" s="16"/>
@@ -17802,8 +18108,8 @@
       <c r="E45" s="19" t="s">
         <v>377</v>
       </c>
-      <c r="F45" s="44" t="s">
-        <v>346</v>
+      <c r="F45" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -17857,8 +18163,8 @@
       <c r="E46" s="19" t="s">
         <v>381</v>
       </c>
-      <c r="F46" s="44" t="s">
-        <v>346</v>
+      <c r="F46" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G46" s="16"/>
       <c r="H46" s="16"/>
@@ -17912,8 +18218,8 @@
       <c r="E47" s="19" t="s">
         <v>385</v>
       </c>
-      <c r="F47" s="44" t="s">
-        <v>346</v>
+      <c r="F47" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G47" s="16"/>
       <c r="H47" s="16"/>
@@ -17967,8 +18273,8 @@
       <c r="E48" s="19" t="s">
         <v>389</v>
       </c>
-      <c r="F48" s="44" t="s">
-        <v>346</v>
+      <c r="F48" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G48" s="16"/>
       <c r="H48" s="16"/>
@@ -18062,8 +18368,8 @@
       <c r="E50" s="19" t="s">
         <v>396</v>
       </c>
-      <c r="F50" s="44" t="s">
-        <v>346</v>
+      <c r="F50" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G50" s="16"/>
       <c r="H50" s="16"/>
@@ -18117,8 +18423,8 @@
       <c r="E51" s="19" t="s">
         <v>402</v>
       </c>
-      <c r="F51" s="44" t="s">
-        <v>346</v>
+      <c r="F51" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G51" s="16"/>
       <c r="H51" s="16"/>
@@ -18172,8 +18478,8 @@
       <c r="E52" s="33" t="s">
         <v>406</v>
       </c>
-      <c r="F52" s="43" t="s">
-        <v>346</v>
+      <c r="F52" s="44" t="s">
+        <v>370</v>
       </c>
       <c r="G52" s="30"/>
       <c r="H52" s="30"/>
@@ -18420,8 +18726,8 @@
       <c r="E58" s="19" t="s">
         <v>421</v>
       </c>
-      <c r="F58" s="44" t="s">
-        <v>346</v>
+      <c r="F58" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G58" s="16"/>
       <c r="H58" s="16"/>
@@ -18475,8 +18781,8 @@
       <c r="E59" s="19" t="s">
         <v>427</v>
       </c>
-      <c r="F59" s="44" t="s">
-        <v>346</v>
+      <c r="F59" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G59" s="16"/>
       <c r="H59" s="16"/>
@@ -18530,8 +18836,8 @@
       <c r="E60" s="19" t="s">
         <v>433</v>
       </c>
-      <c r="F60" s="44" t="s">
-        <v>346</v>
+      <c r="F60" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G60" s="16"/>
       <c r="H60" s="16"/>
@@ -18585,8 +18891,8 @@
       <c r="E61" s="19" t="s">
         <v>439</v>
       </c>
-      <c r="F61" s="44" t="s">
-        <v>346</v>
+      <c r="F61" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G61" s="16"/>
       <c r="H61" s="16"/>
@@ -18640,8 +18946,8 @@
       <c r="E62" s="19" t="s">
         <v>445</v>
       </c>
-      <c r="F62" s="44" t="s">
-        <v>346</v>
+      <c r="F62" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G62" s="16"/>
       <c r="H62" s="16"/>
@@ -18735,8 +19041,8 @@
       <c r="E64" s="33" t="s">
         <v>451</v>
       </c>
-      <c r="F64" s="43" t="s">
-        <v>346</v>
+      <c r="F64" s="44" t="s">
+        <v>370</v>
       </c>
       <c r="G64" s="30"/>
       <c r="H64" s="30"/>
@@ -18778,7 +19084,7 @@
         <v>453</v>
       </c>
       <c r="F65" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G65" s="37"/>
       <c r="H65" s="37"/>
@@ -18833,7 +19139,7 @@
         <v>459</v>
       </c>
       <c r="F66" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G66" s="37"/>
       <c r="H66" s="37"/>
@@ -18888,7 +19194,7 @@
         <v>465</v>
       </c>
       <c r="F67" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G67" s="37"/>
       <c r="H67" s="37"/>
@@ -18943,7 +19249,7 @@
         <v>471</v>
       </c>
       <c r="F68" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G68" s="37"/>
       <c r="H68" s="37"/>
@@ -18998,7 +19304,7 @@
         <v>477</v>
       </c>
       <c r="F69" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G69" s="37"/>
       <c r="H69" s="37"/>
@@ -19053,7 +19359,7 @@
         <v>481</v>
       </c>
       <c r="F70" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G70" s="37"/>
       <c r="H70" s="37"/>
@@ -19108,7 +19414,7 @@
         <v>487</v>
       </c>
       <c r="F71" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G71" s="37"/>
       <c r="H71" s="37"/>
@@ -19163,7 +19469,7 @@
         <v>493</v>
       </c>
       <c r="F72" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G72" s="37"/>
       <c r="H72" s="37"/>
@@ -19217,8 +19523,8 @@
       <c r="E73" s="33" t="s">
         <v>499</v>
       </c>
-      <c r="F73" s="43" t="s">
-        <v>346</v>
+      <c r="F73" s="44" t="s">
+        <v>370</v>
       </c>
       <c r="G73" s="30"/>
       <c r="H73" s="30"/>
@@ -19300,7 +19606,7 @@
         <v>503</v>
       </c>
       <c r="F75" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G75" s="37"/>
       <c r="H75" s="37"/>
@@ -19355,7 +19661,7 @@
         <v>509</v>
       </c>
       <c r="F76" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G76" s="37"/>
       <c r="H76" s="37"/>
@@ -19410,7 +19716,7 @@
         <v>513</v>
       </c>
       <c r="F77" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G77" s="37"/>
       <c r="H77" s="37"/>
@@ -19465,7 +19771,7 @@
         <v>519</v>
       </c>
       <c r="F78" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G78" s="37"/>
       <c r="H78" s="37"/>
@@ -19520,7 +19826,7 @@
         <v>522</v>
       </c>
       <c r="F79" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G79" s="37"/>
       <c r="H79" s="37"/>
@@ -19575,7 +19881,7 @@
         <v>528</v>
       </c>
       <c r="F80" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G80" s="37"/>
       <c r="H80" s="37"/>
@@ -19629,8 +19935,8 @@
       <c r="E81" s="33" t="s">
         <v>534</v>
       </c>
-      <c r="F81" s="43" t="s">
-        <v>346</v>
+      <c r="F81" s="44" t="s">
+        <v>370</v>
       </c>
       <c r="G81" s="30"/>
       <c r="H81" s="30"/>
@@ -19712,7 +20018,7 @@
         <v>536</v>
       </c>
       <c r="F83" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G83" s="37"/>
       <c r="H83" s="37"/>
@@ -19767,7 +20073,7 @@
         <v>542</v>
       </c>
       <c r="F84" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G84" s="37"/>
       <c r="H84" s="37"/>
@@ -19821,8 +20127,8 @@
       <c r="E85" s="19" t="s">
         <v>548</v>
       </c>
-      <c r="F85" s="44" t="s">
-        <v>346</v>
+      <c r="F85" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G85" s="16"/>
       <c r="H85" s="16"/>
@@ -19876,8 +20182,8 @@
       <c r="E86" s="19" t="s">
         <v>554</v>
       </c>
-      <c r="F86" s="44" t="s">
-        <v>346</v>
+      <c r="F86" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G86" s="16"/>
       <c r="H86" s="16"/>
@@ -19931,8 +20237,8 @@
       <c r="E87" s="33" t="s">
         <v>560</v>
       </c>
-      <c r="F87" s="43" t="s">
-        <v>346</v>
+      <c r="F87" s="44" t="s">
+        <v>370</v>
       </c>
       <c r="G87" s="30"/>
       <c r="H87" s="30"/>
@@ -20013,8 +20319,8 @@
       <c r="E89" s="19" t="s">
         <v>562</v>
       </c>
-      <c r="F89" s="44" t="s">
-        <v>346</v>
+      <c r="F89" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G89" s="16"/>
       <c r="H89" s="16"/>
@@ -20068,8 +20374,8 @@
       <c r="E90" s="19" t="s">
         <v>568</v>
       </c>
-      <c r="F90" s="44" t="s">
-        <v>346</v>
+      <c r="F90" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G90" s="16"/>
       <c r="H90" s="16"/>
@@ -20123,8 +20429,8 @@
       <c r="E91" s="19" t="s">
         <v>574</v>
       </c>
-      <c r="F91" s="44" t="s">
-        <v>346</v>
+      <c r="F91" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G91" s="16"/>
       <c r="H91" s="16"/>
@@ -20178,8 +20484,8 @@
       <c r="E92" s="19" t="s">
         <v>580</v>
       </c>
-      <c r="F92" s="44" t="s">
-        <v>346</v>
+      <c r="F92" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G92" s="16"/>
       <c r="H92" s="16"/>
@@ -20233,8 +20539,8 @@
       <c r="E93" s="19" t="s">
         <v>586</v>
       </c>
-      <c r="F93" s="44" t="s">
-        <v>346</v>
+      <c r="F93" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G93" s="16"/>
       <c r="H93" s="16"/>
@@ -20288,8 +20594,8 @@
       <c r="E94" s="33" t="s">
         <v>592</v>
       </c>
-      <c r="F94" s="43" t="s">
-        <v>346</v>
+      <c r="F94" s="44" t="s">
+        <v>370</v>
       </c>
       <c r="G94" s="30"/>
       <c r="H94" s="30"/>
@@ -20330,8 +20636,8 @@
       <c r="E95" s="19" t="s">
         <v>594</v>
       </c>
-      <c r="F95" s="44" t="s">
-        <v>346</v>
+      <c r="F95" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G95" s="16"/>
       <c r="H95" s="16"/>
@@ -20385,8 +20691,8 @@
       <c r="E96" s="19" t="s">
         <v>600</v>
       </c>
-      <c r="F96" s="44" t="s">
-        <v>346</v>
+      <c r="F96" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G96" s="16"/>
       <c r="H96" s="16"/>
@@ -20441,7 +20747,7 @@
         <v>606</v>
       </c>
       <c r="F97" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G97" s="37"/>
       <c r="H97" s="37"/>
@@ -20496,7 +20802,7 @@
         <v>610</v>
       </c>
       <c r="F98" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G98" s="37"/>
       <c r="H98" s="37"/>
@@ -20551,7 +20857,7 @@
         <v>616</v>
       </c>
       <c r="F99" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G99" s="37"/>
       <c r="H99" s="37"/>
@@ -20645,8 +20951,8 @@
       <c r="E101" s="33" t="s">
         <v>622</v>
       </c>
-      <c r="F101" s="43" t="s">
-        <v>346</v>
+      <c r="F101" s="44" t="s">
+        <v>370</v>
       </c>
       <c r="G101" s="30"/>
       <c r="H101" s="30"/>
@@ -20927,8 +21233,8 @@
       <c r="E108" s="19" t="s">
         <v>624</v>
       </c>
-      <c r="F108" s="44" t="s">
-        <v>346</v>
+      <c r="F108" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G108" s="16"/>
       <c r="H108" s="16"/>
@@ -20982,8 +21288,8 @@
       <c r="E109" s="19" t="s">
         <v>630</v>
       </c>
-      <c r="F109" s="44" t="s">
-        <v>346</v>
+      <c r="F109" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G109" s="16"/>
       <c r="H109" s="16"/>
@@ -21037,8 +21343,8 @@
       <c r="E110" s="19" t="s">
         <v>634</v>
       </c>
-      <c r="F110" s="44" t="s">
-        <v>346</v>
+      <c r="F110" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G110" s="16"/>
       <c r="H110" s="16"/>
@@ -21092,8 +21398,8 @@
       <c r="E111" s="19" t="s">
         <v>640</v>
       </c>
-      <c r="F111" s="44" t="s">
-        <v>346</v>
+      <c r="F111" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G111" s="16"/>
       <c r="H111" s="16"/>
@@ -21147,8 +21453,8 @@
       <c r="E112" s="19" t="s">
         <v>644</v>
       </c>
-      <c r="F112" s="44" t="s">
-        <v>346</v>
+      <c r="F112" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G112" s="16"/>
       <c r="H112" s="16"/>
@@ -21202,8 +21508,8 @@
       <c r="E113" s="19" t="s">
         <v>648</v>
       </c>
-      <c r="F113" s="44" t="s">
-        <v>346</v>
+      <c r="F113" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G113" s="16"/>
       <c r="H113" s="16"/>
@@ -21257,8 +21563,8 @@
       <c r="E114" s="19" t="s">
         <v>654</v>
       </c>
-      <c r="F114" s="44" t="s">
-        <v>346</v>
+      <c r="F114" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G114" s="16"/>
       <c r="H114" s="16"/>
@@ -21312,8 +21618,8 @@
       <c r="E115" s="19" t="s">
         <v>660</v>
       </c>
-      <c r="F115" s="44" t="s">
-        <v>346</v>
+      <c r="F115" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G115" s="16"/>
       <c r="H115" s="16"/>
@@ -21368,7 +21674,7 @@
         <v>664</v>
       </c>
       <c r="F116" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G116" s="37"/>
       <c r="H116" s="37"/>
@@ -21423,7 +21729,7 @@
         <v>670</v>
       </c>
       <c r="F117" s="45" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G117" s="37"/>
       <c r="H117" s="37"/>
@@ -21477,8 +21783,8 @@
       <c r="E118" s="33" t="s">
         <v>676</v>
       </c>
-      <c r="F118" s="43" t="s">
-        <v>346</v>
+      <c r="F118" s="44" t="s">
+        <v>370</v>
       </c>
       <c r="G118" s="30"/>
       <c r="H118" s="30"/>
@@ -21519,8 +21825,8 @@
       <c r="E119" s="19" t="s">
         <v>678</v>
       </c>
-      <c r="F119" s="44" t="s">
-        <v>346</v>
+      <c r="F119" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G119" s="16"/>
       <c r="H119" s="16"/>
@@ -21574,8 +21880,8 @@
       <c r="E120" s="19" t="s">
         <v>684</v>
       </c>
-      <c r="F120" s="44" t="s">
-        <v>346</v>
+      <c r="F120" s="43" t="s">
+        <v>370</v>
       </c>
       <c r="G120" s="16"/>
       <c r="H120" s="16"/>
@@ -21629,8 +21935,8 @@
       <c r="E121" s="33" t="s">
         <v>690</v>
       </c>
-      <c r="F121" s="43" t="s">
-        <v>346</v>
+      <c r="F121" s="44" t="s">
+        <v>370</v>
       </c>
       <c r="G121" s="30"/>
       <c r="H121" s="30"/>
@@ -26904,11 +27210,26 @@
         <f aca="false">C107</f>
         <v>18</v>
       </c>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
-      <c r="G9" s="52"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="52"/>
+      <c r="E9" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$27,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="F9" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$28,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="G9" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$29,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="H9" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$30,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="I9" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$31,"open")</f>
+        <v>open</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
@@ -26920,7 +27241,7 @@
       <c r="C10" s="7"/>
       <c r="D10" s="46"/>
       <c r="E10" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F10" s="52"/>
       <c r="G10" s="52"/>
@@ -26937,7 +27258,7 @@
       <c r="C11" s="7"/>
       <c r="D11" s="46"/>
       <c r="E11" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F11" s="52"/>
       <c r="G11" s="52"/>
@@ -26954,7 +27275,7 @@
       <c r="C12" s="7"/>
       <c r="D12" s="46"/>
       <c r="E12" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F12" s="52"/>
       <c r="G12" s="52"/>
@@ -26971,7 +27292,7 @@
       <c r="C13" s="7"/>
       <c r="D13" s="46"/>
       <c r="E13" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F13" s="52"/>
       <c r="G13" s="52"/>
@@ -26988,7 +27309,7 @@
       <c r="C14" s="7"/>
       <c r="D14" s="46"/>
       <c r="E14" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F14" s="52"/>
       <c r="G14" s="52"/>
@@ -27005,7 +27326,7 @@
       <c r="C15" s="7"/>
       <c r="D15" s="46"/>
       <c r="E15" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F15" s="52"/>
       <c r="G15" s="52"/>
@@ -27022,7 +27343,7 @@
       <c r="C16" s="7"/>
       <c r="D16" s="46"/>
       <c r="E16" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="52"/>
@@ -27039,7 +27360,7 @@
       <c r="C17" s="7"/>
       <c r="D17" s="46"/>
       <c r="E17" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F17" s="52"/>
       <c r="G17" s="52"/>
@@ -27056,7 +27377,7 @@
       <c r="C18" s="7"/>
       <c r="D18" s="46"/>
       <c r="E18" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F18" s="52"/>
       <c r="G18" s="52"/>
@@ -31202,7 +31523,7 @@
         <v>6</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C89" s="65" t="n">
         <v>46344</v>
@@ -31219,7 +31540,7 @@
         <v>6</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C90" s="65" t="n">
         <v>46344</v>
@@ -31236,7 +31557,7 @@
         <v>6</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C91" s="65" t="n">
         <v>46344</v>
@@ -31253,7 +31574,7 @@
         <v>6</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C92" s="65" t="n">
         <v>46344</v>
@@ -31270,7 +31591,7 @@
         <v>6</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C93" s="65" t="n">
         <v>46345</v>
@@ -31287,7 +31608,7 @@
         <v>6</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C94" s="65" t="n">
         <v>46345</v>
@@ -31304,7 +31625,7 @@
         <v>6</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C95" s="65" t="n">
         <v>46345</v>
@@ -31321,7 +31642,7 @@
         <v>6</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C96" s="65" t="n">
         <v>46345</v>
@@ -31524,35 +31845,35 @@
         <v>1680</v>
       </c>
       <c r="G2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$27,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$32,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$28,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$33,"open")</f>
         <v>open</v>
       </c>
       <c r="I2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$29,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$34,"open")</f>
         <v>open</v>
       </c>
       <c r="J2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$30,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$35,"open")</f>
         <v>open</v>
       </c>
       <c r="K2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$31,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$36,"open")</f>
         <v>open</v>
       </c>
       <c r="L2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$32,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$37,"open")</f>
         <v>open</v>
       </c>
       <c r="M2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$33,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$38,"open")</f>
         <v>open</v>
       </c>
       <c r="N2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$34,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$39,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -31572,35 +31893,35 @@
         <v>1680</v>
       </c>
       <c r="G3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$35,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$40,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$36,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$41,"open")</f>
         <v>open</v>
       </c>
       <c r="I3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$37,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$42,"open")</f>
         <v>open</v>
       </c>
       <c r="J3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$38,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$43,"open")</f>
         <v>open</v>
       </c>
       <c r="K3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$39,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$44,"open")</f>
         <v>open</v>
       </c>
       <c r="L3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$40,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$45,"open")</f>
         <v>open</v>
       </c>
       <c r="M3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$41,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$46,"open")</f>
         <v>open</v>
       </c>
       <c r="N3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$42,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$47,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -31625,35 +31946,35 @@
         <v>1683</v>
       </c>
       <c r="G4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$43,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$48,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$44,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$49,"open")</f>
         <v>open</v>
       </c>
       <c r="I4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$45,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$50,"open")</f>
         <v>open</v>
       </c>
       <c r="J4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$46,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$51,"open")</f>
         <v>open</v>
       </c>
       <c r="K4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$47,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$52,"open")</f>
         <v>open</v>
       </c>
       <c r="L4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$48,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$53,"open")</f>
         <v>open</v>
       </c>
       <c r="M4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$49,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$54,"open")</f>
         <v>open</v>
       </c>
       <c r="N4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$50,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$55,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -31678,35 +31999,35 @@
         <v>1683</v>
       </c>
       <c r="G5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$51,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$56,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$52,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$57,"open")</f>
         <v>open</v>
       </c>
       <c r="I5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$53,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$58,"open")</f>
         <v>open</v>
       </c>
       <c r="J5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$54,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$59,"open")</f>
         <v>open</v>
       </c>
       <c r="K5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$55,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$60,"open")</f>
         <v>open</v>
       </c>
       <c r="L5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$56,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$61,"open")</f>
         <v>open</v>
       </c>
       <c r="M5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$57,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$62,"open")</f>
         <v>open</v>
       </c>
       <c r="N5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$58,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$63,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -31731,35 +32052,35 @@
         <v>1680</v>
       </c>
       <c r="G6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$59,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$64,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$60,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$65,"open")</f>
         <v>open</v>
       </c>
       <c r="I6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$61,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$66,"open")</f>
         <v>open</v>
       </c>
       <c r="J6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$62,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$67,"open")</f>
         <v>open</v>
       </c>
       <c r="K6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$63,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$68,"open")</f>
         <v>open</v>
       </c>
       <c r="L6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$64,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$69,"open")</f>
         <v>open</v>
       </c>
       <c r="M6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$65,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$70,"open")</f>
         <v>open</v>
       </c>
       <c r="N6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$66,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$71,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -31784,20 +32105,35 @@
         <v>1680</v>
       </c>
       <c r="G7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$67,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$72,"folder")</f>
         <v>folder</v>
       </c>
       <c r="H7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$68,"open")</f>
-        <v>open</v>
-      </c>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
+        <f aca="false">HYPERLINK(Links!$Q$73,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="I7" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$74,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="J7" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$75,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="K7" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$76,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="L7" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$77,"open")</f>
+        <v>open</v>
+      </c>
+      <c r="M7" s="8" t="str">
+        <f aca="false">HYPERLINK(Links!$Q$78,"open")</f>
+        <v>open</v>
+      </c>
       <c r="N7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$69,"folder")</f>
+        <f aca="false">HYPERLINK(Links!$Q$79,"folder")</f>
         <v>folder</v>
       </c>
     </row>
@@ -31819,7 +32155,7 @@
         <v>9</v>
       </c>
       <c r="F8" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
@@ -31848,7 +32184,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
@@ -31877,7 +32213,7 @@
         <v>4</v>
       </c>
       <c r="F10" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
@@ -31906,7 +32242,7 @@
         <v>10</v>
       </c>
       <c r="F11" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
@@ -31935,7 +32271,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
@@ -31964,7 +32300,7 @@
         <v>8</v>
       </c>
       <c r="F13" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
@@ -31993,7 +32329,7 @@
         <v>8</v>
       </c>
       <c r="F14" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
@@ -32022,7 +32358,7 @@
         <v>5</v>
       </c>
       <c r="F15" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
@@ -32051,7 +32387,7 @@
         <v>14</v>
       </c>
       <c r="F16" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
@@ -32080,7 +32416,7 @@
         <v>3</v>
       </c>
       <c r="F17" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
@@ -32109,7 +32445,7 @@
         <v>3</v>
       </c>
       <c r="F18" s="52" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
@@ -32188,27 +32524,27 @@
         <v>1700</v>
       </c>
       <c r="C2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$70,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$80,"open")</f>
         <v>open</v>
       </c>
       <c r="D2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$71,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$81,"open")</f>
         <v>open</v>
       </c>
       <c r="E2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$72,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$82,"open")</f>
         <v>open</v>
       </c>
       <c r="F2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$73,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$83,"open")</f>
         <v>open</v>
       </c>
       <c r="G2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$74,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$84,"open")</f>
         <v>open</v>
       </c>
       <c r="H2" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$75,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$85,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32220,27 +32556,27 @@
         <v>1701</v>
       </c>
       <c r="C3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$76,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$86,"open")</f>
         <v>open</v>
       </c>
       <c r="D3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$77,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$87,"open")</f>
         <v>open</v>
       </c>
       <c r="E3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$78,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$88,"open")</f>
         <v>open</v>
       </c>
       <c r="F3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$79,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$89,"open")</f>
         <v>open</v>
       </c>
       <c r="G3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$80,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$90,"open")</f>
         <v>open</v>
       </c>
       <c r="H3" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$81,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$91,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32252,27 +32588,27 @@
         <v>1702</v>
       </c>
       <c r="C4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$82,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$92,"open")</f>
         <v>open</v>
       </c>
       <c r="D4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$83,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$93,"open")</f>
         <v>open</v>
       </c>
       <c r="E4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$84,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$94,"open")</f>
         <v>open</v>
       </c>
       <c r="F4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$85,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$95,"open")</f>
         <v>open</v>
       </c>
       <c r="G4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$86,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$96,"open")</f>
         <v>open</v>
       </c>
       <c r="H4" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$87,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$97,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32284,27 +32620,27 @@
         <v>1703</v>
       </c>
       <c r="C5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$88,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$98,"open")</f>
         <v>open</v>
       </c>
       <c r="D5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$89,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$99,"open")</f>
         <v>open</v>
       </c>
       <c r="E5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$90,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$100,"open")</f>
         <v>open</v>
       </c>
       <c r="F5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$91,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$101,"open")</f>
         <v>open</v>
       </c>
       <c r="G5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$92,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$102,"open")</f>
         <v>open</v>
       </c>
       <c r="H5" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$93,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$103,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32316,27 +32652,27 @@
         <v>1704</v>
       </c>
       <c r="C6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$94,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$104,"open")</f>
         <v>open</v>
       </c>
       <c r="D6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$95,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$105,"open")</f>
         <v>open</v>
       </c>
       <c r="E6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$96,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$106,"open")</f>
         <v>open</v>
       </c>
       <c r="F6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$97,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$107,"open")</f>
         <v>open</v>
       </c>
       <c r="G6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$98,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$108,"open")</f>
         <v>open</v>
       </c>
       <c r="H6" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$99,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$109,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32348,27 +32684,27 @@
         <v>1705</v>
       </c>
       <c r="C7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$100,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$110,"open")</f>
         <v>open</v>
       </c>
       <c r="D7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$101,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$111,"open")</f>
         <v>open</v>
       </c>
       <c r="E7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$102,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$112,"open")</f>
         <v>open</v>
       </c>
       <c r="F7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$103,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$113,"open")</f>
         <v>open</v>
       </c>
       <c r="G7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$104,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$114,"open")</f>
         <v>open</v>
       </c>
       <c r="H7" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$105,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$115,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32380,27 +32716,27 @@
         <v>1706</v>
       </c>
       <c r="C8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$106,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$116,"open")</f>
         <v>open</v>
       </c>
       <c r="D8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$107,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$117,"open")</f>
         <v>open</v>
       </c>
       <c r="E8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$108,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$118,"open")</f>
         <v>open</v>
       </c>
       <c r="F8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$109,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$119,"open")</f>
         <v>open</v>
       </c>
       <c r="G8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$110,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$120,"open")</f>
         <v>open</v>
       </c>
       <c r="H8" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$111,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$121,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32412,27 +32748,27 @@
         <v>1707</v>
       </c>
       <c r="C9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$112,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$122,"open")</f>
         <v>open</v>
       </c>
       <c r="D9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$113,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$123,"open")</f>
         <v>open</v>
       </c>
       <c r="E9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$114,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$124,"open")</f>
         <v>open</v>
       </c>
       <c r="F9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$115,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$125,"open")</f>
         <v>open</v>
       </c>
       <c r="G9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$116,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$126,"open")</f>
         <v>open</v>
       </c>
       <c r="H9" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$117,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$127,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32444,27 +32780,27 @@
         <v>1708</v>
       </c>
       <c r="C10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$118,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$128,"open")</f>
         <v>open</v>
       </c>
       <c r="D10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$119,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$129,"open")</f>
         <v>open</v>
       </c>
       <c r="E10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$120,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$130,"open")</f>
         <v>open</v>
       </c>
       <c r="F10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$121,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$131,"open")</f>
         <v>open</v>
       </c>
       <c r="G10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$122,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$132,"open")</f>
         <v>open</v>
       </c>
       <c r="H10" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$123,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$133,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32476,27 +32812,27 @@
         <v>1709</v>
       </c>
       <c r="C11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$124,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$134,"open")</f>
         <v>open</v>
       </c>
       <c r="D11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$125,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$135,"open")</f>
         <v>open</v>
       </c>
       <c r="E11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$126,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$136,"open")</f>
         <v>open</v>
       </c>
       <c r="F11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$127,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$137,"open")</f>
         <v>open</v>
       </c>
       <c r="G11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$128,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$138,"open")</f>
         <v>open</v>
       </c>
       <c r="H11" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$129,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$139,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32508,27 +32844,27 @@
         <v>1710</v>
       </c>
       <c r="C12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$130,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$140,"open")</f>
         <v>open</v>
       </c>
       <c r="D12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$131,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$141,"open")</f>
         <v>open</v>
       </c>
       <c r="E12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$132,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$142,"open")</f>
         <v>open</v>
       </c>
       <c r="F12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$133,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$143,"open")</f>
         <v>open</v>
       </c>
       <c r="G12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$134,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$144,"open")</f>
         <v>open</v>
       </c>
       <c r="H12" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$135,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$145,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32540,27 +32876,27 @@
         <v>1711</v>
       </c>
       <c r="C13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$136,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$146,"open")</f>
         <v>open</v>
       </c>
       <c r="D13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$137,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$147,"open")</f>
         <v>open</v>
       </c>
       <c r="E13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$138,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$148,"open")</f>
         <v>open</v>
       </c>
       <c r="F13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$139,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$149,"open")</f>
         <v>open</v>
       </c>
       <c r="G13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$140,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$150,"open")</f>
         <v>open</v>
       </c>
       <c r="H13" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$141,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$151,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32572,27 +32908,27 @@
         <v>1712</v>
       </c>
       <c r="C14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$142,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$152,"open")</f>
         <v>open</v>
       </c>
       <c r="D14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$143,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$153,"open")</f>
         <v>open</v>
       </c>
       <c r="E14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$144,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$154,"open")</f>
         <v>open</v>
       </c>
       <c r="F14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$145,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$155,"open")</f>
         <v>open</v>
       </c>
       <c r="G14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$146,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$156,"open")</f>
         <v>open</v>
       </c>
       <c r="H14" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$147,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$157,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32604,27 +32940,27 @@
         <v>1713</v>
       </c>
       <c r="C15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$148,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$158,"open")</f>
         <v>open</v>
       </c>
       <c r="D15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$149,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$159,"open")</f>
         <v>open</v>
       </c>
       <c r="E15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$150,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$160,"open")</f>
         <v>open</v>
       </c>
       <c r="F15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$151,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$161,"open")</f>
         <v>open</v>
       </c>
       <c r="G15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$152,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$162,"open")</f>
         <v>open</v>
       </c>
       <c r="H15" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$153,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$163,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32636,27 +32972,27 @@
         <v>1714</v>
       </c>
       <c r="C16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$154,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$164,"open")</f>
         <v>open</v>
       </c>
       <c r="D16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$155,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$165,"open")</f>
         <v>open</v>
       </c>
       <c r="E16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$156,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$166,"open")</f>
         <v>open</v>
       </c>
       <c r="F16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$157,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$167,"open")</f>
         <v>open</v>
       </c>
       <c r="G16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$158,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$168,"open")</f>
         <v>open</v>
       </c>
       <c r="H16" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$159,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$169,"open")</f>
         <v>open</v>
       </c>
     </row>
@@ -32668,21 +33004,21 @@
         <v>1715</v>
       </c>
       <c r="C17" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$160,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$170,"open")</f>
         <v>open</v>
       </c>
       <c r="D17" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$161,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$171,"open")</f>
         <v>open</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$162,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$172,"open")</f>
         <v>open</v>
       </c>
       <c r="G17" s="7"/>
       <c r="H17" s="8" t="str">
-        <f aca="false">HYPERLINK(Links!$Q$163,"open")</f>
+        <f aca="false">HYPERLINK(Links!$Q$173,"open")</f>
         <v>open</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruling 53 (Croix, 25 Oct: "The students should be doing the ixls as we do the corresponding lessons, however they are due by the unit assessment."): every lesson's IXL skills are due by the unit's exam — scope_calendar.due() is the first exam day after the run (a thread day the next exam; none after it, the next class); the scope and the due-date sheet regenerated (its words: done as we go, due by the unit test); Units 5 and 6's Lesson Plan lines say due by the unit test (Thread B's by Unit 11's); the master sheet regenerated, 0 problems; ruling 53 in HOUSE STYLE, with Croix's stories/learning-plan answer on M7 Unit 10. Not rebuilt here: Units 4–5 are being rebuilt by the kit-fix session (Windmill 7611a99) — build them on Windmill fbac773 or later so the IXL slide says 'Due by the Unit 5 test.'; Unit 6 at its review.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7ovt6yLjh6QuFV9HBMV4N
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -6340,7 +6340,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 28e8a92c on 25 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 459c3e62 on 25 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -8078,7 +8078,7 @@
       </c>
       <c r="B11" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IFERROR(INDEX('IXL tracker'!$D$5:$D$82,MATCH(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),'IXL tracker'!$G$5:$G$82,0)),"nothing due"))</f>
-        <v>nothing due</v>
+        <v>Add and subtract numbers written in scientific notation (HUR)</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14680,7 +14680,7 @@
         <v>42</v>
       </c>
       <c r="S2" s="21" t="n">
-        <v>46289</v>
+        <v>46310</v>
       </c>
       <c r="T2" s="19" t="s">
         <v>43</v>
@@ -14778,7 +14778,7 @@
         <v>55</v>
       </c>
       <c r="S3" s="21" t="n">
-        <v>46290</v>
+        <v>46310</v>
       </c>
       <c r="T3" s="19" t="s">
         <v>56</v>
@@ -14876,7 +14876,7 @@
         <v>66</v>
       </c>
       <c r="S4" s="21" t="n">
-        <v>46293</v>
+        <v>46310</v>
       </c>
       <c r="T4" s="19" t="s">
         <v>67</v>
@@ -14974,7 +14974,7 @@
         <v>77</v>
       </c>
       <c r="S5" s="21" t="n">
-        <v>46294</v>
+        <v>46310</v>
       </c>
       <c r="T5" s="19" t="s">
         <v>78</v>
@@ -15072,7 +15072,7 @@
         <v>90</v>
       </c>
       <c r="S6" s="21" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="T6" s="19" t="s">
         <v>91</v>
@@ -15170,7 +15170,7 @@
         <v>99</v>
       </c>
       <c r="S7" s="21" t="n">
-        <v>46296</v>
+        <v>46310</v>
       </c>
       <c r="T7" s="19" t="s">
         <v>100</v>
@@ -15354,7 +15354,7 @@
         <v>112</v>
       </c>
       <c r="S10" s="21" t="n">
-        <v>46301</v>
+        <v>46310</v>
       </c>
       <c r="T10" s="19" t="s">
         <v>113</v>
@@ -15452,7 +15452,7 @@
         <v>123</v>
       </c>
       <c r="S11" s="21" t="n">
-        <v>46302</v>
+        <v>46310</v>
       </c>
       <c r="T11" s="19" t="s">
         <v>124</v>
@@ -15550,7 +15550,7 @@
         <v>132</v>
       </c>
       <c r="S12" s="21" t="n">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="T12" s="19" t="s">
         <v>133</v>
@@ -15691,7 +15691,7 @@
         <v>146</v>
       </c>
       <c r="S14" s="21" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="T14" s="19" t="s">
         <v>147</v>
@@ -15924,7 +15924,7 @@
         <v>159</v>
       </c>
       <c r="S18" s="42" t="n">
-        <v>46314</v>
+        <v>46321</v>
       </c>
       <c r="T18" s="40" t="s">
         <v>160</v>
@@ -16022,7 +16022,7 @@
         <v>170</v>
       </c>
       <c r="S19" s="42" t="n">
-        <v>46315</v>
+        <v>46321</v>
       </c>
       <c r="T19" s="40" t="s">
         <v>171</v>
@@ -16120,7 +16120,7 @@
         <v>179</v>
       </c>
       <c r="S20" s="42" t="n">
-        <v>46316</v>
+        <v>46321</v>
       </c>
       <c r="T20" s="40" t="s">
         <v>180</v>
@@ -16218,7 +16218,7 @@
         <v>191</v>
       </c>
       <c r="S21" s="42" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="T21" s="40" t="s">
         <v>192</v>
@@ -16316,7 +16316,7 @@
         <v>191</v>
       </c>
       <c r="S22" s="42" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="T22" s="40" t="s">
         <v>202</v>
@@ -16506,7 +16506,7 @@
         <v>213</v>
       </c>
       <c r="S25" s="21" t="n">
-        <v>46323</v>
+        <v>46331</v>
       </c>
       <c r="T25" s="19" t="s">
         <v>214</v>
@@ -16604,7 +16604,7 @@
         <v>225</v>
       </c>
       <c r="S26" s="21" t="n">
-        <v>46324</v>
+        <v>46331</v>
       </c>
       <c r="T26" s="19" t="s">
         <v>226</v>
@@ -16702,7 +16702,7 @@
         <v>234</v>
       </c>
       <c r="S27" s="21" t="n">
-        <v>46325</v>
+        <v>46331</v>
       </c>
       <c r="T27" s="19" t="s">
         <v>235</v>
@@ -16800,7 +16800,7 @@
         <v>244</v>
       </c>
       <c r="S28" s="21" t="n">
-        <v>46329</v>
+        <v>46331</v>
       </c>
       <c r="T28" s="19" t="s">
         <v>245</v>
@@ -16898,7 +16898,7 @@
         <v>244</v>
       </c>
       <c r="S29" s="21" t="n">
-        <v>46329</v>
+        <v>46331</v>
       </c>
       <c r="T29" s="19" t="s">
         <v>256</v>
@@ -16996,7 +16996,7 @@
         <v>264</v>
       </c>
       <c r="S30" s="21" t="n">
-        <v>46330</v>
+        <v>46331</v>
       </c>
       <c r="T30" s="19" t="s">
         <v>265</v>
@@ -17192,7 +17192,7 @@
         <v>280</v>
       </c>
       <c r="S33" s="42" t="n">
-        <v>46335</v>
+        <v>46343</v>
       </c>
       <c r="T33" s="40" t="s">
         <v>281</v>
@@ -17290,7 +17290,7 @@
         <v>292</v>
       </c>
       <c r="S34" s="42" t="n">
-        <v>46336</v>
+        <v>46343</v>
       </c>
       <c r="T34" s="40" t="s">
         <v>293</v>
@@ -17388,7 +17388,7 @@
         <v>304</v>
       </c>
       <c r="S35" s="42" t="n">
-        <v>46338</v>
+        <v>46343</v>
       </c>
       <c r="T35" s="40" t="s">
         <v>305</v>
@@ -17486,7 +17486,7 @@
         <v>314</v>
       </c>
       <c r="S36" s="42" t="n">
-        <v>46339</v>
+        <v>46343</v>
       </c>
       <c r="T36" s="40" t="s">
         <v>315</v>
@@ -17584,7 +17584,7 @@
         <v>325</v>
       </c>
       <c r="S37" s="42" t="n">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="T37" s="40" t="s">
         <v>326</v>
@@ -17829,7 +17829,7 @@
         <v>348</v>
       </c>
       <c r="S40" s="42" t="n">
-        <v>46345</v>
+        <v>46367</v>
       </c>
       <c r="T40" s="40" t="s">
         <v>349</v>
@@ -17927,7 +17927,7 @@
         <v>359</v>
       </c>
       <c r="S41" s="42" t="n">
-        <v>46346</v>
+        <v>46367</v>
       </c>
       <c r="T41" s="40" t="s">
         <v>360</v>
@@ -18034,7 +18034,7 @@
         <v>371</v>
       </c>
       <c r="S43" s="21" t="n">
-        <v>46358</v>
+        <v>46367</v>
       </c>
       <c r="T43" s="16"/>
       <c r="U43" s="16"/>
@@ -18129,7 +18129,7 @@
         <v>378</v>
       </c>
       <c r="S45" s="21" t="n">
-        <v>46359</v>
+        <v>46367</v>
       </c>
       <c r="T45" s="16"/>
       <c r="U45" s="16"/>
@@ -18184,7 +18184,7 @@
         <v>382</v>
       </c>
       <c r="S46" s="21" t="n">
-        <v>46360</v>
+        <v>46367</v>
       </c>
       <c r="T46" s="16"/>
       <c r="U46" s="16"/>
@@ -18239,7 +18239,7 @@
         <v>386</v>
       </c>
       <c r="S47" s="21" t="n">
-        <v>46363</v>
+        <v>46367</v>
       </c>
       <c r="T47" s="16"/>
       <c r="U47" s="16"/>
@@ -18294,7 +18294,7 @@
         <v>390</v>
       </c>
       <c r="S48" s="21" t="n">
-        <v>46365</v>
+        <v>46367</v>
       </c>
       <c r="T48" s="16"/>
       <c r="U48" s="16"/>
@@ -18389,7 +18389,7 @@
         <v>397</v>
       </c>
       <c r="S50" s="21" t="n">
-        <v>46366</v>
+        <v>46367</v>
       </c>
       <c r="T50" s="16"/>
       <c r="U50" s="16"/>
@@ -18747,7 +18747,7 @@
         <v>422</v>
       </c>
       <c r="S58" s="21" t="n">
-        <v>46394</v>
+        <v>46401</v>
       </c>
       <c r="T58" s="16"/>
       <c r="U58" s="16"/>
@@ -18802,7 +18802,7 @@
         <v>428</v>
       </c>
       <c r="S59" s="21" t="n">
-        <v>46395</v>
+        <v>46401</v>
       </c>
       <c r="T59" s="16"/>
       <c r="U59" s="16"/>
@@ -18857,7 +18857,7 @@
         <v>434</v>
       </c>
       <c r="S60" s="21" t="n">
-        <v>46398</v>
+        <v>46401</v>
       </c>
       <c r="T60" s="16"/>
       <c r="U60" s="16"/>
@@ -18912,7 +18912,7 @@
         <v>440</v>
       </c>
       <c r="S61" s="21" t="n">
-        <v>46399</v>
+        <v>46401</v>
       </c>
       <c r="T61" s="16"/>
       <c r="U61" s="16"/>
@@ -18967,7 +18967,7 @@
         <v>446</v>
       </c>
       <c r="S62" s="21" t="n">
-        <v>46400</v>
+        <v>46401</v>
       </c>
       <c r="T62" s="16"/>
       <c r="U62" s="16"/>
@@ -19104,7 +19104,7 @@
         <v>454</v>
       </c>
       <c r="S65" s="42" t="n">
-        <v>46406</v>
+        <v>46415</v>
       </c>
       <c r="T65" s="37"/>
       <c r="U65" s="37"/>
@@ -19159,7 +19159,7 @@
         <v>460</v>
       </c>
       <c r="S66" s="42" t="n">
-        <v>46407</v>
+        <v>46415</v>
       </c>
       <c r="T66" s="37"/>
       <c r="U66" s="37"/>
@@ -19214,7 +19214,7 @@
         <v>466</v>
       </c>
       <c r="S67" s="42" t="n">
-        <v>46408</v>
+        <v>46415</v>
       </c>
       <c r="T67" s="37"/>
       <c r="U67" s="37"/>
@@ -19269,7 +19269,7 @@
         <v>472</v>
       </c>
       <c r="S68" s="42" t="n">
-        <v>46409</v>
+        <v>46415</v>
       </c>
       <c r="T68" s="37"/>
       <c r="U68" s="37"/>
@@ -19324,7 +19324,7 @@
         <v>478</v>
       </c>
       <c r="S69" s="42" t="n">
-        <v>46412</v>
+        <v>46415</v>
       </c>
       <c r="T69" s="37"/>
       <c r="U69" s="37"/>
@@ -19379,7 +19379,7 @@
         <v>482</v>
       </c>
       <c r="S70" s="42" t="n">
-        <v>46413</v>
+        <v>46415</v>
       </c>
       <c r="T70" s="37"/>
       <c r="U70" s="37"/>
@@ -19434,7 +19434,7 @@
         <v>488</v>
       </c>
       <c r="S71" s="42" t="n">
-        <v>46414</v>
+        <v>46415</v>
       </c>
       <c r="T71" s="37"/>
       <c r="U71" s="37"/>
@@ -19626,7 +19626,7 @@
         <v>504</v>
       </c>
       <c r="S75" s="42" t="n">
-        <v>46420</v>
+        <v>46427</v>
       </c>
       <c r="T75" s="37"/>
       <c r="U75" s="37"/>
@@ -19681,7 +19681,7 @@
         <v>510</v>
       </c>
       <c r="S76" s="42" t="n">
-        <v>46421</v>
+        <v>46427</v>
       </c>
       <c r="T76" s="37"/>
       <c r="U76" s="37"/>
@@ -19736,7 +19736,7 @@
         <v>514</v>
       </c>
       <c r="S77" s="42" t="n">
-        <v>46423</v>
+        <v>46427</v>
       </c>
       <c r="T77" s="37"/>
       <c r="U77" s="37"/>
@@ -19791,7 +19791,7 @@
         <v>514</v>
       </c>
       <c r="S78" s="42" t="n">
-        <v>46423</v>
+        <v>46427</v>
       </c>
       <c r="T78" s="37"/>
       <c r="U78" s="37"/>
@@ -19846,7 +19846,7 @@
         <v>523</v>
       </c>
       <c r="S79" s="42" t="n">
-        <v>46426</v>
+        <v>46427</v>
       </c>
       <c r="T79" s="37"/>
       <c r="U79" s="37"/>
@@ -20038,7 +20038,7 @@
         <v>537</v>
       </c>
       <c r="S83" s="42" t="n">
-        <v>46430</v>
+        <v>46436</v>
       </c>
       <c r="T83" s="37"/>
       <c r="U83" s="37"/>
@@ -20093,7 +20093,7 @@
         <v>543</v>
       </c>
       <c r="S84" s="42" t="n">
-        <v>46434</v>
+        <v>46436</v>
       </c>
       <c r="T84" s="37"/>
       <c r="U84" s="37"/>
@@ -20148,7 +20148,7 @@
         <v>549</v>
       </c>
       <c r="S85" s="21" t="n">
-        <v>46435</v>
+        <v>46436</v>
       </c>
       <c r="T85" s="16"/>
       <c r="U85" s="16"/>
@@ -20340,7 +20340,7 @@
         <v>563</v>
       </c>
       <c r="S89" s="21" t="n">
-        <v>46441</v>
+        <v>46447</v>
       </c>
       <c r="T89" s="16"/>
       <c r="U89" s="16"/>
@@ -20395,7 +20395,7 @@
         <v>569</v>
       </c>
       <c r="S90" s="21" t="n">
-        <v>46442</v>
+        <v>46447</v>
       </c>
       <c r="T90" s="16"/>
       <c r="U90" s="16"/>
@@ -20450,7 +20450,7 @@
         <v>575</v>
       </c>
       <c r="S91" s="21" t="n">
-        <v>46443</v>
+        <v>46447</v>
       </c>
       <c r="T91" s="16"/>
       <c r="U91" s="16"/>
@@ -20505,7 +20505,7 @@
         <v>581</v>
       </c>
       <c r="S92" s="21" t="n">
-        <v>46444</v>
+        <v>46447</v>
       </c>
       <c r="T92" s="16"/>
       <c r="U92" s="16"/>
@@ -20657,7 +20657,7 @@
         <v>595</v>
       </c>
       <c r="S95" s="21" t="n">
-        <v>46449</v>
+        <v>46457</v>
       </c>
       <c r="T95" s="16"/>
       <c r="U95" s="16"/>
@@ -20712,7 +20712,7 @@
         <v>601</v>
       </c>
       <c r="S96" s="21" t="n">
-        <v>46450</v>
+        <v>46457</v>
       </c>
       <c r="T96" s="16"/>
       <c r="U96" s="16"/>
@@ -20767,7 +20767,7 @@
         <v>607</v>
       </c>
       <c r="S97" s="42" t="n">
-        <v>46454</v>
+        <v>46457</v>
       </c>
       <c r="T97" s="37"/>
       <c r="U97" s="37"/>
@@ -20822,7 +20822,7 @@
         <v>611</v>
       </c>
       <c r="S98" s="42" t="n">
-        <v>46455</v>
+        <v>46457</v>
       </c>
       <c r="T98" s="37"/>
       <c r="U98" s="37"/>
@@ -20877,7 +20877,7 @@
         <v>617</v>
       </c>
       <c r="S99" s="42" t="n">
-        <v>46456</v>
+        <v>46457</v>
       </c>
       <c r="T99" s="37"/>
       <c r="U99" s="37"/>
@@ -21254,7 +21254,7 @@
         <v>625</v>
       </c>
       <c r="S108" s="21" t="n">
-        <v>46476</v>
+        <v>46489</v>
       </c>
       <c r="T108" s="16"/>
       <c r="U108" s="16"/>
@@ -21309,7 +21309,7 @@
         <v>631</v>
       </c>
       <c r="S109" s="21" t="n">
-        <v>46477</v>
+        <v>46489</v>
       </c>
       <c r="T109" s="16"/>
       <c r="U109" s="16"/>
@@ -21364,7 +21364,7 @@
         <v>635</v>
       </c>
       <c r="S110" s="21" t="n">
-        <v>46478</v>
+        <v>46489</v>
       </c>
       <c r="T110" s="16"/>
       <c r="U110" s="16"/>
@@ -21419,7 +21419,7 @@
         <v>641</v>
       </c>
       <c r="S111" s="21" t="n">
-        <v>46479</v>
+        <v>46489</v>
       </c>
       <c r="T111" s="16"/>
       <c r="U111" s="16"/>
@@ -21474,7 +21474,7 @@
         <v>645</v>
       </c>
       <c r="S112" s="21" t="n">
-        <v>46482</v>
+        <v>46489</v>
       </c>
       <c r="T112" s="16"/>
       <c r="U112" s="16"/>
@@ -21529,7 +21529,7 @@
         <v>649</v>
       </c>
       <c r="S113" s="21" t="n">
-        <v>46483</v>
+        <v>46489</v>
       </c>
       <c r="T113" s="16"/>
       <c r="U113" s="16"/>
@@ -21584,7 +21584,7 @@
         <v>655</v>
       </c>
       <c r="S114" s="21" t="n">
-        <v>46484</v>
+        <v>46489</v>
       </c>
       <c r="T114" s="16"/>
       <c r="U114" s="16"/>
@@ -21639,7 +21639,7 @@
         <v>661</v>
       </c>
       <c r="S115" s="21" t="n">
-        <v>46485</v>
+        <v>46489</v>
       </c>
       <c r="T115" s="16"/>
       <c r="U115" s="16"/>
@@ -21694,7 +21694,7 @@
         <v>665</v>
       </c>
       <c r="S116" s="42" t="n">
-        <v>46486</v>
+        <v>46489</v>
       </c>
       <c r="T116" s="37"/>
       <c r="U116" s="37"/>
@@ -21846,7 +21846,7 @@
         <v>679</v>
       </c>
       <c r="S119" s="21" t="n">
-        <v>46491</v>
+        <v>46492</v>
       </c>
       <c r="T119" s="16"/>
       <c r="U119" s="16"/>
@@ -22491,7 +22491,7 @@
         <v>67</v>
       </c>
       <c r="G5" s="47" t="n">
-        <v>46289</v>
+        <v>46310</v>
       </c>
       <c r="H5" s="49"/>
       <c r="I5" s="49"/>
@@ -22521,7 +22521,7 @@
         <v>67</v>
       </c>
       <c r="G6" s="47" t="n">
-        <v>46290</v>
+        <v>46310</v>
       </c>
       <c r="H6" s="49"/>
       <c r="I6" s="49"/>
@@ -22551,7 +22551,7 @@
         <v>67</v>
       </c>
       <c r="G7" s="47" t="n">
-        <v>46293</v>
+        <v>46310</v>
       </c>
       <c r="H7" s="49"/>
       <c r="I7" s="49"/>
@@ -22581,7 +22581,7 @@
         <v>67</v>
       </c>
       <c r="G8" s="47" t="n">
-        <v>46294</v>
+        <v>46310</v>
       </c>
       <c r="H8" s="49"/>
       <c r="I8" s="49"/>
@@ -22611,7 +22611,7 @@
         <v>67</v>
       </c>
       <c r="G9" s="47" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="H9" s="49"/>
       <c r="I9" s="49"/>
@@ -22641,7 +22641,7 @@
         <v>67</v>
       </c>
       <c r="G10" s="47" t="n">
-        <v>46296</v>
+        <v>46310</v>
       </c>
       <c r="H10" s="49"/>
       <c r="I10" s="49"/>
@@ -22671,7 +22671,7 @@
         <v>67</v>
       </c>
       <c r="G11" s="47" t="n">
-        <v>46301</v>
+        <v>46310</v>
       </c>
       <c r="H11" s="49"/>
       <c r="I11" s="49"/>
@@ -22701,7 +22701,7 @@
         <v>67</v>
       </c>
       <c r="G12" s="47" t="n">
-        <v>46302</v>
+        <v>46310</v>
       </c>
       <c r="H12" s="49"/>
       <c r="I12" s="49"/>
@@ -22731,7 +22731,7 @@
         <v>67</v>
       </c>
       <c r="G13" s="47" t="n">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="H13" s="49"/>
       <c r="I13" s="49"/>
@@ -22761,7 +22761,7 @@
         <v>67</v>
       </c>
       <c r="G14" s="47" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="H14" s="49"/>
       <c r="I14" s="49"/>
@@ -22791,13 +22791,13 @@
         <v>67</v>
       </c>
       <c r="G15" s="47" t="n">
-        <v>46314</v>
+        <v>46321</v>
       </c>
       <c r="H15" s="49"/>
       <c r="I15" s="49"/>
       <c r="J15" s="7" t="str">
         <f aca="true">IF(I15="✓","done",IF(TODAY()&lt;B15,"upcoming",IF(TODAY()&lt;G15,"open","due — check scores")))</f>
-        <v>due — check scores</v>
+        <v>open</v>
       </c>
       <c r="K15" s="50"/>
     </row>
@@ -22821,13 +22821,13 @@
         <v>67</v>
       </c>
       <c r="G16" s="47" t="n">
-        <v>46315</v>
+        <v>46321</v>
       </c>
       <c r="H16" s="49"/>
       <c r="I16" s="49"/>
       <c r="J16" s="7" t="str">
         <f aca="true">IF(I16="✓","done",IF(TODAY()&lt;B16,"upcoming",IF(TODAY()&lt;G16,"open","due — check scores")))</f>
-        <v>due — check scores</v>
+        <v>open</v>
       </c>
       <c r="K16" s="50"/>
     </row>
@@ -22851,13 +22851,13 @@
         <v>67</v>
       </c>
       <c r="G17" s="47" t="n">
-        <v>46316</v>
+        <v>46321</v>
       </c>
       <c r="H17" s="49"/>
       <c r="I17" s="49"/>
       <c r="J17" s="7" t="str">
         <f aca="true">IF(I17="✓","done",IF(TODAY()&lt;B17,"upcoming",IF(TODAY()&lt;G17,"open","due — check scores")))</f>
-        <v>due — check scores</v>
+        <v>open</v>
       </c>
       <c r="K17" s="50"/>
     </row>
@@ -22881,13 +22881,13 @@
         <v>67</v>
       </c>
       <c r="G18" s="47" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="H18" s="49"/>
       <c r="I18" s="49"/>
       <c r="J18" s="7" t="str">
         <f aca="true">IF(I18="✓","done",IF(TODAY()&lt;B18,"upcoming",IF(TODAY()&lt;G18,"open","due — check scores")))</f>
-        <v>due — check scores</v>
+        <v>open</v>
       </c>
       <c r="K18" s="50"/>
     </row>
@@ -22911,7 +22911,7 @@
         <v>67</v>
       </c>
       <c r="G19" s="47" t="n">
-        <v>46323</v>
+        <v>46331</v>
       </c>
       <c r="H19" s="49"/>
       <c r="I19" s="49"/>
@@ -22941,7 +22941,7 @@
         <v>67</v>
       </c>
       <c r="G20" s="47" t="n">
-        <v>46324</v>
+        <v>46331</v>
       </c>
       <c r="H20" s="49"/>
       <c r="I20" s="49"/>
@@ -22971,7 +22971,7 @@
         <v>67</v>
       </c>
       <c r="G21" s="47" t="n">
-        <v>46325</v>
+        <v>46331</v>
       </c>
       <c r="H21" s="49"/>
       <c r="I21" s="49"/>
@@ -23001,7 +23001,7 @@
         <v>67</v>
       </c>
       <c r="G22" s="47" t="n">
-        <v>46329</v>
+        <v>46331</v>
       </c>
       <c r="H22" s="49"/>
       <c r="I22" s="49"/>
@@ -23031,7 +23031,7 @@
         <v>67</v>
       </c>
       <c r="G23" s="47" t="n">
-        <v>46330</v>
+        <v>46331</v>
       </c>
       <c r="H23" s="49"/>
       <c r="I23" s="49"/>
@@ -23061,7 +23061,7 @@
         <v>67</v>
       </c>
       <c r="G24" s="47" t="n">
-        <v>46335</v>
+        <v>46343</v>
       </c>
       <c r="H24" s="49"/>
       <c r="I24" s="49"/>
@@ -23091,7 +23091,7 @@
         <v>67</v>
       </c>
       <c r="G25" s="47" t="n">
-        <v>46336</v>
+        <v>46343</v>
       </c>
       <c r="H25" s="49"/>
       <c r="I25" s="49"/>
@@ -23121,7 +23121,7 @@
         <v>67</v>
       </c>
       <c r="G26" s="47" t="n">
-        <v>46338</v>
+        <v>46343</v>
       </c>
       <c r="H26" s="49"/>
       <c r="I26" s="49"/>
@@ -23151,7 +23151,7 @@
         <v>67</v>
       </c>
       <c r="G27" s="47" t="n">
-        <v>46339</v>
+        <v>46343</v>
       </c>
       <c r="H27" s="49"/>
       <c r="I27" s="49"/>
@@ -23181,7 +23181,7 @@
         <v>67</v>
       </c>
       <c r="G28" s="47" t="n">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="H28" s="49"/>
       <c r="I28" s="49"/>
@@ -23241,7 +23241,7 @@
         <v>67</v>
       </c>
       <c r="G30" s="47" t="n">
-        <v>46345</v>
+        <v>46367</v>
       </c>
       <c r="H30" s="49"/>
       <c r="I30" s="49"/>
@@ -23271,7 +23271,7 @@
         <v>67</v>
       </c>
       <c r="G31" s="47" t="n">
-        <v>46346</v>
+        <v>46367</v>
       </c>
       <c r="H31" s="49"/>
       <c r="I31" s="49"/>
@@ -23301,7 +23301,7 @@
         <v>67</v>
       </c>
       <c r="G32" s="47" t="n">
-        <v>46358</v>
+        <v>46367</v>
       </c>
       <c r="H32" s="49"/>
       <c r="I32" s="49"/>
@@ -23331,7 +23331,7 @@
         <v>67</v>
       </c>
       <c r="G33" s="47" t="n">
-        <v>46359</v>
+        <v>46367</v>
       </c>
       <c r="H33" s="49"/>
       <c r="I33" s="49"/>
@@ -23361,7 +23361,7 @@
         <v>67</v>
       </c>
       <c r="G34" s="47" t="n">
-        <v>46360</v>
+        <v>46367</v>
       </c>
       <c r="H34" s="49"/>
       <c r="I34" s="49"/>
@@ -23391,7 +23391,7 @@
         <v>67</v>
       </c>
       <c r="G35" s="47" t="n">
-        <v>46363</v>
+        <v>46367</v>
       </c>
       <c r="H35" s="49"/>
       <c r="I35" s="49"/>
@@ -23421,7 +23421,7 @@
         <v>67</v>
       </c>
       <c r="G36" s="47" t="n">
-        <v>46365</v>
+        <v>46367</v>
       </c>
       <c r="H36" s="49"/>
       <c r="I36" s="49"/>
@@ -23451,7 +23451,7 @@
         <v>67</v>
       </c>
       <c r="G37" s="47" t="n">
-        <v>46366</v>
+        <v>46367</v>
       </c>
       <c r="H37" s="49"/>
       <c r="I37" s="49"/>
@@ -23511,7 +23511,7 @@
         <v>67</v>
       </c>
       <c r="G39" s="47" t="n">
-        <v>46394</v>
+        <v>46401</v>
       </c>
       <c r="H39" s="49"/>
       <c r="I39" s="49"/>
@@ -23541,7 +23541,7 @@
         <v>67</v>
       </c>
       <c r="G40" s="47" t="n">
-        <v>46395</v>
+        <v>46401</v>
       </c>
       <c r="H40" s="49"/>
       <c r="I40" s="49"/>
@@ -23571,7 +23571,7 @@
         <v>67</v>
       </c>
       <c r="G41" s="47" t="n">
-        <v>46398</v>
+        <v>46401</v>
       </c>
       <c r="H41" s="49"/>
       <c r="I41" s="49"/>
@@ -23601,7 +23601,7 @@
         <v>67</v>
       </c>
       <c r="G42" s="47" t="n">
-        <v>46399</v>
+        <v>46401</v>
       </c>
       <c r="H42" s="49"/>
       <c r="I42" s="49"/>
@@ -23631,7 +23631,7 @@
         <v>67</v>
       </c>
       <c r="G43" s="47" t="n">
-        <v>46400</v>
+        <v>46401</v>
       </c>
       <c r="H43" s="49"/>
       <c r="I43" s="49"/>
@@ -23661,7 +23661,7 @@
         <v>67</v>
       </c>
       <c r="G44" s="47" t="n">
-        <v>46406</v>
+        <v>46415</v>
       </c>
       <c r="H44" s="49"/>
       <c r="I44" s="49"/>
@@ -23691,7 +23691,7 @@
         <v>67</v>
       </c>
       <c r="G45" s="47" t="n">
-        <v>46407</v>
+        <v>46415</v>
       </c>
       <c r="H45" s="49"/>
       <c r="I45" s="49"/>
@@ -23721,7 +23721,7 @@
         <v>67</v>
       </c>
       <c r="G46" s="47" t="n">
-        <v>46408</v>
+        <v>46415</v>
       </c>
       <c r="H46" s="49"/>
       <c r="I46" s="49"/>
@@ -23751,7 +23751,7 @@
         <v>67</v>
       </c>
       <c r="G47" s="47" t="n">
-        <v>46409</v>
+        <v>46415</v>
       </c>
       <c r="H47" s="49"/>
       <c r="I47" s="49"/>
@@ -23781,7 +23781,7 @@
         <v>67</v>
       </c>
       <c r="G48" s="47" t="n">
-        <v>46412</v>
+        <v>46415</v>
       </c>
       <c r="H48" s="49"/>
       <c r="I48" s="49"/>
@@ -23811,7 +23811,7 @@
         <v>67</v>
       </c>
       <c r="G49" s="47" t="n">
-        <v>46413</v>
+        <v>46415</v>
       </c>
       <c r="H49" s="49"/>
       <c r="I49" s="49"/>
@@ -23841,7 +23841,7 @@
         <v>67</v>
       </c>
       <c r="G50" s="47" t="n">
-        <v>46414</v>
+        <v>46415</v>
       </c>
       <c r="H50" s="49"/>
       <c r="I50" s="49"/>
@@ -23901,7 +23901,7 @@
         <v>67</v>
       </c>
       <c r="G52" s="47" t="n">
-        <v>46420</v>
+        <v>46427</v>
       </c>
       <c r="H52" s="49"/>
       <c r="I52" s="49"/>
@@ -23931,7 +23931,7 @@
         <v>67</v>
       </c>
       <c r="G53" s="47" t="n">
-        <v>46421</v>
+        <v>46427</v>
       </c>
       <c r="H53" s="49"/>
       <c r="I53" s="49"/>
@@ -23961,7 +23961,7 @@
         <v>67</v>
       </c>
       <c r="G54" s="47" t="n">
-        <v>46423</v>
+        <v>46427</v>
       </c>
       <c r="H54" s="49"/>
       <c r="I54" s="49"/>
@@ -23991,7 +23991,7 @@
         <v>67</v>
       </c>
       <c r="G55" s="47" t="n">
-        <v>46426</v>
+        <v>46427</v>
       </c>
       <c r="H55" s="49"/>
       <c r="I55" s="49"/>
@@ -24051,7 +24051,7 @@
         <v>67</v>
       </c>
       <c r="G57" s="47" t="n">
-        <v>46430</v>
+        <v>46436</v>
       </c>
       <c r="H57" s="49"/>
       <c r="I57" s="49"/>
@@ -24081,7 +24081,7 @@
         <v>67</v>
       </c>
       <c r="G58" s="47" t="n">
-        <v>46434</v>
+        <v>46436</v>
       </c>
       <c r="H58" s="49"/>
       <c r="I58" s="49"/>
@@ -24111,7 +24111,7 @@
         <v>67</v>
       </c>
       <c r="G59" s="47" t="n">
-        <v>46435</v>
+        <v>46436</v>
       </c>
       <c r="H59" s="49"/>
       <c r="I59" s="49"/>
@@ -24171,7 +24171,7 @@
         <v>67</v>
       </c>
       <c r="G61" s="47" t="n">
-        <v>46441</v>
+        <v>46447</v>
       </c>
       <c r="H61" s="49"/>
       <c r="I61" s="49"/>
@@ -24201,7 +24201,7 @@
         <v>67</v>
       </c>
       <c r="G62" s="47" t="n">
-        <v>46442</v>
+        <v>46447</v>
       </c>
       <c r="H62" s="49"/>
       <c r="I62" s="49"/>
@@ -24231,7 +24231,7 @@
         <v>67</v>
       </c>
       <c r="G63" s="47" t="n">
-        <v>46443</v>
+        <v>46447</v>
       </c>
       <c r="H63" s="49"/>
       <c r="I63" s="49"/>
@@ -24261,7 +24261,7 @@
         <v>67</v>
       </c>
       <c r="G64" s="47" t="n">
-        <v>46444</v>
+        <v>46447</v>
       </c>
       <c r="H64" s="49"/>
       <c r="I64" s="49"/>
@@ -24321,7 +24321,7 @@
         <v>67</v>
       </c>
       <c r="G66" s="47" t="n">
-        <v>46449</v>
+        <v>46457</v>
       </c>
       <c r="H66" s="49"/>
       <c r="I66" s="49"/>
@@ -24351,7 +24351,7 @@
         <v>67</v>
       </c>
       <c r="G67" s="47" t="n">
-        <v>46450</v>
+        <v>46457</v>
       </c>
       <c r="H67" s="49"/>
       <c r="I67" s="49"/>
@@ -24381,7 +24381,7 @@
         <v>67</v>
       </c>
       <c r="G68" s="47" t="n">
-        <v>46454</v>
+        <v>46457</v>
       </c>
       <c r="H68" s="49"/>
       <c r="I68" s="49"/>
@@ -24411,7 +24411,7 @@
         <v>67</v>
       </c>
       <c r="G69" s="47" t="n">
-        <v>46455</v>
+        <v>46457</v>
       </c>
       <c r="H69" s="49"/>
       <c r="I69" s="49"/>
@@ -24441,7 +24441,7 @@
         <v>67</v>
       </c>
       <c r="G70" s="47" t="n">
-        <v>46456</v>
+        <v>46457</v>
       </c>
       <c r="H70" s="49"/>
       <c r="I70" s="49"/>
@@ -24471,7 +24471,7 @@
         <v>67</v>
       </c>
       <c r="G71" s="47" t="n">
-        <v>46476</v>
+        <v>46489</v>
       </c>
       <c r="H71" s="49"/>
       <c r="I71" s="49"/>
@@ -24501,7 +24501,7 @@
         <v>67</v>
       </c>
       <c r="G72" s="47" t="n">
-        <v>46477</v>
+        <v>46489</v>
       </c>
       <c r="H72" s="49"/>
       <c r="I72" s="49"/>
@@ -24531,7 +24531,7 @@
         <v>67</v>
       </c>
       <c r="G73" s="47" t="n">
-        <v>46478</v>
+        <v>46489</v>
       </c>
       <c r="H73" s="49"/>
       <c r="I73" s="49"/>
@@ -24561,7 +24561,7 @@
         <v>67</v>
       </c>
       <c r="G74" s="47" t="n">
-        <v>46479</v>
+        <v>46489</v>
       </c>
       <c r="H74" s="49"/>
       <c r="I74" s="49"/>
@@ -24591,7 +24591,7 @@
         <v>67</v>
       </c>
       <c r="G75" s="47" t="n">
-        <v>46482</v>
+        <v>46489</v>
       </c>
       <c r="H75" s="49"/>
       <c r="I75" s="49"/>
@@ -24621,7 +24621,7 @@
         <v>67</v>
       </c>
       <c r="G76" s="47" t="n">
-        <v>46483</v>
+        <v>46489</v>
       </c>
       <c r="H76" s="49"/>
       <c r="I76" s="49"/>
@@ -24651,7 +24651,7 @@
         <v>67</v>
       </c>
       <c r="G77" s="47" t="n">
-        <v>46484</v>
+        <v>46489</v>
       </c>
       <c r="H77" s="49"/>
       <c r="I77" s="49"/>
@@ -24681,7 +24681,7 @@
         <v>67</v>
       </c>
       <c r="G78" s="47" t="n">
-        <v>46485</v>
+        <v>46489</v>
       </c>
       <c r="H78" s="49"/>
       <c r="I78" s="49"/>
@@ -24711,7 +24711,7 @@
         <v>67</v>
       </c>
       <c r="G79" s="47" t="n">
-        <v>46486</v>
+        <v>46489</v>
       </c>
       <c r="H79" s="49"/>
       <c r="I79" s="49"/>
@@ -24771,7 +24771,7 @@
         <v>67</v>
       </c>
       <c r="G81" s="47" t="n">
-        <v>46491</v>
+        <v>46492</v>
       </c>
       <c r="H81" s="49"/>
       <c r="I81" s="49"/>

</xml_diff>

<commit_message>
Ruling 53: the master sheet's Today shows an exam day's whole unit of IXL (every skill of the unit — N assignments), and its notes say done as the lessons go, due by the unit's exam (a thread day's by the next exam).
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7ovt6yLjh6QuFV9HBMV4N
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -827,7 +827,7 @@
     <t xml:space="preserve">IXL assigned</t>
   </si>
   <si>
-    <t xml:space="preserve">IXL due at the start of class</t>
+    <t xml:space="preserve">IXL due today</t>
   </si>
   <si>
     <t xml:space="preserve">Closure question</t>
@@ -6331,7 +6331,7 @@
     <t xml:space="preserve">The yellow cells in the IXL tracker are yours. In the live Google Sheet they stay: when a new edition of this sheet is published, the script puts the new contents into the same Google Sheet, so its address and your bookmark stay (should Google ever refuse, it makes a new sheet, and the Status tab of the Windy Hill Drive Index links to it), and it writes your ticks and notes back, lesson by lesson (a copy of them is kept on the Kept tab of the Windy Hill Drive Index). Anything typed anywhere else in this sheet is replaced by the next edition. An Excel copy (.xlsx) carries no ticks.</t>
   </si>
   <si>
-    <t xml:space="preserve">IXL: every skill listed is required, to a SmartScore of 67, due at the start of the next class (ruling 28). Lessons in a row that use the same skills are one assignment, due after the last of them — the IXL due column already shows that date.</t>
+    <t xml:space="preserve">IXL: every skill listed is required, to a SmartScore of 67 (ruling 28); done as the lessons go, and due by the unit's exam (ruling 53, 25 Oct 2026; a thread day's by the next exam). The IXL due column shows that date.</t>
   </si>
   <si>
     <t xml:space="preserve">'No school' days are the holidays in the plan (tools/scope_calendar.py), taken from the board-approved calendar — check them against the school's copy.</t>
@@ -6340,7 +6340,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 459c3e62 on 25 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 3976f039 on 25 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -8077,8 +8077,8 @@
         <v>8</v>
       </c>
       <c r="B11" s="6" t="str">
-        <f aca="false">IF($B$44&gt;131,"",IFERROR(INDEX('IXL tracker'!$D$5:$D$82,MATCH(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),'IXL tracker'!$G$5:$G$82,0)),"nothing due"))</f>
-        <v>Add and subtract numbers written in scientific notation (HUR)</v>
+        <f aca="false">IF($B$44&gt;131,"",IF(COUNTIF('IXL tracker'!$G$5:$G$82,INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44))=0,"nothing due",IF(COUNTIF('IXL tracker'!$G$5:$G$82,INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44))=1,INDEX('IXL tracker'!$D$5:$D$82,MATCH(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),'IXL tracker'!$G$5:$G$82,0)),"every skill of the unit — "&amp;COUNTIF('IXL tracker'!$G$5:$G$82,INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44))&amp;" assignments (IXL tracker)")))</f>
+        <v>every skill of the unit — 4 assignments (IXL tracker)</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Master sheet rebuilt for the ELA PM2 move (Thu 3 Dec); all checks pass.
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7ovt6yLjh6QuFV9HBMV4N
</commit_message>
<xml_diff>
--- a/a7/reference/A7 Master Sheet 2026-27.xlsx
+++ b/a7/reference/A7 Master Sheet 2026-27.xlsx
@@ -1972,31 +1972,31 @@
     <t xml:space="preserve">11.1 Solving Equations</t>
   </si>
   <si>
+    <t xml:space="preserve">11.02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variables on both sides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solve equations with variables on both sides — ZYL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.2 Solving Equations with Variables on Both Sides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One, none, infinitely many solutions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Find the number of solutions — XDE; Create equations with no solutions or infinitely many solutions — 7TY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.3 Solutions to Linear Equations</t>
+  </si>
+  <si>
     <t xml:space="preserve">FAST PM2 (ELA) — no class</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variables on both sides</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solve equations with variables on both sides — ZYL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.2 Solving Equations with Variables on Both Sides</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One, none, infinitely many solutions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Find the number of solutions — XDE; Create equations with no solutions or infinitely many solutions — 7TY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.3 Solutions to Linear Equations</t>
   </si>
   <si>
     <t xml:space="preserve">11.04</t>
@@ -4151,7 +4151,7 @@
     <t xml:space="preserve">11</t>
   </si>
   <si>
-    <t xml:space="preserve">11.01 (Mon 30 Nov); 11.02 (Wed 2 Dec); 11.03 (Thu 3 Dec); 11.04 (Fri 4 Dec)</t>
+    <t xml:space="preserve">11.01 (Mon 30 Nov); 11.02 (Tue 1 Dec); 11.03 (Wed 2 Dec); 11.04 (Fri 4 Dec)</t>
   </si>
   <si>
     <t xml:space="preserve">Q2B, QWE, 8CZ, ZYL, XDE, 7TY, 55K, PGH, HZZ</t>
@@ -5095,16 +5095,16 @@
     <t xml:space="preserve">December 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">1   off
+    <t xml:space="preserve">1   11.02
+Variables on both sides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2   11.03
+One, none, infinitely many solutions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3   off
 FAST PM2 (ELA) — no class</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2   11.02
-Variables on both sides</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3   11.03
-One, none, infinitely many solutions</t>
   </si>
   <si>
     <t xml:space="preserve">4   11.04
@@ -6340,7 +6340,7 @@
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 27b9603b on 25 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
+    <t xml:space="preserve">Generated by tools/master_sheet.py (live Google Drive links) at commit 32c6680e on 31 October 2026, from the calendar table, the IXL due-date sheet, the Source of Truth (benchmark wording), Florida's B.E.S.T. standards (MTR titles), the Math Nation table of contents, the lesson and unit specs, and the package folders. The plan is edited in scope_calendar.py; this file is never edited by hand — except the yellow cells in the IXL tracker, which are yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Where</t>
@@ -6574,16 +6574,16 @@
     <t xml:space="preserve">'Units'!J3</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.02%22</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Units'!K3</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.02%22</t>
+    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.03%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!L3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/drive/search?q=title:%22A7%2011.03%22</t>
   </si>
   <si>
     <t xml:space="preserve">'Units'!M3</t>
@@ -8006,7 +8006,7 @@
       </c>
       <c r="B1" s="2" t="n">
         <f aca="true">TODAY()</f>
-        <v>46320</v>
+        <v>46326</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="B3" s="4" t="str">
         <f aca="true">IF($B$44&gt;131,"The school year has ended.",IF(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44)=TODAY(),"Today's class",IF(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44)&lt;TODAY(),"The PM3 window (3–28 May)","Next class: "&amp;TEXT(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),"dddd d mmmm"))))</f>
-        <v>Next class: Monday 26 October</v>
+        <v>Next class: Monday 2 November</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8024,16 +8024,16 @@
       </c>
       <c r="B5" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,$B$44)&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,$B$44))</f>
-        <v>4.X   Unit 4 exam</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5.08+09   Converting mass, area and volume across systems</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$T$2:$T$132,$B$44)&amp;"")</f>
-        <v/>
+        <v>I can convert mass, volume and area between systems, and square the length ratio for area.</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8042,7 +8042,7 @@
       </c>
       <c r="B7" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$U$2:$U$132,$B$44)&amp;"")</f>
-        <v/>
+        <v>1 ft = 12 in. Why is 1 ft² not 12 in²?</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8051,7 +8051,7 @@
       </c>
       <c r="B8" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$V$2:$V$132,$B$44)&amp;"")</f>
-        <v/>
+        <v>mass and weight, ounce (oz), fluid ounce (fl oz), square units, cubic units</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8060,16 +8060,16 @@
       </c>
       <c r="B9" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$W$2:$W$132,$B$44)&amp;"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>7.AR.3.3</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IF(INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;""="","none",INDEX('Scope &amp; Sequence'!$R$2:$R$132,$B$44)&amp;"   — due "&amp;TEXT(INDEX('Scope &amp; Sequence'!$S$2:$S$132,$B$44),"ddd d mmm")))</f>
-        <v>none</v>
+        <v>Convert between customary and metric systems — E8Z; Compare and convert customary units — 4B8; Compare and convert metric units — HW2   — due Thu 5 Nov</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="B11" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",IF(COUNTIF('IXL tracker'!$G$5:$G$82,INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44))=0,"nothing due",IF(COUNTIF('IXL tracker'!$G$5:$G$82,INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44))=1,INDEX('IXL tracker'!$D$5:$D$82,MATCH(INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44),'IXL tracker'!$G$5:$G$82,0)),"every skill of the unit — "&amp;COUNTIF('IXL tracker'!$G$5:$G$82,INDEX('Scope &amp; Sequence'!$A$2:$A$132,$B$44))&amp;" assignments (IXL tracker)")))</f>
-        <v>every skill of the unit — 4 assignments (IXL tracker)</v>
+        <v>nothing due</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8087,7 +8087,7 @@
       </c>
       <c r="B12" s="6" t="str">
         <f aca="false">IF($B$44&gt;131,"",INDEX('Scope &amp; Sequence'!$Z$2:$Z$132,$B$44)&amp;"")</f>
-        <v/>
+        <v>1 ft = 12 in. Priya says 2 ft³ is 24 in³, because 2 × 12 = 24. Name the error and fix it.</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8101,7 +8101,7 @@
       </c>
       <c r="B15" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$B$2:$B$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,$B$44),INDEX('Scope &amp; Sequence'!$F$2:$F$132,$B$44)&amp;"")))</f>
-        <v>Unit Assessment</v>
+        <v>open</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8110,7 +8110,7 @@
       </c>
       <c r="B16" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$C$2:$C$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$C$2:$C$132,$B$44),INDEX('Scope &amp; Sequence'!$G$2:$G$132,$B$44)&amp;"")))</f>
-        <v>—</v>
+        <v>open</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8119,7 +8119,7 @@
       </c>
       <c r="B17" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$D$2:$D$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$D$2:$D$132,$B$44),INDEX('Scope &amp; Sequence'!$H$2:$H$132,$B$44)&amp;"")))</f>
-        <v>—</v>
+        <v>open</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="B18" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$E$2:$E$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$E$2:$E$132,$B$44),INDEX('Scope &amp; Sequence'!$I$2:$I$132,$B$44)&amp;"")))</f>
-        <v>—</v>
+        <v>open</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8137,7 +8137,7 @@
       </c>
       <c r="B19" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$F$2:$F$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$F$2:$F$132,$B$44),INDEX('Scope &amp; Sequence'!$J$2:$J$132,$B$44)&amp;"")))</f>
-        <v>—</v>
+        <v>open</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8146,7 +8146,7 @@
       </c>
       <c r="B20" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$G$2:$G$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$G$2:$G$132,$B$44),INDEX('Scope &amp; Sequence'!$K$2:$K$132,$B$44)&amp;"")))</f>
-        <v>Assessment key</v>
+        <v>key</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="B21" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$H$2:$H$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$H$2:$H$132,$B$44),INDEX('Scope &amp; Sequence'!$L$2:$L$132,$B$44)&amp;"")))</f>
-        <v>—</v>
+        <v>open</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="B22" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$I$2:$I$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$I$2:$I$132,$B$44),INDEX('Scope &amp; Sequence'!$M$2:$M$132,$B$44)&amp;"")))</f>
-        <v>—</v>
+        <v>key</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8173,7 +8173,7 @@
       </c>
       <c r="B23" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$J$2:$J$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$J$2:$J$132,$B$44),INDEX('Scope &amp; Sequence'!$N$2:$N$132,$B$44)&amp;"")))</f>
-        <v>—</v>
+        <v>open</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="B24" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$K$2:$K$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$K$2:$K$132,$B$44),INDEX('Scope &amp; Sequence'!$O$2:$O$132,$B$44)&amp;"")))</f>
-        <v>—</v>
+        <v>key</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="B26" s="8" t="str">
         <f aca="false">IF($B$44&gt;131,"—",IF(INDEX(Links!$M$2:$M$132,$B$44)&amp;""="","—",HYPERLINK(INDEX(Links!$M$2:$M$132,$B$44),INDEX('Scope &amp; Sequence'!$Q$2:$Q$132,$B$44)&amp;"")))</f>
-        <v>—</v>
+        <v>search</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8222,11 +8222,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="n">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+1)))</f>
-        <v>46322</v>
+        <v>46329</v>
       </c>
       <c r="B30" s="6" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+1))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+1)))</f>
-        <v>5.01   Scale drawings</v>
+        <v>5.10+11   Multi-step proportion problems</v>
       </c>
       <c r="C30" s="8" t="str">
         <f aca="false">IF(($B$44+1)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+1))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+1)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+1))&amp;"")))</f>
@@ -8236,39 +8236,39 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="n">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+2)))</f>
-        <v>46323</v>
+        <v>46330</v>
       </c>
       <c r="B31" s="6" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+2))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+2)))</f>
-        <v>5.02+03   Scale factor: perimeter and area (k and k²)</v>
+        <v>spiral   Spiral day — mixed retrieval from the unit just finished and the two before it</v>
       </c>
       <c r="C31" s="8" t="str">
         <f aca="false">IF(($B$44+2)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+2))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+2)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+2))&amp;"")))</f>
-        <v>open</v>
+        <v>Unit Review</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="n">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+3)))</f>
-        <v>46324</v>
+        <v>46331</v>
       </c>
       <c r="B32" s="6" t="str">
         <f aca="false">IF(($B$44+3)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+3))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+3)))</f>
-        <v>5.04   Real-world scale drawings</v>
+        <v>5.X   Unit 5 exam</v>
       </c>
       <c r="C32" s="8" t="str">
         <f aca="false">IF(($B$44+3)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+3))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+3)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+3))&amp;"")))</f>
-        <v>open</v>
+        <v>Unit Assessment</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+4)))</f>
-        <v>46325</v>
+        <v>46332</v>
       </c>
       <c r="B33" s="6" t="str">
         <f aca="false">IF(($B$44+4)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+4))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+4)))</f>
-        <v>5.06+07   Converting length across systems; currency</v>
+        <v>6.01+02   Triangle Inequality Theorem; converse of the Pythagorean Theorem</v>
       </c>
       <c r="C33" s="8" t="str">
         <f aca="false">IF(($B$44+4)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+4))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+4)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+4))&amp;"")))</f>
@@ -8278,11 +8278,11 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="n">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$A$2:$A$132,($B$44+5)))</f>
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="B34" s="6" t="str">
         <f aca="false">IF(($B$44+5)&gt;131,"",INDEX('Scope &amp; Sequence'!$D$2:$D$132,($B$44+5))&amp;"   "&amp;INDEX('Scope &amp; Sequence'!$E$2:$E$132,($B$44+5)))</f>
-        <v>5.08+09   Converting mass, area and volume across systems</v>
+        <v>6.03   Pythagorean Theorem (memorize)</v>
       </c>
       <c r="C34" s="8" t="str">
         <f aca="false">IF(($B$44+5)&gt;131,"",IF(INDEX(Links!$B$2:$B$132,($B$44+5))&amp;""="","—",HYPERLINK(INDEX(Links!$B$2:$B$132,($B$44+5)),INDEX('Scope &amp; Sequence'!$F$2:$F$132,($B$44+5))&amp;"")))</f>
@@ -8302,7 +8302,7 @@
       </c>
       <c r="B44" s="13" t="n">
         <f aca="true">IF(TODAY()&gt;$B$45,131+1,MIN(COUNTIF('Scope &amp; Sequence'!$A$2:$A$132,"&lt;"&amp;TODAY())+1,131))</f>
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10803,10 +10803,12 @@
       <c r="J44" s="69"/>
       <c r="K44" s="69"/>
       <c r="L44" s="69"/>
-      <c r="M44" s="69"/>
+      <c r="M44" s="69" t="s">
+        <v>1816</v>
+      </c>
       <c r="N44" s="69"/>
       <c r="O44" s="69" t="s">
-        <v>1816</v>
+        <v>1817</v>
       </c>
       <c r="P44" s="69" t="s">
         <v>1744</v>
@@ -10832,11 +10834,11 @@
       <c r="K45" s="69"/>
       <c r="L45" s="69"/>
       <c r="M45" s="69" t="s">
-        <v>1817</v>
+        <v>1818</v>
       </c>
       <c r="N45" s="69"/>
       <c r="O45" s="69" t="s">
-        <v>1818</v>
+        <v>1819</v>
       </c>
       <c r="P45" s="69" t="s">
         <v>1744</v>
@@ -10861,9 +10863,7 @@
       <c r="J46" s="69"/>
       <c r="K46" s="69"/>
       <c r="L46" s="69"/>
-      <c r="M46" s="69" t="s">
-        <v>1819</v>
-      </c>
+      <c r="M46" s="69"/>
       <c r="N46" s="69"/>
       <c r="O46" s="69" t="s">
         <v>1820</v>
@@ -18052,45 +18052,60 @@
         <v>374</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="22" t="n">
+    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="15" t="n">
         <v>46357</v>
       </c>
-      <c r="B44" s="23" t="s">
+      <c r="B44" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="C44" s="24" t="n">
+      <c r="C44" s="17" t="n">
         <v>11</v>
       </c>
-      <c r="D44" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="E44" s="26" t="s">
+      <c r="D44" s="18" t="s">
         <v>375</v>
       </c>
-      <c r="F44" s="23"/>
-      <c r="G44" s="23"/>
-      <c r="H44" s="23"/>
-      <c r="I44" s="23"/>
-      <c r="J44" s="23"/>
-      <c r="K44" s="23"/>
-      <c r="L44" s="23"/>
-      <c r="M44" s="23"/>
-      <c r="N44" s="23"/>
-      <c r="O44" s="23"/>
-      <c r="P44" s="23"/>
-      <c r="Q44" s="23"/>
-      <c r="R44" s="26"/>
-      <c r="S44" s="28"/>
-      <c r="T44" s="23"/>
-      <c r="U44" s="23"/>
-      <c r="V44" s="23"/>
-      <c r="W44" s="26"/>
-      <c r="X44" s="26"/>
-      <c r="Y44" s="23"/>
-      <c r="Z44" s="23"/>
-      <c r="AA44" s="23"/>
-      <c r="AB44" s="26"/>
+      <c r="E44" s="19" t="s">
+        <v>376</v>
+      </c>
+      <c r="F44" s="43" t="s">
+        <v>370</v>
+      </c>
+      <c r="G44" s="16"/>
+      <c r="H44" s="16"/>
+      <c r="I44" s="16"/>
+      <c r="J44" s="16"/>
+      <c r="K44" s="16"/>
+      <c r="L44" s="16"/>
+      <c r="M44" s="16"/>
+      <c r="N44" s="16"/>
+      <c r="O44" s="16"/>
+      <c r="P44" s="16"/>
+      <c r="Q44" s="20" t="str">
+        <f aca="false">HYPERLINK(Links!$M$44,"search")</f>
+        <v>search</v>
+      </c>
+      <c r="R44" s="19" t="s">
+        <v>377</v>
+      </c>
+      <c r="S44" s="21" t="n">
+        <v>46367</v>
+      </c>
+      <c r="T44" s="16"/>
+      <c r="U44" s="16"/>
+      <c r="V44" s="16"/>
+      <c r="W44" s="19" t="s">
+        <v>372</v>
+      </c>
+      <c r="X44" s="19" t="s">
+        <v>373</v>
+      </c>
+      <c r="Y44" s="16"/>
+      <c r="Z44" s="16"/>
+      <c r="AA44" s="16"/>
+      <c r="AB44" s="19" t="s">
+        <v>378</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="15" t="n">
@@ -18103,10 +18118,10 @@
         <v>11</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="E45" s="19" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="F45" s="43" t="s">
         <v>370</v>
@@ -18126,7 +18141,7 @@
         <v>search</v>
       </c>
       <c r="R45" s="19" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="S45" s="21" t="n">
         <v>46367</v>
@@ -18144,63 +18159,48 @@
       <c r="Z45" s="16"/>
       <c r="AA45" s="16"/>
       <c r="AB45" s="19" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="15" t="n">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="22" t="n">
         <v>46359</v>
       </c>
-      <c r="B46" s="16" t="s">
+      <c r="B46" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="C46" s="17" t="n">
+      <c r="C46" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="D46" s="18" t="s">
-        <v>380</v>
-      </c>
-      <c r="E46" s="19" t="s">
-        <v>381</v>
-      </c>
-      <c r="F46" s="43" t="s">
-        <v>370</v>
-      </c>
-      <c r="G46" s="16"/>
-      <c r="H46" s="16"/>
-      <c r="I46" s="16"/>
-      <c r="J46" s="16"/>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="16"/>
-      <c r="O46" s="16"/>
-      <c r="P46" s="16"/>
-      <c r="Q46" s="20" t="str">
-        <f aca="false">HYPERLINK(Links!$M$46,"search")</f>
-        <v>search</v>
-      </c>
-      <c r="R46" s="19" t="s">
-        <v>382</v>
-      </c>
-      <c r="S46" s="21" t="n">
-        <v>46367</v>
-      </c>
-      <c r="T46" s="16"/>
-      <c r="U46" s="16"/>
-      <c r="V46" s="16"/>
-      <c r="W46" s="19" t="s">
-        <v>372</v>
-      </c>
-      <c r="X46" s="19" t="s">
-        <v>373</v>
-      </c>
-      <c r="Y46" s="16"/>
-      <c r="Z46" s="16"/>
-      <c r="AA46" s="16"/>
-      <c r="AB46" s="19" t="s">
+      <c r="D46" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="E46" s="26" t="s">
         <v>383</v>
       </c>
+      <c r="F46" s="23"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="23"/>
+      <c r="K46" s="23"/>
+      <c r="L46" s="23"/>
+      <c r="M46" s="23"/>
+      <c r="N46" s="23"/>
+      <c r="O46" s="23"/>
+      <c r="P46" s="23"/>
+      <c r="Q46" s="23"/>
+      <c r="R46" s="26"/>
+      <c r="S46" s="28"/>
+      <c r="T46" s="23"/>
+      <c r="U46" s="23"/>
+      <c r="V46" s="23"/>
+      <c r="W46" s="26"/>
+      <c r="X46" s="26"/>
+      <c r="Y46" s="23"/>
+      <c r="Z46" s="23"/>
+      <c r="AA46" s="23"/>
+      <c r="AB46" s="26"/>
     </row>
     <row r="47" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="15" t="n">
@@ -22797,7 +22797,7 @@
       <c r="I15" s="49"/>
       <c r="J15" s="7" t="str">
         <f aca="true">IF(I15="✓","done",IF(TODAY()&lt;B15,"upcoming",IF(TODAY()&lt;G15,"open","due — check scores")))</f>
-        <v>open</v>
+        <v>due — check scores</v>
       </c>
       <c r="K15" s="50"/>
     </row>
@@ -22827,7 +22827,7 @@
       <c r="I16" s="49"/>
       <c r="J16" s="7" t="str">
         <f aca="true">IF(I16="✓","done",IF(TODAY()&lt;B16,"upcoming",IF(TODAY()&lt;G16,"open","due — check scores")))</f>
-        <v>open</v>
+        <v>due — check scores</v>
       </c>
       <c r="K16" s="50"/>
     </row>
@@ -22857,7 +22857,7 @@
       <c r="I17" s="49"/>
       <c r="J17" s="7" t="str">
         <f aca="true">IF(I17="✓","done",IF(TODAY()&lt;B17,"upcoming",IF(TODAY()&lt;G17,"open","due — check scores")))</f>
-        <v>open</v>
+        <v>due — check scores</v>
       </c>
       <c r="K17" s="50"/>
     </row>
@@ -22887,7 +22887,7 @@
       <c r="I18" s="49"/>
       <c r="J18" s="7" t="str">
         <f aca="true">IF(I18="✓","done",IF(TODAY()&lt;B18,"upcoming",IF(TODAY()&lt;G18,"open","due — check scores")))</f>
-        <v>open</v>
+        <v>due — check scores</v>
       </c>
       <c r="K18" s="50"/>
     </row>
@@ -22917,7 +22917,7 @@
       <c r="I19" s="49"/>
       <c r="J19" s="7" t="str">
         <f aca="true">IF(I19="✓","done",IF(TODAY()&lt;B19,"upcoming",IF(TODAY()&lt;G19,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>open</v>
       </c>
       <c r="K19" s="50"/>
     </row>
@@ -22947,7 +22947,7 @@
       <c r="I20" s="49"/>
       <c r="J20" s="7" t="str">
         <f aca="true">IF(I20="✓","done",IF(TODAY()&lt;B20,"upcoming",IF(TODAY()&lt;G20,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>open</v>
       </c>
       <c r="K20" s="50"/>
     </row>
@@ -22977,7 +22977,7 @@
       <c r="I21" s="49"/>
       <c r="J21" s="7" t="str">
         <f aca="true">IF(I21="✓","done",IF(TODAY()&lt;B21,"upcoming",IF(TODAY()&lt;G21,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>open</v>
       </c>
       <c r="K21" s="50"/>
     </row>
@@ -23007,7 +23007,7 @@
       <c r="I22" s="49"/>
       <c r="J22" s="7" t="str">
         <f aca="true">IF(I22="✓","done",IF(TODAY()&lt;B22,"upcoming",IF(TODAY()&lt;G22,"open","due — check scores")))</f>
-        <v>upcoming</v>
+        <v>open</v>
       </c>
       <c r="K22" s="50"/>
     </row>
@@ -23316,7 +23316,7 @@
         <v>29</v>
       </c>
       <c r="B33" s="47" t="n">
-        <v>46358</v>
+        <v>46357</v>
       </c>
       <c r="C33" s="48" t="s">
         <v>812</v>
@@ -23346,7 +23346,7 @@
         <v>30</v>
       </c>
       <c r="B34" s="47" t="n">
-        <v>46359</v>
+        <v>46358</v>
       </c>
       <c r="C34" s="48" t="s">
         <v>815</v>
@@ -24862,8 +24862,8 @@
     <hyperlink ref="C30" location="'Scope &amp; Sequence'!D40" display="T-B1 Thread B: angle pairs — supplementary, complementary, vertical, adjacent (16.1)"/>
     <hyperlink ref="C31" location="'Scope &amp; Sequence'!D41" display="T-B2 Thread B: interior and exterior angles of a triangle (16.2)"/>
     <hyperlink ref="C32" location="'Scope &amp; Sequence'!D43" display="11.01 Equations with like terms and the distributive property"/>
-    <hyperlink ref="C33" location="'Scope &amp; Sequence'!D45" display="11.02 Variables on both sides"/>
-    <hyperlink ref="C34" location="'Scope &amp; Sequence'!D46" display="11.03 One, none, infinitely many solutions"/>
+    <hyperlink ref="C33" location="'Scope &amp; Sequence'!D44" display="11.02 Variables on both sides"/>
+    <hyperlink ref="C34" location="'Scope &amp; Sequence'!D45" display="11.03 One, none, infinitely many solutions"/>
     <hyperlink ref="C35" location="'Scope &amp; Sequence'!D47" display="11.04 Multi-step equations"/>
     <hyperlink ref="C36" location="'Scope &amp; Sequence'!D48" display="11.05+06 Systems: which points are solutions; how many solutions"/>
     <hyperlink ref="C37" location="'Scope &amp; Sequence'!D50" display="11.07 Solving systems by graphing"/>
@@ -27389,7 +27389,7 @@
         <v>1266</v>
       </c>
       <c r="B19" s="47" t="n">
-        <v>46357</v>
+        <v>46359</v>
       </c>
       <c r="C19" s="47" t="n">
         <v>46364</v>
@@ -29379,13 +29379,13 @@
     </row>
     <row r="25" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="60"/>
-      <c r="B25" s="61" t="s">
+      <c r="B25" s="59" t="s">
         <v>1363</v>
       </c>
       <c r="C25" s="59" t="s">
         <v>1364</v>
       </c>
-      <c r="D25" s="59" t="s">
+      <c r="D25" s="61" t="s">
         <v>1365</v>
       </c>
       <c r="E25" s="59" t="s">

</xml_diff>